<commit_message>
Revert to hosted repo model + add HTS subset note in B1 sheet
- Revert delivery to salt0401-hosted repo with GitHub Release
- Restore download_latest.bat (curl from Release, auto-opens Excel)
- Remove setup.bat/update.bat (no longer needed)
- Add B1 sheet notes: HTS codes are a selected subset of official TRQ scope
- Simplify guide.html: Laura just downloads, no GitHub account needed

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/canada_trq_tracker.xlsx
+++ b/data/canada_trq_tracker.xlsx
@@ -2495,7 +2495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2526,35 +2526,49 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>B1 imports are matched at the 8-digit tariff item level using the HTS codes listed in the 'HTS code covered' sheet.</t>
+        </is>
+      </c>
+    </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>These HTS codes are a selected subset; the official TRQ product scope may include additional tariff items not tracked here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>Product Category</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>Total Tonnes</t>
         </is>
       </c>
-      <c r="D7" s="1" t="inlineStr">
+      <c r="D9" s="1" t="inlineStr">
         <is>
           <t>Total C$1000</t>
         </is>
       </c>
-      <c r="E7" s="1" t="inlineStr">
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>Avg C$/Tonne</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>B1 data not available for the matching calendar quarter.</t>
         </is>

</xml_diff>

<commit_message>
Weekly TRQ update 2026-03-30
</commit_message>
<xml_diff>
--- a/data/canada_trq_tracker.xlsx
+++ b/data/canada_trq_tracker.xlsx
@@ -9,8 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="non-FTA Q4" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FTA Q4" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B1 Imports" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HTS code covered" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HTS code covered" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B1 Imports" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2495,82 +2495,318 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>B1 Import Data - Calendar Quarter: April 1 to June 30, 2026</t>
+          <t>Hot-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Rebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>7208.10.00.00</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>7214.20.00.00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>NOTE: B1 data reflects actual customs entries using calendar quarters (Jan-Mar, Apr-Jun, etc.).</t>
+          <t>7208.25.00.00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TRQ utilization data uses offset quarters (Mar 26-Jun 26, etc.) and tracks permit issuance, not customs entries.</t>
+          <t>7208.26.00.00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>The two datasets have ~5-6 day boundary misalignment and measure different aspects of the import process.</t>
+          <t>7208.27.00.00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>7214.30.00.00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>B1 imports are matched at the 8-digit tariff item level using the HTS codes listed in the 'HTS code covered' sheet.</t>
+          <t>7208.36.00.00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>7214.91.00.00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>These HTS codes are a selected subset; the official TRQ product scope may include additional tariff items not tracked here.</t>
+          <t>7208.37.00.00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>7214.99.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>7208.38.00.00</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>Product Category</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
-        <is>
-          <t>Country</t>
-        </is>
-      </c>
-      <c r="C9" s="1" t="inlineStr">
-        <is>
-          <t>Total Tonnes</t>
-        </is>
-      </c>
-      <c r="D9" s="1" t="inlineStr">
-        <is>
-          <t>Total C$1000</t>
-        </is>
-      </c>
-      <c r="E9" s="1" t="inlineStr">
-        <is>
-          <t>Avg C$/Tonne</t>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>7208.39.00.00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>7213.10.00.00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>B1 data not available for the matching calendar quarter.</t>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>7213.20.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>7208.40.00.00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>7213.91.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>7208.51.00.00</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>7213.99.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>7208.52.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Cold-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>7216.10.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>7209.15.00.00</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>7216.21.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>7209.16.00.00</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>7216.22.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>7209.17.00.00</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>7216.31.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>7209.18.00.00</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>7216.32.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>7209.25.00.00</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>7216.33.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>7209.26.00.00</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>7216.40.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>7209.27.00.00</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>7216.50.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>7209.28.00.00</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>7216.69.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>7210.41.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>7210.49.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>7210.61.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>7210.69.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>7210.70.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>7210.90.00.00</t>
         </is>
       </c>
     </row>
@@ -2585,318 +2821,82 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Hot-Rolled Sheet</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Rebar</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>7208.10.00.00</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>7214.20.00.00</t>
+          <t>B1 Import Data - Calendar Quarter: April 1 to June 30, 2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>7208.25.00.00</t>
+          <t>NOTE: B1 data reflects actual customs entries using calendar quarters (Jan-Mar, Apr-Jun, etc.).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>7208.26.00.00</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Hot-Rolled Bar</t>
+          <t>TRQ utilization data uses offset quarters (Mar 26-Jun 26, etc.) and tracks permit issuance, not customs entries.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>7208.27.00.00</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>7214.30.00.00</t>
+          <t>The two datasets have ~5-6 day boundary misalignment and measure different aspects of the import process.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>7208.36.00.00</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>7214.91.00.00</t>
+          <t>B1 imports are matched at the 8-digit tariff item level using the HTS codes listed in the 'HTS code covered' sheet.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>7208.37.00.00</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>7214.99.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>7208.38.00.00</t>
+          <t>These HTS codes are a selected subset; the official TRQ product scope may include additional tariff items not tracked here.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>7208.39.00.00</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Wire Rod</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>7213.10.00.00</t>
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Product Category</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>Total Tonnes</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>Total C$1000</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>Avg C$/Tonne</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Steel Plate</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>7213.20.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>7208.40.00.00</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>7213.91.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>7208.51.00.00</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>7213.99.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>7208.52.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Structural Steel</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Cold-Rolled Sheet</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>7216.10.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>7209.15.00.00</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>7216.21.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>7209.16.00.00</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>7216.22.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>7209.17.00.00</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>7216.31.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>7209.18.00.00</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>7216.32.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>7209.25.00.00</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>7216.33.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>7209.26.00.00</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>7216.40.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>7209.27.00.00</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>7216.50.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>7209.28.00.00</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>7216.69.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Coated Steel Sheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>7210.41.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>7210.49.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>7210.61.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>7210.69.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>7210.70.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>7210.90.00.00</t>
+          <t>B1 data not available for the matching calendar quarter.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix 6 bugs found in code review
Critical:
- Fix insert_rows stale row ranges: shift all downstream products' row
  references after inserting a new country row
- Fix Part B b_idx not incremented when section missing, which
  desynchronized all remaining product matching

Important:
- Clear old OVER column values before writing new date data to prevent
  ghost "YES" strings persisting in the date column
- Add bounds check on Part A CSV field access to prevent IndexError
  on malformed/short rows
- Skip KGM mismatch validation when "Max Utilized" to avoid spurious
  warnings on fully-exhausted quotas
- Add month range validation (1-12) for B1 6-cell row parser

Minor:
- Fix workflow release body: remove empty template variable
- Fix guide.html: "~8:00 AM ET" to account for DST variation

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/canada_trq_tracker.xlsx
+++ b/data/canada_trq_tracker.xlsx
@@ -9,8 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="non-FTA Q4" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FTA Q4" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HTS code covered" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B1 Imports" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B1 Imports" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HTS code covered" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2495,318 +2495,82 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Hot-Rolled Sheet</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Rebar</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>7208.10.00.00</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>7214.20.00.00</t>
+          <t>B1 Import Data - Calendar Quarter: April 1 to June 30, 2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>7208.25.00.00</t>
+          <t>NOTE: B1 data reflects actual customs entries using calendar quarters (Jan-Mar, Apr-Jun, etc.).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>7208.26.00.00</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Hot-Rolled Bar</t>
+          <t>TRQ utilization data uses offset quarters (Mar 26-Jun 26, etc.) and tracks permit issuance, not customs entries.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>7208.27.00.00</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>7214.30.00.00</t>
+          <t>The two datasets have ~5-6 day boundary misalignment and measure different aspects of the import process.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>7208.36.00.00</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>7214.91.00.00</t>
+          <t>B1 imports are matched at the 8-digit tariff item level using the HTS codes listed in the 'HTS code covered' sheet.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>7208.37.00.00</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>7214.99.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>7208.38.00.00</t>
+          <t>These HTS codes are a selected subset; the official TRQ product scope may include additional tariff items not tracked here.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>7208.39.00.00</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Wire Rod</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>7213.10.00.00</t>
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Product Category</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>Total Tonnes</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>Total C$1000</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>Avg C$/Tonne</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Steel Plate</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>7213.20.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>7208.40.00.00</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>7213.91.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>7208.51.00.00</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>7213.99.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>7208.52.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Structural Steel</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Cold-Rolled Sheet</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>7216.10.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>7209.15.00.00</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>7216.21.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>7209.16.00.00</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>7216.22.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>7209.17.00.00</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>7216.31.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>7209.18.00.00</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>7216.32.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>7209.25.00.00</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>7216.33.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>7209.26.00.00</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>7216.40.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>7209.27.00.00</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>7216.50.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>7209.28.00.00</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>7216.69.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Coated Steel Sheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>7210.41.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>7210.49.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>7210.61.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>7210.69.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>7210.70.00.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>7210.90.00.00</t>
+          <t>B1 data not available for the matching calendar quarter.</t>
         </is>
       </c>
     </row>
@@ -2821,82 +2585,318 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>B1 Import Data - Calendar Quarter: April 1 to June 30, 2026</t>
+          <t>Hot-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Rebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>7208.10.00.00</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>7214.20.00.00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>NOTE: B1 data reflects actual customs entries using calendar quarters (Jan-Mar, Apr-Jun, etc.).</t>
+          <t>7208.25.00.00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TRQ utilization data uses offset quarters (Mar 26-Jun 26, etc.) and tracks permit issuance, not customs entries.</t>
+          <t>7208.26.00.00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>The two datasets have ~5-6 day boundary misalignment and measure different aspects of the import process.</t>
+          <t>7208.27.00.00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>7214.30.00.00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>B1 imports are matched at the 8-digit tariff item level using the HTS codes listed in the 'HTS code covered' sheet.</t>
+          <t>7208.36.00.00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>7214.91.00.00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>These HTS codes are a selected subset; the official TRQ product scope may include additional tariff items not tracked here.</t>
+          <t>7208.37.00.00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>7214.99.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>7208.38.00.00</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>Product Category</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
-        <is>
-          <t>Country</t>
-        </is>
-      </c>
-      <c r="C9" s="1" t="inlineStr">
-        <is>
-          <t>Total Tonnes</t>
-        </is>
-      </c>
-      <c r="D9" s="1" t="inlineStr">
-        <is>
-          <t>Total C$1000</t>
-        </is>
-      </c>
-      <c r="E9" s="1" t="inlineStr">
-        <is>
-          <t>Avg C$/Tonne</t>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>7208.39.00.00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>7213.10.00.00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>B1 data not available for the matching calendar quarter.</t>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>7213.20.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>7208.40.00.00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>7213.91.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>7208.51.00.00</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>7213.99.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>7208.52.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Cold-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>7216.10.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>7209.15.00.00</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>7216.21.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>7209.16.00.00</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>7216.22.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>7209.17.00.00</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>7216.31.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>7209.18.00.00</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>7216.32.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>7209.25.00.00</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>7216.33.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>7209.26.00.00</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>7216.40.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>7209.27.00.00</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>7216.50.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>7209.28.00.00</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>7216.69.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>7210.41.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>7210.49.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>7210.61.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>7210.69.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>7210.70.00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>7210.90.00.00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Weekly TRQ update 2026-04-06
</commit_message>
<xml_diff>
--- a/data/canada_trq_tracker.xlsx
+++ b/data/canada_trq_tracker.xlsx
@@ -60,13 +60,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,6 +466,11 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>April 6 2026</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
           <t>OVER</t>
         </is>
       </c>
@@ -489,6 +495,9 @@
       <c r="E3" s="4" t="n">
         <v>0.0005</v>
       </c>
+      <c r="F3" s="4" t="n">
+        <v>0.0033</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -510,6 +519,9 @@
       <c r="E4" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="F4" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -531,7 +543,10 @@
       <c r="E5" s="4" t="n">
         <v>0.41</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="4" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -552,6 +567,10 @@
         <f>SUM(E3:E5)</f>
         <v/>
       </c>
+      <c r="F6" s="5">
+        <f>SUM(F3:F5)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -573,6 +592,9 @@
       <c r="E7" s="4" t="n">
         <v>0.3337</v>
       </c>
+      <c r="F7" s="4" t="n">
+        <v>0.3402000000000001</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -592,6 +614,9 @@
         <v>0.36</v>
       </c>
       <c r="E8" s="4" t="n">
+        <v>0.0172</v>
+      </c>
+      <c r="F8" s="4" t="n">
         <v>0.0172</v>
       </c>
     </row>
@@ -610,6 +635,10 @@
         <f>SUM(E7:E8)</f>
         <v/>
       </c>
+      <c r="F9" s="5">
+        <f>SUM(F7:F8)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -631,6 +660,9 @@
       <c r="E10" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="F10" s="4" t="n">
+        <v>0.0008</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -652,6 +684,9 @@
       <c r="E11" s="4" t="n">
         <v>0.0023</v>
       </c>
+      <c r="F11" s="4" t="n">
+        <v>0.0023</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -673,6 +708,9 @@
       <c r="E12" s="4" t="n">
         <v>0.0421</v>
       </c>
+      <c r="F12" s="4" t="n">
+        <v>0.0421</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -692,6 +730,9 @@
         <v>0.92</v>
       </c>
       <c r="E13" s="4" t="n">
+        <v>0.0911</v>
+      </c>
+      <c r="F13" s="4" t="n">
         <v>0.0911</v>
       </c>
     </row>
@@ -710,6 +751,10 @@
         <f>SUM(E10:E13)</f>
         <v/>
       </c>
+      <c r="F14" s="5">
+        <f>SUM(F10:F13)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -731,6 +776,9 @@
       <c r="E15" s="4" t="n">
         <v>0.0021</v>
       </c>
+      <c r="F15" s="4" t="n">
+        <v>0.0025</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -752,6 +800,9 @@
       <c r="E16" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="F16" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -773,6 +824,9 @@
       <c r="E17" s="4" t="n">
         <v>0.011</v>
       </c>
+      <c r="F17" s="4" t="n">
+        <v>0.0135</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -794,6 +848,9 @@
       <c r="E18" s="4" t="n">
         <v>0.0024</v>
       </c>
+      <c r="F18" s="4" t="n">
+        <v>0.0024</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -815,6 +872,9 @@
       <c r="E19" s="4" t="n">
         <v>0.2787</v>
       </c>
+      <c r="F19" s="4" t="n">
+        <v>0.2962</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -836,6 +896,9 @@
       <c r="E20" s="4" t="n">
         <v>0.0086</v>
       </c>
+      <c r="F20" s="4" t="n">
+        <v>0.0086</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -857,6 +920,9 @@
       <c r="E21" s="4" t="n">
         <v>0.0308</v>
       </c>
+      <c r="F21" s="4" t="n">
+        <v>0.0308</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -876,6 +942,9 @@
         <v>0.37</v>
       </c>
       <c r="E22" s="4" t="n">
+        <v>0.0387</v>
+      </c>
+      <c r="F22" s="4" t="n">
         <v>0.0387</v>
       </c>
     </row>
@@ -894,6 +963,10 @@
         <f>SUM(E15:E22)</f>
         <v/>
       </c>
+      <c r="F23" s="5">
+        <f>SUM(F15:F22)</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -915,7 +988,10 @@
       <c r="E24" s="4" t="n">
         <v>0.29</v>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F24" s="4" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="G24" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -941,6 +1017,9 @@
       <c r="E25" s="4" t="n">
         <v>0.1227</v>
       </c>
+      <c r="F25" s="4" t="n">
+        <v>0.1228</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -962,6 +1041,9 @@
       <c r="E26" s="4" t="n">
         <v>0.2394</v>
       </c>
+      <c r="F26" s="4" t="n">
+        <v>0.2394</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -983,6 +1065,9 @@
       <c r="E27" s="4" t="n">
         <v>0.1668</v>
       </c>
+      <c r="F27" s="4" t="n">
+        <v>0.1668</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1004,6 +1089,9 @@
       <c r="E28" s="4" t="n">
         <v>0.0241</v>
       </c>
+      <c r="F28" s="4" t="n">
+        <v>0.0241</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1023,6 +1111,9 @@
         <v>0.29</v>
       </c>
       <c r="E29" s="4" t="n">
+        <v>0.1569</v>
+      </c>
+      <c r="F29" s="4" t="n">
         <v>0.1569</v>
       </c>
     </row>
@@ -1041,6 +1132,10 @@
         <f>SUM(E24:E29)</f>
         <v/>
       </c>
+      <c r="F30" s="5">
+        <f>SUM(F24:F29)</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1062,6 +1157,9 @@
       <c r="E31" s="4" t="n">
         <v>0.0005999999999999999</v>
       </c>
+      <c r="F31" s="4" t="n">
+        <v>0.0021</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1083,6 +1181,9 @@
       <c r="E32" s="4" t="n">
         <v>0.08259999999999999</v>
       </c>
+      <c r="F32" s="4" t="n">
+        <v>0.1359</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1104,6 +1205,9 @@
       <c r="E33" s="4" t="n">
         <v>0.1397</v>
       </c>
+      <c r="F33" s="4" t="n">
+        <v>0.1475</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1124,6 +1228,9 @@
       </c>
       <c r="E34" s="4" t="n">
         <v>0.1438</v>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>0.1892</v>
       </c>
     </row>
     <row r="35">
@@ -1141,6 +1248,10 @@
         <f>SUM(E31:E34)</f>
         <v/>
       </c>
+      <c r="F35" s="5">
+        <f>SUM(F31:F34)</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1160,6 +1271,9 @@
         <v>0.45</v>
       </c>
       <c r="E36" s="4" t="n">
+        <v>0.1514</v>
+      </c>
+      <c r="F36" s="4" t="n">
         <v>0.1514</v>
       </c>
     </row>
@@ -1178,6 +1292,10 @@
         <f>SUM(E36:E36)</f>
         <v/>
       </c>
+      <c r="F37" s="5">
+        <f>SUM(F36:F36)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1199,6 +1317,9 @@
       <c r="E38" s="4" t="n">
         <v>0.0359</v>
       </c>
+      <c r="F38" s="4" t="n">
+        <v>0.0408</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1220,6 +1341,9 @@
       <c r="E39" s="4" t="n">
         <v>0.0177</v>
       </c>
+      <c r="F39" s="4" t="n">
+        <v>0.0236</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1241,6 +1365,9 @@
       <c r="E40" s="4" t="n">
         <v>0.2154</v>
       </c>
+      <c r="F40" s="4" t="n">
+        <v>0.2154</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1262,6 +1389,9 @@
       <c r="E41" s="4" t="n">
         <v>0.5329999999999999</v>
       </c>
+      <c r="F41" s="4" t="n">
+        <v>0.5436</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1276,6 +1406,10 @@
       </c>
       <c r="E42" s="5">
         <f>SUM(E38:E41)</f>
+        <v/>
+      </c>
+      <c r="F42" s="5">
+        <f>SUM(F38:F41)</f>
         <v/>
       </c>
     </row>
@@ -1290,7 +1424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1323,6 +1457,11 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>April 6 2026</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
           <t>OVER</t>
         </is>
       </c>
@@ -1347,6 +1486,9 @@
       <c r="E3" s="4" t="n">
         <v>0.001</v>
       </c>
+      <c r="F3" s="4" t="n">
+        <v>0.0015</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1368,6 +1510,9 @@
       <c r="E4" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="F4" s="4" t="n">
+        <v>0.0002</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1389,6 +1534,9 @@
       <c r="E5" s="4" t="n">
         <v>0.0268</v>
       </c>
+      <c r="F5" s="4" t="n">
+        <v>0.0435</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1410,6 +1558,9 @@
       <c r="E6" s="4" t="n">
         <v>0.0306</v>
       </c>
+      <c r="F6" s="4" t="n">
+        <v>0.0306</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1431,6 +1582,9 @@
       <c r="E7" s="4" t="n">
         <v>0.0446</v>
       </c>
+      <c r="F7" s="4" t="n">
+        <v>0.0446</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1452,6 +1606,9 @@
       <c r="E8" s="4" t="n">
         <v>0.0002</v>
       </c>
+      <c r="F8" s="4" t="n">
+        <v>0.0002</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1473,6 +1630,9 @@
       <c r="E9" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="F9" s="4" t="n">
+        <v>0.0011</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1515,6 +1675,9 @@
       <c r="E11" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="F11" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1524,54 +1687,58 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>9523100</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>0.0012</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>9523100</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>0.0003</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E12" s="5">
+      <c r="E14" s="5">
         <f>SUM(E3:E11)</f>
         <v/>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Steel Plate</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="n">
-        <v>54354900</v>
-      </c>
-      <c r="D13" s="4" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="E13" s="4" t="n">
-        <v>0.0016</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Steel Plate</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Finland</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="n">
-        <v>54354900</v>
-      </c>
-      <c r="D14" s="4" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="E14" s="4" t="n">
-        <v>0.008500000000000001</v>
+      <c r="F14" s="5">
+        <f>SUM(F3:F13)</f>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -1582,7 +1749,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
@@ -1592,7 +1759,10 @@
         <v>0.3</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.0016</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>0.0025</v>
       </c>
     </row>
     <row r="16">
@@ -1603,7 +1773,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
@@ -1613,7 +1783,10 @@
         <v>0.3</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0.0033</v>
+        <v>0.008500000000000001</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>0.0141</v>
       </c>
     </row>
     <row r="17">
@@ -1624,7 +1797,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
@@ -1634,7 +1807,10 @@
         <v>0.3</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>0</v>
+        <v>0.0012</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>0.0012</v>
       </c>
     </row>
     <row r="18">
@@ -1645,7 +1821,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
@@ -1655,7 +1831,10 @@
         <v>0.3</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>0.2889</v>
+        <v>0.0033</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>0.008199999999999999</v>
       </c>
     </row>
     <row r="19">
@@ -1666,7 +1845,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
@@ -1676,7 +1855,10 @@
         <v>0.3</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>0.0892</v>
+        <v>0</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>0.0083</v>
       </c>
     </row>
     <row r="20">
@@ -1687,7 +1869,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
@@ -1697,7 +1879,15 @@
         <v>0.3</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.2889</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -1708,7 +1898,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
@@ -1718,7 +1908,10 @@
         <v>0.3</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>0.0008</v>
+        <v>0.0892</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>0.0892</v>
       </c>
     </row>
     <row r="22">
@@ -1729,175 +1922,192 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>54354900</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>0.0004</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>0.0004</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>54354900</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>0.0128</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>54354900</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>54354900</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>0.0011</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Slovenia</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>54354900</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>0.0001</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E22" s="5">
+      <c r="E27" s="5">
         <f>SUM(E13:E21)</f>
         <v/>
       </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="F27" s="5">
+        <f>SUM(F15:F26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>Cold-Rolled Sheet</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>Sweden</t>
         </is>
       </c>
-      <c r="C23" s="3" t="n">
+      <c r="C28" s="3" t="n">
         <v>1832600</v>
       </c>
-      <c r="D23" s="4" t="n">
+      <c r="D28" s="4" t="n">
         <v>0.32</v>
       </c>
-      <c r="E23" s="4" t="n">
+      <c r="E28" s="4" t="n">
         <v>0.0867</v>
       </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="F28" s="4" t="n">
+        <v>0.0964</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>Cold-Rolled Sheet</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>1832600</v>
+      </c>
+      <c r="D29" s="4" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>0.0795</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Cold-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E24" s="5">
+      <c r="E30" s="5">
         <f>SUM(E23:E23)</f>
         <v/>
       </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Coated Steel Sheet</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Australia</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="n">
-        <v>31128200</v>
-      </c>
-      <c r="D25" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E25" s="4" t="n">
-        <v>0.0003</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Coated Steel Sheet</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Belgium</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="n">
-        <v>31128200</v>
-      </c>
-      <c r="D26" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E26" s="4" t="n">
-        <v>0.0541</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Coated Steel Sheet</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="n">
-        <v>31128200</v>
-      </c>
-      <c r="D27" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E27" s="4" t="n">
-        <v>0.005</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Coated Steel Sheet</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Korea, Republic of</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="n">
-        <v>31128200</v>
-      </c>
-      <c r="D28" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E28" s="4" t="n">
-        <v>0.04019999999999999</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Coated Steel Sheet</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Netherlands</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="n">
-        <v>31128200</v>
-      </c>
-      <c r="D29" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E29" s="4" t="n">
-        <v>0.0251</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Coated Steel Sheet</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Spain</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="n">
-        <v>31128200</v>
-      </c>
-      <c r="D30" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E30" s="4" t="n">
-        <v>0.0007000000000000001</v>
+      <c r="F30" s="5">
+        <f>SUM(F28:F29)</f>
+        <v/>
       </c>
     </row>
     <row r="31">
@@ -1908,7 +2118,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C31" s="3" t="n">
@@ -1918,7 +2128,10 @@
         <v>0.25</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>0.0026</v>
+        <v>0.0003</v>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>0.0003</v>
       </c>
     </row>
     <row r="32">
@@ -1929,322 +2142,363 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>31128200</v>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>0.0541</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>0.0562</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>31128200</v>
+      </c>
+      <c r="D33" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>0.0341</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Korea, Republic of</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="n">
+        <v>31128200</v>
+      </c>
+      <c r="D34" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>0.04019999999999999</v>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>0.0435</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="n">
+        <v>31128200</v>
+      </c>
+      <c r="D35" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>0.0251</v>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>0.0251</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>31128200</v>
+      </c>
+      <c r="D36" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>31128200</v>
+      </c>
+      <c r="D37" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>0.0026</v>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>0.0265</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="n">
+        <v>31128200</v>
+      </c>
+      <c r="D38" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>0.0005</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="n">
+        <v>31128200</v>
+      </c>
+      <c r="D39" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F39" s="4" t="n">
+        <v>0.0064</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="n">
+        <v>31128200</v>
+      </c>
+      <c r="D40" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F40" s="4" t="n">
+        <v>0.0101</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E32" s="5">
+      <c r="E41" s="5">
         <f>SUM(E25:E31)</f>
         <v/>
       </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="F41" s="5">
+        <f>SUM(F31:F40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
         <is>
           <t>Rebar</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="C33" s="3" t="n">
+      <c r="C42" s="3" t="n">
         <v>28710400</v>
       </c>
-      <c r="D33" s="4" t="n">
+      <c r="D42" s="4" t="n">
         <v>0.45</v>
       </c>
-      <c r="E33" s="4" t="n">
+      <c r="E42" s="4" t="n">
         <v>0.1642</v>
       </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="F42" s="4" t="n">
+        <v>0.1642</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
         <is>
           <t>Rebar</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>Greece</t>
         </is>
       </c>
-      <c r="C34" s="3" t="n">
+      <c r="C43" s="3" t="n">
         <v>28710400</v>
       </c>
-      <c r="D34" s="4" t="n">
+      <c r="D43" s="4" t="n">
         <v>0.45</v>
       </c>
-      <c r="E34" s="4" t="n">
+      <c r="E43" s="4" t="n">
         <v>0.3234</v>
       </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="F43" s="4" t="n">
+        <v>0.3234</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t>Rebar</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>Netherlands</t>
         </is>
       </c>
-      <c r="C35" s="3" t="n">
+      <c r="C44" s="3" t="n">
         <v>28710400</v>
       </c>
-      <c r="D35" s="4" t="n">
+      <c r="D44" s="4" t="n">
         <v>0.45</v>
       </c>
-      <c r="E35" s="4" t="n">
+      <c r="E44" s="4" t="n">
         <v>0.0028</v>
       </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="F44" s="4" t="n">
+        <v>0.0028</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
         <is>
           <t>Rebar</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>Peru</t>
         </is>
       </c>
-      <c r="C36" s="3" t="n">
+      <c r="C45" s="3" t="n">
         <v>28710400</v>
       </c>
-      <c r="D36" s="4" t="n">
+      <c r="D45" s="4" t="n">
         <v>0.45</v>
       </c>
-      <c r="E36" s="4" t="n">
+      <c r="E45" s="4" t="n">
         <v>0.1633</v>
       </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="F45" s="4" t="n">
+        <v>0.1633</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t>Rebar</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
-      <c r="C37" s="3" t="n">
+      <c r="C46" s="3" t="n">
         <v>28710400</v>
       </c>
-      <c r="D37" s="4" t="n">
+      <c r="D46" s="4" t="n">
         <v>0.45</v>
       </c>
-      <c r="E37" s="4" t="n">
+      <c r="E46" s="4" t="n">
         <v>0.3462</v>
       </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="F46" s="4" t="n">
+        <v>0.3462</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
         <is>
           <t>Rebar</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E38" s="5">
+      <c r="E47" s="5">
         <f>SUM(E33:E37)</f>
         <v/>
       </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Hot-Rolled Bar</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Czech Republic</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="n">
-        <v>8750300</v>
-      </c>
-      <c r="D39" s="4" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="E39" s="4" t="n">
-        <v>0.0001</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Hot-Rolled Bar</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Denmark</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="n">
-        <v>8750300</v>
-      </c>
-      <c r="D40" s="4" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="E40" s="4" t="n">
-        <v>0.0022</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Hot-Rolled Bar</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="n">
-        <v>8750300</v>
-      </c>
-      <c r="D41" s="4" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="E41" s="4" t="n">
-        <v>0.0017</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Hot-Rolled Bar</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="n">
-        <v>8750300</v>
-      </c>
-      <c r="D42" s="4" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="E42" s="4" t="n">
-        <v>0.0307</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Hot-Rolled Bar</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="n">
-        <v>8750300</v>
-      </c>
-      <c r="D43" s="4" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="E43" s="4" t="n">
-        <v>0.001</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Hot-Rolled Bar</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Korea, Republic of</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="n">
-        <v>8750300</v>
-      </c>
-      <c r="D44" s="4" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="E44" s="4" t="n">
-        <v>0.07519999999999999</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Hot-Rolled Bar</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Slovenia</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="n">
-        <v>8750300</v>
-      </c>
-      <c r="D45" s="4" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="E45" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Hot-Rolled Bar</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Spain</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="n">
-        <v>8750300</v>
-      </c>
-      <c r="D46" s="4" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="E46" s="4" t="n">
-        <v>0.009899999999999999</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Hot-Rolled Bar</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Sweden</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="n">
-        <v>8750300</v>
-      </c>
-      <c r="D47" s="4" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="E47" s="4" t="n">
-        <v>0</v>
+      <c r="F47" s="5">
+        <f>SUM(F33:F37)</f>
+        <v/>
       </c>
     </row>
     <row r="48">
@@ -2255,232 +2509,592 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
+          <t>Czech Republic</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="n">
+        <v>8750300</v>
+      </c>
+      <c r="D48" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="E48" s="4" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="F48" s="4" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="n">
+        <v>8750300</v>
+      </c>
+      <c r="D49" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="E49" s="4" t="n">
+        <v>0.0022</v>
+      </c>
+      <c r="F49" s="4" t="n">
+        <v>0.0022</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="n">
+        <v>8750300</v>
+      </c>
+      <c r="D50" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="E50" s="4" t="n">
+        <v>0.0017</v>
+      </c>
+      <c r="F50" s="4" t="n">
+        <v>0.0017</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="n">
+        <v>8750300</v>
+      </c>
+      <c r="D51" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="E51" s="4" t="n">
+        <v>0.0307</v>
+      </c>
+      <c r="F51" s="4" t="n">
+        <v>0.0633</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="n">
+        <v>8750300</v>
+      </c>
+      <c r="D52" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="E52" s="4" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="F52" s="4" t="n">
+        <v>0.0021</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Korea, Republic of</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="n">
+        <v>8750300</v>
+      </c>
+      <c r="D53" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="E53" s="4" t="n">
+        <v>0.07519999999999999</v>
+      </c>
+      <c r="F53" s="4" t="n">
+        <v>0.127</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Slovenia</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="n">
+        <v>8750300</v>
+      </c>
+      <c r="D54" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="E54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="n">
+        <v>8750300</v>
+      </c>
+      <c r="D55" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="E55" s="4" t="n">
+        <v>0.009899999999999999</v>
+      </c>
+      <c r="F55" s="4" t="n">
+        <v>0.0876</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="n">
+        <v>8750300</v>
+      </c>
+      <c r="D56" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="E56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="n">
+        <v>8750300</v>
+      </c>
+      <c r="D57" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F57" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Romania</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="n">
+        <v>8750300</v>
+      </c>
+      <c r="D58" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F58" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E48" s="5">
+      <c r="E59" s="5">
         <f>SUM(E39:E47)</f>
         <v/>
       </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="F59" s="5">
+        <f>SUM(F48:F58)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
         <is>
           <t>Wire Rod</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B60" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="C49" s="3" t="n">
+      <c r="C60" s="3" t="n">
         <v>16514800</v>
       </c>
-      <c r="D49" s="4" t="n">
+      <c r="D60" s="4" t="n">
         <v>0.59</v>
       </c>
-      <c r="E49" s="4" t="n">
+      <c r="E60" s="4" t="n">
         <v>0.0011</v>
       </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="F60" s="4" t="n">
+        <v>0.0751</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
         <is>
           <t>Wire Rod</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t>Korea, Republic of</t>
         </is>
       </c>
-      <c r="C50" s="3" t="n">
+      <c r="C61" s="3" t="n">
         <v>16514800</v>
       </c>
-      <c r="D50" s="4" t="n">
+      <c r="D61" s="4" t="n">
         <v>0.59</v>
       </c>
-      <c r="E50" s="4" t="n">
+      <c r="E61" s="4" t="n">
         <v>0.0122</v>
       </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="F61" s="4" t="n">
+        <v>0.0122</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
         <is>
           <t>Wire Rod</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B62" t="inlineStr">
         <is>
           <t>Netherlands</t>
         </is>
       </c>
-      <c r="C51" s="3" t="n">
+      <c r="C62" s="3" t="n">
         <v>16514800</v>
       </c>
-      <c r="D51" s="4" t="n">
+      <c r="D62" s="4" t="n">
         <v>0.59</v>
       </c>
-      <c r="E51" s="4" t="n">
+      <c r="E62" s="4" t="n">
         <v>0.008800000000000001</v>
       </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="F62" s="4" t="n">
+        <v>0.0176</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
         <is>
           <t>Wire Rod</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="n">
+        <v>16514800</v>
+      </c>
+      <c r="D63" s="4" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="F63" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E52" s="5">
+      <c r="E64" s="5">
         <f>SUM(E49:E51)</f>
         <v/>
       </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="F64" s="5">
+        <f>SUM(F60:F63)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
         <is>
           <t>Structural Steel</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B65" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="C53" s="3" t="n">
+      <c r="C65" s="3" t="n">
         <v>3467600</v>
       </c>
-      <c r="D53" s="4" t="n">
+      <c r="D65" s="4" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="E53" s="4" t="n">
+      <c r="E65" s="4" t="n">
         <v>0.0001</v>
       </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="F65" s="4" t="n">
+        <v>0.0001</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
         <is>
           <t>Structural Steel</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B66" t="inlineStr">
         <is>
           <t>Italy</t>
         </is>
       </c>
-      <c r="C54" s="3" t="n">
+      <c r="C66" s="3" t="n">
         <v>3467600</v>
       </c>
-      <c r="D54" s="4" t="n">
+      <c r="D66" s="4" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="E54" s="4" t="n">
+      <c r="E66" s="4" t="n">
         <v>0.0011</v>
       </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="F66" s="4" t="n">
+        <v>0.0073</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
         <is>
           <t>Structural Steel</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B67" t="inlineStr">
         <is>
           <t>Poland</t>
         </is>
       </c>
-      <c r="C55" s="3" t="n">
+      <c r="C67" s="3" t="n">
         <v>3467600</v>
       </c>
-      <c r="D55" s="4" t="n">
+      <c r="D67" s="4" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="E55" s="4" t="n">
+      <c r="E67" s="4" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="F67" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
         <is>
           <t>Structural Steel</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B68" t="inlineStr">
         <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="C56" s="3" t="n">
+      <c r="C68" s="3" t="n">
         <v>3467600</v>
       </c>
-      <c r="D56" s="4" t="n">
+      <c r="D68" s="4" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="E56" s="4" t="n">
+      <c r="E68" s="4" t="n">
         <v>0.0191</v>
       </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="F68" s="4" t="n">
+        <v>0.0191</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
         <is>
           <t>Structural Steel</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B69" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="C57" s="3" t="n">
+      <c r="C69" s="3" t="n">
         <v>3467600</v>
       </c>
-      <c r="D57" s="4" t="n">
+      <c r="D69" s="4" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="E57" s="4" t="n">
+      <c r="E69" s="4" t="n">
         <v>0.007900000000000001</v>
       </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="F69" s="4" t="n">
+        <v>0.007900000000000001</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
         <is>
           <t>Structural Steel</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B70" t="inlineStr">
         <is>
           <t>Vietnam</t>
         </is>
       </c>
-      <c r="C58" s="3" t="n">
+      <c r="C70" s="3" t="n">
         <v>3467600</v>
       </c>
-      <c r="D58" s="4" t="n">
+      <c r="D70" s="4" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="E58" s="4" t="n">
+      <c r="E70" s="4" t="n">
         <v>0.3604</v>
       </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="F70" s="4" t="n">
+        <v>0.3604</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
         <is>
           <t>Structural Steel</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Korea, Republic of</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D71" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="F71" s="4" t="n">
+        <v>0.0421</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D72" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="F72" s="4" t="n">
+        <v>0.0001</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E59" s="5">
+      <c r="E73" s="5">
         <f>SUM(E53:E58)</f>
+        <v/>
+      </c>
+      <c r="F73" s="5">
+        <f>SUM(F65:F72)</f>
         <v/>
       </c>
     </row>
@@ -2821,7 +3435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2893,11 +3507,2566 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>10.93</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>397.9871912168344</v>
+      </c>
+    </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>B1 data not available for the matching calendar quarter.</t>
-        </is>
+          <t>Hot-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>102.11</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>171.34</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>1677.994319851141</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>343.02</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>272.3</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>793.8312634831789</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Korea, Republic of</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>1756.41</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>1337.35</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>761.4110600600089</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>32.75</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>1760.752688172043</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>71.09999999999999</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>97.78999999999999</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>1375.386779184247</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>24736.99000000001</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>37963.62</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>1534.69035642574</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>633.1</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>657.24</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>1038.129837308482</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>346.21</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>664.45</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>1919.210883567777</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>2814.44</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>2707.8</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>962.1096914483874</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>2119.047619047619</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>2051.31</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>6915.08</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>3371.055569367867</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>3007.1</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>3666.78</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>1219.374147850088</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>141.02</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>333.88</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>2367.60743156999</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>4.140000000000001</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>2379.310344827587</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>9.879999999999999</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>2115.384615384616</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Korea, Republic of</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>11695.79</v>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>13727.43</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>1173.70694925268</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Malaysia</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>1160.84</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>1173.79</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <v>1011.155714827194</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>614.54</v>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>1255.25</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>2042.584697497315</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>22.77</v>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="E30" s="6" t="n">
+        <v>2828.282828282829</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>23.49</v>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>89.52</v>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v>3810.983397190294</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>725.13</v>
+      </c>
+      <c r="D32" s="6" t="n">
+        <v>670.12</v>
+      </c>
+      <c r="E32" s="6" t="n">
+        <v>924.1377408188877</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="n">
+        <v>27.77</v>
+      </c>
+      <c r="D33" s="6" t="n">
+        <v>6.82</v>
+      </c>
+      <c r="E33" s="6" t="n">
+        <v>245.5887648541592</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="n">
+        <v>5.83</v>
+      </c>
+      <c r="D34" s="6" t="n">
+        <v>28.01</v>
+      </c>
+      <c r="E34" s="6" t="n">
+        <v>4804.459691252144</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="n">
+        <v>16955.68</v>
+      </c>
+      <c r="D35" s="6" t="n">
+        <v>30083.11999999999</v>
+      </c>
+      <c r="E35" s="6" t="n">
+        <v>1774.220792088551</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Cold-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="D36" s="6" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="E36" s="6" t="n">
+        <v>4416.666666666667</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Cold-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="n">
+        <v>30.99</v>
+      </c>
+      <c r="D37" s="6" t="n">
+        <v>61.46999999999999</v>
+      </c>
+      <c r="E37" s="6" t="n">
+        <v>1983.543078412391</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Cold-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="n">
+        <v>34.08</v>
+      </c>
+      <c r="D38" s="6" t="n">
+        <v>83.56000000000002</v>
+      </c>
+      <c r="E38" s="6" t="n">
+        <v>2451.877934272301</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Cold-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Korea, Republic of</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D39" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Cold-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="n">
+        <v>6.26</v>
+      </c>
+      <c r="D40" s="6" t="n">
+        <v>26.97</v>
+      </c>
+      <c r="E40" s="6" t="n">
+        <v>4308.306709265175</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Cold-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Pakistan</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="n">
+        <v>227.27</v>
+      </c>
+      <c r="D41" s="6" t="n">
+        <v>274.06</v>
+      </c>
+      <c r="E41" s="6" t="n">
+        <v>1205.878470541646</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Cold-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="n">
+        <v>631.48</v>
+      </c>
+      <c r="D42" s="6" t="n">
+        <v>1015.23</v>
+      </c>
+      <c r="E42" s="6" t="n">
+        <v>1607.699372901754</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Cold-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="n">
+        <v>240.83</v>
+      </c>
+      <c r="D43" s="6" t="n">
+        <v>407.72</v>
+      </c>
+      <c r="E43" s="6" t="n">
+        <v>1692.978449528713</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Cold-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="n">
+        <v>682.4400000000001</v>
+      </c>
+      <c r="D44" s="6" t="n">
+        <v>782.05</v>
+      </c>
+      <c r="E44" s="6" t="n">
+        <v>1145.96154973331</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Cold-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="n">
+        <v>61.92</v>
+      </c>
+      <c r="D45" s="6" t="n">
+        <v>75.73</v>
+      </c>
+      <c r="E45" s="6" t="n">
+        <v>1223.029715762274</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Cold-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="n">
+        <v>19458.11</v>
+      </c>
+      <c r="D46" s="6" t="n">
+        <v>34979.60999999999</v>
+      </c>
+      <c r="E46" s="6" t="n">
+        <v>1797.68795633286</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="n">
+        <v>2082.86</v>
+      </c>
+      <c r="D47" s="6" t="n">
+        <v>2259.27</v>
+      </c>
+      <c r="E47" s="6" t="n">
+        <v>1084.696042940956</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="n">
+        <v>240.71</v>
+      </c>
+      <c r="D48" s="6" t="n">
+        <v>3547.61</v>
+      </c>
+      <c r="E48" s="6" t="n">
+        <v>14738.10809688006</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="n">
+        <v>1097.23</v>
+      </c>
+      <c r="D49" s="6" t="n">
+        <v>2030.54</v>
+      </c>
+      <c r="E49" s="6" t="n">
+        <v>1850.60561596019</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="n">
+        <v>1247.42</v>
+      </c>
+      <c r="D50" s="6" t="n">
+        <v>1836.53</v>
+      </c>
+      <c r="E50" s="6" t="n">
+        <v>1472.262750316653</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="n">
+        <v>52.75</v>
+      </c>
+      <c r="D51" s="6" t="n">
+        <v>158.51</v>
+      </c>
+      <c r="E51" s="6" t="n">
+        <v>3004.928909952607</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="n">
+        <v>256.4299999999999</v>
+      </c>
+      <c r="D52" s="6" t="n">
+        <v>547.1199999999999</v>
+      </c>
+      <c r="E52" s="6" t="n">
+        <v>2133.603712514137</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="n">
+        <v>1994.65</v>
+      </c>
+      <c r="D53" s="6" t="n">
+        <v>3876.01</v>
+      </c>
+      <c r="E53" s="6" t="n">
+        <v>1943.203068207455</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="n">
+        <v>7.52</v>
+      </c>
+      <c r="D54" s="6" t="n">
+        <v>21.57</v>
+      </c>
+      <c r="E54" s="6" t="n">
+        <v>2868.351063829787</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="n">
+        <v>370.58</v>
+      </c>
+      <c r="D55" s="6" t="n">
+        <v>1223.97</v>
+      </c>
+      <c r="E55" s="6" t="n">
+        <v>3302.849587133683</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="n">
+        <v>301.32</v>
+      </c>
+      <c r="D56" s="6" t="n">
+        <v>562.62</v>
+      </c>
+      <c r="E56" s="6" t="n">
+        <v>1867.184388689765</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Korea, Republic of</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="n">
+        <v>19958.56</v>
+      </c>
+      <c r="D57" s="6" t="n">
+        <v>31146.28</v>
+      </c>
+      <c r="E57" s="6" t="n">
+        <v>1560.547454325362</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Malaysia</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="n">
+        <v>597.22</v>
+      </c>
+      <c r="D58" s="6" t="n">
+        <v>677.98</v>
+      </c>
+      <c r="E58" s="6" t="n">
+        <v>1135.226549680185</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="n">
+        <v>217.16</v>
+      </c>
+      <c r="D59" s="6" t="n">
+        <v>342.85</v>
+      </c>
+      <c r="E59" s="6" t="n">
+        <v>1578.789832381654</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="n">
+        <v>157.8</v>
+      </c>
+      <c r="D60" s="6" t="n">
+        <v>256.68</v>
+      </c>
+      <c r="E60" s="6" t="n">
+        <v>1626.615969581749</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="n">
+        <v>860.5</v>
+      </c>
+      <c r="D61" s="6" t="n">
+        <v>2076.12</v>
+      </c>
+      <c r="E61" s="6" t="n">
+        <v>2412.690296339338</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Pakistan</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="n">
+        <v>1455.29</v>
+      </c>
+      <c r="D62" s="6" t="n">
+        <v>1727.26</v>
+      </c>
+      <c r="E62" s="6" t="n">
+        <v>1186.883713898948</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="D63" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="E63" s="6" t="n">
+        <v>2151.394422310757</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="n">
+        <v>99.50999999999999</v>
+      </c>
+      <c r="D64" s="6" t="n">
+        <v>291.25</v>
+      </c>
+      <c r="E64" s="6" t="n">
+        <v>2926.841523464979</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Saudi Arabia</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="n">
+        <v>175.3</v>
+      </c>
+      <c r="D65" s="6" t="n">
+        <v>218.79</v>
+      </c>
+      <c r="E65" s="6" t="n">
+        <v>1248.088990302339</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="n">
+        <v>297.41</v>
+      </c>
+      <c r="D66" s="6" t="n">
+        <v>406.74</v>
+      </c>
+      <c r="E66" s="6" t="n">
+        <v>1367.60700716183</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="n">
+        <v>7469.95</v>
+      </c>
+      <c r="D67" s="6" t="n">
+        <v>8780.879999999999</v>
+      </c>
+      <c r="E67" s="6" t="n">
+        <v>1175.493811872904</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="n">
+        <v>308.38</v>
+      </c>
+      <c r="D68" s="6" t="n">
+        <v>402.99</v>
+      </c>
+      <c r="E68" s="6" t="n">
+        <v>1306.796809131591</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="n">
+        <v>85.08</v>
+      </c>
+      <c r="D69" s="6" t="n">
+        <v>129.62</v>
+      </c>
+      <c r="E69" s="6" t="n">
+        <v>1523.50728725905</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="n">
+        <v>3651.25</v>
+      </c>
+      <c r="D70" s="6" t="n">
+        <v>4974.879999999999</v>
+      </c>
+      <c r="E70" s="6" t="n">
+        <v>1362.514207463197</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="n">
+        <v>57197.30999999998</v>
+      </c>
+      <c r="D71" s="6" t="n">
+        <v>110282.55</v>
+      </c>
+      <c r="E71" s="6" t="n">
+        <v>1928.107283366999</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="n">
+        <v>1461.61</v>
+      </c>
+      <c r="D72" s="6" t="n">
+        <v>2099.690000000001</v>
+      </c>
+      <c r="E72" s="6" t="n">
+        <v>1436.55968418388</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Rebar</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Cambodia</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="n">
+        <v>3899.08</v>
+      </c>
+      <c r="D73" s="6" t="n">
+        <v>2995.72</v>
+      </c>
+      <c r="E73" s="6" t="n">
+        <v>768.3145767719565</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Rebar</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="n">
+        <v>156.65</v>
+      </c>
+      <c r="D74" s="6" t="n">
+        <v>65.61</v>
+      </c>
+      <c r="E74" s="6" t="n">
+        <v>418.8317906160231</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Rebar</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Czechia</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="D75" s="6" t="n">
+        <v>81.67</v>
+      </c>
+      <c r="E75" s="6" t="n">
+        <v>1856.136363636364</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Rebar</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="n">
+        <v>12083.72</v>
+      </c>
+      <c r="D76" s="6" t="n">
+        <v>11452.17</v>
+      </c>
+      <c r="E76" s="6" t="n">
+        <v>947.7354655685502</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Rebar</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Greece</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="n">
+        <v>2957.11</v>
+      </c>
+      <c r="D77" s="6" t="n">
+        <v>2514.12</v>
+      </c>
+      <c r="E77" s="6" t="n">
+        <v>850.1949538569752</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Rebar</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="n">
+        <v>1879.78</v>
+      </c>
+      <c r="D78" s="6" t="n">
+        <v>1188.11</v>
+      </c>
+      <c r="E78" s="6" t="n">
+        <v>632.0473672451033</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Rebar</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="n">
+        <v>3899.08</v>
+      </c>
+      <c r="D79" s="6" t="n">
+        <v>3015.8</v>
+      </c>
+      <c r="E79" s="6" t="n">
+        <v>773.4645095766181</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Rebar</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="n">
+        <v>7317.469999999999</v>
+      </c>
+      <c r="D80" s="6" t="n">
+        <v>8917.290000000001</v>
+      </c>
+      <c r="E80" s="6" t="n">
+        <v>1218.630209621632</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Rebar</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="n">
+        <v>2391.98</v>
+      </c>
+      <c r="D81" s="6" t="n">
+        <v>2225.46</v>
+      </c>
+      <c r="E81" s="6" t="n">
+        <v>930.3840333113153</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Rebar</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="n">
+        <v>4384.48</v>
+      </c>
+      <c r="D82" s="6" t="n">
+        <v>4625.09</v>
+      </c>
+      <c r="E82" s="6" t="n">
+        <v>1054.87765938036</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Rebar</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="n">
+        <v>324.21</v>
+      </c>
+      <c r="D83" s="6" t="n">
+        <v>504.71</v>
+      </c>
+      <c r="E83" s="6" t="n">
+        <v>1556.737916782333</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Rebar</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="n">
+        <v>439.91</v>
+      </c>
+      <c r="D84" s="6" t="n">
+        <v>464.35</v>
+      </c>
+      <c r="E84" s="6" t="n">
+        <v>1055.556818440135</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Rebar</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="n">
+        <v>2038.59</v>
+      </c>
+      <c r="D85" s="6" t="n">
+        <v>3070.56</v>
+      </c>
+      <c r="E85" s="6" t="n">
+        <v>1506.21753270643</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="C86" s="6" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="D86" s="6" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="E86" s="6" t="n">
+        <v>3261.904761904762</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="n">
+        <v>13.53</v>
+      </c>
+      <c r="D87" s="6" t="n">
+        <v>26.23</v>
+      </c>
+      <c r="E87" s="6" t="n">
+        <v>1938.654841093865</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C88" s="6" t="n">
+        <v>251.04</v>
+      </c>
+      <c r="D88" s="6" t="n">
+        <v>225.12</v>
+      </c>
+      <c r="E88" s="6" t="n">
+        <v>896.7495219885277</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Czechia</t>
+        </is>
+      </c>
+      <c r="C89" s="6" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="D89" s="6" t="n">
+        <v>15.24</v>
+      </c>
+      <c r="E89" s="6" t="n">
+        <v>1953.846153846154</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C90" s="6" t="n">
+        <v>114.53</v>
+      </c>
+      <c r="D90" s="6" t="n">
+        <v>144.92</v>
+      </c>
+      <c r="E90" s="6" t="n">
+        <v>1265.345324369161</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="C91" s="6" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="D91" s="6" t="n">
+        <v>5.81</v>
+      </c>
+      <c r="E91" s="6" t="n">
+        <v>1363.849765258216</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="n">
+        <v>10.78</v>
+      </c>
+      <c r="D92" s="6" t="n">
+        <v>27.53</v>
+      </c>
+      <c r="E92" s="6" t="n">
+        <v>2553.803339517625</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Korea, Republic of</t>
+        </is>
+      </c>
+      <c r="C93" s="6" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="D93" s="6" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="E93" s="6" t="n">
+        <v>4941.176470588235</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C94" s="6" t="n">
+        <v>776.99</v>
+      </c>
+      <c r="D94" s="6" t="n">
+        <v>1062.9</v>
+      </c>
+      <c r="E94" s="6" t="n">
+        <v>1367.971273761567</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Romania</t>
+        </is>
+      </c>
+      <c r="C95" s="6" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="D95" s="6" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="E95" s="6" t="n">
+        <v>4101.449275362319</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C96" s="6" t="n">
+        <v>58.38</v>
+      </c>
+      <c r="D96" s="6" t="n">
+        <v>101.44</v>
+      </c>
+      <c r="E96" s="6" t="n">
+        <v>1737.581363480644</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="C97" s="6" t="n">
+        <v>1647.26</v>
+      </c>
+      <c r="D97" s="6" t="n">
+        <v>1590.47</v>
+      </c>
+      <c r="E97" s="6" t="n">
+        <v>965.5245680706144</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="n">
+        <v>1677.88</v>
+      </c>
+      <c r="D98" s="6" t="n">
+        <v>1868.25</v>
+      </c>
+      <c r="E98" s="6" t="n">
+        <v>1113.458650201444</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C99" s="6" t="n">
+        <v>10.04</v>
+      </c>
+      <c r="D99" s="6" t="n">
+        <v>43.44</v>
+      </c>
+      <c r="E99" s="6" t="n">
+        <v>4326.693227091633</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="n">
+        <v>6327.199999999999</v>
+      </c>
+      <c r="D100" s="6" t="n">
+        <v>11487.06</v>
+      </c>
+      <c r="E100" s="6" t="n">
+        <v>1815.50448855734</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="C101" s="6" t="n">
+        <v>1314.16</v>
+      </c>
+      <c r="D101" s="6" t="n">
+        <v>1770.94</v>
+      </c>
+      <c r="E101" s="6" t="n">
+        <v>1347.5832470932</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C102" s="6" t="n">
+        <v>205.63</v>
+      </c>
+      <c r="D102" s="6" t="n">
+        <v>139.64</v>
+      </c>
+      <c r="E102" s="6" t="n">
+        <v>679.0837912755923</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C103" s="6" t="n">
+        <v>4488.21</v>
+      </c>
+      <c r="D103" s="6" t="n">
+        <v>6577.24</v>
+      </c>
+      <c r="E103" s="6" t="n">
+        <v>1465.448363601525</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Greece</t>
+        </is>
+      </c>
+      <c r="C104" s="6" t="n">
+        <v>198.08</v>
+      </c>
+      <c r="D104" s="6" t="n">
+        <v>175.53</v>
+      </c>
+      <c r="E104" s="6" t="n">
+        <v>886.1571082390952</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Malaysia</t>
+        </is>
+      </c>
+      <c r="C105" s="6" t="n">
+        <v>12348.33</v>
+      </c>
+      <c r="D105" s="6" t="n">
+        <v>12312.31</v>
+      </c>
+      <c r="E105" s="6" t="n">
+        <v>997.083006366043</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C106" s="6" t="n">
+        <v>593.8200000000001</v>
+      </c>
+      <c r="D106" s="6" t="n">
+        <v>703.6800000000001</v>
+      </c>
+      <c r="E106" s="6" t="n">
+        <v>1185.005557239568</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C107" s="6" t="n">
+        <v>185.81</v>
+      </c>
+      <c r="D107" s="6" t="n">
+        <v>243.39</v>
+      </c>
+      <c r="E107" s="6" t="n">
+        <v>1309.886443140843</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C108" s="6" t="n">
+        <v>1722.13</v>
+      </c>
+      <c r="D108" s="6" t="n">
+        <v>1452.3</v>
+      </c>
+      <c r="E108" s="6" t="n">
+        <v>843.3161259602934</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C109" s="6" t="n">
+        <v>20.52</v>
+      </c>
+      <c r="D109" s="6" t="n">
+        <v>28.52</v>
+      </c>
+      <c r="E109" s="6" t="n">
+        <v>1389.863547758285</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C110" s="6" t="n">
+        <v>8887.820000000002</v>
+      </c>
+      <c r="D110" s="6" t="n">
+        <v>12105.48</v>
+      </c>
+      <c r="E110" s="6" t="n">
+        <v>1362.030284141668</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C111" s="6" t="n">
+        <v>1871.11</v>
+      </c>
+      <c r="D111" s="6" t="n">
+        <v>1741.11</v>
+      </c>
+      <c r="E111" s="6" t="n">
+        <v>930.522524063257</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Czechia</t>
+        </is>
+      </c>
+      <c r="C112" s="6" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="D112" s="6" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="E112" s="6" t="n">
+        <v>4250</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="C113" s="6" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="D113" s="6" t="n">
+        <v>6.87</v>
+      </c>
+      <c r="E113" s="6" t="n">
+        <v>3271.428571428571</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C114" s="6" t="n">
+        <v>20.41</v>
+      </c>
+      <c r="D114" s="6" t="n">
+        <v>41.37</v>
+      </c>
+      <c r="E114" s="6" t="n">
+        <v>2026.947574718276</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C115" s="6" t="n">
+        <v>177.25</v>
+      </c>
+      <c r="D115" s="6" t="n">
+        <v>673.3299999999999</v>
+      </c>
+      <c r="E115" s="6" t="n">
+        <v>3798.758815232722</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="C116" s="6" t="n">
+        <v>221.75</v>
+      </c>
+      <c r="D116" s="6" t="n">
+        <v>484.19</v>
+      </c>
+      <c r="E116" s="6" t="n">
+        <v>2183.494926719278</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C117" s="6" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="D117" s="6" t="n">
+        <v>95.00999999999999</v>
+      </c>
+      <c r="E117" s="6" t="n">
+        <v>3345.422535211267</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="C118" s="6" t="n">
+        <v>115.61</v>
+      </c>
+      <c r="D118" s="6" t="n">
+        <v>238.04</v>
+      </c>
+      <c r="E118" s="6" t="n">
+        <v>2058.991436726927</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Korea, Republic of</t>
+        </is>
+      </c>
+      <c r="C119" s="6" t="n">
+        <v>17759.65</v>
+      </c>
+      <c r="D119" s="6" t="n">
+        <v>19078.07</v>
+      </c>
+      <c r="E119" s="6" t="n">
+        <v>1074.236823360821</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Luxembourg</t>
+        </is>
+      </c>
+      <c r="C120" s="6" t="n">
+        <v>4468.509999999999</v>
+      </c>
+      <c r="D120" s="6" t="n">
+        <v>6739.87</v>
+      </c>
+      <c r="E120" s="6" t="n">
+        <v>1508.303662742167</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C121" s="6" t="n">
+        <v>8204.919999999998</v>
+      </c>
+      <c r="D121" s="6" t="n">
+        <v>11006.31</v>
+      </c>
+      <c r="E121" s="6" t="n">
+        <v>1341.428069987276</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="C122" s="6" t="n">
+        <v>11.76</v>
+      </c>
+      <c r="D122" s="6" t="n">
+        <v>27.41</v>
+      </c>
+      <c r="E122" s="6" t="n">
+        <v>2330.78231292517</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="C123" s="6" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="D123" s="6" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="E123" s="6" t="n">
+        <v>3891.304347826087</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C124" s="6" t="n">
+        <v>13113.65</v>
+      </c>
+      <c r="D124" s="6" t="n">
+        <v>13899.15</v>
+      </c>
+      <c r="E124" s="6" t="n">
+        <v>1059.899417782234</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="C125" s="6" t="n">
+        <v>1119.84</v>
+      </c>
+      <c r="D125" s="6" t="n">
+        <v>1082.06</v>
+      </c>
+      <c r="E125" s="6" t="n">
+        <v>966.2630375767966</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C126" s="6" t="n">
+        <v>8477.610000000001</v>
+      </c>
+      <c r="D126" s="6" t="n">
+        <v>7530.9</v>
+      </c>
+      <c r="E126" s="6" t="n">
+        <v>888.3281962722983</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C127" s="6" t="n">
+        <v>3180.37</v>
+      </c>
+      <c r="D127" s="6" t="n">
+        <v>3831.62</v>
+      </c>
+      <c r="E127" s="6" t="n">
+        <v>1204.771771837868</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="C128" s="6" t="n">
+        <v>321.25</v>
+      </c>
+      <c r="D128" s="6" t="n">
+        <v>729.84</v>
+      </c>
+      <c r="E128" s="6" t="n">
+        <v>2271.875486381323</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C129" s="6" t="n">
+        <v>8529.469999999999</v>
+      </c>
+      <c r="D129" s="6" t="n">
+        <v>9778.500000000002</v>
+      </c>
+      <c r="E129" s="6" t="n">
+        <v>1146.437000188758</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C130" s="6" t="n">
+        <v>14377.29</v>
+      </c>
+      <c r="D130" s="6" t="n">
+        <v>31020.93</v>
+      </c>
+      <c r="E130" s="6" t="n">
+        <v>2157.634018650246</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="C131" s="6" t="n">
+        <v>48.44</v>
+      </c>
+      <c r="D131" s="6" t="n">
+        <v>45.15</v>
+      </c>
+      <c r="E131" s="6" t="n">
+        <v>932.0809248554914</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Weekly TRQ update 2026-04-13
</commit_message>
<xml_diff>
--- a/data/canada_trq_tracker.xlsx
+++ b/data/canada_trq_tracker.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,6 +471,11 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>April 13 2026</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
           <t>OVER</t>
         </is>
       </c>
@@ -498,6 +503,9 @@
       <c r="F3" s="4" t="n">
         <v>0.0033</v>
       </c>
+      <c r="G3" s="4" t="n">
+        <v>0.0043</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -522,6 +530,9 @@
       <c r="F4" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="G4" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -546,7 +557,10 @@
       <c r="F5" s="4" t="n">
         <v>0.41</v>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="4" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -571,6 +585,10 @@
         <f>SUM(F3:F5)</f>
         <v/>
       </c>
+      <c r="G6" s="5">
+        <f>SUM(G3:G5)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -595,6 +613,9 @@
       <c r="F7" s="4" t="n">
         <v>0.3402000000000001</v>
       </c>
+      <c r="G7" s="4" t="n">
+        <v>0.3408</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -617,6 +638,9 @@
         <v>0.0172</v>
       </c>
       <c r="F8" s="4" t="n">
+        <v>0.0172</v>
+      </c>
+      <c r="G8" s="4" t="n">
         <v>0.0172</v>
       </c>
     </row>
@@ -639,6 +663,10 @@
         <f>SUM(F7:F8)</f>
         <v/>
       </c>
+      <c r="G9" s="5">
+        <f>SUM(G7:G8)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -663,6 +691,9 @@
       <c r="F10" s="4" t="n">
         <v>0.0008</v>
       </c>
+      <c r="G10" s="4" t="n">
+        <v>0.0018</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -687,6 +718,9 @@
       <c r="F11" s="4" t="n">
         <v>0.0023</v>
       </c>
+      <c r="G11" s="4" t="n">
+        <v>0.0024</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -711,6 +745,9 @@
       <c r="F12" s="4" t="n">
         <v>0.0421</v>
       </c>
+      <c r="G12" s="4" t="n">
+        <v>0.0421</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -733,6 +770,9 @@
         <v>0.0911</v>
       </c>
       <c r="F13" s="4" t="n">
+        <v>0.0911</v>
+      </c>
+      <c r="G13" s="4" t="n">
         <v>0.0911</v>
       </c>
     </row>
@@ -755,6 +795,10 @@
         <f>SUM(F10:F13)</f>
         <v/>
       </c>
+      <c r="G14" s="5">
+        <f>SUM(G10:G13)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -779,6 +823,9 @@
       <c r="F15" s="4" t="n">
         <v>0.0025</v>
       </c>
+      <c r="G15" s="4" t="n">
+        <v>0.0059</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -803,6 +850,9 @@
       <c r="F16" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="G16" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -827,6 +877,9 @@
       <c r="F17" s="4" t="n">
         <v>0.0135</v>
       </c>
+      <c r="G17" s="4" t="n">
+        <v>0.0135</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -851,6 +904,9 @@
       <c r="F18" s="4" t="n">
         <v>0.0024</v>
       </c>
+      <c r="G18" s="4" t="n">
+        <v>0.0046</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -875,6 +931,9 @@
       <c r="F19" s="4" t="n">
         <v>0.2962</v>
       </c>
+      <c r="G19" s="4" t="n">
+        <v>0.2962</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -899,6 +958,9 @@
       <c r="F20" s="4" t="n">
         <v>0.0086</v>
       </c>
+      <c r="G20" s="4" t="n">
+        <v>0.0086</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -923,6 +985,9 @@
       <c r="F21" s="4" t="n">
         <v>0.0308</v>
       </c>
+      <c r="G21" s="4" t="n">
+        <v>0.0308</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -945,6 +1010,9 @@
         <v>0.0387</v>
       </c>
       <c r="F22" s="4" t="n">
+        <v>0.0387</v>
+      </c>
+      <c r="G22" s="4" t="n">
         <v>0.0387</v>
       </c>
     </row>
@@ -967,6 +1035,10 @@
         <f>SUM(F15:F22)</f>
         <v/>
       </c>
+      <c r="G23" s="5">
+        <f>SUM(G15:G22)</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -991,7 +1063,10 @@
       <c r="F24" s="4" t="n">
         <v>0.29</v>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G24" s="4" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="H24" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -1020,6 +1095,9 @@
       <c r="F25" s="4" t="n">
         <v>0.1228</v>
       </c>
+      <c r="G25" s="4" t="n">
+        <v>0.1228</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1044,6 +1122,9 @@
       <c r="F26" s="4" t="n">
         <v>0.2394</v>
       </c>
+      <c r="G26" s="4" t="n">
+        <v>0.2394</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1068,6 +1149,9 @@
       <c r="F27" s="4" t="n">
         <v>0.1668</v>
       </c>
+      <c r="G27" s="4" t="n">
+        <v>0.1668</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1092,6 +1176,9 @@
       <c r="F28" s="4" t="n">
         <v>0.0241</v>
       </c>
+      <c r="G28" s="4" t="n">
+        <v>0.0241</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1114,6 +1201,9 @@
         <v>0.1569</v>
       </c>
       <c r="F29" s="4" t="n">
+        <v>0.1569</v>
+      </c>
+      <c r="G29" s="4" t="n">
         <v>0.1569</v>
       </c>
     </row>
@@ -1136,6 +1226,10 @@
         <f>SUM(F24:F29)</f>
         <v/>
       </c>
+      <c r="G30" s="5">
+        <f>SUM(G24:G29)</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1160,6 +1254,9 @@
       <c r="F31" s="4" t="n">
         <v>0.0021</v>
       </c>
+      <c r="G31" s="4" t="n">
+        <v>0.0154</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1184,6 +1281,9 @@
       <c r="F32" s="4" t="n">
         <v>0.1359</v>
       </c>
+      <c r="G32" s="4" t="n">
+        <v>0.2337</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1208,6 +1308,9 @@
       <c r="F33" s="4" t="n">
         <v>0.1475</v>
       </c>
+      <c r="G33" s="4" t="n">
+        <v>0.31</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1232,6 +1335,9 @@
       <c r="F34" s="4" t="n">
         <v>0.1892</v>
       </c>
+      <c r="G34" s="4" t="n">
+        <v>0.1892</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1241,40 +1347,41 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="n">
+        <v>7281700</v>
+      </c>
+      <c r="D35" s="4" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="G35" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E35" s="5">
+      <c r="E36" s="5">
         <f>SUM(E31:E34)</f>
         <v/>
       </c>
-      <c r="F35" s="5">
+      <c r="F36" s="5">
         <f>SUM(F31:F34)</f>
         <v/>
       </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Wire Rod</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Türkiye</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="n">
-        <v>1571700</v>
-      </c>
-      <c r="D36" s="4" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="E36" s="4" t="n">
-        <v>0.1514</v>
-      </c>
-      <c r="F36" s="4" t="n">
-        <v>0.1514</v>
+      <c r="G36" s="5">
+        <f>SUM(G31:G35)</f>
+        <v/>
       </c>
     </row>
     <row r="37">
@@ -1285,40 +1392,47 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>1571700</v>
+      </c>
+      <c r="D37" s="4" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>0.1514</v>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>0.1514</v>
+      </c>
+      <c r="G37" s="4" t="n">
+        <v>0.1514</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E37" s="5">
+      <c r="E38" s="5">
         <f>SUM(E36:E36)</f>
         <v/>
       </c>
-      <c r="F37" s="5">
+      <c r="F38" s="5">
         <f>SUM(F36:F36)</f>
         <v/>
       </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Structural Steel</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>China</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="n">
-        <v>4674200</v>
-      </c>
-      <c r="D38" s="4" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="E38" s="4" t="n">
-        <v>0.0359</v>
-      </c>
-      <c r="F38" s="4" t="n">
-        <v>0.0408</v>
+      <c r="G38" s="5">
+        <f>SUM(G36:G36)</f>
+        <v/>
       </c>
     </row>
     <row r="39">
@@ -1329,7 +1443,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C39" s="3" t="n">
@@ -1339,10 +1453,13 @@
         <v>0.55</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>0.0177</v>
+        <v>0.0359</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>0.0236</v>
+        <v>0.0408</v>
+      </c>
+      <c r="G39" s="4" t="n">
+        <v>0.0412</v>
       </c>
     </row>
     <row r="40">
@@ -1353,7 +1470,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C40" s="3" t="n">
@@ -1363,10 +1480,13 @@
         <v>0.55</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>0.2154</v>
+        <v>0.0177</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>0.2154</v>
+        <v>0.0236</v>
+      </c>
+      <c r="G40" s="4" t="n">
+        <v>0.0236</v>
       </c>
     </row>
     <row r="41">
@@ -1377,7 +1497,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C41" s="3" t="n">
@@ -1387,10 +1507,13 @@
         <v>0.55</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>0.5329999999999999</v>
+        <v>0.2154</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>0.5436</v>
+        <v>0.2154</v>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>0.3917</v>
       </c>
     </row>
     <row r="42">
@@ -1401,15 +1524,46 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="n">
+        <v>4674200</v>
+      </c>
+      <c r="D42" s="4" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="E42" s="4" t="n">
+        <v>0.5329999999999999</v>
+      </c>
+      <c r="F42" s="4" t="n">
+        <v>0.5436</v>
+      </c>
+      <c r="G42" s="4" t="n">
+        <v>0.5436</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E42" s="5">
+      <c r="E43" s="5">
         <f>SUM(E38:E41)</f>
         <v/>
       </c>
-      <c r="F42" s="5">
+      <c r="F43" s="5">
         <f>SUM(F38:F41)</f>
+        <v/>
+      </c>
+      <c r="G43" s="5">
+        <f>SUM(G38:G41)</f>
         <v/>
       </c>
     </row>
@@ -1424,7 +1578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G73"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1462,6 +1616,11 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>April 13 2026</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
           <t>OVER</t>
         </is>
       </c>
@@ -1489,6 +1648,9 @@
       <c r="F3" s="4" t="n">
         <v>0.0015</v>
       </c>
+      <c r="G3" s="4" t="n">
+        <v>0.0015</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1513,6 +1675,9 @@
       <c r="F4" s="4" t="n">
         <v>0.0002</v>
       </c>
+      <c r="G4" s="4" t="n">
+        <v>0.1158</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1537,6 +1702,9 @@
       <c r="F5" s="4" t="n">
         <v>0.0435</v>
       </c>
+      <c r="G5" s="4" t="n">
+        <v>0.115</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1561,6 +1729,9 @@
       <c r="F6" s="4" t="n">
         <v>0.0306</v>
       </c>
+      <c r="G6" s="4" t="n">
+        <v>0.0306</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1585,6 +1756,9 @@
       <c r="F7" s="4" t="n">
         <v>0.0446</v>
       </c>
+      <c r="G7" s="4" t="n">
+        <v>0.0623</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1609,6 +1783,9 @@
       <c r="F8" s="4" t="n">
         <v>0.0002</v>
       </c>
+      <c r="G8" s="4" t="n">
+        <v>0.0003</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1633,6 +1810,9 @@
       <c r="F9" s="4" t="n">
         <v>0.0011</v>
       </c>
+      <c r="G9" s="4" t="n">
+        <v>0.0011</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1678,6 +1858,9 @@
       <c r="F11" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="G11" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1699,6 +1882,9 @@
       <c r="F12" s="4" t="n">
         <v>0.0012</v>
       </c>
+      <c r="G12" s="4" t="n">
+        <v>0.0012</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1718,6 +1904,9 @@
         <v>0.67</v>
       </c>
       <c r="F13" s="4" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="G13" s="4" t="n">
         <v>0.0003</v>
       </c>
     </row>
@@ -1740,6 +1929,10 @@
         <f>SUM(F3:F13)</f>
         <v/>
       </c>
+      <c r="G14" s="5">
+        <f>SUM(G3:G13)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1764,6 +1957,9 @@
       <c r="F15" s="4" t="n">
         <v>0.0025</v>
       </c>
+      <c r="G15" s="4" t="n">
+        <v>0.005500000000000001</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1788,6 +1984,9 @@
       <c r="F16" s="4" t="n">
         <v>0.0141</v>
       </c>
+      <c r="G16" s="4" t="n">
+        <v>0.022</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1812,6 +2011,9 @@
       <c r="F17" s="4" t="n">
         <v>0.0012</v>
       </c>
+      <c r="G17" s="4" t="n">
+        <v>0.0018</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1836,6 +2038,9 @@
       <c r="F18" s="4" t="n">
         <v>0.008199999999999999</v>
       </c>
+      <c r="G18" s="4" t="n">
+        <v>0.2861</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1860,6 +2065,9 @@
       <c r="F19" s="4" t="n">
         <v>0.0083</v>
       </c>
+      <c r="G19" s="4" t="n">
+        <v>0.0572</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1884,7 +2092,10 @@
       <c r="F20" s="4" t="n">
         <v>0.3</v>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H20" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -1913,6 +2124,9 @@
       <c r="F21" s="4" t="n">
         <v>0.0892</v>
       </c>
+      <c r="G21" s="4" t="n">
+        <v>0.0892</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1937,6 +2151,9 @@
       <c r="F22" s="4" t="n">
         <v>0.0004</v>
       </c>
+      <c r="G22" s="4" t="n">
+        <v>0.0004</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1961,6 +2178,9 @@
       <c r="F23" s="4" t="n">
         <v>0.0128</v>
       </c>
+      <c r="G23" s="4" t="n">
+        <v>0.0315</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1982,6 +2202,9 @@
       <c r="F24" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="G24" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2003,6 +2226,9 @@
       <c r="F25" s="4" t="n">
         <v>0.0011</v>
       </c>
+      <c r="G25" s="4" t="n">
+        <v>0.0019</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2023,6 +2249,9 @@
       </c>
       <c r="F26" s="4" t="n">
         <v>0.0001</v>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>0.0003</v>
       </c>
     </row>
     <row r="27">
@@ -2044,6 +2273,10 @@
         <f>SUM(F15:F26)</f>
         <v/>
       </c>
+      <c r="G27" s="5">
+        <f>SUM(G15:G26)</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2068,6 +2301,9 @@
       <c r="F28" s="4" t="n">
         <v>0.0964</v>
       </c>
+      <c r="G28" s="4" t="n">
+        <v>0.1823</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2088,6 +2324,9 @@
       </c>
       <c r="F29" s="4" t="n">
         <v>0.0795</v>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>0.123</v>
       </c>
     </row>
     <row r="30">
@@ -2109,6 +2348,10 @@
         <f>SUM(F28:F29)</f>
         <v/>
       </c>
+      <c r="G30" s="5">
+        <f>SUM(G28:G29)</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2133,6 +2376,9 @@
       <c r="F31" s="4" t="n">
         <v>0.0003</v>
       </c>
+      <c r="G31" s="4" t="n">
+        <v>0.0003</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2157,6 +2403,9 @@
       <c r="F32" s="4" t="n">
         <v>0.0562</v>
       </c>
+      <c r="G32" s="4" t="n">
+        <v>0.0793</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2181,6 +2430,9 @@
       <c r="F33" s="4" t="n">
         <v>0.0341</v>
       </c>
+      <c r="G33" s="4" t="n">
+        <v>0.0385</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2205,6 +2457,9 @@
       <c r="F34" s="4" t="n">
         <v>0.0435</v>
       </c>
+      <c r="G34" s="4" t="n">
+        <v>0.0435</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2229,6 +2484,9 @@
       <c r="F35" s="4" t="n">
         <v>0.0251</v>
       </c>
+      <c r="G35" s="4" t="n">
+        <v>0.0282</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2253,6 +2511,9 @@
       <c r="F36" s="4" t="n">
         <v>0.0007000000000000001</v>
       </c>
+      <c r="G36" s="4" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2277,6 +2538,9 @@
       <c r="F37" s="4" t="n">
         <v>0.0265</v>
       </c>
+      <c r="G37" s="4" t="n">
+        <v>0.0302</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2298,6 +2562,9 @@
       <c r="F38" s="4" t="n">
         <v>0.0005</v>
       </c>
+      <c r="G38" s="4" t="n">
+        <v>0.0008</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2319,6 +2586,9 @@
       <c r="F39" s="4" t="n">
         <v>0.0064</v>
       </c>
+      <c r="G39" s="4" t="n">
+        <v>0.0142</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2340,6 +2610,9 @@
       <c r="F40" s="4" t="n">
         <v>0.0101</v>
       </c>
+      <c r="G40" s="4" t="n">
+        <v>0.0101</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2349,40 +2622,41 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
+          <t>Slovenia</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="n">
+        <v>31128200</v>
+      </c>
+      <c r="D41" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>0.0003</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E41" s="5">
+      <c r="E42" s="5">
         <f>SUM(E25:E31)</f>
         <v/>
       </c>
-      <c r="F41" s="5">
+      <c r="F42" s="5">
         <f>SUM(F31:F40)</f>
         <v/>
       </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Rebar</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="n">
-        <v>28710400</v>
-      </c>
-      <c r="D42" s="4" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="E42" s="4" t="n">
-        <v>0.1642</v>
-      </c>
-      <c r="F42" s="4" t="n">
-        <v>0.1642</v>
+      <c r="G42" s="5">
+        <f>SUM(G31:G41)</f>
+        <v/>
       </c>
     </row>
     <row r="43">
@@ -2393,7 +2667,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Greece</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C43" s="3" t="n">
@@ -2403,10 +2677,13 @@
         <v>0.45</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>0.3234</v>
+        <v>0.1642</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>0.3234</v>
+        <v>0.1642</v>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>0.1642</v>
       </c>
     </row>
     <row r="44">
@@ -2417,7 +2694,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Greece</t>
         </is>
       </c>
       <c r="C44" s="3" t="n">
@@ -2427,10 +2704,13 @@
         <v>0.45</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>0.0028</v>
+        <v>0.3234</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>0.0028</v>
+        <v>0.3234</v>
+      </c>
+      <c r="G44" s="4" t="n">
+        <v>0.3234</v>
       </c>
     </row>
     <row r="45">
@@ -2441,7 +2721,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Peru</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C45" s="3" t="n">
@@ -2451,10 +2731,13 @@
         <v>0.45</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>0.1633</v>
+        <v>0.0028</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>0.1633</v>
+        <v>0.0028</v>
+      </c>
+      <c r="G45" s="4" t="n">
+        <v>0.0028</v>
       </c>
     </row>
     <row r="46">
@@ -2465,7 +2748,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Peru</t>
         </is>
       </c>
       <c r="C46" s="3" t="n">
@@ -2475,10 +2758,13 @@
         <v>0.45</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>0.3462</v>
+        <v>0.1633</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>0.3462</v>
+        <v>0.1633</v>
+      </c>
+      <c r="G46" s="4" t="n">
+        <v>0.1633</v>
       </c>
     </row>
     <row r="47">
@@ -2489,40 +2775,47 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="n">
+        <v>28710400</v>
+      </c>
+      <c r="D47" s="4" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>0.3462</v>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>0.3462</v>
+      </c>
+      <c r="G47" s="4" t="n">
+        <v>0.3462</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Rebar</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E47" s="5">
+      <c r="E48" s="5">
         <f>SUM(E33:E37)</f>
         <v/>
       </c>
-      <c r="F47" s="5">
+      <c r="F48" s="5">
         <f>SUM(F33:F37)</f>
         <v/>
       </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Hot-Rolled Bar</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Czech Republic</t>
-        </is>
-      </c>
-      <c r="C48" s="3" t="n">
-        <v>8750300</v>
-      </c>
-      <c r="D48" s="4" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="E48" s="4" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="F48" s="4" t="n">
-        <v>0.0007000000000000001</v>
+      <c r="G48" s="5">
+        <f>SUM(G42:G46)</f>
+        <v/>
       </c>
     </row>
     <row r="49">
@@ -2533,7 +2826,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C49" s="3" t="n">
@@ -2543,10 +2836,13 @@
         <v>0.58</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>0.0022</v>
+        <v>0.0001</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>0.0022</v>
+        <v>0.0007000000000000001</v>
+      </c>
+      <c r="G49" s="4" t="n">
+        <v>0.0016</v>
       </c>
     </row>
     <row r="50">
@@ -2557,7 +2853,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="C50" s="3" t="n">
@@ -2567,10 +2863,13 @@
         <v>0.58</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>0.0017</v>
+        <v>0.0022</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>0.0017</v>
+        <v>0.0022</v>
+      </c>
+      <c r="G50" s="4" t="n">
+        <v>0.0022</v>
       </c>
     </row>
     <row r="51">
@@ -2581,7 +2880,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C51" s="3" t="n">
@@ -2591,10 +2890,13 @@
         <v>0.58</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>0.0307</v>
+        <v>0.0017</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>0.0633</v>
+        <v>0.0017</v>
+      </c>
+      <c r="G51" s="4" t="n">
+        <v>0.0017</v>
       </c>
     </row>
     <row r="52">
@@ -2605,7 +2907,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C52" s="3" t="n">
@@ -2615,10 +2917,13 @@
         <v>0.58</v>
       </c>
       <c r="E52" s="4" t="n">
-        <v>0.001</v>
+        <v>0.0307</v>
       </c>
       <c r="F52" s="4" t="n">
-        <v>0.0021</v>
+        <v>0.0633</v>
+      </c>
+      <c r="G52" s="4" t="n">
+        <v>0.0793</v>
       </c>
     </row>
     <row r="53">
@@ -2629,7 +2934,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C53" s="3" t="n">
@@ -2639,10 +2944,13 @@
         <v>0.58</v>
       </c>
       <c r="E53" s="4" t="n">
-        <v>0.07519999999999999</v>
+        <v>0.001</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>0.127</v>
+        <v>0.0021</v>
+      </c>
+      <c r="G53" s="4" t="n">
+        <v>0.0029</v>
       </c>
     </row>
     <row r="54">
@@ -2653,7 +2961,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C54" s="3" t="n">
@@ -2663,10 +2971,13 @@
         <v>0.58</v>
       </c>
       <c r="E54" s="4" t="n">
-        <v>0</v>
+        <v>0.07519999999999999</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>0</v>
+        <v>0.127</v>
+      </c>
+      <c r="G54" s="4" t="n">
+        <v>0.1355</v>
       </c>
     </row>
     <row r="55">
@@ -2677,7 +2988,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="C55" s="3" t="n">
@@ -2687,10 +2998,13 @@
         <v>0.58</v>
       </c>
       <c r="E55" s="4" t="n">
-        <v>0.009899999999999999</v>
+        <v>0</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>0.0876</v>
+        <v>0</v>
+      </c>
+      <c r="G55" s="4" t="n">
+        <v>0.0002</v>
       </c>
     </row>
     <row r="56">
@@ -2701,7 +3015,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C56" s="3" t="n">
@@ -2711,10 +3025,13 @@
         <v>0.58</v>
       </c>
       <c r="E56" s="4" t="n">
-        <v>0</v>
+        <v>0.009899999999999999</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>0</v>
+        <v>0.0876</v>
+      </c>
+      <c r="G56" s="4" t="n">
+        <v>0.1008</v>
       </c>
     </row>
     <row r="57">
@@ -2725,7 +3042,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C57" s="3" t="n">
@@ -2734,9 +3051,15 @@
       <c r="D57" s="4" t="n">
         <v>0.58</v>
       </c>
+      <c r="E57" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="F57" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="G57" s="4" t="n">
+        <v>0.0016</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2746,7 +3069,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C58" s="3" t="n">
@@ -2758,6 +3081,9 @@
       <c r="F58" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="G58" s="4" t="n">
+        <v>0.0206</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2767,64 +3093,65 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
+          <t>Romania</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="n">
+        <v>8750300</v>
+      </c>
+      <c r="D59" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F59" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="4" t="n">
+        <v>0.0017</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="n">
+        <v>8750300</v>
+      </c>
+      <c r="D60" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="G60" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E59" s="5">
+      <c r="E61" s="5">
         <f>SUM(E39:E47)</f>
         <v/>
       </c>
-      <c r="F59" s="5">
+      <c r="F61" s="5">
         <f>SUM(F48:F58)</f>
         <v/>
       </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Wire Rod</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="C60" s="3" t="n">
-        <v>16514800</v>
-      </c>
-      <c r="D60" s="4" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="E60" s="4" t="n">
-        <v>0.0011</v>
-      </c>
-      <c r="F60" s="4" t="n">
-        <v>0.0751</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Wire Rod</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Korea, Republic of</t>
-        </is>
-      </c>
-      <c r="C61" s="3" t="n">
-        <v>16514800</v>
-      </c>
-      <c r="D61" s="4" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="E61" s="4" t="n">
-        <v>0.0122</v>
-      </c>
-      <c r="F61" s="4" t="n">
-        <v>0.0122</v>
+      <c r="G61" s="5">
+        <f>SUM(G49:G60)</f>
+        <v/>
       </c>
     </row>
     <row r="62">
@@ -2835,7 +3162,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C62" s="3" t="n">
@@ -2845,10 +3172,13 @@
         <v>0.59</v>
       </c>
       <c r="E62" s="4" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.0011</v>
       </c>
       <c r="F62" s="4" t="n">
-        <v>0.0176</v>
+        <v>0.0751</v>
+      </c>
+      <c r="G62" s="4" t="n">
+        <v>0.1416</v>
       </c>
     </row>
     <row r="63">
@@ -2859,7 +3189,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C63" s="3" t="n">
@@ -2868,8 +3198,14 @@
       <c r="D63" s="4" t="n">
         <v>0.59</v>
       </c>
+      <c r="E63" s="4" t="n">
+        <v>0.0122</v>
+      </c>
       <c r="F63" s="4" t="n">
-        <v>0</v>
+        <v>0.0122</v>
+      </c>
+      <c r="G63" s="4" t="n">
+        <v>0.0434</v>
       </c>
     </row>
     <row r="64">
@@ -2880,64 +3216,71 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="n">
+        <v>16514800</v>
+      </c>
+      <c r="D64" s="4" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="E64" s="4" t="n">
+        <v>0.008800000000000001</v>
+      </c>
+      <c r="F64" s="4" t="n">
+        <v>0.0176</v>
+      </c>
+      <c r="G64" s="4" t="n">
+        <v>0.0147</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="n">
+        <v>16514800</v>
+      </c>
+      <c r="D65" s="4" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="F65" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E64" s="5">
+      <c r="E66" s="5">
         <f>SUM(E49:E51)</f>
         <v/>
       </c>
-      <c r="F64" s="5">
+      <c r="F66" s="5">
         <f>SUM(F60:F63)</f>
         <v/>
       </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Structural Steel</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="C65" s="3" t="n">
-        <v>3467600</v>
-      </c>
-      <c r="D65" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="E65" s="4" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="F65" s="4" t="n">
-        <v>0.0001</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Structural Steel</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="C66" s="3" t="n">
-        <v>3467600</v>
-      </c>
-      <c r="D66" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="E66" s="4" t="n">
-        <v>0.0011</v>
-      </c>
-      <c r="F66" s="4" t="n">
-        <v>0.0073</v>
+      <c r="G66" s="5">
+        <f>SUM(G60:G63)</f>
+        <v/>
       </c>
     </row>
     <row r="67">
@@ -2948,7 +3291,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C67" s="3" t="n">
@@ -2958,10 +3301,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E67" s="4" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="F67" s="4" t="n">
-        <v>0</v>
+        <v>0.0001</v>
+      </c>
+      <c r="G67" s="4" t="n">
+        <v>0.0017</v>
       </c>
     </row>
     <row r="68">
@@ -2972,7 +3318,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C68" s="3" t="n">
@@ -2982,10 +3328,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E68" s="4" t="n">
-        <v>0.0191</v>
+        <v>0.0011</v>
       </c>
       <c r="F68" s="4" t="n">
-        <v>0.0191</v>
+        <v>0.0073</v>
+      </c>
+      <c r="G68" s="4" t="n">
+        <v>0.0075</v>
       </c>
     </row>
     <row r="69">
@@ -2996,7 +3345,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C69" s="3" t="n">
@@ -3006,10 +3355,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E69" s="4" t="n">
-        <v>0.007900000000000001</v>
+        <v>0</v>
       </c>
       <c r="F69" s="4" t="n">
-        <v>0.007900000000000001</v>
+        <v>0</v>
+      </c>
+      <c r="G69" s="4" t="n">
+        <v>0.0001</v>
       </c>
     </row>
     <row r="70">
@@ -3020,7 +3372,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C70" s="3" t="n">
@@ -3030,10 +3382,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E70" s="4" t="n">
-        <v>0.3604</v>
+        <v>0.0191</v>
       </c>
       <c r="F70" s="4" t="n">
-        <v>0.3604</v>
+        <v>0.0191</v>
+      </c>
+      <c r="G70" s="4" t="n">
+        <v>0.0191</v>
       </c>
     </row>
     <row r="71">
@@ -3044,7 +3399,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C71" s="3" t="n">
@@ -3053,8 +3408,14 @@
       <c r="D71" s="4" t="n">
         <v>0.6899999999999999</v>
       </c>
+      <c r="E71" s="4" t="n">
+        <v>0.007900000000000001</v>
+      </c>
       <c r="F71" s="4" t="n">
-        <v>0.0421</v>
+        <v>0.007900000000000001</v>
+      </c>
+      <c r="G71" s="4" t="n">
+        <v>0.0142</v>
       </c>
     </row>
     <row r="72">
@@ -3065,7 +3426,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C72" s="3" t="n">
@@ -3074,8 +3435,14 @@
       <c r="D72" s="4" t="n">
         <v>0.6899999999999999</v>
       </c>
+      <c r="E72" s="4" t="n">
+        <v>0.3604</v>
+      </c>
       <c r="F72" s="4" t="n">
-        <v>0.0001</v>
+        <v>0.3604</v>
+      </c>
+      <c r="G72" s="4" t="n">
+        <v>0.3604</v>
       </c>
     </row>
     <row r="73">
@@ -3086,15 +3453,67 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
+          <t>Korea, Republic of</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D73" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="F73" s="4" t="n">
+        <v>0.0421</v>
+      </c>
+      <c r="G73" s="4" t="n">
+        <v>0.0421</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D74" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="F74" s="4" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="G74" s="4" t="n">
+        <v>0.0001</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E73" s="5">
+      <c r="E75" s="5">
         <f>SUM(E53:E58)</f>
         <v/>
       </c>
-      <c r="F73" s="5">
+      <c r="F75" s="5">
         <f>SUM(F65:F72)</f>
+        <v/>
+      </c>
+      <c r="G75" s="5">
+        <f>SUM(G65:G72)</f>
         <v/>
       </c>
     </row>
@@ -3435,7 +3854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E131"/>
+  <dimension ref="A1:E137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3519,13 +3938,13 @@
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>10.93</v>
+        <v>13.31</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>4.35</v>
+        <v>5.07</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>397.9871912168344</v>
+        <v>380.9166040570999</v>
       </c>
     </row>
     <row r="11">
@@ -3540,13 +3959,13 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>102.11</v>
+        <v>515.33</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>171.34</v>
+        <v>667.6300000000001</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>1677.994319851141</v>
+        <v>1295.538780975297</v>
       </c>
     </row>
     <row r="12">
@@ -3603,13 +4022,13 @@
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>1756.41</v>
+        <v>4145.04</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>1337.35</v>
+        <v>3123.96</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>761.4110600600089</v>
+        <v>753.6622083260958</v>
       </c>
     </row>
     <row r="15">
@@ -3645,13 +4064,13 @@
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>71.09999999999999</v>
+        <v>517.73</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>97.78999999999999</v>
+        <v>644.96</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1375.386779184247</v>
+        <v>1245.745852085064</v>
       </c>
     </row>
     <row r="17">
@@ -3662,38 +4081,38 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>24736.99000000001</v>
+        <v>1129.4</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>37963.62</v>
+        <v>866.98</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>1534.69035642574</v>
+        <v>767.6465379847706</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Steel Plate</t>
+          <t>Hot-Rolled Sheet</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>633.1</v>
+        <v>29177.21</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>657.24</v>
+        <v>45065.73999999999</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1038.129837308482</v>
+        <v>1544.552751959491</v>
       </c>
     </row>
     <row r="19">
@@ -3704,17 +4123,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>346.21</v>
+        <v>633.1</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>664.45</v>
+        <v>657.24</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>1919.210883567777</v>
+        <v>1038.129837308482</v>
       </c>
     </row>
     <row r="20">
@@ -3725,17 +4144,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>2814.44</v>
+        <v>346.21</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>2707.8</v>
+        <v>664.45</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>962.1096914483874</v>
+        <v>1919.210883567777</v>
       </c>
     </row>
     <row r="21">
@@ -3746,17 +4165,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>0.84</v>
+        <v>3230.12</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>1.78</v>
+        <v>3078.239999999999</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>2119.047619047619</v>
+        <v>952.9800750436515</v>
       </c>
     </row>
     <row r="22">
@@ -3767,17 +4186,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>2051.31</v>
+        <v>0.84</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>6915.08</v>
+        <v>1.78</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>3371.055569367867</v>
+        <v>2119.047619047619</v>
       </c>
     </row>
     <row r="23">
@@ -3788,17 +4207,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>3007.1</v>
+        <v>2762.83</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>3666.78</v>
+        <v>8893.600000000002</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>1219.374147850088</v>
+        <v>3219.018180633626</v>
       </c>
     </row>
     <row r="24">
@@ -3809,17 +4228,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>141.02</v>
+        <v>3007.1</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>333.88</v>
+        <v>3666.78</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>2367.60743156999</v>
+        <v>1219.374147850088</v>
       </c>
     </row>
     <row r="25">
@@ -3830,17 +4249,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C25" s="6" t="n">
-        <v>1.74</v>
+        <v>165</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>4.140000000000001</v>
+        <v>368.13</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>2379.310344827587</v>
+        <v>2231.090909090909</v>
       </c>
     </row>
     <row r="26">
@@ -3851,17 +4270,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>9.879999999999999</v>
+        <v>1.74</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>20.9</v>
+        <v>4.140000000000001</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>2115.384615384616</v>
+        <v>2379.310344827587</v>
       </c>
     </row>
     <row r="27">
@@ -3872,17 +4291,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>11695.79</v>
+        <v>11.95</v>
       </c>
       <c r="D27" s="6" t="n">
-        <v>13727.43</v>
+        <v>27.64</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>1173.70694925268</v>
+        <v>2312.970711297071</v>
       </c>
     </row>
     <row r="28">
@@ -3893,17 +4312,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>1160.84</v>
+        <v>13028.15</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>1173.79</v>
+        <v>15185.58999999999</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>1011.155714827194</v>
+        <v>1165.598338981359</v>
       </c>
     </row>
     <row r="29">
@@ -3914,17 +4333,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>614.54</v>
+        <v>4263.77</v>
       </c>
       <c r="D29" s="6" t="n">
-        <v>1255.25</v>
+        <v>4469.190000000001</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>2042.584697497315</v>
+        <v>1048.178020859474</v>
       </c>
     </row>
     <row r="30">
@@ -3935,17 +4354,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>22.77</v>
+        <v>704.16</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>64.40000000000001</v>
+        <v>1384.4</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>2828.282828282829</v>
+        <v>1966.030447625539</v>
       </c>
     </row>
     <row r="31">
@@ -3956,17 +4375,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C31" s="6" t="n">
-        <v>23.49</v>
+        <v>22.77</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>89.52</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="E31" s="6" t="n">
-        <v>3810.983397190294</v>
+        <v>2828.282828282829</v>
       </c>
     </row>
     <row r="32">
@@ -3977,17 +4396,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>725.13</v>
+        <v>23.49</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>670.12</v>
+        <v>89.52</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>924.1377408188877</v>
+        <v>3810.983397190294</v>
       </c>
     </row>
     <row r="33">
@@ -3998,17 +4417,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C33" s="6" t="n">
-        <v>27.77</v>
+        <v>1256.14</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>6.82</v>
+        <v>1161.6</v>
       </c>
       <c r="E33" s="6" t="n">
-        <v>245.5887648541592</v>
+        <v>924.7376884742146</v>
       </c>
     </row>
     <row r="34">
@@ -4019,17 +4438,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C34" s="6" t="n">
-        <v>5.83</v>
+        <v>27.77</v>
       </c>
       <c r="D34" s="6" t="n">
-        <v>28.01</v>
+        <v>6.82</v>
       </c>
       <c r="E34" s="6" t="n">
-        <v>4804.459691252144</v>
+        <v>245.5887648541592</v>
       </c>
     </row>
     <row r="35">
@@ -4040,38 +4459,38 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C35" s="6" t="n">
-        <v>16955.68</v>
+        <v>5.83</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>30083.11999999999</v>
+        <v>28.01</v>
       </c>
       <c r="E35" s="6" t="n">
-        <v>1774.220792088551</v>
+        <v>4804.459691252144</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Cold-Rolled Sheet</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C36" s="6" t="n">
-        <v>2.28</v>
+        <v>18765.25</v>
       </c>
       <c r="D36" s="6" t="n">
-        <v>10.07</v>
+        <v>33508.98999999998</v>
       </c>
       <c r="E36" s="6" t="n">
-        <v>4416.666666666667</v>
+        <v>1785.693769067824</v>
       </c>
     </row>
     <row r="37">
@@ -4082,17 +4501,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C37" s="6" t="n">
-        <v>30.99</v>
+        <v>2.79</v>
       </c>
       <c r="D37" s="6" t="n">
-        <v>61.46999999999999</v>
+        <v>10.74</v>
       </c>
       <c r="E37" s="6" t="n">
-        <v>1983.543078412391</v>
+        <v>3849.462365591398</v>
       </c>
     </row>
     <row r="38">
@@ -4103,17 +4522,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C38" s="6" t="n">
-        <v>34.08</v>
+        <v>35.62</v>
       </c>
       <c r="D38" s="6" t="n">
-        <v>83.56000000000002</v>
+        <v>70.01000000000001</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>2451.877934272301</v>
+        <v>1965.468837731612</v>
       </c>
     </row>
     <row r="39">
@@ -4124,17 +4543,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C39" s="6" t="n">
-        <v>0.25</v>
+        <v>54.14</v>
       </c>
       <c r="D39" s="6" t="n">
-        <v>0.35</v>
+        <v>131.16</v>
       </c>
       <c r="E39" s="6" t="n">
-        <v>1400</v>
+        <v>2422.60805319542</v>
       </c>
     </row>
     <row r="40">
@@ -4145,17 +4564,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C40" s="6" t="n">
-        <v>6.26</v>
+        <v>0.25</v>
       </c>
       <c r="D40" s="6" t="n">
-        <v>26.97</v>
+        <v>0.35</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>4308.306709265175</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="41">
@@ -4166,17 +4585,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C41" s="6" t="n">
-        <v>227.27</v>
+        <v>6.26</v>
       </c>
       <c r="D41" s="6" t="n">
-        <v>274.06</v>
+        <v>26.97</v>
       </c>
       <c r="E41" s="6" t="n">
-        <v>1205.878470541646</v>
+        <v>4308.306709265175</v>
       </c>
     </row>
     <row r="42">
@@ -4187,17 +4606,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="C42" s="6" t="n">
-        <v>631.48</v>
+        <v>227.27</v>
       </c>
       <c r="D42" s="6" t="n">
-        <v>1015.23</v>
+        <v>274.06</v>
       </c>
       <c r="E42" s="6" t="n">
-        <v>1607.699372901754</v>
+        <v>1205.878470541646</v>
       </c>
     </row>
     <row r="43">
@@ -4208,17 +4627,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C43" s="6" t="n">
-        <v>240.83</v>
+        <v>701.76</v>
       </c>
       <c r="D43" s="6" t="n">
-        <v>407.72</v>
+        <v>1173.86</v>
       </c>
       <c r="E43" s="6" t="n">
-        <v>1692.978449528713</v>
+        <v>1672.737118103055</v>
       </c>
     </row>
     <row r="44">
@@ -4229,17 +4648,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C44" s="6" t="n">
-        <v>682.4400000000001</v>
+        <v>896.8299999999999</v>
       </c>
       <c r="D44" s="6" t="n">
-        <v>782.05</v>
+        <v>969.67</v>
       </c>
       <c r="E44" s="6" t="n">
-        <v>1145.96154973331</v>
+        <v>1081.219406130482</v>
       </c>
     </row>
     <row r="45">
@@ -4250,17 +4669,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C45" s="6" t="n">
-        <v>61.92</v>
+        <v>682.4400000000001</v>
       </c>
       <c r="D45" s="6" t="n">
-        <v>75.73</v>
+        <v>782.05</v>
       </c>
       <c r="E45" s="6" t="n">
-        <v>1223.029715762274</v>
+        <v>1145.96154973331</v>
       </c>
     </row>
     <row r="46">
@@ -4271,38 +4690,38 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C46" s="6" t="n">
-        <v>19458.11</v>
+        <v>1734.44</v>
       </c>
       <c r="D46" s="6" t="n">
-        <v>34979.60999999999</v>
+        <v>1532.54</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>1797.68795633286</v>
+        <v>883.5935518092294</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C47" s="6" t="n">
-        <v>2082.86</v>
+        <v>23464.85</v>
       </c>
       <c r="D47" s="6" t="n">
-        <v>2259.27</v>
+        <v>41945.93</v>
       </c>
       <c r="E47" s="6" t="n">
-        <v>1084.696042940956</v>
+        <v>1787.6069951438</v>
       </c>
     </row>
     <row r="48">
@@ -4313,17 +4732,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C48" s="6" t="n">
-        <v>240.71</v>
+        <v>2102.71</v>
       </c>
       <c r="D48" s="6" t="n">
-        <v>3547.61</v>
+        <v>2324.73</v>
       </c>
       <c r="E48" s="6" t="n">
-        <v>14738.10809688006</v>
+        <v>1105.587551302842</v>
       </c>
     </row>
     <row r="49">
@@ -4334,17 +4753,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="C49" s="6" t="n">
-        <v>1097.23</v>
+        <v>240.71</v>
       </c>
       <c r="D49" s="6" t="n">
-        <v>2030.54</v>
+        <v>3547.61</v>
       </c>
       <c r="E49" s="6" t="n">
-        <v>1850.60561596019</v>
+        <v>14738.10809688006</v>
       </c>
     </row>
     <row r="50">
@@ -4355,17 +4774,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C50" s="6" t="n">
-        <v>1247.42</v>
+        <v>1686.27</v>
       </c>
       <c r="D50" s="6" t="n">
-        <v>1836.53</v>
+        <v>3082.800000000001</v>
       </c>
       <c r="E50" s="6" t="n">
-        <v>1472.262750316653</v>
+        <v>1828.17698233379</v>
       </c>
     </row>
     <row r="51">
@@ -4376,17 +4795,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C51" s="6" t="n">
-        <v>52.75</v>
+        <v>1532.05</v>
       </c>
       <c r="D51" s="6" t="n">
-        <v>158.51</v>
+        <v>2225.27</v>
       </c>
       <c r="E51" s="6" t="n">
-        <v>3004.928909952607</v>
+        <v>1452.4787050031</v>
       </c>
     </row>
     <row r="52">
@@ -4397,17 +4816,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C52" s="6" t="n">
-        <v>256.4299999999999</v>
+        <v>52.75</v>
       </c>
       <c r="D52" s="6" t="n">
-        <v>547.1199999999999</v>
+        <v>158.51</v>
       </c>
       <c r="E52" s="6" t="n">
-        <v>2133.603712514137</v>
+        <v>3004.928909952607</v>
       </c>
     </row>
     <row r="53">
@@ -4418,17 +4837,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C53" s="6" t="n">
-        <v>1994.65</v>
+        <v>256.4299999999999</v>
       </c>
       <c r="D53" s="6" t="n">
-        <v>3876.01</v>
+        <v>547.1199999999999</v>
       </c>
       <c r="E53" s="6" t="n">
-        <v>1943.203068207455</v>
+        <v>2133.603712514137</v>
       </c>
     </row>
     <row r="54">
@@ -4439,17 +4858,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C54" s="6" t="n">
-        <v>7.52</v>
+        <v>19.09</v>
       </c>
       <c r="D54" s="6" t="n">
-        <v>21.57</v>
+        <v>57.17</v>
       </c>
       <c r="E54" s="6" t="n">
-        <v>2868.351063829787</v>
+        <v>2994.76165531692</v>
       </c>
     </row>
     <row r="55">
@@ -4460,17 +4879,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C55" s="6" t="n">
-        <v>370.58</v>
+        <v>2666.57</v>
       </c>
       <c r="D55" s="6" t="n">
-        <v>1223.97</v>
+        <v>5166.57</v>
       </c>
       <c r="E55" s="6" t="n">
-        <v>3302.849587133683</v>
+        <v>1937.533985606978</v>
       </c>
     </row>
     <row r="56">
@@ -4481,17 +4900,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C56" s="6" t="n">
-        <v>301.32</v>
+        <v>22.04</v>
       </c>
       <c r="D56" s="6" t="n">
-        <v>562.62</v>
+        <v>73.03</v>
       </c>
       <c r="E56" s="6" t="n">
-        <v>1867.184388689765</v>
+        <v>3313.520871143376</v>
       </c>
     </row>
     <row r="57">
@@ -4502,17 +4921,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C57" s="6" t="n">
-        <v>19958.56</v>
+        <v>395.29</v>
       </c>
       <c r="D57" s="6" t="n">
-        <v>31146.28</v>
+        <v>1318.63</v>
       </c>
       <c r="E57" s="6" t="n">
-        <v>1560.547454325362</v>
+        <v>3335.854688962534</v>
       </c>
     </row>
     <row r="58">
@@ -4523,17 +4942,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C58" s="6" t="n">
-        <v>597.22</v>
+        <v>558.91</v>
       </c>
       <c r="D58" s="6" t="n">
-        <v>677.98</v>
+        <v>1088.48</v>
       </c>
       <c r="E58" s="6" t="n">
-        <v>1135.226549680185</v>
+        <v>1947.504965021202</v>
       </c>
     </row>
     <row r="59">
@@ -4544,17 +4963,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C59" s="6" t="n">
-        <v>217.16</v>
+        <v>37153.22</v>
       </c>
       <c r="D59" s="6" t="n">
-        <v>342.85</v>
+        <v>57365.08</v>
       </c>
       <c r="E59" s="6" t="n">
-        <v>1578.789832381654</v>
+        <v>1544.013681721261</v>
       </c>
     </row>
     <row r="60">
@@ -4565,17 +4984,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C60" s="6" t="n">
-        <v>157.8</v>
+        <v>597.22</v>
       </c>
       <c r="D60" s="6" t="n">
-        <v>256.68</v>
+        <v>677.98</v>
       </c>
       <c r="E60" s="6" t="n">
-        <v>1626.615969581749</v>
+        <v>1135.226549680185</v>
       </c>
     </row>
     <row r="61">
@@ -4586,17 +5005,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C61" s="6" t="n">
-        <v>860.5</v>
+        <v>394.15</v>
       </c>
       <c r="D61" s="6" t="n">
-        <v>2076.12</v>
+        <v>637.4400000000001</v>
       </c>
       <c r="E61" s="6" t="n">
-        <v>2412.690296339338</v>
+        <v>1617.252315108461</v>
       </c>
     </row>
     <row r="62">
@@ -4607,17 +5026,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>Morocco</t>
         </is>
       </c>
       <c r="C62" s="6" t="n">
-        <v>1455.29</v>
+        <v>157.8</v>
       </c>
       <c r="D62" s="6" t="n">
-        <v>1727.26</v>
+        <v>256.68</v>
       </c>
       <c r="E62" s="6" t="n">
-        <v>1186.883713898948</v>
+        <v>1626.615969581749</v>
       </c>
     </row>
     <row r="63">
@@ -4628,17 +5047,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C63" s="6" t="n">
-        <v>25.1</v>
+        <v>1166.08</v>
       </c>
       <c r="D63" s="6" t="n">
-        <v>54</v>
+        <v>2601.2</v>
       </c>
       <c r="E63" s="6" t="n">
-        <v>2151.394422310757</v>
+        <v>2230.721734357848</v>
       </c>
     </row>
     <row r="64">
@@ -4649,17 +5068,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="C64" s="6" t="n">
-        <v>99.50999999999999</v>
+        <v>1455.29</v>
       </c>
       <c r="D64" s="6" t="n">
-        <v>291.25</v>
+        <v>1727.26</v>
       </c>
       <c r="E64" s="6" t="n">
-        <v>2926.841523464979</v>
+        <v>1186.883713898948</v>
       </c>
     </row>
     <row r="65">
@@ -4670,17 +5089,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C65" s="6" t="n">
-        <v>175.3</v>
+        <v>25.1</v>
       </c>
       <c r="D65" s="6" t="n">
-        <v>218.79</v>
+        <v>54</v>
       </c>
       <c r="E65" s="6" t="n">
-        <v>1248.088990302339</v>
+        <v>2151.394422310757</v>
       </c>
     </row>
     <row r="66">
@@ -4691,17 +5110,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="C66" s="6" t="n">
-        <v>297.41</v>
+        <v>99.50999999999999</v>
       </c>
       <c r="D66" s="6" t="n">
-        <v>406.74</v>
+        <v>291.25</v>
       </c>
       <c r="E66" s="6" t="n">
-        <v>1367.60700716183</v>
+        <v>2926.841523464979</v>
       </c>
     </row>
     <row r="67">
@@ -4712,17 +5131,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="C67" s="6" t="n">
-        <v>7469.95</v>
+        <v>219.82</v>
       </c>
       <c r="D67" s="6" t="n">
-        <v>8780.879999999999</v>
+        <v>274.41</v>
       </c>
       <c r="E67" s="6" t="n">
-        <v>1175.493811872904</v>
+        <v>1248.339550541352</v>
       </c>
     </row>
     <row r="68">
@@ -4733,17 +5152,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C68" s="6" t="n">
-        <v>308.38</v>
+        <v>297.41</v>
       </c>
       <c r="D68" s="6" t="n">
-        <v>402.99</v>
+        <v>406.74</v>
       </c>
       <c r="E68" s="6" t="n">
-        <v>1306.796809131591</v>
+        <v>1367.60700716183</v>
       </c>
     </row>
     <row r="69">
@@ -4754,17 +5173,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="C69" s="6" t="n">
-        <v>85.08</v>
+        <v>0</v>
       </c>
       <c r="D69" s="6" t="n">
-        <v>129.62</v>
+        <v>0</v>
       </c>
       <c r="E69" s="6" t="n">
-        <v>1523.50728725905</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70">
@@ -4775,17 +5194,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C70" s="6" t="n">
-        <v>3651.25</v>
+        <v>15863.96</v>
       </c>
       <c r="D70" s="6" t="n">
-        <v>4974.879999999999</v>
+        <v>20216.67</v>
       </c>
       <c r="E70" s="6" t="n">
-        <v>1362.514207463197</v>
+        <v>1274.377267718779</v>
       </c>
     </row>
     <row r="71">
@@ -4796,17 +5215,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C71" s="6" t="n">
-        <v>57197.30999999998</v>
+        <v>308.38</v>
       </c>
       <c r="D71" s="6" t="n">
-        <v>110282.55</v>
+        <v>402.99</v>
       </c>
       <c r="E71" s="6" t="n">
-        <v>1928.107283366999</v>
+        <v>1306.796809131591</v>
       </c>
     </row>
     <row r="72">
@@ -4817,80 +5236,80 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C72" s="6" t="n">
-        <v>1461.61</v>
+        <v>4504.51</v>
       </c>
       <c r="D72" s="6" t="n">
-        <v>2099.690000000001</v>
+        <v>4830.77</v>
       </c>
       <c r="E72" s="6" t="n">
-        <v>1436.55968418388</v>
+        <v>1072.429631635849</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Cambodia</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="C73" s="6" t="n">
-        <v>3899.08</v>
+        <v>4173.55</v>
       </c>
       <c r="D73" s="6" t="n">
-        <v>2995.72</v>
+        <v>5582.879999999999</v>
       </c>
       <c r="E73" s="6" t="n">
-        <v>768.3145767719565</v>
+        <v>1337.681350409124</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C74" s="6" t="n">
-        <v>156.65</v>
+        <v>63768.26999999997</v>
       </c>
       <c r="D74" s="6" t="n">
-        <v>65.61</v>
+        <v>123401.21</v>
       </c>
       <c r="E74" s="6" t="n">
-        <v>418.8317906160231</v>
+        <v>1935.150663488284</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C75" s="6" t="n">
-        <v>44</v>
+        <v>1776.87</v>
       </c>
       <c r="D75" s="6" t="n">
-        <v>81.67</v>
+        <v>2549.12</v>
       </c>
       <c r="E75" s="6" t="n">
-        <v>1856.136363636364</v>
+        <v>1434.61254903285</v>
       </c>
     </row>
     <row r="76">
@@ -4901,17 +5320,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Cambodia</t>
         </is>
       </c>
       <c r="C76" s="6" t="n">
-        <v>12083.72</v>
+        <v>13898.96</v>
       </c>
       <c r="D76" s="6" t="n">
-        <v>11452.17</v>
+        <v>11272.91</v>
       </c>
       <c r="E76" s="6" t="n">
-        <v>947.7354655685502</v>
+        <v>811.061403155344</v>
       </c>
     </row>
     <row r="77">
@@ -4922,17 +5341,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Greece</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C77" s="6" t="n">
-        <v>2957.11</v>
+        <v>156.65</v>
       </c>
       <c r="D77" s="6" t="n">
-        <v>2514.12</v>
+        <v>65.61</v>
       </c>
       <c r="E77" s="6" t="n">
-        <v>850.1949538569752</v>
+        <v>418.8317906160231</v>
       </c>
     </row>
     <row r="78">
@@ -4943,17 +5362,17 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="C78" s="6" t="n">
-        <v>1879.78</v>
+        <v>44</v>
       </c>
       <c r="D78" s="6" t="n">
-        <v>1188.11</v>
+        <v>81.67</v>
       </c>
       <c r="E78" s="6" t="n">
-        <v>632.0473672451033</v>
+        <v>1856.136363636364</v>
       </c>
     </row>
     <row r="79">
@@ -4964,17 +5383,17 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C79" s="6" t="n">
-        <v>3899.08</v>
+        <v>12083.72</v>
       </c>
       <c r="D79" s="6" t="n">
-        <v>3015.8</v>
+        <v>11452.17</v>
       </c>
       <c r="E79" s="6" t="n">
-        <v>773.4645095766181</v>
+        <v>947.7354655685502</v>
       </c>
     </row>
     <row r="80">
@@ -4985,17 +5404,17 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Greece</t>
         </is>
       </c>
       <c r="C80" s="6" t="n">
-        <v>7317.469999999999</v>
+        <v>11145.09</v>
       </c>
       <c r="D80" s="6" t="n">
-        <v>8917.290000000001</v>
+        <v>9520.82</v>
       </c>
       <c r="E80" s="6" t="n">
-        <v>1218.630209621632</v>
+        <v>854.2613832638408</v>
       </c>
     </row>
     <row r="81">
@@ -5006,17 +5425,17 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Peru</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C81" s="6" t="n">
-        <v>2391.98</v>
+        <v>1879.78</v>
       </c>
       <c r="D81" s="6" t="n">
-        <v>2225.46</v>
+        <v>1188.11</v>
       </c>
       <c r="E81" s="6" t="n">
-        <v>930.3840333113153</v>
+        <v>632.0473672451033</v>
       </c>
     </row>
     <row r="82">
@@ -5027,17 +5446,17 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="C82" s="6" t="n">
-        <v>4384.48</v>
+        <v>3899.08</v>
       </c>
       <c r="D82" s="6" t="n">
-        <v>4625.09</v>
+        <v>3015.8</v>
       </c>
       <c r="E82" s="6" t="n">
-        <v>1054.87765938036</v>
+        <v>773.4645095766181</v>
       </c>
     </row>
     <row r="83">
@@ -5048,17 +5467,17 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C83" s="6" t="n">
-        <v>324.21</v>
+        <v>7815.87</v>
       </c>
       <c r="D83" s="6" t="n">
-        <v>504.71</v>
+        <v>9533.76</v>
       </c>
       <c r="E83" s="6" t="n">
-        <v>1556.737916782333</v>
+        <v>1219.795109181703</v>
       </c>
     </row>
     <row r="84">
@@ -5069,17 +5488,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Peru</t>
         </is>
       </c>
       <c r="C84" s="6" t="n">
-        <v>439.91</v>
+        <v>7080.98</v>
       </c>
       <c r="D84" s="6" t="n">
-        <v>464.35</v>
+        <v>6563.85</v>
       </c>
       <c r="E84" s="6" t="n">
-        <v>1055.556818440135</v>
+        <v>926.9691483382244</v>
       </c>
     </row>
     <row r="85">
@@ -5090,101 +5509,101 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="C85" s="6" t="n">
-        <v>2038.59</v>
+        <v>9938.370000000001</v>
       </c>
       <c r="D85" s="6" t="n">
-        <v>3070.56</v>
+        <v>8618.030000000001</v>
       </c>
       <c r="E85" s="6" t="n">
-        <v>1506.21753270643</v>
+        <v>867.1472283684346</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="C86" s="6" t="n">
-        <v>0.42</v>
+        <v>4384.48</v>
       </c>
       <c r="D86" s="6" t="n">
-        <v>1.37</v>
+        <v>4625.09</v>
       </c>
       <c r="E86" s="6" t="n">
-        <v>3261.904761904762</v>
+        <v>1054.87765938036</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C87" s="6" t="n">
-        <v>13.53</v>
+        <v>324.21</v>
       </c>
       <c r="D87" s="6" t="n">
-        <v>26.23</v>
+        <v>504.71</v>
       </c>
       <c r="E87" s="6" t="n">
-        <v>1938.654841093865</v>
+        <v>1556.737916782333</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="C88" s="6" t="n">
-        <v>251.04</v>
+        <v>1811.46</v>
       </c>
       <c r="D88" s="6" t="n">
-        <v>225.12</v>
+        <v>1874.02</v>
       </c>
       <c r="E88" s="6" t="n">
-        <v>896.7495219885277</v>
+        <v>1034.535678403056</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C89" s="6" t="n">
-        <v>7.8</v>
+        <v>2379.76</v>
       </c>
       <c r="D89" s="6" t="n">
-        <v>15.24</v>
+        <v>3587.98</v>
       </c>
       <c r="E89" s="6" t="n">
-        <v>1953.846153846154</v>
+        <v>1507.706659495075</v>
       </c>
     </row>
     <row r="90">
@@ -5195,17 +5614,17 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C90" s="6" t="n">
-        <v>114.53</v>
+        <v>0.42</v>
       </c>
       <c r="D90" s="6" t="n">
-        <v>144.92</v>
+        <v>1.37</v>
       </c>
       <c r="E90" s="6" t="n">
-        <v>1265.345324369161</v>
+        <v>3261.904761904762</v>
       </c>
     </row>
     <row r="91">
@@ -5216,17 +5635,17 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C91" s="6" t="n">
-        <v>4.26</v>
+        <v>13.53</v>
       </c>
       <c r="D91" s="6" t="n">
-        <v>5.81</v>
+        <v>26.23</v>
       </c>
       <c r="E91" s="6" t="n">
-        <v>1363.849765258216</v>
+        <v>1938.654841093865</v>
       </c>
     </row>
     <row r="92">
@@ -5237,17 +5656,17 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C92" s="6" t="n">
-        <v>10.78</v>
+        <v>302.23</v>
       </c>
       <c r="D92" s="6" t="n">
-        <v>27.53</v>
+        <v>311.01</v>
       </c>
       <c r="E92" s="6" t="n">
-        <v>2553.803339517625</v>
+        <v>1029.050722959336</v>
       </c>
     </row>
     <row r="93">
@@ -5258,17 +5677,17 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="C93" s="6" t="n">
-        <v>0.17</v>
+        <v>7.96</v>
       </c>
       <c r="D93" s="6" t="n">
-        <v>0.84</v>
+        <v>15.56</v>
       </c>
       <c r="E93" s="6" t="n">
-        <v>4941.176470588235</v>
+        <v>1954.773869346734</v>
       </c>
     </row>
     <row r="94">
@@ -5279,17 +5698,17 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="C94" s="6" t="n">
-        <v>776.99</v>
+        <v>19.32</v>
       </c>
       <c r="D94" s="6" t="n">
-        <v>1062.9</v>
+        <v>39.73</v>
       </c>
       <c r="E94" s="6" t="n">
-        <v>1367.971273761567</v>
+        <v>2056.418219461698</v>
       </c>
     </row>
     <row r="95">
@@ -5300,17 +5719,17 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C95" s="6" t="n">
-        <v>0.6899999999999999</v>
+        <v>166.15</v>
       </c>
       <c r="D95" s="6" t="n">
-        <v>2.83</v>
+        <v>212.56</v>
       </c>
       <c r="E95" s="6" t="n">
-        <v>4101.449275362319</v>
+        <v>1279.325910321998</v>
       </c>
     </row>
     <row r="96">
@@ -5321,17 +5740,17 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C96" s="6" t="n">
-        <v>58.38</v>
+        <v>4.26</v>
       </c>
       <c r="D96" s="6" t="n">
-        <v>101.44</v>
+        <v>5.81</v>
       </c>
       <c r="E96" s="6" t="n">
-        <v>1737.581363480644</v>
+        <v>1363.849765258216</v>
       </c>
     </row>
     <row r="97">
@@ -5342,17 +5761,17 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C97" s="6" t="n">
-        <v>1647.26</v>
+        <v>11.83</v>
       </c>
       <c r="D97" s="6" t="n">
-        <v>1590.47</v>
+        <v>30.95</v>
       </c>
       <c r="E97" s="6" t="n">
-        <v>965.5245680706144</v>
+        <v>2616.229923922232</v>
       </c>
     </row>
     <row r="98">
@@ -5363,17 +5782,17 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C98" s="6" t="n">
-        <v>1677.88</v>
+        <v>0.63</v>
       </c>
       <c r="D98" s="6" t="n">
-        <v>1868.25</v>
+        <v>1.97</v>
       </c>
       <c r="E98" s="6" t="n">
-        <v>1113.458650201444</v>
+        <v>3126.984126984127</v>
       </c>
     </row>
     <row r="99">
@@ -5384,17 +5803,17 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C99" s="6" t="n">
-        <v>10.04</v>
+        <v>797.6600000000001</v>
       </c>
       <c r="D99" s="6" t="n">
-        <v>43.44</v>
+        <v>1062.6</v>
       </c>
       <c r="E99" s="6" t="n">
-        <v>4326.693227091633</v>
+        <v>1332.146528596144</v>
       </c>
     </row>
     <row r="100">
@@ -5405,122 +5824,122 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="C100" s="6" t="n">
-        <v>6327.199999999999</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="D100" s="6" t="n">
-        <v>11487.06</v>
+        <v>2.83</v>
       </c>
       <c r="E100" s="6" t="n">
-        <v>1815.50448855734</v>
+        <v>4101.449275362319</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C101" s="6" t="n">
-        <v>1314.16</v>
+        <v>77.03999999999999</v>
       </c>
       <c r="D101" s="6" t="n">
-        <v>1770.94</v>
+        <v>134.76</v>
       </c>
       <c r="E101" s="6" t="n">
-        <v>1347.5832470932</v>
+        <v>1749.221183800624</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C102" s="6" t="n">
-        <v>205.63</v>
+        <v>2452.06</v>
       </c>
       <c r="D102" s="6" t="n">
-        <v>139.64</v>
+        <v>2368.9</v>
       </c>
       <c r="E102" s="6" t="n">
-        <v>679.0837912755923</v>
+        <v>966.0856585891047</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C103" s="6" t="n">
-        <v>4488.21</v>
+        <v>2190.81</v>
       </c>
       <c r="D103" s="6" t="n">
-        <v>6577.24</v>
+        <v>2332.4</v>
       </c>
       <c r="E103" s="6" t="n">
-        <v>1465.448363601525</v>
+        <v>1064.629064136096</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Greece</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C104" s="6" t="n">
-        <v>198.08</v>
+        <v>10.47</v>
       </c>
       <c r="D104" s="6" t="n">
-        <v>175.53</v>
+        <v>45.46</v>
       </c>
       <c r="E104" s="6" t="n">
-        <v>886.1571082390952</v>
+        <v>4341.929321872015</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C105" s="6" t="n">
-        <v>12348.33</v>
+        <v>6790.009999999999</v>
       </c>
       <c r="D105" s="6" t="n">
-        <v>12312.31</v>
+        <v>12268.18</v>
       </c>
       <c r="E105" s="6" t="n">
-        <v>997.083006366043</v>
+        <v>1806.798517233406</v>
       </c>
     </row>
     <row r="106">
@@ -5531,17 +5950,17 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C106" s="6" t="n">
-        <v>593.8200000000001</v>
+        <v>1314.16</v>
       </c>
       <c r="D106" s="6" t="n">
-        <v>703.6800000000001</v>
+        <v>1770.94</v>
       </c>
       <c r="E106" s="6" t="n">
-        <v>1185.005557239568</v>
+        <v>1347.5832470932</v>
       </c>
     </row>
     <row r="107">
@@ -5552,17 +5971,17 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C107" s="6" t="n">
-        <v>185.81</v>
+        <v>205.63</v>
       </c>
       <c r="D107" s="6" t="n">
-        <v>243.39</v>
+        <v>139.64</v>
       </c>
       <c r="E107" s="6" t="n">
-        <v>1309.886443140843</v>
+        <v>679.0837912755923</v>
       </c>
     </row>
     <row r="108">
@@ -5573,17 +5992,17 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C108" s="6" t="n">
-        <v>1722.13</v>
+        <v>7282.92</v>
       </c>
       <c r="D108" s="6" t="n">
-        <v>1452.3</v>
+        <v>10975.99</v>
       </c>
       <c r="E108" s="6" t="n">
-        <v>843.3161259602934</v>
+        <v>1507.086443349645</v>
       </c>
     </row>
     <row r="109">
@@ -5594,17 +6013,17 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Greece</t>
         </is>
       </c>
       <c r="C109" s="6" t="n">
-        <v>20.52</v>
+        <v>1217.18</v>
       </c>
       <c r="D109" s="6" t="n">
-        <v>28.52</v>
+        <v>1078.62</v>
       </c>
       <c r="E109" s="6" t="n">
-        <v>1389.863547758285</v>
+        <v>886.1630983092065</v>
       </c>
     </row>
     <row r="110">
@@ -5615,122 +6034,122 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C110" s="6" t="n">
-        <v>8887.820000000002</v>
+        <v>12348.33</v>
       </c>
       <c r="D110" s="6" t="n">
-        <v>12105.48</v>
+        <v>12312.31</v>
       </c>
       <c r="E110" s="6" t="n">
-        <v>1362.030284141668</v>
+        <v>997.083006366043</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C111" s="6" t="n">
-        <v>1871.11</v>
+        <v>674.6899999999998</v>
       </c>
       <c r="D111" s="6" t="n">
-        <v>1741.11</v>
+        <v>801.9900000000001</v>
       </c>
       <c r="E111" s="6" t="n">
-        <v>930.522524063257</v>
+        <v>1188.679245283019</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C112" s="6" t="n">
-        <v>0.08</v>
+        <v>185.81</v>
       </c>
       <c r="D112" s="6" t="n">
-        <v>0.34</v>
+        <v>243.39</v>
       </c>
       <c r="E112" s="6" t="n">
-        <v>4250</v>
+        <v>1309.886443140843</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C113" s="6" t="n">
-        <v>2.1</v>
+        <v>1722.13</v>
       </c>
       <c r="D113" s="6" t="n">
-        <v>6.87</v>
+        <v>1452.3</v>
       </c>
       <c r="E113" s="6" t="n">
-        <v>3271.428571428571</v>
+        <v>843.3161259602934</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C114" s="6" t="n">
-        <v>20.41</v>
+        <v>41.24</v>
       </c>
       <c r="D114" s="6" t="n">
-        <v>41.37</v>
+        <v>57.11</v>
       </c>
       <c r="E114" s="6" t="n">
-        <v>2026.947574718276</v>
+        <v>1384.820562560621</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C115" s="6" t="n">
-        <v>177.25</v>
+        <v>9673.599999999999</v>
       </c>
       <c r="D115" s="6" t="n">
-        <v>673.3299999999999</v>
+        <v>13220.43</v>
       </c>
       <c r="E115" s="6" t="n">
-        <v>3798.758815232722</v>
+        <v>1366.650471386041</v>
       </c>
     </row>
     <row r="116">
@@ -5741,17 +6160,17 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C116" s="6" t="n">
-        <v>221.75</v>
+        <v>2854.6</v>
       </c>
       <c r="D116" s="6" t="n">
-        <v>484.19</v>
+        <v>2533.12</v>
       </c>
       <c r="E116" s="6" t="n">
-        <v>2183.494926719278</v>
+        <v>887.3817697750999</v>
       </c>
     </row>
     <row r="117">
@@ -5762,17 +6181,17 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="C117" s="6" t="n">
-        <v>28.4</v>
+        <v>0.08</v>
       </c>
       <c r="D117" s="6" t="n">
-        <v>95.00999999999999</v>
+        <v>0.34</v>
       </c>
       <c r="E117" s="6" t="n">
-        <v>3345.422535211267</v>
+        <v>4250</v>
       </c>
     </row>
     <row r="118">
@@ -5783,17 +6202,17 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="C118" s="6" t="n">
-        <v>115.61</v>
+        <v>2.1</v>
       </c>
       <c r="D118" s="6" t="n">
-        <v>238.04</v>
+        <v>6.87</v>
       </c>
       <c r="E118" s="6" t="n">
-        <v>2058.991436726927</v>
+        <v>3271.428571428571</v>
       </c>
     </row>
     <row r="119">
@@ -5804,17 +6223,17 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C119" s="6" t="n">
-        <v>17759.65</v>
+        <v>20.41</v>
       </c>
       <c r="D119" s="6" t="n">
-        <v>19078.07</v>
+        <v>41.37</v>
       </c>
       <c r="E119" s="6" t="n">
-        <v>1074.236823360821</v>
+        <v>2026.947574718276</v>
       </c>
     </row>
     <row r="120">
@@ -5825,17 +6244,17 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C120" s="6" t="n">
-        <v>4468.509999999999</v>
+        <v>180.55</v>
       </c>
       <c r="D120" s="6" t="n">
-        <v>6739.87</v>
+        <v>686.2099999999999</v>
       </c>
       <c r="E120" s="6" t="n">
-        <v>1508.303662742167</v>
+        <v>3800.664635834949</v>
       </c>
     </row>
     <row r="121">
@@ -5846,17 +6265,17 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C121" s="6" t="n">
-        <v>8204.919999999998</v>
+        <v>276.78</v>
       </c>
       <c r="D121" s="6" t="n">
-        <v>11006.31</v>
+        <v>557.1</v>
       </c>
       <c r="E121" s="6" t="n">
-        <v>1341.428069987276</v>
+        <v>2012.789941469759</v>
       </c>
     </row>
     <row r="122">
@@ -5867,17 +6286,17 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Panama</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C122" s="6" t="n">
-        <v>11.76</v>
+        <v>31.83</v>
       </c>
       <c r="D122" s="6" t="n">
-        <v>27.41</v>
+        <v>110.5</v>
       </c>
       <c r="E122" s="6" t="n">
-        <v>2330.78231292517</v>
+        <v>3471.567703424443</v>
       </c>
     </row>
     <row r="123">
@@ -5888,17 +6307,17 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C123" s="6" t="n">
-        <v>0.46</v>
+        <v>115.61</v>
       </c>
       <c r="D123" s="6" t="n">
-        <v>1.79</v>
+        <v>238.04</v>
       </c>
       <c r="E123" s="6" t="n">
-        <v>3891.304347826087</v>
+        <v>2058.991436726927</v>
       </c>
     </row>
     <row r="124">
@@ -5909,17 +6328,17 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C124" s="6" t="n">
-        <v>13113.65</v>
+        <v>29106.32</v>
       </c>
       <c r="D124" s="6" t="n">
-        <v>13899.15</v>
+        <v>31748.18</v>
       </c>
       <c r="E124" s="6" t="n">
-        <v>1059.899417782234</v>
+        <v>1090.765854288691</v>
       </c>
     </row>
     <row r="125">
@@ -5930,17 +6349,17 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Luxembourg</t>
         </is>
       </c>
       <c r="C125" s="6" t="n">
-        <v>1119.84</v>
+        <v>10421.4</v>
       </c>
       <c r="D125" s="6" t="n">
-        <v>1082.06</v>
+        <v>15291.51</v>
       </c>
       <c r="E125" s="6" t="n">
-        <v>966.2630375767966</v>
+        <v>1467.318210605101</v>
       </c>
     </row>
     <row r="126">
@@ -5951,17 +6370,17 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C126" s="6" t="n">
-        <v>8477.610000000001</v>
+        <v>9479.65</v>
       </c>
       <c r="D126" s="6" t="n">
-        <v>7530.9</v>
+        <v>12727.56</v>
       </c>
       <c r="E126" s="6" t="n">
-        <v>888.3281962722983</v>
+        <v>1342.619189527039</v>
       </c>
     </row>
     <row r="127">
@@ -5972,17 +6391,17 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Oman</t>
         </is>
       </c>
       <c r="C127" s="6" t="n">
-        <v>3180.37</v>
+        <v>149.33</v>
       </c>
       <c r="D127" s="6" t="n">
-        <v>3831.62</v>
+        <v>126.64</v>
       </c>
       <c r="E127" s="6" t="n">
-        <v>1204.771771837868</v>
+        <v>848.0546440768767</v>
       </c>
     </row>
     <row r="128">
@@ -5993,17 +6412,17 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Panama</t>
         </is>
       </c>
       <c r="C128" s="6" t="n">
-        <v>321.25</v>
+        <v>11.76</v>
       </c>
       <c r="D128" s="6" t="n">
-        <v>729.84</v>
+        <v>27.41</v>
       </c>
       <c r="E128" s="6" t="n">
-        <v>2271.875486381323</v>
+        <v>2330.78231292517</v>
       </c>
     </row>
     <row r="129">
@@ -6014,17 +6433,17 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C129" s="6" t="n">
-        <v>8529.469999999999</v>
+        <v>0.52</v>
       </c>
       <c r="D129" s="6" t="n">
-        <v>9778.500000000002</v>
+        <v>2.05</v>
       </c>
       <c r="E129" s="6" t="n">
-        <v>1146.437000188758</v>
+        <v>3942.307692307693</v>
       </c>
     </row>
     <row r="130">
@@ -6035,17 +6454,17 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C130" s="6" t="n">
-        <v>14377.29</v>
+        <v>13134.23</v>
       </c>
       <c r="D130" s="6" t="n">
-        <v>31020.93</v>
+        <v>13980.22</v>
       </c>
       <c r="E130" s="6" t="n">
-        <v>2157.634018650246</v>
+        <v>1064.411084623917</v>
       </c>
     </row>
     <row r="131">
@@ -6056,17 +6475,143 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="C131" s="6" t="n">
+        <v>2110.63</v>
+      </c>
+      <c r="D131" s="6" t="n">
+        <v>2060.19</v>
+      </c>
+      <c r="E131" s="6" t="n">
+        <v>976.1019221748955</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C132" s="6" t="n">
+        <v>8477.610000000001</v>
+      </c>
+      <c r="D132" s="6" t="n">
+        <v>7530.9</v>
+      </c>
+      <c r="E132" s="6" t="n">
+        <v>888.3281962722983</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C133" s="6" t="n">
+        <v>5361.25</v>
+      </c>
+      <c r="D133" s="6" t="n">
+        <v>6273.17</v>
+      </c>
+      <c r="E133" s="6" t="n">
+        <v>1170.094660760084</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="C134" s="6" t="n">
+        <v>7790.639999999999</v>
+      </c>
+      <c r="D134" s="6" t="n">
+        <v>8569.17</v>
+      </c>
+      <c r="E134" s="6" t="n">
+        <v>1099.931456208989</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C135" s="6" t="n">
+        <v>8533.51</v>
+      </c>
+      <c r="D135" s="6" t="n">
+        <v>9798.160000000002</v>
+      </c>
+      <c r="E135" s="6" t="n">
+        <v>1148.198103711134</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C136" s="6" t="n">
+        <v>17033.72</v>
+      </c>
+      <c r="D136" s="6" t="n">
+        <v>36661.47999999999</v>
+      </c>
+      <c r="E136" s="6" t="n">
+        <v>2152.288519477835</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
           <t>Vietnam</t>
         </is>
       </c>
-      <c r="C131" s="6" t="n">
-        <v>48.44</v>
-      </c>
-      <c r="D131" s="6" t="n">
-        <v>45.15</v>
-      </c>
-      <c r="E131" s="6" t="n">
-        <v>932.0809248554914</v>
+      <c r="C137" s="6" t="n">
+        <v>952.6800000000001</v>
+      </c>
+      <c r="D137" s="6" t="n">
+        <v>939.7900000000001</v>
+      </c>
+      <c r="E137" s="6" t="n">
+        <v>986.4697484989714</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Weekly TRQ update 2026-04-27
</commit_message>
<xml_diff>
--- a/data/canada_trq_tracker.xlsx
+++ b/data/canada_trq_tracker.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,6 +481,11 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
+          <t>April 27 2026</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>OVER</t>
         </is>
       </c>
@@ -514,6 +519,9 @@
       <c r="H3" s="4" t="n">
         <v>0.0053</v>
       </c>
+      <c r="I3" s="4" t="n">
+        <v>0.0054</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -544,6 +552,9 @@
       <c r="H4" s="4" t="n">
         <v>0.0018</v>
       </c>
+      <c r="I4" s="4" t="n">
+        <v>0.0018</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -574,7 +585,10 @@
       <c r="H5" s="4" t="n">
         <v>0.41</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="4" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -607,6 +621,10 @@
         <f>SUM(H3:H5)</f>
         <v/>
       </c>
+      <c r="I6" s="5">
+        <f>SUM(I3:I5)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -637,6 +655,14 @@
       <c r="H7" s="4" t="n">
         <v>0.353</v>
       </c>
+      <c r="I7" s="4" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -667,6 +693,9 @@
       <c r="H8" s="4" t="n">
         <v>0.0172</v>
       </c>
+      <c r="I8" s="4" t="n">
+        <v>0.0172</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -695,6 +724,10 @@
         <f>SUM(H7:H8)</f>
         <v/>
       </c>
+      <c r="I9" s="5">
+        <f>SUM(I7:I8)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -725,6 +758,9 @@
       <c r="H10" s="4" t="n">
         <v>0.0024</v>
       </c>
+      <c r="I10" s="4" t="n">
+        <v>0.0024</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -755,6 +791,9 @@
       <c r="H11" s="4" t="n">
         <v>0.0024</v>
       </c>
+      <c r="I11" s="4" t="n">
+        <v>0.0026</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -785,6 +824,9 @@
       <c r="H12" s="4" t="n">
         <v>0.0421</v>
       </c>
+      <c r="I12" s="4" t="n">
+        <v>0.0421</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -815,6 +857,9 @@
       <c r="H13" s="4" t="n">
         <v>0.2512</v>
       </c>
+      <c r="I13" s="4" t="n">
+        <v>0.2512</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -836,6 +881,9 @@
       <c r="H14" s="4" t="n">
         <v>0.0133</v>
       </c>
+      <c r="I14" s="4" t="n">
+        <v>0.0262</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -864,6 +912,10 @@
         <f>SUM(H10:H14)</f>
         <v/>
       </c>
+      <c r="I15" s="5">
+        <f>SUM(I10:I14)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -894,6 +946,9 @@
       <c r="H16" s="4" t="n">
         <v>0.007900000000000001</v>
       </c>
+      <c r="I16" s="4" t="n">
+        <v>0.008</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -924,6 +979,9 @@
       <c r="H17" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="I17" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -954,6 +1012,9 @@
       <c r="H18" s="4" t="n">
         <v>0.0135</v>
       </c>
+      <c r="I18" s="4" t="n">
+        <v>0.0135</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -984,6 +1045,9 @@
       <c r="H19" s="4" t="n">
         <v>0.0119</v>
       </c>
+      <c r="I19" s="4" t="n">
+        <v>0.0119</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1014,6 +1078,9 @@
       <c r="H20" s="4" t="n">
         <v>0.3641</v>
       </c>
+      <c r="I20" s="4" t="n">
+        <v>0.3695000000000001</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1044,6 +1111,9 @@
       <c r="H21" s="4" t="n">
         <v>0.0086</v>
       </c>
+      <c r="I21" s="4" t="n">
+        <v>0.1327</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1074,6 +1144,9 @@
       <c r="H22" s="4" t="n">
         <v>0.3262</v>
       </c>
+      <c r="I22" s="4" t="n">
+        <v>0.3262</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1104,6 +1177,9 @@
       <c r="H23" s="4" t="n">
         <v>0.0455</v>
       </c>
+      <c r="I23" s="4" t="n">
+        <v>0.0455</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1125,6 +1201,9 @@
       <c r="H24" s="4" t="n">
         <v>0.0025</v>
       </c>
+      <c r="I24" s="4" t="n">
+        <v>0.0025</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1153,6 +1232,10 @@
         <f>SUM(H16:H24)</f>
         <v/>
       </c>
+      <c r="I25" s="5">
+        <f>SUM(I16:I24)</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1183,7 +1266,10 @@
       <c r="H26" s="4" t="n">
         <v>0.29</v>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="I26" s="4" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="J26" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -1218,6 +1304,9 @@
       <c r="H27" s="4" t="n">
         <v>0.1228</v>
       </c>
+      <c r="I27" s="4" t="n">
+        <v>0.1228</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1248,6 +1337,9 @@
       <c r="H28" s="4" t="n">
         <v>0.2394</v>
       </c>
+      <c r="I28" s="4" t="n">
+        <v>0.2394</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1278,6 +1370,9 @@
       <c r="H29" s="4" t="n">
         <v>0.1668</v>
       </c>
+      <c r="I29" s="4" t="n">
+        <v>0.1668</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1308,6 +1403,9 @@
       <c r="H30" s="4" t="n">
         <v>0.0241</v>
       </c>
+      <c r="I30" s="4" t="n">
+        <v>0.0241</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1338,6 +1436,9 @@
       <c r="H31" s="4" t="n">
         <v>0.1569</v>
       </c>
+      <c r="I31" s="4" t="n">
+        <v>0.1569</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1366,6 +1467,10 @@
         <f>SUM(H24:H29)</f>
         <v/>
       </c>
+      <c r="I32" s="5">
+        <f>SUM(I26:I31)</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1396,6 +1501,9 @@
       <c r="H33" s="4" t="n">
         <v>0.016</v>
       </c>
+      <c r="I33" s="4" t="n">
+        <v>0.0162</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1426,6 +1534,9 @@
       <c r="H34" s="4" t="n">
         <v>0.2784</v>
       </c>
+      <c r="I34" s="4" t="n">
+        <v>0.2784</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1456,6 +1567,9 @@
       <c r="H35" s="4" t="n">
         <v>0.3114</v>
       </c>
+      <c r="I35" s="4" t="n">
+        <v>0.3114</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1486,6 +1600,9 @@
       <c r="H36" s="4" t="n">
         <v>0.2078</v>
       </c>
+      <c r="I36" s="4" t="n">
+        <v>0.2264</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1510,6 +1627,9 @@
       <c r="H37" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="I37" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1538,6 +1658,10 @@
         <f>SUM(H31:H35)</f>
         <v/>
       </c>
+      <c r="I38" s="5">
+        <f>SUM(I33:I37)</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1568,6 +1692,9 @@
       <c r="H39" s="4" t="n">
         <v>0.1514</v>
       </c>
+      <c r="I39" s="4" t="n">
+        <v>0.1514</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1577,54 +1704,49 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E40" s="5">
-        <f>SUM(E36:E36)</f>
-        <v/>
-      </c>
-      <c r="F40" s="5">
-        <f>SUM(F36:F36)</f>
-        <v/>
-      </c>
-      <c r="G40" s="5">
-        <f>SUM(G36:G36)</f>
-        <v/>
-      </c>
-      <c r="H40" s="5">
-        <f>SUM(H37:H37)</f>
-        <v/>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="n">
+        <v>1571700</v>
+      </c>
+      <c r="D40" s="4" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="I40" s="4" t="n">
+        <v>0.3047</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>China</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="n">
-        <v>4674200</v>
-      </c>
-      <c r="D41" s="4" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="E41" s="4" t="n">
-        <v>0.0359</v>
-      </c>
-      <c r="F41" s="4" t="n">
-        <v>0.0408</v>
-      </c>
-      <c r="G41" s="4" t="n">
-        <v>0.0412</v>
-      </c>
-      <c r="H41" s="4" t="n">
-        <v>0.0412</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E41" s="5">
+        <f>SUM(E36:E36)</f>
+        <v/>
+      </c>
+      <c r="F41" s="5">
+        <f>SUM(F36:F36)</f>
+        <v/>
+      </c>
+      <c r="G41" s="5">
+        <f>SUM(G36:G36)</f>
+        <v/>
+      </c>
+      <c r="H41" s="5">
+        <f>SUM(H37:H37)</f>
+        <v/>
+      </c>
+      <c r="I41" s="5">
+        <f>SUM(I39:I40)</f>
+        <v/>
       </c>
     </row>
     <row r="42">
@@ -1635,7 +1757,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C42" s="3" t="n">
@@ -1645,16 +1767,19 @@
         <v>0.55</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>0.0177</v>
+        <v>0.0359</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>0.0236</v>
+        <v>0.0408</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>0.0236</v>
+        <v>0.0412</v>
       </c>
       <c r="H42" s="4" t="n">
-        <v>0.0236</v>
+        <v>0.0412</v>
+      </c>
+      <c r="I42" s="4" t="n">
+        <v>0.0412</v>
       </c>
     </row>
     <row r="43">
@@ -1665,7 +1790,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C43" s="3" t="n">
@@ -1675,16 +1800,19 @@
         <v>0.55</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>0.2154</v>
+        <v>0.0177</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>0.2154</v>
+        <v>0.0236</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>0.3917</v>
+        <v>0.0236</v>
       </c>
       <c r="H43" s="4" t="n">
-        <v>0.3917</v>
+        <v>0.0236</v>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>0.0236</v>
       </c>
     </row>
     <row r="44">
@@ -1695,7 +1823,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C44" s="3" t="n">
@@ -1705,16 +1833,19 @@
         <v>0.55</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>0.5329999999999999</v>
+        <v>0.2154</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>0.5436</v>
+        <v>0.2154</v>
       </c>
       <c r="G44" s="4" t="n">
-        <v>0.5436</v>
+        <v>0.3917</v>
       </c>
       <c r="H44" s="4" t="n">
-        <v>0.5436</v>
+        <v>0.3917</v>
+      </c>
+      <c r="I44" s="4" t="n">
+        <v>0.3917</v>
       </c>
     </row>
     <row r="45">
@@ -1725,23 +1856,60 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="n">
+        <v>4674200</v>
+      </c>
+      <c r="D45" s="4" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="E45" s="4" t="n">
+        <v>0.5329999999999999</v>
+      </c>
+      <c r="F45" s="4" t="n">
+        <v>0.5436</v>
+      </c>
+      <c r="G45" s="4" t="n">
+        <v>0.5436</v>
+      </c>
+      <c r="H45" s="4" t="n">
+        <v>0.5436</v>
+      </c>
+      <c r="I45" s="4" t="n">
+        <v>0.5436</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E45" s="5">
+      <c r="E46" s="5">
         <f>SUM(E38:E41)</f>
         <v/>
       </c>
-      <c r="F45" s="5">
+      <c r="F46" s="5">
         <f>SUM(F38:F41)</f>
         <v/>
       </c>
-      <c r="G45" s="5">
+      <c r="G46" s="5">
         <f>SUM(G38:G41)</f>
         <v/>
       </c>
-      <c r="H45" s="5">
+      <c r="H46" s="5">
         <f>SUM(H39:H42)</f>
+        <v/>
+      </c>
+      <c r="I46" s="5">
+        <f>SUM(I41:I44)</f>
         <v/>
       </c>
     </row>
@@ -1756,7 +1924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I83"/>
+  <dimension ref="A1:J90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1804,6 +1972,11 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
+          <t>April 27 2026</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>OVER</t>
         </is>
       </c>
@@ -1837,6 +2010,9 @@
       <c r="H3" s="4" t="n">
         <v>0.0018</v>
       </c>
+      <c r="I3" s="4" t="n">
+        <v>0.003</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1867,6 +2043,9 @@
       <c r="H4" s="4" t="n">
         <v>0.1162</v>
       </c>
+      <c r="I4" s="4" t="n">
+        <v>0.1164</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1897,6 +2076,9 @@
       <c r="H5" s="4" t="n">
         <v>0.115</v>
       </c>
+      <c r="I5" s="4" t="n">
+        <v>0.115</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1927,6 +2109,9 @@
       <c r="H6" s="4" t="n">
         <v>0.1652</v>
       </c>
+      <c r="I6" s="4" t="n">
+        <v>0.3186</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1957,6 +2142,9 @@
       <c r="H7" s="4" t="n">
         <v>0.0623</v>
       </c>
+      <c r="I7" s="4" t="n">
+        <v>0.0667</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1987,6 +2175,9 @@
       <c r="H8" s="4" t="n">
         <v>0.0004</v>
       </c>
+      <c r="I8" s="4" t="n">
+        <v>0.0008</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2017,6 +2208,9 @@
       <c r="H9" s="4" t="n">
         <v>0.0011</v>
       </c>
+      <c r="I9" s="4" t="n">
+        <v>0.0143</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2041,6 +2235,9 @@
       <c r="H10" s="4" t="n">
         <v>0.0013</v>
       </c>
+      <c r="I10" s="4" t="n">
+        <v>0.0031</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2071,6 +2268,9 @@
       <c r="H11" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="I11" s="4" t="n">
+        <v>0.0004</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2098,6 +2298,9 @@
       <c r="H12" s="4" t="n">
         <v>0.0012</v>
       </c>
+      <c r="I12" s="4" t="n">
+        <v>0.0012</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2125,6 +2328,9 @@
       <c r="H13" s="4" t="n">
         <v>0.0003</v>
       </c>
+      <c r="I13" s="4" t="n">
+        <v>0.0003</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2146,6 +2352,9 @@
       <c r="H14" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="I14" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2155,84 +2364,70 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E15" s="5">
-        <f>SUM(E3:E11)</f>
-        <v/>
-      </c>
-      <c r="F15" s="5">
-        <f>SUM(F3:F13)</f>
-        <v/>
-      </c>
-      <c r="G15" s="5">
-        <f>SUM(G3:G13)</f>
-        <v/>
-      </c>
-      <c r="H15" s="5">
-        <f>SUM(H3:H14)</f>
-        <v/>
+          <t>Czech Republic</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>9523100</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>0.0001</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Steel Plate</t>
+          <t>Hot-Rolled Sheet</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>54354900</v>
+        <v>9523100</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="E16" s="4" t="n">
-        <v>0.0016</v>
-      </c>
-      <c r="F16" s="4" t="n">
-        <v>0.0025</v>
-      </c>
-      <c r="G16" s="4" t="n">
-        <v>0.005500000000000001</v>
-      </c>
-      <c r="H16" s="4" t="n">
-        <v>0.0134</v>
+        <v>0.67</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>0.2405</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Steel Plate</t>
+          <t>Hot-Rolled Sheet</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Finland</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="n">
-        <v>54354900</v>
-      </c>
-      <c r="D17" s="4" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>0.008500000000000001</v>
-      </c>
-      <c r="F17" s="4" t="n">
-        <v>0.0141</v>
-      </c>
-      <c r="G17" s="4" t="n">
-        <v>0.022</v>
-      </c>
-      <c r="H17" s="4" t="n">
-        <v>0.0229</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E17" s="5">
+        <f>SUM(E3:E11)</f>
+        <v/>
+      </c>
+      <c r="F17" s="5">
+        <f>SUM(F3:F13)</f>
+        <v/>
+      </c>
+      <c r="G17" s="5">
+        <f>SUM(G3:G13)</f>
+        <v/>
+      </c>
+      <c r="H17" s="5">
+        <f>SUM(H3:H14)</f>
+        <v/>
+      </c>
+      <c r="I17" s="5">
+        <f>SUM(I3:I16)</f>
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -2243,7 +2438,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
@@ -2253,16 +2448,19 @@
         <v>0.3</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.0016</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.0025</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.0018</v>
+        <v>0.005500000000000001</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>0.0142</v>
+        <v>0.0134</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>0.0151</v>
       </c>
     </row>
     <row r="19">
@@ -2273,7 +2471,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
@@ -2283,16 +2481,19 @@
         <v>0.3</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>0.0033</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>0.008199999999999999</v>
+        <v>0.0141</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>0.2861</v>
+        <v>0.022</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>0.0267</v>
+        <v>0.0229</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>0.0243</v>
       </c>
     </row>
     <row r="20">
@@ -2303,7 +2504,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
@@ -2313,16 +2514,19 @@
         <v>0.3</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>0</v>
+        <v>0.0012</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>0.0083</v>
+        <v>0.0012</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.0572</v>
+        <v>0.0018</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>0.0572</v>
+        <v>0.0142</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>0.0142</v>
       </c>
     </row>
     <row r="21">
@@ -2333,7 +2537,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
@@ -2343,21 +2547,19 @@
         <v>0.3</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>0.2889</v>
+        <v>0.0033</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>0.3</v>
+        <v>0.008199999999999999</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>0.3</v>
+        <v>0.2861</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
+        <v>0.0267</v>
+      </c>
+      <c r="I21" s="4" t="n">
+        <v>0.0384</v>
       </c>
     </row>
     <row r="22">
@@ -2368,7 +2570,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C22" s="3" t="n">
@@ -2378,16 +2580,19 @@
         <v>0.3</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>0.0892</v>
+        <v>0</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>0.0892</v>
+        <v>0.0083</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>0.0892</v>
+        <v>0.0572</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>0.1138</v>
+        <v>0.0572</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>0.1041</v>
       </c>
     </row>
     <row r="23">
@@ -2398,7 +2603,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C23" s="3" t="n">
@@ -2408,16 +2613,24 @@
         <v>0.3</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.2889</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.3</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.3</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.3</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -2428,7 +2641,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C24" s="3" t="n">
@@ -2438,16 +2651,19 @@
         <v>0.3</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>0.0008</v>
+        <v>0.0892</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>0.0128</v>
+        <v>0.0892</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>0.0315</v>
+        <v>0.0892</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>0.0338</v>
+        <v>0.1138</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>0.1668</v>
       </c>
     </row>
     <row r="25">
@@ -2458,7 +2674,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C25" s="3" t="n">
@@ -2467,14 +2683,20 @@
       <c r="D25" s="4" t="n">
         <v>0.3</v>
       </c>
+      <c r="E25" s="4" t="n">
+        <v>0.0004</v>
+      </c>
       <c r="F25" s="4" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>0.0226</v>
+        <v>0.0004</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>0.0004</v>
       </c>
     </row>
     <row r="26">
@@ -2485,7 +2707,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C26" s="3" t="n">
@@ -2494,14 +2716,20 @@
       <c r="D26" s="4" t="n">
         <v>0.3</v>
       </c>
+      <c r="E26" s="4" t="n">
+        <v>0.0008</v>
+      </c>
       <c r="F26" s="4" t="n">
-        <v>0.0011</v>
+        <v>0.0128</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>0.0019</v>
+        <v>0.0315</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>0.0022</v>
+        <v>0.0338</v>
+      </c>
+      <c r="I26" s="4" t="n">
+        <v>0.0366</v>
       </c>
     </row>
     <row r="27">
@@ -2512,7 +2740,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C27" s="3" t="n">
@@ -2522,13 +2750,16 @@
         <v>0.3</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.0003</v>
+        <v>0</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>0.0003</v>
+        <v>0.0226</v>
+      </c>
+      <c r="I27" s="4" t="n">
+        <v>0.0226</v>
       </c>
     </row>
     <row r="28">
@@ -2539,7 +2770,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C28" s="3" t="n">
@@ -2548,8 +2779,17 @@
       <c r="D28" s="4" t="n">
         <v>0.3</v>
       </c>
+      <c r="F28" s="4" t="n">
+        <v>0.0011</v>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>0.0019</v>
+      </c>
       <c r="H28" s="4" t="n">
-        <v>0.0226</v>
+        <v>0.0022</v>
+      </c>
+      <c r="I28" s="4" t="n">
+        <v>0.0026</v>
       </c>
     </row>
     <row r="29">
@@ -2560,81 +2800,82 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E29" s="5">
-        <f>SUM(E13:E21)</f>
-        <v/>
-      </c>
-      <c r="F29" s="5">
-        <f>SUM(F15:F26)</f>
-        <v/>
-      </c>
-      <c r="G29" s="5">
-        <f>SUM(G15:G26)</f>
-        <v/>
-      </c>
-      <c r="H29" s="5">
-        <f>SUM(H16:H28)</f>
-        <v/>
+          <t>Slovenia</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>54354900</v>
+      </c>
+      <c r="D29" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="H29" s="4" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="I29" s="4" t="n">
+        <v>0.0003</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Cold-Rolled Sheet</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C30" s="3" t="n">
-        <v>1832600</v>
+        <v>54354900</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="E30" s="4" t="n">
-        <v>0.0867</v>
-      </c>
-      <c r="F30" s="4" t="n">
-        <v>0.0964</v>
-      </c>
-      <c r="G30" s="4" t="n">
-        <v>0.1823</v>
+        <v>0.3</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>0.1823</v>
+        <v>0.0226</v>
+      </c>
+      <c r="I30" s="4" t="n">
+        <v>0.0226</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Cold-Rolled Sheet</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="n">
-        <v>1832600</v>
-      </c>
-      <c r="D31" s="4" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="F31" s="4" t="n">
-        <v>0.0795</v>
-      </c>
-      <c r="G31" s="4" t="n">
-        <v>0.123</v>
-      </c>
-      <c r="H31" s="4" t="n">
-        <v>0.1251</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E31" s="5">
+        <f>SUM(E13:E21)</f>
+        <v/>
+      </c>
+      <c r="F31" s="5">
+        <f>SUM(F15:F26)</f>
+        <v/>
+      </c>
+      <c r="G31" s="5">
+        <f>SUM(G15:G26)</f>
+        <v/>
+      </c>
+      <c r="H31" s="5">
+        <f>SUM(H16:H28)</f>
+        <v/>
+      </c>
+      <c r="I31" s="5">
+        <f>SUM(I16:I28)</f>
+        <v/>
       </c>
     </row>
     <row r="32">
@@ -2645,7 +2886,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C32" s="3" t="n">
@@ -2654,8 +2895,20 @@
       <c r="D32" s="4" t="n">
         <v>0.32</v>
       </c>
+      <c r="E32" s="4" t="n">
+        <v>0.0867</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>0.0964</v>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>0.1823</v>
+      </c>
       <c r="H32" s="4" t="n">
-        <v>0.1992</v>
+        <v>0.1823</v>
+      </c>
+      <c r="I32" s="4" t="n">
+        <v>0.1823</v>
       </c>
     </row>
     <row r="33">
@@ -2666,30 +2919,32 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E33" s="5">
-        <f>SUM(E23:E23)</f>
-        <v/>
-      </c>
-      <c r="F33" s="5">
-        <f>SUM(F28:F29)</f>
-        <v/>
-      </c>
-      <c r="G33" s="5">
-        <f>SUM(G28:G29)</f>
-        <v/>
-      </c>
-      <c r="H33" s="5">
-        <f>SUM(H30:H32)</f>
-        <v/>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>1832600</v>
+      </c>
+      <c r="D33" s="4" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>0.0795</v>
+      </c>
+      <c r="G33" s="4" t="n">
+        <v>0.123</v>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>0.1251</v>
+      </c>
+      <c r="I33" s="4" t="n">
+        <v>0.2272</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2698,82 +2953,69 @@
         </is>
       </c>
       <c r="C34" s="3" t="n">
-        <v>31128200</v>
+        <v>1832600</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E34" s="4" t="n">
-        <v>0.0003</v>
-      </c>
-      <c r="F34" s="4" t="n">
-        <v>0.0003</v>
-      </c>
-      <c r="G34" s="4" t="n">
-        <v>0.0003</v>
+        <v>0.32</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>0.0003</v>
+        <v>0.1992</v>
+      </c>
+      <c r="I34" s="4" t="n">
+        <v>0.1992</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="C35" s="3" t="n">
-        <v>31128200</v>
+        <v>1832600</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E35" s="4" t="n">
-        <v>0.0541</v>
-      </c>
-      <c r="F35" s="4" t="n">
-        <v>0.0562</v>
-      </c>
-      <c r="G35" s="4" t="n">
-        <v>0.0793</v>
-      </c>
-      <c r="H35" s="4" t="n">
-        <v>0.0793</v>
+        <v>0.32</v>
+      </c>
+      <c r="I35" s="4" t="n">
+        <v>0.0008</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="n">
-        <v>31128200</v>
-      </c>
-      <c r="D36" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E36" s="4" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="F36" s="4" t="n">
-        <v>0.0341</v>
-      </c>
-      <c r="G36" s="4" t="n">
-        <v>0.0385</v>
-      </c>
-      <c r="H36" s="4" t="n">
-        <v>0.0407</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E36" s="5">
+        <f>SUM(E23:E23)</f>
+        <v/>
+      </c>
+      <c r="F36" s="5">
+        <f>SUM(F28:F29)</f>
+        <v/>
+      </c>
+      <c r="G36" s="5">
+        <f>SUM(G28:G29)</f>
+        <v/>
+      </c>
+      <c r="H36" s="5">
+        <f>SUM(H30:H32)</f>
+        <v/>
+      </c>
+      <c r="I36" s="5">
+        <f>SUM(I32:I35)</f>
+        <v/>
       </c>
     </row>
     <row r="37">
@@ -2784,7 +3026,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C37" s="3" t="n">
@@ -2794,16 +3036,19 @@
         <v>0.25</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>0.04019999999999999</v>
+        <v>0.0003</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>0.0435</v>
+        <v>0.0003</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>0.0435</v>
+        <v>0.0003</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>0.06909999999999999</v>
+        <v>0.0003</v>
+      </c>
+      <c r="I37" s="4" t="n">
+        <v>0.0003</v>
       </c>
     </row>
     <row r="38">
@@ -2814,7 +3059,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C38" s="3" t="n">
@@ -2824,16 +3069,19 @@
         <v>0.25</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>0.0251</v>
+        <v>0.0541</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>0.0251</v>
+        <v>0.0562</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>0.0282</v>
+        <v>0.0793</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>0.0282</v>
+        <v>0.0793</v>
+      </c>
+      <c r="I38" s="4" t="n">
+        <v>0.1136</v>
       </c>
     </row>
     <row r="39">
@@ -2844,7 +3092,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C39" s="3" t="n">
@@ -2854,16 +3102,19 @@
         <v>0.25</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>0.0007000000000000001</v>
+        <v>0.005</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>0.0007000000000000001</v>
+        <v>0.0341</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>0.0007000000000000001</v>
+        <v>0.0385</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>0.0007000000000000001</v>
+        <v>0.0407</v>
+      </c>
+      <c r="I39" s="4" t="n">
+        <v>0.0601</v>
       </c>
     </row>
     <row r="40">
@@ -2874,7 +3125,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C40" s="3" t="n">
@@ -2884,16 +3135,19 @@
         <v>0.25</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>0.0026</v>
+        <v>0.04019999999999999</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>0.0265</v>
+        <v>0.0435</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>0.0302</v>
+        <v>0.0435</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>0.0356</v>
+        <v>0.06909999999999999</v>
+      </c>
+      <c r="I40" s="4" t="n">
+        <v>0.06909999999999999</v>
       </c>
     </row>
     <row r="41">
@@ -2904,7 +3158,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C41" s="3" t="n">
@@ -2913,14 +3167,20 @@
       <c r="D41" s="4" t="n">
         <v>0.25</v>
       </c>
+      <c r="E41" s="4" t="n">
+        <v>0.0251</v>
+      </c>
       <c r="F41" s="4" t="n">
-        <v>0.0005</v>
+        <v>0.0251</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>0.0008</v>
+        <v>0.0282</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>0.0011</v>
+        <v>0.0282</v>
+      </c>
+      <c r="I41" s="4" t="n">
+        <v>0.0469</v>
       </c>
     </row>
     <row r="42">
@@ -2931,7 +3191,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C42" s="3" t="n">
@@ -2940,14 +3200,20 @@
       <c r="D42" s="4" t="n">
         <v>0.25</v>
       </c>
+      <c r="E42" s="4" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
       <c r="F42" s="4" t="n">
-        <v>0.0064</v>
+        <v>0.0007000000000000001</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>0.0142</v>
+        <v>0.0007000000000000001</v>
       </c>
       <c r="H42" s="4" t="n">
-        <v>0.0142</v>
+        <v>0.0007000000000000001</v>
+      </c>
+      <c r="I42" s="4" t="n">
+        <v>0.0007000000000000001</v>
       </c>
     </row>
     <row r="43">
@@ -2958,7 +3224,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C43" s="3" t="n">
@@ -2967,14 +3233,20 @@
       <c r="D43" s="4" t="n">
         <v>0.25</v>
       </c>
+      <c r="E43" s="4" t="n">
+        <v>0.0026</v>
+      </c>
       <c r="F43" s="4" t="n">
-        <v>0.0101</v>
+        <v>0.0265</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>0.0101</v>
+        <v>0.0302</v>
       </c>
       <c r="H43" s="4" t="n">
-        <v>0.0101</v>
+        <v>0.0356</v>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>0.0458</v>
       </c>
     </row>
     <row r="44">
@@ -2985,7 +3257,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="C44" s="3" t="n">
@@ -2994,11 +3266,17 @@
       <c r="D44" s="4" t="n">
         <v>0.25</v>
       </c>
+      <c r="F44" s="4" t="n">
+        <v>0.0005</v>
+      </c>
       <c r="G44" s="4" t="n">
-        <v>0.0003</v>
+        <v>0.0008</v>
       </c>
       <c r="H44" s="4" t="n">
-        <v>0.0003</v>
+        <v>0.0011</v>
+      </c>
+      <c r="I44" s="4" t="n">
+        <v>0.0011</v>
       </c>
     </row>
     <row r="45">
@@ -3009,7 +3287,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C45" s="3" t="n">
@@ -3018,8 +3296,17 @@
       <c r="D45" s="4" t="n">
         <v>0.25</v>
       </c>
+      <c r="F45" s="4" t="n">
+        <v>0.0064</v>
+      </c>
+      <c r="G45" s="4" t="n">
+        <v>0.0142</v>
+      </c>
       <c r="H45" s="4" t="n">
-        <v>0.0014</v>
+        <v>0.0142</v>
+      </c>
+      <c r="I45" s="4" t="n">
+        <v>0.0142</v>
       </c>
     </row>
     <row r="46">
@@ -3030,7 +3317,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>New Zealand</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C46" s="3" t="n">
@@ -3039,8 +3326,17 @@
       <c r="D46" s="4" t="n">
         <v>0.25</v>
       </c>
+      <c r="F46" s="4" t="n">
+        <v>0.0101</v>
+      </c>
+      <c r="G46" s="4" t="n">
+        <v>0.0101</v>
+      </c>
       <c r="H46" s="4" t="n">
-        <v>0.0157</v>
+        <v>0.0101</v>
+      </c>
+      <c r="I46" s="4" t="n">
+        <v>0.0137</v>
       </c>
     </row>
     <row r="47">
@@ -3051,7 +3347,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="C47" s="3" t="n">
@@ -3060,8 +3356,14 @@
       <c r="D47" s="4" t="n">
         <v>0.25</v>
       </c>
+      <c r="G47" s="4" t="n">
+        <v>0.0003</v>
+      </c>
       <c r="H47" s="4" t="n">
-        <v>0.0192</v>
+        <v>0.0003</v>
+      </c>
+      <c r="I47" s="4" t="n">
+        <v>0.0003</v>
       </c>
     </row>
     <row r="48">
@@ -3072,174 +3374,142 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E48" s="5">
-        <f>SUM(E25:E31)</f>
-        <v/>
-      </c>
-      <c r="F48" s="5">
-        <f>SUM(F31:F40)</f>
-        <v/>
-      </c>
-      <c r="G48" s="5">
-        <f>SUM(G31:G41)</f>
-        <v/>
-      </c>
-      <c r="H48" s="5">
-        <f>SUM(H34:H47)</f>
-        <v/>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="n">
+        <v>31128200</v>
+      </c>
+      <c r="D48" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H48" s="4" t="n">
+        <v>0.0014</v>
+      </c>
+      <c r="I48" s="4" t="n">
+        <v>0.0014</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>New Zealand</t>
         </is>
       </c>
       <c r="C49" s="3" t="n">
-        <v>28710400</v>
+        <v>31128200</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="E49" s="4" t="n">
-        <v>0.1642</v>
-      </c>
-      <c r="F49" s="4" t="n">
-        <v>0.1642</v>
-      </c>
-      <c r="G49" s="4" t="n">
-        <v>0.1642</v>
+        <v>0.25</v>
       </c>
       <c r="H49" s="4" t="n">
-        <v>0.1642</v>
+        <v>0.0157</v>
+      </c>
+      <c r="I49" s="4" t="n">
+        <v>0.0157</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Greece</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C50" s="3" t="n">
-        <v>28710400</v>
+        <v>31128200</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="E50" s="4" t="n">
-        <v>0.3234</v>
-      </c>
-      <c r="F50" s="4" t="n">
-        <v>0.3234</v>
-      </c>
-      <c r="G50" s="4" t="n">
-        <v>0.3234</v>
+        <v>0.25</v>
       </c>
       <c r="H50" s="4" t="n">
-        <v>0.3234</v>
+        <v>0.0192</v>
+      </c>
+      <c r="I50" s="4" t="n">
+        <v>0.0192</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C51" s="3" t="n">
-        <v>28710400</v>
+        <v>31128200</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="E51" s="4" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="F51" s="4" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="G51" s="4" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="H51" s="4" t="n">
-        <v>0.0028</v>
+        <v>0.25</v>
+      </c>
+      <c r="I51" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Peru</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C52" s="3" t="n">
-        <v>28710400</v>
+        <v>31128200</v>
       </c>
       <c r="D52" s="4" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="E52" s="4" t="n">
-        <v>0.1633</v>
-      </c>
-      <c r="F52" s="4" t="n">
-        <v>0.1633</v>
-      </c>
-      <c r="G52" s="4" t="n">
-        <v>0.1633</v>
-      </c>
-      <c r="H52" s="4" t="n">
-        <v>0.1633</v>
+        <v>0.25</v>
+      </c>
+      <c r="I52" s="4" t="n">
+        <v>0.0258</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="n">
-        <v>28710400</v>
-      </c>
-      <c r="D53" s="4" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="E53" s="4" t="n">
-        <v>0.3462</v>
-      </c>
-      <c r="F53" s="4" t="n">
-        <v>0.3462</v>
-      </c>
-      <c r="G53" s="4" t="n">
-        <v>0.3462</v>
-      </c>
-      <c r="H53" s="4" t="n">
-        <v>0.3462</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E53" s="5">
+        <f>SUM(E25:E31)</f>
+        <v/>
+      </c>
+      <c r="F53" s="5">
+        <f>SUM(F31:F40)</f>
+        <v/>
+      </c>
+      <c r="G53" s="5">
+        <f>SUM(G31:G41)</f>
+        <v/>
+      </c>
+      <c r="H53" s="5">
+        <f>SUM(H34:H47)</f>
+        <v/>
+      </c>
+      <c r="I53" s="5">
+        <f>SUM(I37:I52)</f>
+        <v/>
       </c>
     </row>
     <row r="54">
@@ -3250,174 +3520,193 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E54" s="5">
-        <f>SUM(E33:E37)</f>
-        <v/>
-      </c>
-      <c r="F54" s="5">
-        <f>SUM(F33:F37)</f>
-        <v/>
-      </c>
-      <c r="G54" s="5">
-        <f>SUM(G42:G46)</f>
-        <v/>
-      </c>
-      <c r="H54" s="5">
-        <f>SUM(H43:H47)</f>
-        <v/>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="n">
+        <v>28710400</v>
+      </c>
+      <c r="D54" s="4" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E54" s="4" t="n">
+        <v>0.1642</v>
+      </c>
+      <c r="F54" s="4" t="n">
+        <v>0.1642</v>
+      </c>
+      <c r="G54" s="4" t="n">
+        <v>0.1642</v>
+      </c>
+      <c r="H54" s="4" t="n">
+        <v>0.1642</v>
+      </c>
+      <c r="I54" s="4" t="n">
+        <v>0.1642</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Greece</t>
         </is>
       </c>
       <c r="C55" s="3" t="n">
-        <v>8750300</v>
+        <v>28710400</v>
       </c>
       <c r="D55" s="4" t="n">
-        <v>0.58</v>
+        <v>0.45</v>
       </c>
       <c r="E55" s="4" t="n">
-        <v>0.0001</v>
+        <v>0.3234</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>0.0007000000000000001</v>
+        <v>0.3234</v>
       </c>
       <c r="G55" s="4" t="n">
-        <v>0.0016</v>
+        <v>0.3234</v>
       </c>
       <c r="H55" s="4" t="n">
-        <v>0.0021</v>
+        <v>0.3234</v>
+      </c>
+      <c r="I55" s="4" t="n">
+        <v>0.3234</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C56" s="3" t="n">
-        <v>8750300</v>
+        <v>28710400</v>
       </c>
       <c r="D56" s="4" t="n">
-        <v>0.58</v>
+        <v>0.45</v>
       </c>
       <c r="E56" s="4" t="n">
-        <v>0.0022</v>
+        <v>0.0028</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>0.0022</v>
+        <v>0.0028</v>
       </c>
       <c r="G56" s="4" t="n">
-        <v>0.0022</v>
+        <v>0.0028</v>
       </c>
       <c r="H56" s="4" t="n">
-        <v>0.0022</v>
+        <v>0.0028</v>
+      </c>
+      <c r="I56" s="4" t="n">
+        <v>0.0028</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Peru</t>
         </is>
       </c>
       <c r="C57" s="3" t="n">
-        <v>8750300</v>
+        <v>28710400</v>
       </c>
       <c r="D57" s="4" t="n">
-        <v>0.58</v>
+        <v>0.45</v>
       </c>
       <c r="E57" s="4" t="n">
-        <v>0.0017</v>
+        <v>0.1633</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>0.0017</v>
+        <v>0.1633</v>
       </c>
       <c r="G57" s="4" t="n">
-        <v>0.0017</v>
+        <v>0.1633</v>
       </c>
       <c r="H57" s="4" t="n">
-        <v>0.0017</v>
+        <v>0.1633</v>
+      </c>
+      <c r="I57" s="4" t="n">
+        <v>0.1633</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="C58" s="3" t="n">
-        <v>8750300</v>
+        <v>28710400</v>
       </c>
       <c r="D58" s="4" t="n">
-        <v>0.58</v>
+        <v>0.45</v>
       </c>
       <c r="E58" s="4" t="n">
-        <v>0.0307</v>
+        <v>0.3462</v>
       </c>
       <c r="F58" s="4" t="n">
-        <v>0.0633</v>
+        <v>0.3462</v>
       </c>
       <c r="G58" s="4" t="n">
-        <v>0.0793</v>
+        <v>0.3462</v>
       </c>
       <c r="H58" s="4" t="n">
-        <v>0.07969999999999999</v>
+        <v>0.3462</v>
+      </c>
+      <c r="I58" s="4" t="n">
+        <v>0.3462</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="C59" s="3" t="n">
-        <v>8750300</v>
-      </c>
-      <c r="D59" s="4" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="E59" s="4" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="F59" s="4" t="n">
-        <v>0.0021</v>
-      </c>
-      <c r="G59" s="4" t="n">
-        <v>0.0029</v>
-      </c>
-      <c r="H59" s="4" t="n">
-        <v>0.0069</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E59" s="5">
+        <f>SUM(E33:E37)</f>
+        <v/>
+      </c>
+      <c r="F59" s="5">
+        <f>SUM(F33:F37)</f>
+        <v/>
+      </c>
+      <c r="G59" s="5">
+        <f>SUM(G42:G46)</f>
+        <v/>
+      </c>
+      <c r="H59" s="5">
+        <f>SUM(H43:H47)</f>
+        <v/>
+      </c>
+      <c r="I59" s="5">
+        <f>SUM(I49:I53)</f>
+        <v/>
       </c>
     </row>
     <row r="60">
@@ -3428,7 +3717,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C60" s="3" t="n">
@@ -3438,16 +3727,19 @@
         <v>0.58</v>
       </c>
       <c r="E60" s="4" t="n">
-        <v>0.07519999999999999</v>
+        <v>0.0001</v>
       </c>
       <c r="F60" s="4" t="n">
-        <v>0.127</v>
+        <v>0.0007000000000000001</v>
       </c>
       <c r="G60" s="4" t="n">
-        <v>0.1355</v>
+        <v>0.0016</v>
       </c>
       <c r="H60" s="4" t="n">
-        <v>0.1376</v>
+        <v>0.0021</v>
+      </c>
+      <c r="I60" s="4" t="n">
+        <v>0.0023</v>
       </c>
     </row>
     <row r="61">
@@ -3458,7 +3750,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="C61" s="3" t="n">
@@ -3468,16 +3760,19 @@
         <v>0.58</v>
       </c>
       <c r="E61" s="4" t="n">
-        <v>0</v>
+        <v>0.0022</v>
       </c>
       <c r="F61" s="4" t="n">
-        <v>0</v>
+        <v>0.0022</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0.0002</v>
+        <v>0.0022</v>
       </c>
       <c r="H61" s="4" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0022</v>
+      </c>
+      <c r="I61" s="4" t="n">
+        <v>0.0022</v>
       </c>
     </row>
     <row r="62">
@@ -3488,7 +3783,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C62" s="3" t="n">
@@ -3498,16 +3793,19 @@
         <v>0.58</v>
       </c>
       <c r="E62" s="4" t="n">
-        <v>0.009899999999999999</v>
+        <v>0.0017</v>
       </c>
       <c r="F62" s="4" t="n">
-        <v>0.0876</v>
+        <v>0.0017</v>
       </c>
       <c r="G62" s="4" t="n">
-        <v>0.1008</v>
+        <v>0.0017</v>
       </c>
       <c r="H62" s="4" t="n">
-        <v>0.1247</v>
+        <v>0.0017</v>
+      </c>
+      <c r="I62" s="4" t="n">
+        <v>0.0017</v>
       </c>
     </row>
     <row r="63">
@@ -3518,7 +3816,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C63" s="3" t="n">
@@ -3528,16 +3826,19 @@
         <v>0.58</v>
       </c>
       <c r="E63" s="4" t="n">
-        <v>0</v>
+        <v>0.0307</v>
       </c>
       <c r="F63" s="4" t="n">
-        <v>0</v>
+        <v>0.0633</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>0.0016</v>
+        <v>0.0793</v>
       </c>
       <c r="H63" s="4" t="n">
-        <v>0.0016</v>
+        <v>0.07969999999999999</v>
+      </c>
+      <c r="I63" s="4" t="n">
+        <v>0.08070000000000001</v>
       </c>
     </row>
     <row r="64">
@@ -3548,7 +3849,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C64" s="3" t="n">
@@ -3557,14 +3858,20 @@
       <c r="D64" s="4" t="n">
         <v>0.58</v>
       </c>
+      <c r="E64" s="4" t="n">
+        <v>0.001</v>
+      </c>
       <c r="F64" s="4" t="n">
-        <v>0</v>
+        <v>0.0021</v>
       </c>
       <c r="G64" s="4" t="n">
-        <v>0.0206</v>
+        <v>0.0029</v>
       </c>
       <c r="H64" s="4" t="n">
-        <v>0.0365</v>
+        <v>0.0069</v>
+      </c>
+      <c r="I64" s="4" t="n">
+        <v>0.009000000000000001</v>
       </c>
     </row>
     <row r="65">
@@ -3575,7 +3882,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C65" s="3" t="n">
@@ -3584,14 +3891,20 @@
       <c r="D65" s="4" t="n">
         <v>0.58</v>
       </c>
+      <c r="E65" s="4" t="n">
+        <v>0.07519999999999999</v>
+      </c>
       <c r="F65" s="4" t="n">
-        <v>0</v>
+        <v>0.127</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>0.0017</v>
+        <v>0.1355</v>
       </c>
       <c r="H65" s="4" t="n">
-        <v>0.0017</v>
+        <v>0.1376</v>
+      </c>
+      <c r="I65" s="4" t="n">
+        <v>0.1384</v>
       </c>
     </row>
     <row r="66">
@@ -3602,7 +3915,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="C66" s="3" t="n">
@@ -3611,11 +3924,20 @@
       <c r="D66" s="4" t="n">
         <v>0.58</v>
       </c>
+      <c r="E66" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="G66" s="4" t="n">
-        <v>0</v>
+        <v>0.0002</v>
       </c>
       <c r="H66" s="4" t="n">
-        <v>0</v>
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="I66" s="4" t="n">
+        <v>0.0005999999999999999</v>
       </c>
     </row>
     <row r="67">
@@ -3626,7 +3948,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C67" s="3" t="n">
@@ -3635,8 +3957,20 @@
       <c r="D67" s="4" t="n">
         <v>0.58</v>
       </c>
+      <c r="E67" s="4" t="n">
+        <v>0.009899999999999999</v>
+      </c>
+      <c r="F67" s="4" t="n">
+        <v>0.0876</v>
+      </c>
+      <c r="G67" s="4" t="n">
+        <v>0.1008</v>
+      </c>
       <c r="H67" s="4" t="n">
-        <v>0</v>
+        <v>0.1247</v>
+      </c>
+      <c r="I67" s="4" t="n">
+        <v>0.1478</v>
       </c>
     </row>
     <row r="68">
@@ -3647,168 +3981,167 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E68" s="5">
-        <f>SUM(E39:E47)</f>
-        <v/>
-      </c>
-      <c r="F68" s="5">
-        <f>SUM(F48:F58)</f>
-        <v/>
-      </c>
-      <c r="G68" s="5">
-        <f>SUM(G49:G60)</f>
-        <v/>
-      </c>
-      <c r="H68" s="5">
-        <f>SUM(H55:H67)</f>
-        <v/>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="n">
+        <v>8750300</v>
+      </c>
+      <c r="D68" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="E68" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" s="4" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="H68" s="4" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="I68" s="4" t="n">
+        <v>0.0016</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C69" s="3" t="n">
-        <v>16514800</v>
+        <v>8750300</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="E69" s="4" t="n">
-        <v>0.0011</v>
+        <v>0.58</v>
       </c>
       <c r="F69" s="4" t="n">
-        <v>0.0751</v>
+        <v>0</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>0.1416</v>
+        <v>0.0206</v>
       </c>
       <c r="H69" s="4" t="n">
-        <v>0.1597</v>
+        <v>0.0365</v>
+      </c>
+      <c r="I69" s="4" t="n">
+        <v>0.0587</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="C70" s="3" t="n">
-        <v>16514800</v>
+        <v>8750300</v>
       </c>
       <c r="D70" s="4" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="E70" s="4" t="n">
-        <v>0.0122</v>
+        <v>0.58</v>
       </c>
       <c r="F70" s="4" t="n">
-        <v>0.0122</v>
+        <v>0</v>
       </c>
       <c r="G70" s="4" t="n">
-        <v>0.0434</v>
+        <v>0.0017</v>
       </c>
       <c r="H70" s="4" t="n">
-        <v>0.0434</v>
+        <v>0.0017</v>
+      </c>
+      <c r="I70" s="4" t="n">
+        <v>0.0018</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C71" s="3" t="n">
-        <v>16514800</v>
+        <v>8750300</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="E71" s="4" t="n">
-        <v>0.008800000000000001</v>
-      </c>
-      <c r="F71" s="4" t="n">
-        <v>0.0176</v>
+        <v>0.58</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>0.0147</v>
+        <v>0</v>
       </c>
       <c r="H71" s="4" t="n">
-        <v>0.0204</v>
+        <v>0</v>
+      </c>
+      <c r="I71" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="C72" s="3" t="n">
-        <v>16514800</v>
+        <v>8750300</v>
       </c>
       <c r="D72" s="4" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="F72" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G72" s="4" t="n">
-        <v>0</v>
+        <v>0.58</v>
       </c>
       <c r="H72" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="I72" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C73" s="3" t="n">
-        <v>16514800</v>
+        <v>8750300</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="H73" s="4" t="n">
-        <v>0.4907</v>
+        <v>0.58</v>
+      </c>
+      <c r="I73" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3817,26 +4150,30 @@
         </is>
       </c>
       <c r="E74" s="5">
-        <f>SUM(E49:E51)</f>
+        <f>SUM(E39:E47)</f>
         <v/>
       </c>
       <c r="F74" s="5">
-        <f>SUM(F60:F63)</f>
+        <f>SUM(F48:F58)</f>
         <v/>
       </c>
       <c r="G74" s="5">
-        <f>SUM(G60:G63)</f>
+        <f>SUM(G49:G60)</f>
         <v/>
       </c>
       <c r="H74" s="5">
-        <f>SUM(H69:H73)</f>
+        <f>SUM(H55:H67)</f>
+        <v/>
+      </c>
+      <c r="I74" s="5">
+        <f>SUM(I60:I73)</f>
         <v/>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3845,172 +4182,177 @@
         </is>
       </c>
       <c r="C75" s="3" t="n">
-        <v>3467600</v>
+        <v>16514800</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.59</v>
       </c>
       <c r="E75" s="4" t="n">
-        <v>0.0001</v>
+        <v>0.0011</v>
       </c>
       <c r="F75" s="4" t="n">
-        <v>0.0001</v>
+        <v>0.0751</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>0.0017</v>
+        <v>0.1416</v>
       </c>
       <c r="H75" s="4" t="n">
-        <v>0.0072</v>
+        <v>0.1597</v>
+      </c>
+      <c r="I75" s="4" t="n">
+        <v>0.2349</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C76" s="3" t="n">
-        <v>3467600</v>
+        <v>16514800</v>
       </c>
       <c r="D76" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.59</v>
       </c>
       <c r="E76" s="4" t="n">
-        <v>0.0011</v>
+        <v>0.0122</v>
       </c>
       <c r="F76" s="4" t="n">
-        <v>0.0073</v>
+        <v>0.0122</v>
       </c>
       <c r="G76" s="4" t="n">
-        <v>0.0075</v>
+        <v>0.0434</v>
       </c>
       <c r="H76" s="4" t="n">
-        <v>0.0075</v>
+        <v>0.0434</v>
+      </c>
+      <c r="I76" s="4" t="n">
+        <v>0.0434</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C77" s="3" t="n">
-        <v>3467600</v>
+        <v>16514800</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.59</v>
       </c>
       <c r="E77" s="4" t="n">
-        <v>0</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="F77" s="4" t="n">
-        <v>0</v>
+        <v>0.0176</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>0.0001</v>
+        <v>0.0147</v>
       </c>
       <c r="H77" s="4" t="n">
-        <v>0.0001</v>
+        <v>0.0204</v>
+      </c>
+      <c r="I77" s="4" t="n">
+        <v>0.0234</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C78" s="3" t="n">
-        <v>3467600</v>
+        <v>16514800</v>
       </c>
       <c r="D78" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="E78" s="4" t="n">
-        <v>0.0191</v>
+        <v>0.59</v>
       </c>
       <c r="F78" s="4" t="n">
-        <v>0.0191</v>
+        <v>0</v>
       </c>
       <c r="G78" s="4" t="n">
-        <v>0.0191</v>
+        <v>0</v>
       </c>
       <c r="H78" s="4" t="n">
-        <v>0.0191</v>
+        <v>0</v>
+      </c>
+      <c r="I78" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C79" s="3" t="n">
-        <v>3467600</v>
+        <v>16514800</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="E79" s="4" t="n">
-        <v>0.007900000000000001</v>
-      </c>
-      <c r="F79" s="4" t="n">
-        <v>0.007900000000000001</v>
-      </c>
-      <c r="G79" s="4" t="n">
-        <v>0.0142</v>
+        <v>0.59</v>
       </c>
       <c r="H79" s="4" t="n">
-        <v>0.0151</v>
+        <v>0.4907</v>
+      </c>
+      <c r="I79" s="4" t="n">
+        <v>0.4907</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Vietnam</t>
-        </is>
-      </c>
-      <c r="C80" s="3" t="n">
-        <v>3467600</v>
-      </c>
-      <c r="D80" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="E80" s="4" t="n">
-        <v>0.3604</v>
-      </c>
-      <c r="F80" s="4" t="n">
-        <v>0.3604</v>
-      </c>
-      <c r="G80" s="4" t="n">
-        <v>0.3604</v>
-      </c>
-      <c r="H80" s="4" t="n">
-        <v>0.3604</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E80" s="5">
+        <f>SUM(E49:E51)</f>
+        <v/>
+      </c>
+      <c r="F80" s="5">
+        <f>SUM(F60:F63)</f>
+        <v/>
+      </c>
+      <c r="G80" s="5">
+        <f>SUM(G60:G63)</f>
+        <v/>
+      </c>
+      <c r="H80" s="5">
+        <f>SUM(H69:H73)</f>
+        <v/>
+      </c>
+      <c r="I80" s="5">
+        <f>SUM(I69:I73)</f>
+        <v/>
       </c>
     </row>
     <row r="81">
@@ -4021,7 +4363,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C81" s="3" t="n">
@@ -4030,14 +4372,20 @@
       <c r="D81" s="4" t="n">
         <v>0.6899999999999999</v>
       </c>
+      <c r="E81" s="4" t="n">
+        <v>0.0001</v>
+      </c>
       <c r="F81" s="4" t="n">
-        <v>0.0421</v>
+        <v>0.0001</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>0.0421</v>
+        <v>0.0017</v>
       </c>
       <c r="H81" s="4" t="n">
-        <v>0.5844</v>
+        <v>0.0072</v>
+      </c>
+      <c r="I81" s="4" t="n">
+        <v>0.0072</v>
       </c>
     </row>
     <row r="82">
@@ -4048,7 +4396,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C82" s="3" t="n">
@@ -4057,14 +4405,20 @@
       <c r="D82" s="4" t="n">
         <v>0.6899999999999999</v>
       </c>
+      <c r="E82" s="4" t="n">
+        <v>0.0011</v>
+      </c>
       <c r="F82" s="4" t="n">
-        <v>0.0001</v>
+        <v>0.0073</v>
       </c>
       <c r="G82" s="4" t="n">
-        <v>0.0001</v>
+        <v>0.0075</v>
       </c>
       <c r="H82" s="4" t="n">
-        <v>0.0001</v>
+        <v>0.0075</v>
+      </c>
+      <c r="I82" s="4" t="n">
+        <v>0.0075</v>
       </c>
     </row>
     <row r="83">
@@ -4075,23 +4429,240 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D83" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E83" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F83" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" s="4" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H83" s="4" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="I83" s="4" t="n">
+        <v>0.0001</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D84" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E84" s="4" t="n">
+        <v>0.0191</v>
+      </c>
+      <c r="F84" s="4" t="n">
+        <v>0.0191</v>
+      </c>
+      <c r="G84" s="4" t="n">
+        <v>0.0191</v>
+      </c>
+      <c r="H84" s="4" t="n">
+        <v>0.0191</v>
+      </c>
+      <c r="I84" s="4" t="n">
+        <v>0.0191</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D85" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E85" s="4" t="n">
+        <v>0.007900000000000001</v>
+      </c>
+      <c r="F85" s="4" t="n">
+        <v>0.007900000000000001</v>
+      </c>
+      <c r="G85" s="4" t="n">
+        <v>0.0142</v>
+      </c>
+      <c r="H85" s="4" t="n">
+        <v>0.0151</v>
+      </c>
+      <c r="I85" s="4" t="n">
+        <v>0.0151</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D86" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E86" s="4" t="n">
+        <v>0.3604</v>
+      </c>
+      <c r="F86" s="4" t="n">
+        <v>0.3604</v>
+      </c>
+      <c r="G86" s="4" t="n">
+        <v>0.3604</v>
+      </c>
+      <c r="H86" s="4" t="n">
+        <v>0.3604</v>
+      </c>
+      <c r="I86" s="4" t="n">
+        <v>0.3604</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Korea, Republic of</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D87" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="F87" s="4" t="n">
+        <v>0.0421</v>
+      </c>
+      <c r="G87" s="4" t="n">
+        <v>0.0421</v>
+      </c>
+      <c r="H87" s="4" t="n">
+        <v>0.5844</v>
+      </c>
+      <c r="I87" s="4" t="n">
+        <v>0.5844</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D88" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="F88" s="4" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="G88" s="4" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H88" s="4" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="I88" s="4" t="n">
+        <v>0.0001</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D89" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="I89" s="4" t="n">
+        <v>0.0062</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E83" s="5">
+      <c r="E90" s="5">
         <f>SUM(E53:E58)</f>
         <v/>
       </c>
-      <c r="F83" s="5">
+      <c r="F90" s="5">
         <f>SUM(F65:F72)</f>
         <v/>
       </c>
-      <c r="G83" s="5">
+      <c r="G90" s="5">
         <f>SUM(G65:G72)</f>
         <v/>
       </c>
-      <c r="H83" s="5">
+      <c r="H90" s="5">
         <f>SUM(H67:H74)</f>
+        <v/>
+      </c>
+      <c r="I90" s="5">
+        <f>SUM(I81:I89)</f>
         <v/>
       </c>
     </row>
@@ -4537,13 +5108,13 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>515.33</v>
+        <v>701.49</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>667.6300000000001</v>
+        <v>902.5799999999999</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>1295.538780975297</v>
+        <v>1286.661249625796</v>
       </c>
     </row>
     <row r="12">
@@ -4684,13 +5255,13 @@
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>31674.81</v>
+        <v>33500.76</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>49138.93</v>
+        <v>52033.31</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1551.356740577133</v>
+        <v>1553.197897599935</v>
       </c>
     </row>
     <row r="19">
@@ -4747,13 +5318,13 @@
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>3477.129999999999</v>
+        <v>3480.079999999999</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>3332.26</v>
+        <v>3337.64</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>958.3363290989984</v>
+        <v>959.0699064389325</v>
       </c>
     </row>
     <row r="22">
@@ -4789,13 +5360,13 @@
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>2793.25</v>
+        <v>3312.37</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>8942.680000000002</v>
+        <v>10253.76</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>3201.532265282378</v>
+        <v>3095.596204530291</v>
       </c>
     </row>
     <row r="24">
@@ -4831,13 +5402,13 @@
         </is>
       </c>
       <c r="C25" s="6" t="n">
-        <v>165</v>
+        <v>353.8699999999999</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>368.13</v>
+        <v>724.9</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>2231.090909090909</v>
+        <v>2048.492384208891</v>
       </c>
     </row>
     <row r="26">
@@ -4894,13 +5465,13 @@
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>18805.76</v>
+        <v>21188.62000000001</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>21858.64</v>
+        <v>24838.52</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>1162.337496596787</v>
+        <v>1172.257560898256</v>
       </c>
     </row>
     <row r="29">
@@ -4915,13 +5486,13 @@
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>4263.77</v>
+        <v>8281.609999999999</v>
       </c>
       <c r="D29" s="6" t="n">
-        <v>4469.190000000001</v>
+        <v>9673.280000000002</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>1048.178020859474</v>
+        <v>1168.043411848663</v>
       </c>
     </row>
     <row r="30">
@@ -4936,13 +5507,13 @@
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>732.39</v>
+        <v>772.9499999999999</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>1447.88</v>
+        <v>1520.46</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>1976.92486243668</v>
+        <v>1967.08713370852</v>
       </c>
     </row>
     <row r="31">
@@ -4978,13 +5549,13 @@
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>23.49</v>
+        <v>43.97</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>89.52</v>
+        <v>176.39</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>3810.983397190294</v>
+        <v>4011.598817375484</v>
       </c>
     </row>
     <row r="33">
@@ -5062,13 +5633,13 @@
         </is>
       </c>
       <c r="C36" s="6" t="n">
-        <v>19646.05999999999</v>
+        <v>20357.18</v>
       </c>
       <c r="D36" s="6" t="n">
-        <v>34998.26999999999</v>
+        <v>36507.71999999999</v>
       </c>
       <c r="E36" s="6" t="n">
-        <v>1781.439637260601</v>
+        <v>1793.358412117985</v>
       </c>
     </row>
     <row r="37">
@@ -5104,13 +5675,13 @@
         </is>
       </c>
       <c r="C38" s="6" t="n">
-        <v>38.46</v>
+        <v>44.18</v>
       </c>
       <c r="D38" s="6" t="n">
-        <v>74.95</v>
+        <v>84.58000000000001</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>1948.777951118045</v>
+        <v>1914.440923494794</v>
       </c>
     </row>
     <row r="39">
@@ -5209,13 +5780,13 @@
         </is>
       </c>
       <c r="C43" s="6" t="n">
-        <v>929.72</v>
+        <v>982.1199999999999</v>
       </c>
       <c r="D43" s="6" t="n">
-        <v>1689.16</v>
+        <v>1806.86</v>
       </c>
       <c r="E43" s="6" t="n">
-        <v>1816.848083293895</v>
+        <v>1839.754816112084</v>
       </c>
     </row>
     <row r="44">
@@ -5293,13 +5864,13 @@
         </is>
       </c>
       <c r="C47" s="6" t="n">
-        <v>24862.74</v>
+        <v>25989.26</v>
       </c>
       <c r="D47" s="6" t="n">
-        <v>44334.33</v>
+        <v>46340.7</v>
       </c>
       <c r="E47" s="6" t="n">
-        <v>1783.163480774846</v>
+        <v>1783.071160933401</v>
       </c>
     </row>
     <row r="48">
@@ -5356,13 +5927,13 @@
         </is>
       </c>
       <c r="C50" s="6" t="n">
-        <v>1709.76</v>
+        <v>2436.199999999999</v>
       </c>
       <c r="D50" s="6" t="n">
-        <v>3123.33</v>
+        <v>4223.150000000001</v>
       </c>
       <c r="E50" s="6" t="n">
-        <v>1826.76516002246</v>
+        <v>1733.498891716609</v>
       </c>
     </row>
     <row r="51">
@@ -5377,13 +5948,13 @@
         </is>
       </c>
       <c r="C51" s="6" t="n">
-        <v>1645.56</v>
+        <v>1788.34</v>
       </c>
       <c r="D51" s="6" t="n">
-        <v>2337.23</v>
+        <v>2573.59</v>
       </c>
       <c r="E51" s="6" t="n">
-        <v>1420.324995746129</v>
+        <v>1439.094355659438</v>
       </c>
     </row>
     <row r="52">
@@ -5461,13 +6032,13 @@
         </is>
       </c>
       <c r="C55" s="6" t="n">
-        <v>2666.57</v>
+        <v>2841.62</v>
       </c>
       <c r="D55" s="6" t="n">
-        <v>5166.57</v>
+        <v>5524.5</v>
       </c>
       <c r="E55" s="6" t="n">
-        <v>1937.533985606978</v>
+        <v>1944.137499032242</v>
       </c>
     </row>
     <row r="56">
@@ -5503,13 +6074,13 @@
         </is>
       </c>
       <c r="C57" s="6" t="n">
-        <v>418.66</v>
+        <v>438.4999999999999</v>
       </c>
       <c r="D57" s="6" t="n">
-        <v>1413.93</v>
+        <v>1479.24</v>
       </c>
       <c r="E57" s="6" t="n">
-        <v>3377.275115845794</v>
+        <v>3373.409350057013</v>
       </c>
     </row>
     <row r="58">
@@ -5545,13 +6116,13 @@
         </is>
       </c>
       <c r="C59" s="6" t="n">
-        <v>37383.03999999999</v>
+        <v>41577.75</v>
       </c>
       <c r="D59" s="6" t="n">
-        <v>57790.36</v>
+        <v>64358.31</v>
       </c>
       <c r="E59" s="6" t="n">
-        <v>1545.897818903974</v>
+        <v>1547.902664285585</v>
       </c>
     </row>
     <row r="60">
@@ -5650,13 +6221,13 @@
         </is>
       </c>
       <c r="C64" s="6" t="n">
-        <v>1660.52</v>
+        <v>1707.3</v>
       </c>
       <c r="D64" s="6" t="n">
-        <v>1962.11</v>
+        <v>2027.08</v>
       </c>
       <c r="E64" s="6" t="n">
-        <v>1181.623828680172</v>
+        <v>1187.301587301587</v>
       </c>
     </row>
     <row r="65">
@@ -5881,13 +6452,13 @@
         </is>
       </c>
       <c r="C75" s="6" t="n">
-        <v>67346.60999999999</v>
+        <v>70249.56000000001</v>
       </c>
       <c r="D75" s="6" t="n">
-        <v>130332.61</v>
+        <v>136049.08</v>
       </c>
       <c r="E75" s="6" t="n">
-        <v>1935.251232393138</v>
+        <v>1936.653838116566</v>
       </c>
     </row>
     <row r="76">
@@ -5944,13 +6515,13 @@
         </is>
       </c>
       <c r="C78" s="6" t="n">
-        <v>156.65</v>
+        <v>96.05</v>
       </c>
       <c r="D78" s="6" t="n">
-        <v>65.61</v>
+        <v>42.23999999999999</v>
       </c>
       <c r="E78" s="6" t="n">
-        <v>418.8317906160231</v>
+        <v>439.7709526288391</v>
       </c>
     </row>
     <row r="79">
@@ -6070,13 +6641,13 @@
         </is>
       </c>
       <c r="C84" s="6" t="n">
-        <v>8233.98</v>
+        <v>9474.679999999998</v>
       </c>
       <c r="D84" s="6" t="n">
-        <v>10066.76</v>
+        <v>11611.21</v>
       </c>
       <c r="E84" s="6" t="n">
-        <v>1222.587375728384</v>
+        <v>1225.498908670267</v>
       </c>
     </row>
     <row r="85">
@@ -6196,13 +6767,13 @@
         </is>
       </c>
       <c r="C90" s="6" t="n">
-        <v>2494.79</v>
+        <v>2599.41</v>
       </c>
       <c r="D90" s="6" t="n">
-        <v>3722.74</v>
+        <v>3834.54</v>
       </c>
       <c r="E90" s="6" t="n">
-        <v>1492.205756797165</v>
+        <v>1475.157824275509</v>
       </c>
     </row>
     <row r="91">
@@ -6238,13 +6809,13 @@
         </is>
       </c>
       <c r="C92" s="6" t="n">
-        <v>13.53</v>
+        <v>17.33</v>
       </c>
       <c r="D92" s="6" t="n">
-        <v>26.23</v>
+        <v>33.38</v>
       </c>
       <c r="E92" s="6" t="n">
-        <v>1938.654841093865</v>
+        <v>1926.139642238892</v>
       </c>
     </row>
     <row r="93">
@@ -6280,13 +6851,13 @@
         </is>
       </c>
       <c r="C94" s="6" t="n">
-        <v>7.96</v>
+        <v>9.08</v>
       </c>
       <c r="D94" s="6" t="n">
-        <v>15.56</v>
+        <v>19.74</v>
       </c>
       <c r="E94" s="6" t="n">
-        <v>1954.773869346734</v>
+        <v>2174.008810572688</v>
       </c>
     </row>
     <row r="95">
@@ -6322,13 +6893,13 @@
         </is>
       </c>
       <c r="C96" s="6" t="n">
-        <v>166.15</v>
+        <v>183.16</v>
       </c>
       <c r="D96" s="6" t="n">
-        <v>212.56</v>
+        <v>232.4</v>
       </c>
       <c r="E96" s="6" t="n">
-        <v>1279.325910321998</v>
+        <v>1268.835990390915</v>
       </c>
     </row>
     <row r="97">
@@ -6406,13 +6977,13 @@
         </is>
       </c>
       <c r="C100" s="6" t="n">
-        <v>881.3600000000001</v>
+        <v>885.2500000000001</v>
       </c>
       <c r="D100" s="6" t="n">
-        <v>1178.4</v>
+        <v>1183.22</v>
       </c>
       <c r="E100" s="6" t="n">
-        <v>1337.024598348007</v>
+        <v>1336.59418243434</v>
       </c>
     </row>
     <row r="101">
@@ -6490,13 +7061,13 @@
         </is>
       </c>
       <c r="C104" s="6" t="n">
-        <v>2817.869999999999</v>
+        <v>3544.67</v>
       </c>
       <c r="D104" s="6" t="n">
-        <v>2934.43</v>
+        <v>3772.210000000001</v>
       </c>
       <c r="E104" s="6" t="n">
-        <v>1041.364576790271</v>
+        <v>1064.192153289305</v>
       </c>
     </row>
     <row r="105">
@@ -6511,13 +7082,13 @@
         </is>
       </c>
       <c r="C105" s="6" t="n">
-        <v>10.47</v>
+        <v>11.31</v>
       </c>
       <c r="D105" s="6" t="n">
-        <v>45.46</v>
+        <v>49.19</v>
       </c>
       <c r="E105" s="6" t="n">
-        <v>4341.929321872015</v>
+        <v>4349.248452696728</v>
       </c>
     </row>
     <row r="106">
@@ -6532,13 +7103,13 @@
         </is>
       </c>
       <c r="C106" s="6" t="n">
-        <v>6958.569999999999</v>
+        <v>7335.619999999998</v>
       </c>
       <c r="D106" s="6" t="n">
-        <v>12687.37</v>
+        <v>13530.13</v>
       </c>
       <c r="E106" s="6" t="n">
-        <v>1823.272597674522</v>
+        <v>1844.442596535808</v>
       </c>
     </row>
     <row r="107">
@@ -6553,13 +7124,13 @@
         </is>
       </c>
       <c r="C107" s="6" t="n">
-        <v>1314.16</v>
+        <v>1793.11</v>
       </c>
       <c r="D107" s="6" t="n">
-        <v>1770.94</v>
+        <v>2380.65</v>
       </c>
       <c r="E107" s="6" t="n">
-        <v>1347.5832470932</v>
+        <v>1327.665341222792</v>
       </c>
     </row>
     <row r="108">
@@ -6595,13 +7166,13 @@
         </is>
       </c>
       <c r="C109" s="6" t="n">
-        <v>7581.570000000001</v>
+        <v>8887.280000000001</v>
       </c>
       <c r="D109" s="6" t="n">
-        <v>11476.33</v>
+        <v>13544.8</v>
       </c>
       <c r="E109" s="6" t="n">
-        <v>1513.714177934122</v>
+        <v>1524.065855919922</v>
       </c>
     </row>
     <row r="110">
@@ -6721,13 +7292,13 @@
         </is>
       </c>
       <c r="C115" s="6" t="n">
-        <v>41.24</v>
+        <v>172.62</v>
       </c>
       <c r="D115" s="6" t="n">
-        <v>57.11</v>
+        <v>215.33</v>
       </c>
       <c r="E115" s="6" t="n">
-        <v>1384.820562560621</v>
+        <v>1247.422083188506</v>
       </c>
     </row>
     <row r="116">
@@ -6742,13 +7313,13 @@
         </is>
       </c>
       <c r="C116" s="6" t="n">
-        <v>10183.38</v>
+        <v>11101.05</v>
       </c>
       <c r="D116" s="6" t="n">
-        <v>13938.61</v>
+        <v>15132.32</v>
       </c>
       <c r="E116" s="6" t="n">
-        <v>1368.760666890561</v>
+        <v>1363.143126100684</v>
       </c>
     </row>
     <row r="117">
@@ -6763,13 +7334,13 @@
         </is>
       </c>
       <c r="C117" s="6" t="n">
-        <v>2854.6</v>
+        <v>3454.909999999999</v>
       </c>
       <c r="D117" s="6" t="n">
-        <v>2533.12</v>
+        <v>3040.07</v>
       </c>
       <c r="E117" s="6" t="n">
-        <v>887.3817697750999</v>
+        <v>879.9274076604023</v>
       </c>
     </row>
     <row r="118">
@@ -6826,13 +7397,13 @@
         </is>
       </c>
       <c r="C120" s="6" t="n">
-        <v>20.41</v>
+        <v>20.58</v>
       </c>
       <c r="D120" s="6" t="n">
-        <v>41.37</v>
+        <v>42</v>
       </c>
       <c r="E120" s="6" t="n">
-        <v>2026.947574718276</v>
+        <v>2040.816326530612</v>
       </c>
     </row>
     <row r="121">
@@ -6847,13 +7418,13 @@
         </is>
       </c>
       <c r="C121" s="6" t="n">
-        <v>214.46</v>
+        <v>385.36</v>
       </c>
       <c r="D121" s="6" t="n">
-        <v>780.6399999999999</v>
+        <v>1237.33</v>
       </c>
       <c r="E121" s="6" t="n">
-        <v>3640.026112095496</v>
+        <v>3210.841810255346</v>
       </c>
     </row>
     <row r="122">
@@ -6889,13 +7460,13 @@
         </is>
       </c>
       <c r="C123" s="6" t="n">
-        <v>32.1</v>
+        <v>38.63</v>
       </c>
       <c r="D123" s="6" t="n">
-        <v>111.78</v>
+        <v>137.75</v>
       </c>
       <c r="E123" s="6" t="n">
-        <v>3482.242990654206</v>
+        <v>3565.881439295884</v>
       </c>
     </row>
     <row r="124">
@@ -6910,13 +7481,13 @@
         </is>
       </c>
       <c r="C124" s="6" t="n">
-        <v>115.61</v>
+        <v>2155.06</v>
       </c>
       <c r="D124" s="6" t="n">
-        <v>238.04</v>
+        <v>2631.22</v>
       </c>
       <c r="E124" s="6" t="n">
-        <v>2058.991436726927</v>
+        <v>1220.949764739729</v>
       </c>
     </row>
     <row r="125">
@@ -6931,13 +7502,13 @@
         </is>
       </c>
       <c r="C125" s="6" t="n">
-        <v>29106.32</v>
+        <v>39026.88</v>
       </c>
       <c r="D125" s="6" t="n">
-        <v>31748.18</v>
+        <v>42887.60000000001</v>
       </c>
       <c r="E125" s="6" t="n">
-        <v>1090.765854288691</v>
+        <v>1098.924638608057</v>
       </c>
     </row>
     <row r="126">
@@ -6952,13 +7523,13 @@
         </is>
       </c>
       <c r="C126" s="6" t="n">
-        <v>11902.06</v>
+        <v>11920.74</v>
       </c>
       <c r="D126" s="6" t="n">
-        <v>17791.8</v>
+        <v>17871.43</v>
       </c>
       <c r="E126" s="6" t="n">
-        <v>1494.850471262958</v>
+        <v>1499.187969874353</v>
       </c>
     </row>
     <row r="127">
@@ -6973,13 +7544,13 @@
         </is>
       </c>
       <c r="C127" s="6" t="n">
-        <v>10507.86</v>
+        <v>11348.22</v>
       </c>
       <c r="D127" s="6" t="n">
-        <v>14134.31</v>
+        <v>15303.37</v>
       </c>
       <c r="E127" s="6" t="n">
-        <v>1345.117845117845</v>
+        <v>1348.526024345668</v>
       </c>
     </row>
     <row r="128">
@@ -7036,13 +7607,13 @@
         </is>
       </c>
       <c r="C130" s="6" t="n">
-        <v>0.5900000000000001</v>
+        <v>0.6500000000000001</v>
       </c>
       <c r="D130" s="6" t="n">
-        <v>2.31</v>
+        <v>2.57</v>
       </c>
       <c r="E130" s="6" t="n">
-        <v>3915.254237288135</v>
+        <v>3953.846153846153</v>
       </c>
     </row>
     <row r="131">
@@ -7057,13 +7628,13 @@
         </is>
       </c>
       <c r="C131" s="6" t="n">
-        <v>13134.23</v>
+        <v>18144.85</v>
       </c>
       <c r="D131" s="6" t="n">
-        <v>13980.22</v>
+        <v>19259.58</v>
       </c>
       <c r="E131" s="6" t="n">
-        <v>1064.411084623917</v>
+        <v>1061.435062841523</v>
       </c>
     </row>
     <row r="132">
@@ -7141,13 +7712,13 @@
         </is>
       </c>
       <c r="C135" s="6" t="n">
-        <v>5547.570000000001</v>
+        <v>7919.14</v>
       </c>
       <c r="D135" s="6" t="n">
-        <v>6493.690000000001</v>
+        <v>9321.07</v>
       </c>
       <c r="E135" s="6" t="n">
-        <v>1170.546743889667</v>
+        <v>1177.030586654611</v>
       </c>
     </row>
     <row r="136">
@@ -7183,13 +7754,13 @@
         </is>
       </c>
       <c r="C137" s="6" t="n">
-        <v>8533.469999999999</v>
+        <v>14836.05</v>
       </c>
       <c r="D137" s="6" t="n">
-        <v>9794.780000000002</v>
+        <v>17153.31</v>
       </c>
       <c r="E137" s="6" t="n">
-        <v>1147.807398397135</v>
+        <v>1156.191169482443</v>
       </c>
     </row>
     <row r="138">
@@ -7204,13 +7775,13 @@
         </is>
       </c>
       <c r="C138" s="6" t="n">
-        <v>18655.03</v>
+        <v>20114.18999999999</v>
       </c>
       <c r="D138" s="6" t="n">
-        <v>40435.90000000001</v>
+        <v>44059.39</v>
       </c>
       <c r="E138" s="6" t="n">
-        <v>2167.560170098896</v>
+        <v>2190.463051209123</v>
       </c>
     </row>
     <row r="139">

</xml_diff>

<commit_message>
Weekly TRQ update 2026-06-01
</commit_message>
<xml_diff>
--- a/data/canada_trq_tracker.xlsx
+++ b/data/canada_trq_tracker.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O52"/>
+  <dimension ref="A1:P52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,6 +511,11 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
+          <t>June 1 2026</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
           <t>OVER</t>
         </is>
       </c>
@@ -562,6 +567,9 @@
       <c r="N3" s="4" t="n">
         <v>0.0329</v>
       </c>
+      <c r="O3" s="4" t="n">
+        <v>0.0329</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -610,6 +618,9 @@
       <c r="N4" s="4" t="n">
         <v>0.0019</v>
       </c>
+      <c r="O4" s="4" t="n">
+        <v>0.0019</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -658,7 +669,10 @@
       <c r="N5" s="4" t="n">
         <v>0.41</v>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O5" s="4" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="P5" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -696,6 +710,9 @@
       <c r="N6" s="4" t="n">
         <v>0.0002</v>
       </c>
+      <c r="O6" s="4" t="n">
+        <v>0.0002</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -748,6 +765,10 @@
         <f>SUM(N3:N6)</f>
         <v/>
       </c>
+      <c r="O7" s="5">
+        <f>SUM(O3:O6)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -796,7 +817,10 @@
       <c r="N8" s="4" t="n">
         <v>0.36</v>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="O8" s="4" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="P8" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -849,6 +873,9 @@
       <c r="N9" s="4" t="n">
         <v>0.0369</v>
       </c>
+      <c r="O9" s="4" t="n">
+        <v>0.0369</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -882,6 +909,9 @@
       <c r="N10" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="O10" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -934,6 +964,10 @@
         <f>SUM(N8:N10)</f>
         <v/>
       </c>
+      <c r="O11" s="5">
+        <f>SUM(O8:O10)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -982,6 +1016,9 @@
       <c r="N12" s="4" t="n">
         <v>0.0062</v>
       </c>
+      <c r="O12" s="4" t="n">
+        <v>0.0062</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1030,6 +1067,9 @@
       <c r="N13" s="4" t="n">
         <v>0.0113</v>
       </c>
+      <c r="O13" s="4" t="n">
+        <v>0.0113</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1078,6 +1118,9 @@
       <c r="N14" s="4" t="n">
         <v>0.5147999999999999</v>
       </c>
+      <c r="O14" s="4" t="n">
+        <v>0.5147999999999999</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1126,6 +1169,9 @@
       <c r="N15" s="4" t="n">
         <v>0.2512</v>
       </c>
+      <c r="O15" s="4" t="n">
+        <v>0.2512</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1165,6 +1211,9 @@
       <c r="N16" s="4" t="n">
         <v>0.0426</v>
       </c>
+      <c r="O16" s="4" t="n">
+        <v>0.0426</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1189,6 +1238,9 @@
       <c r="N17" s="4" t="n">
         <v>0.0067</v>
       </c>
+      <c r="O17" s="4" t="n">
+        <v>0.0067</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1241,6 +1293,10 @@
         <f>SUM(N12:N17)</f>
         <v/>
       </c>
+      <c r="O18" s="5">
+        <f>SUM(O12:O17)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1289,6 +1345,9 @@
       <c r="N19" s="4" t="n">
         <v>0.0092</v>
       </c>
+      <c r="O19" s="4" t="n">
+        <v>0.0092</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1337,6 +1396,9 @@
       <c r="N20" s="4" t="n">
         <v>0.0005</v>
       </c>
+      <c r="O20" s="4" t="n">
+        <v>0.0005</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1385,6 +1447,9 @@
       <c r="N21" s="4" t="n">
         <v>0.0532</v>
       </c>
+      <c r="O21" s="4" t="n">
+        <v>0.0532</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1433,6 +1498,9 @@
       <c r="N22" s="4" t="n">
         <v>0.0119</v>
       </c>
+      <c r="O22" s="4" t="n">
+        <v>0.0119</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1481,6 +1549,9 @@
       <c r="N23" s="4" t="n">
         <v>0.3695000000000001</v>
       </c>
+      <c r="O23" s="4" t="n">
+        <v>0.3695000000000001</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1529,6 +1600,9 @@
       <c r="N24" s="4" t="n">
         <v>0.1384</v>
       </c>
+      <c r="O24" s="4" t="n">
+        <v>0.1384</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1577,6 +1651,9 @@
       <c r="N25" s="4" t="n">
         <v>0.3262</v>
       </c>
+      <c r="O25" s="4" t="n">
+        <v>0.3262</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1625,6 +1702,9 @@
       <c r="N26" s="4" t="n">
         <v>0.05599999999999999</v>
       </c>
+      <c r="O26" s="4" t="n">
+        <v>0.05599999999999999</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1664,6 +1744,9 @@
       <c r="N27" s="4" t="n">
         <v>0.0207</v>
       </c>
+      <c r="O27" s="4" t="n">
+        <v>0.0207</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1697,6 +1780,9 @@
       <c r="N28" s="4" t="n">
         <v>0.0077</v>
       </c>
+      <c r="O28" s="4" t="n">
+        <v>0.0077</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1724,6 +1810,9 @@
       <c r="N29" s="4" t="n">
         <v>0.0008</v>
       </c>
+      <c r="O29" s="4" t="n">
+        <v>0.0008</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1776,6 +1865,10 @@
         <f>SUM(N19:N29)</f>
         <v/>
       </c>
+      <c r="O30" s="5">
+        <f>SUM(O19:O29)</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1824,7 +1917,10 @@
       <c r="N31" s="4" t="n">
         <v>0.29</v>
       </c>
-      <c r="O31" t="inlineStr">
+      <c r="O31" s="4" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="P31" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -1877,6 +1973,9 @@
       <c r="N32" s="4" t="n">
         <v>0.1228</v>
       </c>
+      <c r="O32" s="4" t="n">
+        <v>0.1228</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1925,6 +2024,9 @@
       <c r="N33" s="4" t="n">
         <v>0.2394</v>
       </c>
+      <c r="O33" s="4" t="n">
+        <v>0.2394</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1973,6 +2075,9 @@
       <c r="N34" s="4" t="n">
         <v>0.1668</v>
       </c>
+      <c r="O34" s="4" t="n">
+        <v>0.1668</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2021,6 +2126,9 @@
       <c r="N35" s="4" t="n">
         <v>0.0241</v>
       </c>
+      <c r="O35" s="4" t="n">
+        <v>0.0241</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2069,6 +2177,9 @@
       <c r="N36" s="4" t="n">
         <v>0.1569</v>
       </c>
+      <c r="O36" s="4" t="n">
+        <v>0.1569</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2121,6 +2232,10 @@
         <f>SUM(N31:N36)</f>
         <v/>
       </c>
+      <c r="O37" s="5">
+        <f>SUM(O31:O36)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2169,6 +2284,9 @@
       <c r="N38" s="4" t="n">
         <v>0.0524</v>
       </c>
+      <c r="O38" s="4" t="n">
+        <v>0.0524</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2217,6 +2335,9 @@
       <c r="N39" s="4" t="n">
         <v>0.3131</v>
       </c>
+      <c r="O39" s="4" t="n">
+        <v>0.3131</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2265,6 +2386,9 @@
       <c r="N40" s="4" t="n">
         <v>0.3890999999999999</v>
       </c>
+      <c r="O40" s="4" t="n">
+        <v>0.3890999999999999</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2313,6 +2437,9 @@
       <c r="N41" s="4" t="n">
         <v>0.196</v>
       </c>
+      <c r="O41" s="4" t="n">
+        <v>0.196</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2355,6 +2482,9 @@
       <c r="N42" s="4" t="n">
         <v>0.0005</v>
       </c>
+      <c r="O42" s="4" t="n">
+        <v>0.0005</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2407,6 +2537,10 @@
         <f>SUM(N38:N42)</f>
         <v/>
       </c>
+      <c r="O43" s="5">
+        <f>SUM(O38:O42)</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2455,6 +2589,9 @@
       <c r="N44" s="4" t="n">
         <v>0.442</v>
       </c>
+      <c r="O44" s="4" t="n">
+        <v>0.442</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2491,7 +2628,10 @@
       <c r="N45" s="4" t="n">
         <v>0.45</v>
       </c>
-      <c r="O45" t="inlineStr">
+      <c r="O45" s="4" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="P45" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -2529,6 +2669,9 @@
       <c r="N46" s="4" t="n">
         <v>0.0024</v>
       </c>
+      <c r="O46" s="4" t="n">
+        <v>0.0024</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2581,6 +2724,10 @@
         <f>SUM(N44:N46)</f>
         <v/>
       </c>
+      <c r="O47" s="5">
+        <f>SUM(O44:O46)</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2629,6 +2776,9 @@
       <c r="N48" s="4" t="n">
         <v>0.0412</v>
       </c>
+      <c r="O48" s="4" t="n">
+        <v>0.0412</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2677,6 +2827,9 @@
       <c r="N49" s="4" t="n">
         <v>0.0236</v>
       </c>
+      <c r="O49" s="4" t="n">
+        <v>0.0236</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2725,6 +2878,9 @@
       <c r="N50" s="4" t="n">
         <v>0.3917</v>
       </c>
+      <c r="O50" s="4" t="n">
+        <v>0.3917</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2773,6 +2929,9 @@
       <c r="N51" s="4" t="n">
         <v>0.1041</v>
       </c>
+      <c r="O51" s="4" t="n">
+        <v>0.1041</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2823,6 +2982,10 @@
       </c>
       <c r="N52" s="5">
         <f>SUM(N48:N51)</f>
+        <v/>
+      </c>
+      <c r="O52" s="5">
+        <f>SUM(O48:O51)</f>
         <v/>
       </c>
     </row>
@@ -2837,7 +3000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O94"/>
+  <dimension ref="A1:P94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2915,6 +3078,11 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
+          <t>June 1 2026</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
           <t>OVER</t>
         </is>
       </c>
@@ -2966,6 +3134,9 @@
       <c r="N3" s="4" t="n">
         <v>0.003</v>
       </c>
+      <c r="O3" s="4" t="n">
+        <v>0.003</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3014,6 +3185,9 @@
       <c r="N4" s="4" t="n">
         <v>0.1164</v>
       </c>
+      <c r="O4" s="4" t="n">
+        <v>0.1164</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3062,6 +3236,9 @@
       <c r="N5" s="4" t="n">
         <v>0.115</v>
       </c>
+      <c r="O5" s="4" t="n">
+        <v>0.115</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3110,6 +3287,9 @@
       <c r="N6" s="4" t="n">
         <v>0.4198</v>
       </c>
+      <c r="O6" s="4" t="n">
+        <v>0.4198</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3158,6 +3338,9 @@
       <c r="N7" s="4" t="n">
         <v>0.07429999999999999</v>
       </c>
+      <c r="O7" s="4" t="n">
+        <v>0.07429999999999999</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3206,6 +3389,9 @@
       <c r="N8" s="4" t="n">
         <v>0.0008</v>
       </c>
+      <c r="O8" s="4" t="n">
+        <v>0.0008</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3254,6 +3440,9 @@
       <c r="N9" s="4" t="n">
         <v>0.0143</v>
       </c>
+      <c r="O9" s="4" t="n">
+        <v>0.0143</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3296,6 +3485,9 @@
       <c r="N10" s="4" t="n">
         <v>0.014</v>
       </c>
+      <c r="O10" s="4" t="n">
+        <v>0.014</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3344,6 +3536,9 @@
       <c r="N11" s="4" t="n">
         <v>0.0004</v>
       </c>
+      <c r="O11" s="4" t="n">
+        <v>0.0004</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3389,6 +3584,9 @@
       <c r="N12" s="4" t="n">
         <v>0.0012</v>
       </c>
+      <c r="O12" s="4" t="n">
+        <v>0.0012</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3434,6 +3632,9 @@
       <c r="N13" s="4" t="n">
         <v>0.0003</v>
       </c>
+      <c r="O13" s="4" t="n">
+        <v>0.0003</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3473,6 +3674,9 @@
       <c r="N14" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="O14" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3509,6 +3713,9 @@
       <c r="N15" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="O15" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3545,6 +3752,9 @@
       <c r="N16" s="4" t="n">
         <v>0.2405</v>
       </c>
+      <c r="O16" s="4" t="n">
+        <v>0.2405</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3597,6 +3807,10 @@
         <f>SUM(N3:N16)</f>
         <v/>
       </c>
+      <c r="O17" s="5">
+        <f>SUM(O3:O16)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3645,6 +3859,9 @@
       <c r="N18" s="4" t="n">
         <v>0.0199</v>
       </c>
+      <c r="O18" s="4" t="n">
+        <v>0.0199</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3693,6 +3910,9 @@
       <c r="N19" s="4" t="n">
         <v>0.031</v>
       </c>
+      <c r="O19" s="4" t="n">
+        <v>0.031</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3741,6 +3961,9 @@
       <c r="N20" s="4" t="n">
         <v>0.0741</v>
       </c>
+      <c r="O20" s="4" t="n">
+        <v>0.0741</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3789,6 +4012,9 @@
       <c r="N21" s="4" t="n">
         <v>0.154</v>
       </c>
+      <c r="O21" s="4" t="n">
+        <v>0.154</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3837,6 +4063,9 @@
       <c r="N22" s="4" t="n">
         <v>0.1063</v>
       </c>
+      <c r="O22" s="4" t="n">
+        <v>0.1063</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3885,7 +4114,10 @@
       <c r="N23" s="4" t="n">
         <v>0.3</v>
       </c>
-      <c r="O23" t="inlineStr">
+      <c r="O23" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="P23" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -3938,6 +4170,9 @@
       <c r="N24" s="4" t="n">
         <v>0.1668</v>
       </c>
+      <c r="O24" s="4" t="n">
+        <v>0.1668</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3986,6 +4221,9 @@
       <c r="N25" s="4" t="n">
         <v>0.0005</v>
       </c>
+      <c r="O25" s="4" t="n">
+        <v>0.0005</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4034,6 +4272,9 @@
       <c r="N26" s="4" t="n">
         <v>0.0694</v>
       </c>
+      <c r="O26" s="4" t="n">
+        <v>0.0694</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4079,6 +4320,9 @@
       <c r="N27" s="4" t="n">
         <v>0.0317</v>
       </c>
+      <c r="O27" s="4" t="n">
+        <v>0.0317</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4124,6 +4368,9 @@
       <c r="N28" s="4" t="n">
         <v>0.0073</v>
       </c>
+      <c r="O28" s="4" t="n">
+        <v>0.0073</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4169,6 +4416,9 @@
       <c r="N29" s="4" t="n">
         <v>0.0005999999999999999</v>
       </c>
+      <c r="O29" s="4" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4208,6 +4458,9 @@
       <c r="N30" s="4" t="n">
         <v>0.0226</v>
       </c>
+      <c r="O30" s="4" t="n">
+        <v>0.0226</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4238,6 +4491,9 @@
       <c r="N31" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="O31" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4290,6 +4546,10 @@
         <f>SUM(N18:N31)</f>
         <v/>
       </c>
+      <c r="O32" s="5">
+        <f>SUM(O18:O31)</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4338,6 +4598,9 @@
       <c r="N33" s="4" t="n">
         <v>0.258</v>
       </c>
+      <c r="O33" s="4" t="n">
+        <v>0.258</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4383,6 +4646,9 @@
       <c r="N34" s="4" t="n">
         <v>0.236</v>
       </c>
+      <c r="O34" s="4" t="n">
+        <v>0.236</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4422,6 +4688,9 @@
       <c r="N35" s="4" t="n">
         <v>0.1992</v>
       </c>
+      <c r="O35" s="4" t="n">
+        <v>0.1992</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4458,6 +4727,9 @@
       <c r="N36" s="4" t="n">
         <v>0.0011</v>
       </c>
+      <c r="O36" s="4" t="n">
+        <v>0.0011</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4488,6 +4760,9 @@
       <c r="N37" s="4" t="n">
         <v>0.3057</v>
       </c>
+      <c r="O37" s="4" t="n">
+        <v>0.3057</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4540,6 +4815,10 @@
         <f>SUM(N33:N37)</f>
         <v/>
       </c>
+      <c r="O38" s="5">
+        <f>SUM(O33:O37)</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4588,6 +4867,9 @@
       <c r="N39" s="4" t="n">
         <v>0.0015</v>
       </c>
+      <c r="O39" s="4" t="n">
+        <v>0.0015</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4636,6 +4918,9 @@
       <c r="N40" s="4" t="n">
         <v>0.1686</v>
       </c>
+      <c r="O40" s="4" t="n">
+        <v>0.1686</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4684,6 +4969,9 @@
       <c r="N41" s="4" t="n">
         <v>0.2496</v>
       </c>
+      <c r="O41" s="4" t="n">
+        <v>0.2496</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4732,6 +5020,9 @@
       <c r="N42" s="4" t="n">
         <v>0.09910000000000001</v>
       </c>
+      <c r="O42" s="4" t="n">
+        <v>0.09910000000000001</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -4780,6 +5071,9 @@
       <c r="N43" s="4" t="n">
         <v>0.0842</v>
       </c>
+      <c r="O43" s="4" t="n">
+        <v>0.0842</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4828,6 +5122,9 @@
       <c r="N44" s="4" t="n">
         <v>0.0007000000000000001</v>
       </c>
+      <c r="O44" s="4" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4876,6 +5173,9 @@
       <c r="N45" s="4" t="n">
         <v>0.0876</v>
       </c>
+      <c r="O45" s="4" t="n">
+        <v>0.0876</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4921,6 +5221,9 @@
       <c r="N46" s="4" t="n">
         <v>0.0014</v>
       </c>
+      <c r="O46" s="4" t="n">
+        <v>0.0014</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4966,6 +5269,9 @@
       <c r="N47" s="4" t="n">
         <v>0.0354</v>
       </c>
+      <c r="O47" s="4" t="n">
+        <v>0.0354</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5011,6 +5317,9 @@
       <c r="N48" s="4" t="n">
         <v>0.028</v>
       </c>
+      <c r="O48" s="4" t="n">
+        <v>0.028</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5053,6 +5362,9 @@
       <c r="N49" s="4" t="n">
         <v>0.0003</v>
       </c>
+      <c r="O49" s="4" t="n">
+        <v>0.0003</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5092,6 +5404,9 @@
       <c r="N50" s="4" t="n">
         <v>0.0014</v>
       </c>
+      <c r="O50" s="4" t="n">
+        <v>0.0014</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5131,6 +5446,9 @@
       <c r="N51" s="4" t="n">
         <v>0.0157</v>
       </c>
+      <c r="O51" s="4" t="n">
+        <v>0.0157</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5170,6 +5488,9 @@
       <c r="N52" s="4" t="n">
         <v>0.0215</v>
       </c>
+      <c r="O52" s="4" t="n">
+        <v>0.0215</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5206,6 +5527,9 @@
       <c r="N53" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="O53" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5242,6 +5566,9 @@
       <c r="N54" s="4" t="n">
         <v>0.0258</v>
       </c>
+      <c r="O54" s="4" t="n">
+        <v>0.0258</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5294,6 +5621,10 @@
         <f>SUM(N39:N54)</f>
         <v/>
       </c>
+      <c r="O55" s="5">
+        <f>SUM(O39:O54)</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5342,6 +5673,9 @@
       <c r="N56" s="4" t="n">
         <v>0.1642</v>
       </c>
+      <c r="O56" s="4" t="n">
+        <v>0.1642</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5390,6 +5724,9 @@
       <c r="N57" s="4" t="n">
         <v>0.3234</v>
       </c>
+      <c r="O57" s="4" t="n">
+        <v>0.3234</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5438,6 +5775,9 @@
       <c r="N58" s="4" t="n">
         <v>0.0028</v>
       </c>
+      <c r="O58" s="4" t="n">
+        <v>0.0028</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5486,6 +5826,9 @@
       <c r="N59" s="4" t="n">
         <v>0.1633</v>
       </c>
+      <c r="O59" s="4" t="n">
+        <v>0.1633</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5534,6 +5877,9 @@
       <c r="N60" s="4" t="n">
         <v>0.3462</v>
       </c>
+      <c r="O60" s="4" t="n">
+        <v>0.3462</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5586,6 +5932,10 @@
         <f>SUM(N56:N60)</f>
         <v/>
       </c>
+      <c r="O61" s="5">
+        <f>SUM(O56:O60)</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5634,6 +5984,9 @@
       <c r="N62" s="4" t="n">
         <v>0.0048</v>
       </c>
+      <c r="O62" s="4" t="n">
+        <v>0.0048</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -5682,6 +6035,9 @@
       <c r="N63" s="4" t="n">
         <v>0.0022</v>
       </c>
+      <c r="O63" s="4" t="n">
+        <v>0.0022</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5730,6 +6086,9 @@
       <c r="N64" s="4" t="n">
         <v>0.0017</v>
       </c>
+      <c r="O64" s="4" t="n">
+        <v>0.0017</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5778,6 +6137,9 @@
       <c r="N65" s="4" t="n">
         <v>0.3172</v>
       </c>
+      <c r="O65" s="4" t="n">
+        <v>0.3172</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5826,6 +6188,9 @@
       <c r="N66" s="4" t="n">
         <v>0.0106</v>
       </c>
+      <c r="O66" s="4" t="n">
+        <v>0.0106</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5874,6 +6239,9 @@
       <c r="N67" s="4" t="n">
         <v>0.1639</v>
       </c>
+      <c r="O67" s="4" t="n">
+        <v>0.1639</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5922,6 +6290,9 @@
       <c r="N68" s="4" t="n">
         <v>0.0015</v>
       </c>
+      <c r="O68" s="4" t="n">
+        <v>0.0015</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5970,6 +6341,9 @@
       <c r="N69" s="4" t="n">
         <v>0.2238</v>
       </c>
+      <c r="O69" s="4" t="n">
+        <v>0.2238</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -6018,6 +6392,9 @@
       <c r="N70" s="4" t="n">
         <v>0.0017</v>
       </c>
+      <c r="O70" s="4" t="n">
+        <v>0.0017</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -6063,6 +6440,9 @@
       <c r="N71" s="4" t="n">
         <v>0.1891</v>
       </c>
+      <c r="O71" s="4" t="n">
+        <v>0.1891</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6108,6 +6488,9 @@
       <c r="N72" s="4" t="n">
         <v>0.0018</v>
       </c>
+      <c r="O72" s="4" t="n">
+        <v>0.0018</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -6150,6 +6533,9 @@
       <c r="N73" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="O73" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -6189,6 +6575,9 @@
       <c r="N74" s="4" t="n">
         <v>0.0002</v>
       </c>
+      <c r="O74" s="4" t="n">
+        <v>0.0002</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -6225,6 +6614,9 @@
       <c r="N75" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="O75" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -6246,6 +6638,9 @@
       <c r="N76" s="4" t="n">
         <v>0.0019</v>
       </c>
+      <c r="O76" s="4" t="n">
+        <v>0.0019</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -6298,6 +6693,10 @@
         <f>SUM(N62:N76)</f>
         <v/>
       </c>
+      <c r="O77" s="5">
+        <f>SUM(O62:O76)</f>
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6346,6 +6745,9 @@
       <c r="N78" s="4" t="n">
         <v>0.318</v>
       </c>
+      <c r="O78" s="4" t="n">
+        <v>0.318</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6394,6 +6796,9 @@
       <c r="N79" s="4" t="n">
         <v>0.0941</v>
       </c>
+      <c r="O79" s="4" t="n">
+        <v>0.0941</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6442,6 +6847,9 @@
       <c r="N80" s="4" t="n">
         <v>0.0307</v>
       </c>
+      <c r="O80" s="4" t="n">
+        <v>0.0307</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6487,6 +6895,9 @@
       <c r="N81" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="O81" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6526,6 +6937,9 @@
       <c r="N82" s="4" t="n">
         <v>0.4907</v>
       </c>
+      <c r="O82" s="4" t="n">
+        <v>0.4907</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6556,6 +6970,9 @@
       <c r="N83" s="4" t="n">
         <v>0.0044</v>
       </c>
+      <c r="O83" s="4" t="n">
+        <v>0.0044</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -6608,6 +7025,10 @@
         <f>SUM(N77:N82)</f>
         <v/>
       </c>
+      <c r="O84" s="5">
+        <f>SUM(O78:O83)</f>
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6656,6 +7077,9 @@
       <c r="N85" s="4" t="n">
         <v>0.0072</v>
       </c>
+      <c r="O85" s="4" t="n">
+        <v>0.0072</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6704,6 +7128,9 @@
       <c r="N86" s="4" t="n">
         <v>0.0075</v>
       </c>
+      <c r="O86" s="4" t="n">
+        <v>0.0075</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6752,6 +7179,9 @@
       <c r="N87" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="O87" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6800,6 +7230,9 @@
       <c r="N88" s="4" t="n">
         <v>0.0191</v>
       </c>
+      <c r="O88" s="4" t="n">
+        <v>0.0191</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6848,6 +7281,9 @@
       <c r="N89" s="4" t="n">
         <v>0.0151</v>
       </c>
+      <c r="O89" s="4" t="n">
+        <v>0.0151</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -6896,6 +7332,9 @@
       <c r="N90" s="4" t="n">
         <v>0.3604</v>
       </c>
+      <c r="O90" s="4" t="n">
+        <v>0.3604</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -6941,6 +7380,9 @@
       <c r="N91" s="4" t="n">
         <v>0.5844</v>
       </c>
+      <c r="O91" s="4" t="n">
+        <v>0.5844</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -6986,6 +7428,9 @@
       <c r="N92" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="O92" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -7022,6 +7467,9 @@
       <c r="N93" s="4" t="n">
         <v>0.0062</v>
       </c>
+      <c r="O93" s="4" t="n">
+        <v>0.0062</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -7072,6 +7520,10 @@
       </c>
       <c r="N94" s="5">
         <f>SUM(N84:N92)</f>
+        <v/>
+      </c>
+      <c r="O94" s="5">
+        <f>SUM(O85:O93)</f>
         <v/>
       </c>
     </row>
@@ -7412,7 +7864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E117"/>
+  <dimension ref="A1:E120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7545,13 +7997,13 @@
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>2161.37</v>
+        <v>3125.41</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>1721.53</v>
+        <v>2478.809999999999</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>796.4994424832397</v>
+        <v>793.1151432931998</v>
       </c>
     </row>
     <row r="13">
@@ -7608,13 +8060,13 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>15629.66</v>
+        <v>17874.19</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>25084.05000000001</v>
+        <v>28660.25000000001</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>1604.900554458639</v>
+        <v>1603.443288898686</v>
       </c>
     </row>
     <row r="16">
@@ -7692,13 +8144,13 @@
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>381.77</v>
+        <v>382.2400000000001</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>402.77</v>
+        <v>404.07</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>1055.006941352123</v>
+        <v>1057.110715780661</v>
       </c>
     </row>
     <row r="20">
@@ -7713,13 +8165,13 @@
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>861.6799999999998</v>
+        <v>933.4</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>2517.58</v>
+        <v>2829.57</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>2921.711076037509</v>
+        <v>3031.465609599315</v>
       </c>
     </row>
     <row r="21">
@@ -7755,13 +8207,13 @@
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>310.68</v>
+        <v>310.93</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>627.87</v>
+        <v>628.1899999999999</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>2020.954036307455</v>
+        <v>2020.358279998713</v>
       </c>
     </row>
     <row r="23">
@@ -7797,13 +8249,13 @@
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>16671.75</v>
+        <v>16672.35</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>19026.49</v>
+        <v>19027.7</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>1141.241321396974</v>
+        <v>1141.272825966345</v>
       </c>
     </row>
     <row r="25">
@@ -7839,13 +8291,13 @@
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>262.05</v>
+        <v>286.73</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>554.13</v>
+        <v>592.9499999999999</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>2114.596451058958</v>
+        <v>2067.973354723956</v>
       </c>
     </row>
     <row r="27">
@@ -7877,17 +8329,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>20.48</v>
+        <v>4.109999999999999</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>86.87</v>
+        <v>9.25</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>4241.69921875</v>
+        <v>2250.608272506083</v>
       </c>
     </row>
     <row r="29">
@@ -7898,17 +8350,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>531.0100000000001</v>
+        <v>20.48</v>
       </c>
       <c r="D29" s="6" t="n">
-        <v>491.4800000000001</v>
+        <v>86.87</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>925.5569574960923</v>
+        <v>4241.69921875</v>
       </c>
     </row>
     <row r="30">
@@ -7919,38 +8371,38 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>8506.030000000004</v>
+        <v>531.0100000000001</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>16258.8</v>
+        <v>491.4800000000001</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>1911.443999139433</v>
+        <v>925.5569574960923</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Cold-Rolled Sheet</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C31" s="6" t="n">
-        <v>365.06</v>
+        <v>9787.210000000001</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>355.54</v>
+        <v>18590.28</v>
       </c>
       <c r="E31" s="6" t="n">
-        <v>973.9220949980823</v>
+        <v>1899.446318205086</v>
       </c>
     </row>
     <row r="32">
@@ -7961,17 +8413,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>0.51</v>
+        <v>365.06</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>0.67</v>
+        <v>355.54</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>1313.725490196078</v>
+        <v>973.9220949980823</v>
       </c>
     </row>
     <row r="33">
@@ -7982,17 +8434,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C33" s="6" t="n">
-        <v>38.36</v>
+        <v>0.51</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>59.45000000000001</v>
+        <v>0.67</v>
       </c>
       <c r="E33" s="6" t="n">
-        <v>1549.791449426486</v>
+        <v>1313.725490196078</v>
       </c>
     </row>
     <row r="34">
@@ -8003,17 +8455,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C34" s="6" t="n">
-        <v>35.28</v>
+        <v>42.7</v>
       </c>
       <c r="D34" s="6" t="n">
-        <v>81.73999999999999</v>
+        <v>68.26000000000001</v>
       </c>
       <c r="E34" s="6" t="n">
-        <v>2316.893424036281</v>
+        <v>1598.594847775176</v>
       </c>
     </row>
     <row r="35">
@@ -8024,17 +8476,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C35" s="6" t="n">
-        <v>795.15</v>
+        <v>36.19</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>1174.87</v>
+        <v>84.06</v>
       </c>
       <c r="E35" s="6" t="n">
-        <v>1477.545117273471</v>
+        <v>2322.741088698536</v>
       </c>
     </row>
     <row r="36">
@@ -8045,17 +8497,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C36" s="6" t="n">
-        <v>438.39</v>
+        <v>795.15</v>
       </c>
       <c r="D36" s="6" t="n">
-        <v>942.6799999999999</v>
+        <v>1174.87</v>
       </c>
       <c r="E36" s="6" t="n">
-        <v>2150.322771961039</v>
+        <v>1477.545117273471</v>
       </c>
     </row>
     <row r="37">
@@ -8066,17 +8518,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C37" s="6" t="n">
-        <v>259.4</v>
+        <v>0.86</v>
       </c>
       <c r="D37" s="6" t="n">
-        <v>216.61</v>
+        <v>3.13</v>
       </c>
       <c r="E37" s="6" t="n">
-        <v>835.0424055512723</v>
+        <v>3639.53488372093</v>
       </c>
     </row>
     <row r="38">
@@ -8087,17 +8539,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C38" s="6" t="n">
-        <v>5881.17</v>
+        <v>438.39</v>
       </c>
       <c r="D38" s="6" t="n">
-        <v>5165.24</v>
+        <v>942.6799999999999</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>878.2674195780771</v>
+        <v>2150.322771961039</v>
       </c>
     </row>
     <row r="39">
@@ -8108,17 +8560,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C39" s="6" t="n">
-        <v>11032.39</v>
+        <v>259.4</v>
       </c>
       <c r="D39" s="6" t="n">
-        <v>19228.37000000001</v>
+        <v>216.61</v>
       </c>
       <c r="E39" s="6" t="n">
-        <v>1742.901583428432</v>
+        <v>835.0424055512723</v>
       </c>
     </row>
     <row r="40">
@@ -8129,59 +8581,59 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C40" s="6" t="n">
-        <v>0.4</v>
+        <v>5881.17</v>
       </c>
       <c r="D40" s="6" t="n">
-        <v>0.64</v>
+        <v>5165.24</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>1600</v>
+        <v>878.2674195780771</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C41" s="6" t="n">
-        <v>170.56</v>
+        <v>12406.71</v>
       </c>
       <c r="D41" s="6" t="n">
-        <v>371.76</v>
+        <v>21804.84</v>
       </c>
       <c r="E41" s="6" t="n">
-        <v>2179.643527204503</v>
+        <v>1757.503802377906</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C42" s="6" t="n">
-        <v>1340.68</v>
+        <v>0.4</v>
       </c>
       <c r="D42" s="6" t="n">
-        <v>2141.28</v>
+        <v>0.64</v>
       </c>
       <c r="E42" s="6" t="n">
-        <v>1597.159650326699</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="43">
@@ -8192,17 +8644,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C43" s="6" t="n">
-        <v>14.96</v>
+        <v>208.06</v>
       </c>
       <c r="D43" s="6" t="n">
-        <v>45.9</v>
+        <v>729.5799999999999</v>
       </c>
       <c r="E43" s="6" t="n">
-        <v>3068.181818181818</v>
+        <v>3506.584639046428</v>
       </c>
     </row>
     <row r="44">
@@ -8213,17 +8665,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C44" s="6" t="n">
-        <v>805.9300000000001</v>
+        <v>1381.93</v>
       </c>
       <c r="D44" s="6" t="n">
-        <v>1092.53</v>
+        <v>2214.59</v>
       </c>
       <c r="E44" s="6" t="n">
-        <v>1355.614011142407</v>
+        <v>1602.534137040226</v>
       </c>
     </row>
     <row r="45">
@@ -8234,17 +8686,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C45" s="6" t="n">
-        <v>17.7</v>
+        <v>14.96</v>
       </c>
       <c r="D45" s="6" t="n">
-        <v>48.98</v>
+        <v>45.9</v>
       </c>
       <c r="E45" s="6" t="n">
-        <v>2767.231638418079</v>
+        <v>3068.181818181818</v>
       </c>
     </row>
     <row r="46">
@@ -8255,17 +8707,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C46" s="6" t="n">
-        <v>4.63</v>
+        <v>958.76</v>
       </c>
       <c r="D46" s="6" t="n">
-        <v>10.26</v>
+        <v>1305.55</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>2215.98272138229</v>
+        <v>1361.706787934415</v>
       </c>
     </row>
     <row r="47">
@@ -8276,17 +8728,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C47" s="6" t="n">
-        <v>11.28</v>
+        <v>17.7</v>
       </c>
       <c r="D47" s="6" t="n">
-        <v>46.33</v>
+        <v>48.98</v>
       </c>
       <c r="E47" s="6" t="n">
-        <v>4107.269503546099</v>
+        <v>2767.231638418079</v>
       </c>
     </row>
     <row r="48">
@@ -8297,17 +8749,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="C48" s="6" t="n">
-        <v>111.46</v>
+        <v>4.63</v>
       </c>
       <c r="D48" s="6" t="n">
-        <v>330.41</v>
+        <v>10.26</v>
       </c>
       <c r="E48" s="6" t="n">
-        <v>2964.3818410192</v>
+        <v>2215.98272138229</v>
       </c>
     </row>
     <row r="49">
@@ -8318,17 +8770,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C49" s="6" t="n">
-        <v>2680.25</v>
+        <v>11.28</v>
       </c>
       <c r="D49" s="6" t="n">
-        <v>5396.6</v>
+        <v>46.33</v>
       </c>
       <c r="E49" s="6" t="n">
-        <v>2013.468892827161</v>
+        <v>4107.269503546099</v>
       </c>
     </row>
     <row r="50">
@@ -8339,17 +8791,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C50" s="6" t="n">
-        <v>11.93</v>
+        <v>111.46</v>
       </c>
       <c r="D50" s="6" t="n">
-        <v>33.91</v>
+        <v>330.41</v>
       </c>
       <c r="E50" s="6" t="n">
-        <v>2842.414082145851</v>
+        <v>2964.3818410192</v>
       </c>
     </row>
     <row r="51">
@@ -8360,17 +8812,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C51" s="6" t="n">
-        <v>340.13</v>
+        <v>2774.73</v>
       </c>
       <c r="D51" s="6" t="n">
-        <v>471.82</v>
+        <v>5586.42</v>
       </c>
       <c r="E51" s="6" t="n">
-        <v>1387.175491723753</v>
+        <v>2013.320214939832</v>
       </c>
     </row>
     <row r="52">
@@ -8381,17 +8833,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C52" s="6" t="n">
-        <v>43.21</v>
+        <v>13.67</v>
       </c>
       <c r="D52" s="6" t="n">
-        <v>160.61</v>
+        <v>39.3</v>
       </c>
       <c r="E52" s="6" t="n">
-        <v>3716.963665818098</v>
+        <v>2874.908558888077</v>
       </c>
     </row>
     <row r="53">
@@ -8402,17 +8854,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="C53" s="6" t="n">
-        <v>524.28</v>
+        <v>340.13</v>
       </c>
       <c r="D53" s="6" t="n">
-        <v>1086.98</v>
+        <v>471.82</v>
       </c>
       <c r="E53" s="6" t="n">
-        <v>2073.281452658885</v>
+        <v>1387.175491723753</v>
       </c>
     </row>
     <row r="54">
@@ -8423,17 +8875,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C54" s="6" t="n">
-        <v>7978.940000000001</v>
+        <v>98.31</v>
       </c>
       <c r="D54" s="6" t="n">
-        <v>12760.64</v>
+        <v>300.11</v>
       </c>
       <c r="E54" s="6" t="n">
-        <v>1599.290131270569</v>
+        <v>3052.690468924829</v>
       </c>
     </row>
     <row r="55">
@@ -8444,17 +8896,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C55" s="6" t="n">
-        <v>28.85</v>
+        <v>842.0400000000001</v>
       </c>
       <c r="D55" s="6" t="n">
-        <v>47.97</v>
+        <v>1849.62</v>
       </c>
       <c r="E55" s="6" t="n">
-        <v>1662.738301559792</v>
+        <v>2196.593986033918</v>
       </c>
     </row>
     <row r="56">
@@ -8465,17 +8917,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C56" s="6" t="n">
-        <v>721.0599999999999</v>
+        <v>9201.209999999999</v>
       </c>
       <c r="D56" s="6" t="n">
-        <v>1658.96</v>
+        <v>14232.45</v>
       </c>
       <c r="E56" s="6" t="n">
-        <v>2300.723934207972</v>
+        <v>1546.801996693913</v>
       </c>
     </row>
     <row r="57">
@@ -8486,17 +8938,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C57" s="6" t="n">
-        <v>516.9000000000001</v>
+        <v>28.85</v>
       </c>
       <c r="D57" s="6" t="n">
-        <v>786.5</v>
+        <v>47.97</v>
       </c>
       <c r="E57" s="6" t="n">
-        <v>1521.570903462952</v>
+        <v>1662.738301559792</v>
       </c>
     </row>
     <row r="58">
@@ -8507,17 +8959,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>New Zealand</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C58" s="6" t="n">
-        <v>489.25</v>
+        <v>1002.95</v>
       </c>
       <c r="D58" s="6" t="n">
-        <v>567.84</v>
+        <v>2328.91</v>
       </c>
       <c r="E58" s="6" t="n">
-        <v>1160.633622892182</v>
+        <v>2322.059923226482</v>
       </c>
     </row>
     <row r="59">
@@ -8528,17 +8980,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C59" s="6" t="n">
-        <v>252.01</v>
+        <v>648.9700000000001</v>
       </c>
       <c r="D59" s="6" t="n">
-        <v>299.82</v>
+        <v>1088.52</v>
       </c>
       <c r="E59" s="6" t="n">
-        <v>1189.714693861355</v>
+        <v>1677.304035625683</v>
       </c>
     </row>
     <row r="60">
@@ -8549,17 +9001,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>New Zealand</t>
         </is>
       </c>
       <c r="C60" s="6" t="n">
-        <v>48.67</v>
+        <v>489.25</v>
       </c>
       <c r="D60" s="6" t="n">
-        <v>57.52</v>
+        <v>567.84</v>
       </c>
       <c r="E60" s="6" t="n">
-        <v>1181.836860489007</v>
+        <v>1160.633622892182</v>
       </c>
     </row>
     <row r="61">
@@ -8570,17 +9022,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="C61" s="6" t="n">
-        <v>63.97</v>
+        <v>996.73</v>
       </c>
       <c r="D61" s="6" t="n">
-        <v>81.75</v>
+        <v>1032.71</v>
       </c>
       <c r="E61" s="6" t="n">
-        <v>1277.942785680788</v>
+        <v>1036.098040592738</v>
       </c>
     </row>
     <row r="62">
@@ -8591,17 +9043,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C62" s="6" t="n">
-        <v>10021.7</v>
+        <v>48.67</v>
       </c>
       <c r="D62" s="6" t="n">
-        <v>13593.73</v>
+        <v>57.52</v>
       </c>
       <c r="E62" s="6" t="n">
-        <v>1356.429547881098</v>
+        <v>1181.836860489007</v>
       </c>
     </row>
     <row r="63">
@@ -8612,17 +9064,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="C63" s="6" t="n">
-        <v>2485.74</v>
+        <v>63.97</v>
       </c>
       <c r="D63" s="6" t="n">
-        <v>3113.53</v>
+        <v>81.75</v>
       </c>
       <c r="E63" s="6" t="n">
-        <v>1252.556582747995</v>
+        <v>1277.942785680788</v>
       </c>
     </row>
     <row r="64">
@@ -8633,17 +9085,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C64" s="6" t="n">
-        <v>11334.39</v>
+        <v>10579.12</v>
       </c>
       <c r="D64" s="6" t="n">
-        <v>12765.71</v>
+        <v>14302.06</v>
       </c>
       <c r="E64" s="6" t="n">
-        <v>1126.281167314695</v>
+        <v>1351.913958816991</v>
       </c>
     </row>
     <row r="65">
@@ -8654,17 +9106,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Ukraine</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C65" s="6" t="n">
-        <v>17.65</v>
+        <v>2485.74</v>
       </c>
       <c r="D65" s="6" t="n">
-        <v>68.54000000000001</v>
+        <v>3113.53</v>
       </c>
       <c r="E65" s="6" t="n">
-        <v>3883.28611898017</v>
+        <v>1252.556582747995</v>
       </c>
     </row>
     <row r="66">
@@ -8675,17 +9127,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C66" s="6" t="n">
-        <v>901.9299999999999</v>
+        <v>11334.39</v>
       </c>
       <c r="D66" s="6" t="n">
-        <v>1027.67</v>
+        <v>12765.71</v>
       </c>
       <c r="E66" s="6" t="n">
-        <v>1139.412149501625</v>
+        <v>1126.281167314695</v>
       </c>
     </row>
     <row r="67">
@@ -8696,17 +9148,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Ukraine</t>
         </is>
       </c>
       <c r="C67" s="6" t="n">
-        <v>26712.7</v>
+        <v>17.65</v>
       </c>
       <c r="D67" s="6" t="n">
-        <v>51182.78</v>
+        <v>68.54000000000001</v>
       </c>
       <c r="E67" s="6" t="n">
-        <v>1916.046674428268</v>
+        <v>3883.28611898017</v>
       </c>
     </row>
     <row r="68">
@@ -8717,59 +9169,59 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="C68" s="6" t="n">
-        <v>1189.02</v>
+        <v>901.9299999999999</v>
       </c>
       <c r="D68" s="6" t="n">
-        <v>1275.32</v>
+        <v>1027.67</v>
       </c>
       <c r="E68" s="6" t="n">
-        <v>1072.580780811088</v>
+        <v>1139.412149501625</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Cambodia</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C69" s="6" t="n">
-        <v>6038.5</v>
+        <v>31932.43</v>
       </c>
       <c r="D69" s="6" t="n">
-        <v>4639.469999999999</v>
+        <v>60709.84999999999</v>
       </c>
       <c r="E69" s="6" t="n">
-        <v>768.3149788854846</v>
+        <v>1901.197309443722</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C70" s="6" t="n">
-        <v>18.06</v>
+        <v>1189.02</v>
       </c>
       <c r="D70" s="6" t="n">
-        <v>14.86</v>
+        <v>1275.32</v>
       </c>
       <c r="E70" s="6" t="n">
-        <v>822.8128460686601</v>
+        <v>1072.580780811088</v>
       </c>
     </row>
     <row r="71">
@@ -8780,17 +9232,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Cambodia</t>
         </is>
       </c>
       <c r="C71" s="6" t="n">
-        <v>339.7</v>
+        <v>6038.5</v>
       </c>
       <c r="D71" s="6" t="n">
-        <v>381.9399999999999</v>
+        <v>4639.469999999999</v>
       </c>
       <c r="E71" s="6" t="n">
-        <v>1124.345010303208</v>
+        <v>768.3149788854846</v>
       </c>
     </row>
     <row r="72">
@@ -8801,17 +9253,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C72" s="6" t="n">
-        <v>1311.26</v>
+        <v>18.06</v>
       </c>
       <c r="D72" s="6" t="n">
-        <v>1218.72</v>
+        <v>14.86</v>
       </c>
       <c r="E72" s="6" t="n">
-        <v>929.4266583286305</v>
+        <v>822.8128460686601</v>
       </c>
     </row>
     <row r="73">
@@ -8822,17 +9274,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C73" s="6" t="n">
-        <v>3218.63</v>
+        <v>354.29</v>
       </c>
       <c r="D73" s="6" t="n">
-        <v>2489.5</v>
+        <v>438.73</v>
       </c>
       <c r="E73" s="6" t="n">
-        <v>773.4657292077685</v>
+        <v>1238.335826582743</v>
       </c>
     </row>
     <row r="74">
@@ -8843,17 +9295,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C74" s="6" t="n">
-        <v>23718.24</v>
+        <v>1311.26</v>
       </c>
       <c r="D74" s="6" t="n">
-        <v>25502.29</v>
+        <v>1218.72</v>
       </c>
       <c r="E74" s="6" t="n">
-        <v>1075.218481641133</v>
+        <v>929.4266583286305</v>
       </c>
     </row>
     <row r="75">
@@ -8864,17 +9316,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="C75" s="6" t="n">
-        <v>52.75</v>
+        <v>3218.63</v>
       </c>
       <c r="D75" s="6" t="n">
-        <v>53.87</v>
+        <v>2489.5</v>
       </c>
       <c r="E75" s="6" t="n">
-        <v>1021.232227488152</v>
+        <v>773.4657292077685</v>
       </c>
     </row>
     <row r="76">
@@ -8885,59 +9337,59 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C76" s="6" t="n">
-        <v>898.76</v>
+        <v>24659.24</v>
       </c>
       <c r="D76" s="6" t="n">
-        <v>1924.14</v>
+        <v>26715.55</v>
       </c>
       <c r="E76" s="6" t="n">
-        <v>2140.882994347768</v>
+        <v>1083.38902577695</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="C77" s="6" t="n">
-        <v>778.64</v>
+        <v>52.75</v>
       </c>
       <c r="D77" s="6" t="n">
-        <v>746.96</v>
+        <v>53.87</v>
       </c>
       <c r="E77" s="6" t="n">
-        <v>959.3136751258605</v>
+        <v>1021.232227488152</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C78" s="6" t="n">
-        <v>179.09</v>
+        <v>1068.9</v>
       </c>
       <c r="D78" s="6" t="n">
-        <v>176.14</v>
+        <v>2105.6</v>
       </c>
       <c r="E78" s="6" t="n">
-        <v>983.5278351666759</v>
+        <v>1969.875573018992</v>
       </c>
     </row>
     <row r="79">
@@ -8948,17 +9400,17 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C79" s="6" t="n">
-        <v>1.12</v>
+        <v>781.04</v>
       </c>
       <c r="D79" s="6" t="n">
-        <v>4.18</v>
+        <v>750.46</v>
       </c>
       <c r="E79" s="6" t="n">
-        <v>3732.142857142857</v>
+        <v>960.8470756939465</v>
       </c>
     </row>
     <row r="80">
@@ -8969,17 +9421,17 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C80" s="6" t="n">
-        <v>19.32</v>
+        <v>204.65</v>
       </c>
       <c r="D80" s="6" t="n">
-        <v>39.73</v>
+        <v>219.29</v>
       </c>
       <c r="E80" s="6" t="n">
-        <v>2056.418219461698</v>
+        <v>1071.536770095285</v>
       </c>
     </row>
     <row r="81">
@@ -8990,17 +9442,17 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="C81" s="6" t="n">
-        <v>585.71</v>
+        <v>1.12</v>
       </c>
       <c r="D81" s="6" t="n">
-        <v>916.8199999999999</v>
+        <v>4.18</v>
       </c>
       <c r="E81" s="6" t="n">
-        <v>1565.313892540677</v>
+        <v>3732.142857142857</v>
       </c>
     </row>
     <row r="82">
@@ -9011,17 +9463,17 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="C82" s="6" t="n">
-        <v>25.36</v>
+        <v>19.32</v>
       </c>
       <c r="D82" s="6" t="n">
-        <v>68.78</v>
+        <v>39.73</v>
       </c>
       <c r="E82" s="6" t="n">
-        <v>2712.145110410094</v>
+        <v>2056.418219461698</v>
       </c>
     </row>
     <row r="83">
@@ -9032,17 +9484,17 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C83" s="6" t="n">
-        <v>5.119999999999999</v>
+        <v>585.71</v>
       </c>
       <c r="D83" s="6" t="n">
-        <v>10.47</v>
+        <v>916.97</v>
       </c>
       <c r="E83" s="6" t="n">
-        <v>2044.921875</v>
+        <v>1565.569991975551</v>
       </c>
     </row>
     <row r="84">
@@ -9053,17 +9505,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C84" s="6" t="n">
-        <v>886.27</v>
+        <v>3.2</v>
       </c>
       <c r="D84" s="6" t="n">
-        <v>1190.37</v>
+        <v>4</v>
       </c>
       <c r="E84" s="6" t="n">
-        <v>1343.123427397971</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="85">
@@ -9074,17 +9526,17 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C85" s="6" t="n">
-        <v>1.16</v>
+        <v>25.36</v>
       </c>
       <c r="D85" s="6" t="n">
-        <v>5.25</v>
+        <v>68.78</v>
       </c>
       <c r="E85" s="6" t="n">
-        <v>4525.862068965516</v>
+        <v>2712.145110410094</v>
       </c>
     </row>
     <row r="86">
@@ -9095,17 +9547,17 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C86" s="6" t="n">
-        <v>17.73</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="D86" s="6" t="n">
-        <v>35.48</v>
+        <v>18.05</v>
       </c>
       <c r="E86" s="6" t="n">
-        <v>2001.128031584885</v>
+        <v>2069.954128440367</v>
       </c>
     </row>
     <row r="87">
@@ -9116,17 +9568,17 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C87" s="6" t="n">
-        <v>1448.87</v>
+        <v>905.08</v>
       </c>
       <c r="D87" s="6" t="n">
-        <v>1394.15</v>
+        <v>1216.57</v>
       </c>
       <c r="E87" s="6" t="n">
-        <v>962.2326364684203</v>
+        <v>1344.157422548283</v>
       </c>
     </row>
     <row r="88">
@@ -9137,17 +9589,17 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="C88" s="6" t="n">
-        <v>1258.61</v>
+        <v>1.27</v>
       </c>
       <c r="D88" s="6" t="n">
-        <v>1198.64</v>
+        <v>5.95</v>
       </c>
       <c r="E88" s="6" t="n">
-        <v>952.3521980597641</v>
+        <v>4685.039370078739</v>
       </c>
     </row>
     <row r="89">
@@ -9158,17 +9610,17 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C89" s="6" t="n">
-        <v>7.02</v>
+        <v>25.4</v>
       </c>
       <c r="D89" s="6" t="n">
-        <v>31.11</v>
+        <v>49.81</v>
       </c>
       <c r="E89" s="6" t="n">
-        <v>4431.623931623932</v>
+        <v>1961.023622047244</v>
       </c>
     </row>
     <row r="90">
@@ -9179,80 +9631,80 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C90" s="6" t="n">
-        <v>1655.93</v>
+        <v>1448.87</v>
       </c>
       <c r="D90" s="6" t="n">
-        <v>3483.12</v>
+        <v>1394.15</v>
       </c>
       <c r="E90" s="6" t="n">
-        <v>2103.422246109437</v>
+        <v>962.2326364684203</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C91" s="6" t="n">
-        <v>931.79</v>
+        <v>1277.28</v>
       </c>
       <c r="D91" s="6" t="n">
-        <v>1241.13</v>
+        <v>1216.36</v>
       </c>
       <c r="E91" s="6" t="n">
-        <v>1331.984674658453</v>
+        <v>952.3048979080546</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C92" s="6" t="n">
-        <v>5.78</v>
+        <v>10.8</v>
       </c>
       <c r="D92" s="6" t="n">
-        <v>10.29</v>
+        <v>47.44</v>
       </c>
       <c r="E92" s="6" t="n">
-        <v>1780.276816608997</v>
+        <v>4392.592592592593</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C93" s="6" t="n">
-        <v>6027.879999999999</v>
+        <v>1782</v>
       </c>
       <c r="D93" s="6" t="n">
-        <v>9226.099999999999</v>
+        <v>3771.49</v>
       </c>
       <c r="E93" s="6" t="n">
-        <v>1530.571278791217</v>
+        <v>2116.436588103255</v>
       </c>
     </row>
     <row r="94">
@@ -9263,17 +9715,17 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C94" s="6" t="n">
-        <v>8103.91</v>
+        <v>931.79</v>
       </c>
       <c r="D94" s="6" t="n">
-        <v>5812.44</v>
+        <v>1241.13</v>
       </c>
       <c r="E94" s="6" t="n">
-        <v>717.2389624267792</v>
+        <v>1331.984674658453</v>
       </c>
     </row>
     <row r="95">
@@ -9284,17 +9736,17 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C95" s="6" t="n">
-        <v>171.22</v>
+        <v>5.78</v>
       </c>
       <c r="D95" s="6" t="n">
-        <v>228.5</v>
+        <v>10.29</v>
       </c>
       <c r="E95" s="6" t="n">
-        <v>1334.540357434879</v>
+        <v>1780.276816608997</v>
       </c>
     </row>
     <row r="96">
@@ -9305,17 +9757,17 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C96" s="6" t="n">
-        <v>386.36</v>
+        <v>6257.499999999999</v>
       </c>
       <c r="D96" s="6" t="n">
-        <v>468.08</v>
+        <v>9524.9</v>
       </c>
       <c r="E96" s="6" t="n">
-        <v>1211.51257894192</v>
+        <v>1522.157411106672</v>
       </c>
     </row>
     <row r="97">
@@ -9326,17 +9778,17 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C97" s="6" t="n">
-        <v>288.96</v>
+        <v>8103.91</v>
       </c>
       <c r="D97" s="6" t="n">
-        <v>328.76</v>
+        <v>5812.44</v>
       </c>
       <c r="E97" s="6" t="n">
-        <v>1137.735326688815</v>
+        <v>717.2389624267792</v>
       </c>
     </row>
     <row r="98">
@@ -9347,80 +9799,80 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C98" s="6" t="n">
-        <v>4624.31</v>
+        <v>256.94</v>
       </c>
       <c r="D98" s="6" t="n">
-        <v>6631.430000000001</v>
+        <v>334.05</v>
       </c>
       <c r="E98" s="6" t="n">
-        <v>1434.036645467108</v>
+        <v>1300.108974857943</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C99" s="6" t="n">
-        <v>1579.73</v>
+        <v>482.54</v>
       </c>
       <c r="D99" s="6" t="n">
-        <v>1367.22</v>
+        <v>588</v>
       </c>
       <c r="E99" s="6" t="n">
-        <v>865.4770118944374</v>
+        <v>1218.551829900112</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C100" s="6" t="n">
-        <v>0.17</v>
+        <v>288.96</v>
       </c>
       <c r="D100" s="6" t="n">
-        <v>0.63</v>
+        <v>328.76</v>
       </c>
       <c r="E100" s="6" t="n">
-        <v>3705.882352941176</v>
+        <v>1137.735326688815</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C101" s="6" t="n">
-        <v>499.68</v>
+        <v>5283.169999999999</v>
       </c>
       <c r="D101" s="6" t="n">
-        <v>1681.03</v>
+        <v>7492.090000000001</v>
       </c>
       <c r="E101" s="6" t="n">
-        <v>3364.213096381684</v>
+        <v>1418.105039209414</v>
       </c>
     </row>
     <row r="102">
@@ -9431,17 +9883,17 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C102" s="6" t="n">
-        <v>55.17</v>
+        <v>1584.38</v>
       </c>
       <c r="D102" s="6" t="n">
-        <v>81.37</v>
+        <v>1372.53</v>
       </c>
       <c r="E102" s="6" t="n">
-        <v>1474.89577669023</v>
+        <v>866.288390411391</v>
       </c>
     </row>
     <row r="103">
@@ -9452,17 +9904,17 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C103" s="6" t="n">
-        <v>7.37</v>
+        <v>0.17</v>
       </c>
       <c r="D103" s="6" t="n">
-        <v>29.81</v>
+        <v>0.63</v>
       </c>
       <c r="E103" s="6" t="n">
-        <v>4044.776119402985</v>
+        <v>3705.882352941176</v>
       </c>
     </row>
     <row r="104">
@@ -9473,17 +9925,17 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C104" s="6" t="n">
-        <v>2542.16</v>
+        <v>499.68</v>
       </c>
       <c r="D104" s="6" t="n">
-        <v>2991.16</v>
+        <v>1681.03</v>
       </c>
       <c r="E104" s="6" t="n">
-        <v>1176.621455769897</v>
+        <v>3364.213096381684</v>
       </c>
     </row>
     <row r="105">
@@ -9494,17 +9946,17 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C105" s="6" t="n">
-        <v>34144.79</v>
+        <v>55.17</v>
       </c>
       <c r="D105" s="6" t="n">
-        <v>34109.59</v>
+        <v>81.37</v>
       </c>
       <c r="E105" s="6" t="n">
-        <v>998.9690960172841</v>
+        <v>1474.89577669023</v>
       </c>
     </row>
     <row r="106">
@@ -9515,17 +9967,17 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C106" s="6" t="n">
-        <v>6022.950000000001</v>
+        <v>8.18</v>
       </c>
       <c r="D106" s="6" t="n">
-        <v>10125.49</v>
+        <v>33.53</v>
       </c>
       <c r="E106" s="6" t="n">
-        <v>1681.151263085365</v>
+        <v>4099.022004889976</v>
       </c>
     </row>
     <row r="107">
@@ -9536,17 +9988,17 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C107" s="6" t="n">
-        <v>6118.65</v>
+        <v>4717.8</v>
       </c>
       <c r="D107" s="6" t="n">
-        <v>8472.690000000001</v>
+        <v>5541.98</v>
       </c>
       <c r="E107" s="6" t="n">
-        <v>1384.731926160182</v>
+        <v>1174.695832803425</v>
       </c>
     </row>
     <row r="108">
@@ -9557,17 +10009,17 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C108" s="6" t="n">
-        <v>0.44</v>
+        <v>49328.85999999999</v>
       </c>
       <c r="D108" s="6" t="n">
-        <v>1.8</v>
+        <v>49713.03999999999</v>
       </c>
       <c r="E108" s="6" t="n">
-        <v>4090.909090909091</v>
+        <v>1007.788138627165</v>
       </c>
     </row>
     <row r="109">
@@ -9578,17 +10030,17 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Luxembourg</t>
         </is>
       </c>
       <c r="C109" s="6" t="n">
-        <v>5036.15</v>
+        <v>6022.950000000001</v>
       </c>
       <c r="D109" s="6" t="n">
-        <v>5376.8</v>
+        <v>10125.49</v>
       </c>
       <c r="E109" s="6" t="n">
-        <v>1067.640955888923</v>
+        <v>1681.151263085365</v>
       </c>
     </row>
     <row r="110">
@@ -9599,17 +10051,17 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C110" s="6" t="n">
-        <v>0.12</v>
+        <v>7962.869999999999</v>
       </c>
       <c r="D110" s="6" t="n">
-        <v>0.59</v>
+        <v>10964.77</v>
       </c>
       <c r="E110" s="6" t="n">
-        <v>4916.666666666667</v>
+        <v>1376.98719180396</v>
       </c>
     </row>
     <row r="111">
@@ -9620,17 +10072,17 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C111" s="6" t="n">
-        <v>887.71</v>
+        <v>0.96</v>
       </c>
       <c r="D111" s="6" t="n">
-        <v>852.09</v>
+        <v>3.83</v>
       </c>
       <c r="E111" s="6" t="n">
-        <v>959.8742832681844</v>
+        <v>3989.583333333333</v>
       </c>
     </row>
     <row r="112">
@@ -9641,17 +10093,17 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C112" s="6" t="n">
-        <v>6378.700000000001</v>
+        <v>5036.45</v>
       </c>
       <c r="D112" s="6" t="n">
-        <v>5627.59</v>
+        <v>5378</v>
       </c>
       <c r="E112" s="6" t="n">
-        <v>882.2471663505102</v>
+        <v>1067.815624100309</v>
       </c>
     </row>
     <row r="113">
@@ -9662,17 +10114,17 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C113" s="6" t="n">
-        <v>2904.849999999999</v>
+        <v>0.12</v>
       </c>
       <c r="D113" s="6" t="n">
-        <v>4140.07</v>
+        <v>0.59</v>
       </c>
       <c r="E113" s="6" t="n">
-        <v>1425.226775909255</v>
+        <v>4916.666666666667</v>
       </c>
     </row>
     <row r="114">
@@ -9683,17 +10135,17 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C114" s="6" t="n">
-        <v>7469.389999999999</v>
+        <v>887.71</v>
       </c>
       <c r="D114" s="6" t="n">
-        <v>7839.33</v>
+        <v>852.09</v>
       </c>
       <c r="E114" s="6" t="n">
-        <v>1049.527471453492</v>
+        <v>959.8742832681844</v>
       </c>
     </row>
     <row r="115">
@@ -9704,17 +10156,17 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C115" s="6" t="n">
-        <v>6314.309999999999</v>
+        <v>6378.700000000001</v>
       </c>
       <c r="D115" s="6" t="n">
-        <v>7393.599999999999</v>
+        <v>5627.59</v>
       </c>
       <c r="E115" s="6" t="n">
-        <v>1170.927623129051</v>
+        <v>882.2471663505102</v>
       </c>
     </row>
     <row r="116">
@@ -9725,17 +10177,17 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C116" s="6" t="n">
-        <v>10159.72</v>
+        <v>2913.529999999999</v>
       </c>
       <c r="D116" s="6" t="n">
-        <v>24648.45</v>
+        <v>4148.74</v>
       </c>
       <c r="E116" s="6" t="n">
-        <v>2426.095404204052</v>
+        <v>1423.956506368564</v>
       </c>
     </row>
     <row r="117">
@@ -9746,16 +10198,79 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="C117" s="6" t="n">
+        <v>7469.389999999999</v>
+      </c>
+      <c r="D117" s="6" t="n">
+        <v>7839.33</v>
+      </c>
+      <c r="E117" s="6" t="n">
+        <v>1049.527471453492</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C118" s="6" t="n">
+        <v>6316.48</v>
+      </c>
+      <c r="D118" s="6" t="n">
+        <v>7401.58</v>
+      </c>
+      <c r="E118" s="6" t="n">
+        <v>1171.788717766858</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C119" s="6" t="n">
+        <v>11701.85</v>
+      </c>
+      <c r="D119" s="6" t="n">
+        <v>28649.04</v>
+      </c>
+      <c r="E119" s="6" t="n">
+        <v>2448.248781175626</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
           <t>Vietnam</t>
         </is>
       </c>
-      <c r="C117" s="6" t="n">
+      <c r="C120" s="6" t="n">
         <v>345.42</v>
       </c>
-      <c r="D117" s="6" t="n">
+      <c r="D120" s="6" t="n">
         <v>331.78</v>
       </c>
-      <c r="E117" s="6" t="n">
+      <c r="E120" s="6" t="n">
         <v>960.51184065775</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Weekly TRQ update 2026-06-15
</commit_message>
<xml_diff>
--- a/data/canada_trq_tracker.xlsx
+++ b/data/canada_trq_tracker.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q52"/>
+  <dimension ref="A1:R54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -521,6 +521,11 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
+          <t>June 15 2026</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
           <t>OVER</t>
         </is>
       </c>
@@ -578,6 +583,9 @@
       <c r="P3" s="4" t="n">
         <v>0.0361</v>
       </c>
+      <c r="Q3" s="4" t="n">
+        <v>0.0382</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -632,6 +640,9 @@
       <c r="P4" s="4" t="n">
         <v>0.0019</v>
       </c>
+      <c r="Q4" s="4" t="n">
+        <v>0.0033</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -686,7 +697,10 @@
       <c r="P5" s="4" t="n">
         <v>0.41</v>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="Q5" s="4" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="R5" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -730,6 +744,9 @@
       <c r="P6" s="4" t="n">
         <v>0.0002</v>
       </c>
+      <c r="Q6" s="4" t="n">
+        <v>0.0002</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -790,6 +807,10 @@
         <f>SUM(P3:P6)</f>
         <v/>
       </c>
+      <c r="Q7" s="5">
+        <f>SUM(Q3:Q6)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -844,7 +865,10 @@
       <c r="P8" s="4" t="n">
         <v>0.36</v>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="Q8" s="4" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="R8" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -903,6 +927,9 @@
       <c r="P9" s="4" t="n">
         <v>0.0369</v>
       </c>
+      <c r="Q9" s="4" t="n">
+        <v>0.0369</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -942,6 +969,9 @@
       <c r="P10" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="Q10" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1002,6 +1032,10 @@
         <f>SUM(P8:P10)</f>
         <v/>
       </c>
+      <c r="Q11" s="5">
+        <f>SUM(Q8:Q10)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1056,6 +1090,9 @@
       <c r="P12" s="4" t="n">
         <v>0.0063</v>
       </c>
+      <c r="Q12" s="4" t="n">
+        <v>0.0063</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1110,6 +1147,9 @@
       <c r="P13" s="4" t="n">
         <v>0.0113</v>
       </c>
+      <c r="Q13" s="4" t="n">
+        <v>0.0113</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1164,6 +1204,9 @@
       <c r="P14" s="4" t="n">
         <v>0.6692</v>
       </c>
+      <c r="Q14" s="4" t="n">
+        <v>0.6692</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1218,6 +1261,9 @@
       <c r="P15" s="4" t="n">
         <v>0.2512</v>
       </c>
+      <c r="Q15" s="4" t="n">
+        <v>0.2512</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1263,6 +1309,9 @@
       <c r="P16" s="4" t="n">
         <v>0.0552</v>
       </c>
+      <c r="Q16" s="4" t="n">
+        <v>0.0552</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1293,6 +1342,9 @@
       <c r="P17" s="4" t="n">
         <v>0.0067</v>
       </c>
+      <c r="Q17" s="4" t="n">
+        <v>0.0067</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1353,6 +1405,10 @@
         <f>SUM(P12:P17)</f>
         <v/>
       </c>
+      <c r="Q18" s="5">
+        <f>SUM(Q12:Q17)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1407,6 +1463,9 @@
       <c r="P19" s="4" t="n">
         <v>0.0092</v>
       </c>
+      <c r="Q19" s="4" t="n">
+        <v>0.0092</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1461,6 +1520,9 @@
       <c r="P20" s="4" t="n">
         <v>0.0005</v>
       </c>
+      <c r="Q20" s="4" t="n">
+        <v>0.0005</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1515,6 +1577,9 @@
       <c r="P21" s="4" t="n">
         <v>0.0532</v>
       </c>
+      <c r="Q21" s="4" t="n">
+        <v>0.0532</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1569,6 +1634,9 @@
       <c r="P22" s="4" t="n">
         <v>0.0119</v>
       </c>
+      <c r="Q22" s="4" t="n">
+        <v>0.0119</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1623,6 +1691,9 @@
       <c r="P23" s="4" t="n">
         <v>0.3695000000000001</v>
       </c>
+      <c r="Q23" s="4" t="n">
+        <v>0.3695000000000001</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1677,6 +1748,9 @@
       <c r="P24" s="4" t="n">
         <v>0.1384</v>
       </c>
+      <c r="Q24" s="4" t="n">
+        <v>0.1384</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1731,6 +1805,9 @@
       <c r="P25" s="4" t="n">
         <v>0.3262</v>
       </c>
+      <c r="Q25" s="4" t="n">
+        <v>0.3262</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1785,6 +1862,9 @@
       <c r="P26" s="4" t="n">
         <v>0.05599999999999999</v>
       </c>
+      <c r="Q26" s="4" t="n">
+        <v>0.05599999999999999</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1830,6 +1910,9 @@
       <c r="P27" s="4" t="n">
         <v>0.0207</v>
       </c>
+      <c r="Q27" s="4" t="n">
+        <v>0.0207</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1902,6 +1985,9 @@
       <c r="P29" s="4" t="n">
         <v>0.0008</v>
       </c>
+      <c r="Q29" s="4" t="n">
+        <v>0.0008</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1962,6 +2048,10 @@
         <f>SUM(P19:P29)</f>
         <v/>
       </c>
+      <c r="Q30" s="5">
+        <f>SUM(Q19:Q29)</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2016,7 +2106,10 @@
       <c r="P31" s="4" t="n">
         <v>0.29</v>
       </c>
-      <c r="Q31" t="inlineStr">
+      <c r="Q31" s="4" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="R31" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -2075,6 +2168,9 @@
       <c r="P32" s="4" t="n">
         <v>0.1228</v>
       </c>
+      <c r="Q32" s="4" t="n">
+        <v>0.1228</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2129,6 +2225,9 @@
       <c r="P33" s="4" t="n">
         <v>0.2394</v>
       </c>
+      <c r="Q33" s="4" t="n">
+        <v>0.2394</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2183,6 +2282,9 @@
       <c r="P34" s="4" t="n">
         <v>0.1668</v>
       </c>
+      <c r="Q34" s="4" t="n">
+        <v>0.1668</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2237,6 +2339,9 @@
       <c r="P35" s="4" t="n">
         <v>0.0241</v>
       </c>
+      <c r="Q35" s="4" t="n">
+        <v>0.0241</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2291,6 +2396,9 @@
       <c r="P36" s="4" t="n">
         <v>0.1569</v>
       </c>
+      <c r="Q36" s="4" t="n">
+        <v>0.1569</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2351,6 +2459,10 @@
         <f>SUM(P31:P36)</f>
         <v/>
       </c>
+      <c r="Q37" s="5">
+        <f>SUM(Q31:Q36)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2405,6 +2517,9 @@
       <c r="P38" s="4" t="n">
         <v>0.0684</v>
       </c>
+      <c r="Q38" s="4" t="n">
+        <v>0.0684</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2459,6 +2574,9 @@
       <c r="P39" s="4" t="n">
         <v>0.3214</v>
       </c>
+      <c r="Q39" s="4" t="n">
+        <v>0.3214</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2513,6 +2631,9 @@
       <c r="P40" s="4" t="n">
         <v>0.3890999999999999</v>
       </c>
+      <c r="Q40" s="4" t="n">
+        <v>0.3890999999999999</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2567,6 +2688,9 @@
       <c r="P41" s="4" t="n">
         <v>0.2185</v>
       </c>
+      <c r="Q41" s="4" t="n">
+        <v>0.212</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2615,6 +2739,9 @@
       <c r="P42" s="4" t="n">
         <v>0.0005</v>
       </c>
+      <c r="Q42" s="4" t="n">
+        <v>0.0005</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2675,6 +2802,10 @@
         <f>SUM(P38:P42)</f>
         <v/>
       </c>
+      <c r="Q43" s="5">
+        <f>SUM(Q38:Q42)</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2729,6 +2860,9 @@
       <c r="P44" s="4" t="n">
         <v>0.442</v>
       </c>
+      <c r="Q44" s="4" t="n">
+        <v>0.442</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2771,7 +2905,10 @@
       <c r="P45" s="4" t="n">
         <v>0.45</v>
       </c>
-      <c r="Q45" t="inlineStr">
+      <c r="Q45" s="4" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="R45" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -2815,6 +2952,9 @@
       <c r="P46" s="4" t="n">
         <v>0.0024</v>
       </c>
+      <c r="Q46" s="4" t="n">
+        <v>0.0024</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2875,6 +3015,10 @@
         <f>SUM(P44:P46)</f>
         <v/>
       </c>
+      <c r="Q47" s="5">
+        <f>SUM(Q44:Q46)</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2929,6 +3073,9 @@
       <c r="P48" s="4" t="n">
         <v>0.04269999999999999</v>
       </c>
+      <c r="Q48" s="4" t="n">
+        <v>0.08810000000000001</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2983,6 +3130,9 @@
       <c r="P49" s="4" t="n">
         <v>0.0236</v>
       </c>
+      <c r="Q49" s="4" t="n">
+        <v>0.0353</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3037,6 +3187,9 @@
       <c r="P50" s="4" t="n">
         <v>0.3917</v>
       </c>
+      <c r="Q50" s="4" t="n">
+        <v>0.3962</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3091,6 +3244,9 @@
       <c r="P51" s="4" t="n">
         <v>0.1041</v>
       </c>
+      <c r="Q51" s="4" t="n">
+        <v>0.2693</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3100,55 +3256,101 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
+          <t>Oman</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="n">
+        <v>4674200</v>
+      </c>
+      <c r="D52" s="4" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="Q52" s="4" t="n">
+        <v>0.0108</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="n">
+        <v>4674200</v>
+      </c>
+      <c r="D53" s="4" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="Q53" s="4" t="n">
+        <v>0.04269999999999999</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E52" s="5">
+      <c r="E54" s="5">
         <f>SUM(E38:E41)</f>
         <v/>
       </c>
-      <c r="F52" s="5">
+      <c r="F54" s="5">
         <f>SUM(F38:F41)</f>
         <v/>
       </c>
-      <c r="G52" s="5">
+      <c r="G54" s="5">
         <f>SUM(G38:G41)</f>
         <v/>
       </c>
-      <c r="H52" s="5">
+      <c r="H54" s="5">
         <f>SUM(H39:H42)</f>
         <v/>
       </c>
-      <c r="I52" s="5">
+      <c r="I54" s="5">
         <f>SUM(I41:I44)</f>
         <v/>
       </c>
-      <c r="J52" s="5">
+      <c r="J54" s="5">
         <f>SUM(J42:J45)</f>
         <v/>
       </c>
-      <c r="K52" s="5">
+      <c r="K54" s="5">
         <f>SUM(K46:K49)</f>
         <v/>
       </c>
-      <c r="L52" s="5">
+      <c r="L54" s="5">
         <f>SUM(L46:L49)</f>
         <v/>
       </c>
-      <c r="M52" s="5">
+      <c r="M54" s="5">
         <f>SUM(M47:M50)</f>
         <v/>
       </c>
-      <c r="N52" s="5">
+      <c r="N54" s="5">
         <f>SUM(N48:N51)</f>
         <v/>
       </c>
-      <c r="O52" s="5">
+      <c r="O54" s="5">
         <f>SUM(O48:O51)</f>
         <v/>
       </c>
-      <c r="P52" s="5">
+      <c r="P54" s="5">
         <f>SUM(P48:P51)</f>
+        <v/>
+      </c>
+      <c r="Q54" s="5">
+        <f>SUM(Q48:Q53)</f>
         <v/>
       </c>
     </row>
@@ -3163,7 +3365,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q96"/>
+  <dimension ref="A1:R96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3251,6 +3453,11 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
+          <t>June 15 2026</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
           <t>OVER</t>
         </is>
       </c>
@@ -3308,6 +3515,9 @@
       <c r="P3" s="4" t="n">
         <v>0.003</v>
       </c>
+      <c r="Q3" s="4" t="n">
+        <v>0.003</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3362,6 +3572,9 @@
       <c r="P4" s="4" t="n">
         <v>0.1164</v>
       </c>
+      <c r="Q4" s="4" t="n">
+        <v>0.1164</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3416,6 +3629,9 @@
       <c r="P5" s="4" t="n">
         <v>0.115</v>
       </c>
+      <c r="Q5" s="4" t="n">
+        <v>0.115</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3470,6 +3686,9 @@
       <c r="P6" s="4" t="n">
         <v>0.4198</v>
       </c>
+      <c r="Q6" s="4" t="n">
+        <v>0.4198</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3524,6 +3743,9 @@
       <c r="P7" s="4" t="n">
         <v>0.07429999999999999</v>
       </c>
+      <c r="Q7" s="4" t="n">
+        <v>0.07429999999999999</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3578,6 +3800,9 @@
       <c r="P8" s="4" t="n">
         <v>0.0008</v>
       </c>
+      <c r="Q8" s="4" t="n">
+        <v>0.0008</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3632,6 +3857,9 @@
       <c r="P9" s="4" t="n">
         <v>0.0143</v>
       </c>
+      <c r="Q9" s="4" t="n">
+        <v>0.0143</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3680,6 +3908,9 @@
       <c r="P10" s="4" t="n">
         <v>0.014</v>
       </c>
+      <c r="Q10" s="4" t="n">
+        <v>0.014</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3734,6 +3965,9 @@
       <c r="P11" s="4" t="n">
         <v>0.0004</v>
       </c>
+      <c r="Q11" s="4" t="n">
+        <v>0.0004</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3785,6 +4019,9 @@
       <c r="P12" s="4" t="n">
         <v>0.0012</v>
       </c>
+      <c r="Q12" s="4" t="n">
+        <v>0.0012</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3836,6 +4073,9 @@
       <c r="P13" s="4" t="n">
         <v>0.0003</v>
       </c>
+      <c r="Q13" s="4" t="n">
+        <v>0.0003</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3881,6 +4121,9 @@
       <c r="P14" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="Q14" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3923,6 +4166,9 @@
       <c r="P15" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="Q15" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3965,6 +4211,9 @@
       <c r="P16" s="4" t="n">
         <v>0.2405</v>
       </c>
+      <c r="Q16" s="4" t="n">
+        <v>0.2405</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4025,6 +4274,10 @@
         <f>SUM(P3:P16)</f>
         <v/>
       </c>
+      <c r="Q17" s="5">
+        <f>SUM(Q3:Q16)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4079,6 +4332,9 @@
       <c r="P18" s="4" t="n">
         <v>0.0338</v>
       </c>
+      <c r="Q18" s="4" t="n">
+        <v>0.0338</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4133,6 +4389,9 @@
       <c r="P19" s="4" t="n">
         <v>0.031</v>
       </c>
+      <c r="Q19" s="4" t="n">
+        <v>0.031</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4187,6 +4446,9 @@
       <c r="P20" s="4" t="n">
         <v>0.0741</v>
       </c>
+      <c r="Q20" s="4" t="n">
+        <v>0.0741</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4241,6 +4503,9 @@
       <c r="P21" s="4" t="n">
         <v>0.154</v>
       </c>
+      <c r="Q21" s="4" t="n">
+        <v>0.154</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4295,6 +4560,9 @@
       <c r="P22" s="4" t="n">
         <v>0.1063</v>
       </c>
+      <c r="Q22" s="4" t="n">
+        <v>0.1063</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4349,7 +4617,10 @@
       <c r="P23" s="4" t="n">
         <v>0.3</v>
       </c>
-      <c r="Q23" t="inlineStr">
+      <c r="Q23" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="R23" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -4408,6 +4679,9 @@
       <c r="P24" s="4" t="n">
         <v>0.1668</v>
       </c>
+      <c r="Q24" s="4" t="n">
+        <v>0.1668</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4462,6 +4736,9 @@
       <c r="P25" s="4" t="n">
         <v>0.0005</v>
       </c>
+      <c r="Q25" s="4" t="n">
+        <v>0.0005</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4516,6 +4793,9 @@
       <c r="P26" s="4" t="n">
         <v>0.0694</v>
       </c>
+      <c r="Q26" s="4" t="n">
+        <v>0.06900000000000001</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4567,6 +4847,9 @@
       <c r="P27" s="4" t="n">
         <v>0.0317</v>
       </c>
+      <c r="Q27" s="4" t="n">
+        <v>0.0317</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4618,6 +4901,9 @@
       <c r="P28" s="4" t="n">
         <v>0.0073</v>
       </c>
+      <c r="Q28" s="4" t="n">
+        <v>0.0073</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4669,6 +4955,9 @@
       <c r="P29" s="4" t="n">
         <v>0.0005999999999999999</v>
       </c>
+      <c r="Q29" s="4" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4714,6 +5003,9 @@
       <c r="P30" s="4" t="n">
         <v>0.0226</v>
       </c>
+      <c r="Q30" s="4" t="n">
+        <v>0.0226</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4750,6 +5042,9 @@
       <c r="P31" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="Q31" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4810,6 +5105,10 @@
         <f>SUM(P18:P31)</f>
         <v/>
       </c>
+      <c r="Q32" s="5">
+        <f>SUM(Q18:Q31)</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4864,6 +5163,9 @@
       <c r="P33" s="4" t="n">
         <v>0.258</v>
       </c>
+      <c r="Q33" s="4" t="n">
+        <v>0.258</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4915,6 +5217,9 @@
       <c r="P34" s="4" t="n">
         <v>0.236</v>
       </c>
+      <c r="Q34" s="4" t="n">
+        <v>0.236</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4960,6 +5265,9 @@
       <c r="P35" s="4" t="n">
         <v>0.1992</v>
       </c>
+      <c r="Q35" s="4" t="n">
+        <v>0.1992</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5002,6 +5310,9 @@
       <c r="P36" s="4" t="n">
         <v>0.0011</v>
       </c>
+      <c r="Q36" s="4" t="n">
+        <v>0.0011</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5038,6 +5349,9 @@
       <c r="P37" s="4" t="n">
         <v>0.3057</v>
       </c>
+      <c r="Q37" s="4" t="n">
+        <v>0.3057</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5098,6 +5412,10 @@
         <f>SUM(P33:P37)</f>
         <v/>
       </c>
+      <c r="Q38" s="5">
+        <f>SUM(Q33:Q37)</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5152,6 +5470,9 @@
       <c r="P39" s="4" t="n">
         <v>0.166</v>
       </c>
+      <c r="Q39" s="4" t="n">
+        <v>0.166</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5206,6 +5527,9 @@
       <c r="P40" s="4" t="n">
         <v>0.1686</v>
       </c>
+      <c r="Q40" s="4" t="n">
+        <v>0.1686</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5260,6 +5584,9 @@
       <c r="P41" s="4" t="n">
         <v>0.2496</v>
       </c>
+      <c r="Q41" s="4" t="n">
+        <v>0.2496</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5314,6 +5641,9 @@
       <c r="P42" s="4" t="n">
         <v>0.09910000000000001</v>
       </c>
+      <c r="Q42" s="4" t="n">
+        <v>0.09910000000000001</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5368,6 +5698,9 @@
       <c r="P43" s="4" t="n">
         <v>0.0849</v>
       </c>
+      <c r="Q43" s="4" t="n">
+        <v>0.0849</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5422,6 +5755,9 @@
       <c r="P44" s="4" t="n">
         <v>0.0007000000000000001</v>
       </c>
+      <c r="Q44" s="4" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5476,6 +5812,9 @@
       <c r="P45" s="4" t="n">
         <v>0.0906</v>
       </c>
+      <c r="Q45" s="4" t="n">
+        <v>0.0906</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5527,6 +5866,9 @@
       <c r="P46" s="4" t="n">
         <v>0.0014</v>
       </c>
+      <c r="Q46" s="4" t="n">
+        <v>0.0014</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5578,6 +5920,9 @@
       <c r="P47" s="4" t="n">
         <v>0.0354</v>
       </c>
+      <c r="Q47" s="4" t="n">
+        <v>0.0354</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5629,6 +5974,9 @@
       <c r="P48" s="4" t="n">
         <v>0.028</v>
       </c>
+      <c r="Q48" s="4" t="n">
+        <v>0.028</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5677,6 +6025,9 @@
       <c r="P49" s="4" t="n">
         <v>0.0003</v>
       </c>
+      <c r="Q49" s="4" t="n">
+        <v>0.0003</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5722,6 +6073,9 @@
       <c r="P50" s="4" t="n">
         <v>0.0014</v>
       </c>
+      <c r="Q50" s="4" t="n">
+        <v>0.0014</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5767,6 +6121,9 @@
       <c r="P51" s="4" t="n">
         <v>0.0157</v>
       </c>
+      <c r="Q51" s="4" t="n">
+        <v>0.0157</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5812,6 +6169,9 @@
       <c r="P52" s="4" t="n">
         <v>0.0215</v>
       </c>
+      <c r="Q52" s="4" t="n">
+        <v>0.0215</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5854,6 +6214,9 @@
       <c r="P53" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="Q53" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5896,6 +6259,9 @@
       <c r="P54" s="4" t="n">
         <v>0.0258</v>
       </c>
+      <c r="Q54" s="4" t="n">
+        <v>0.0258</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5956,6 +6322,10 @@
         <f>SUM(P39:P54)</f>
         <v/>
       </c>
+      <c r="Q55" s="5">
+        <f>SUM(Q39:Q54)</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -6010,6 +6380,9 @@
       <c r="P56" s="4" t="n">
         <v>0.1642</v>
       </c>
+      <c r="Q56" s="4" t="n">
+        <v>0.1642</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -6064,6 +6437,9 @@
       <c r="P57" s="4" t="n">
         <v>0.3234</v>
       </c>
+      <c r="Q57" s="4" t="n">
+        <v>0.3234</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -6118,6 +6494,9 @@
       <c r="P58" s="4" t="n">
         <v>0.0028</v>
       </c>
+      <c r="Q58" s="4" t="n">
+        <v>0.0028</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -6172,6 +6551,9 @@
       <c r="P59" s="4" t="n">
         <v>0.1633</v>
       </c>
+      <c r="Q59" s="4" t="n">
+        <v>0.1633</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6226,6 +6608,9 @@
       <c r="P60" s="4" t="n">
         <v>0.3462</v>
       </c>
+      <c r="Q60" s="4" t="n">
+        <v>0.3462</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6286,6 +6671,10 @@
         <f>SUM(P56:P60)</f>
         <v/>
       </c>
+      <c r="Q61" s="5">
+        <f>SUM(Q56:Q60)</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -6340,6 +6729,9 @@
       <c r="P62" s="4" t="n">
         <v>0.004500000000000001</v>
       </c>
+      <c r="Q62" s="4" t="n">
+        <v>0.004500000000000001</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -6394,6 +6786,9 @@
       <c r="P63" s="4" t="n">
         <v>0.0022</v>
       </c>
+      <c r="Q63" s="4" t="n">
+        <v>0.0022</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -6448,6 +6843,9 @@
       <c r="P64" s="4" t="n">
         <v>0.0018</v>
       </c>
+      <c r="Q64" s="4" t="n">
+        <v>0.0018</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -6502,6 +6900,9 @@
       <c r="P65" s="4" t="n">
         <v>0.3186</v>
       </c>
+      <c r="Q65" s="4" t="n">
+        <v>0.3186</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -6556,6 +6957,9 @@
       <c r="P66" s="4" t="n">
         <v>0.0108</v>
       </c>
+      <c r="Q66" s="4" t="n">
+        <v>0.0108</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -6610,6 +7014,9 @@
       <c r="P67" s="4" t="n">
         <v>0.1648</v>
       </c>
+      <c r="Q67" s="4" t="n">
+        <v>0.1648</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -6664,6 +7071,9 @@
       <c r="P68" s="4" t="n">
         <v>0.0015</v>
       </c>
+      <c r="Q68" s="4" t="n">
+        <v>0.0015</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -6718,6 +7128,9 @@
       <c r="P69" s="4" t="n">
         <v>0.2402</v>
       </c>
+      <c r="Q69" s="4" t="n">
+        <v>0.2402</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -6772,6 +7185,9 @@
       <c r="P70" s="4" t="n">
         <v>0.0017</v>
       </c>
+      <c r="Q70" s="4" t="n">
+        <v>0.0017</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -6823,6 +7239,9 @@
       <c r="P71" s="4" t="n">
         <v>0.2269</v>
       </c>
+      <c r="Q71" s="4" t="n">
+        <v>0.2399</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6874,6 +7293,9 @@
       <c r="P72" s="4" t="n">
         <v>0.0066</v>
       </c>
+      <c r="Q72" s="4" t="n">
+        <v>0.0066</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -6922,6 +7344,9 @@
       <c r="P73" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="Q73" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -6967,6 +7392,9 @@
       <c r="P74" s="4" t="n">
         <v>0.0002</v>
       </c>
+      <c r="Q74" s="4" t="n">
+        <v>0.0002</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -7009,6 +7437,9 @@
       <c r="P75" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="Q75" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -7036,6 +7467,9 @@
       <c r="P76" s="4" t="n">
         <v>0.0019</v>
       </c>
+      <c r="Q76" s="4" t="n">
+        <v>0.0019</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -7057,6 +7491,9 @@
       <c r="P77" s="4" t="n">
         <v>0.0005</v>
       </c>
+      <c r="Q77" s="4" t="n">
+        <v>0.0005</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -7078,6 +7515,9 @@
       <c r="P78" s="4" t="n">
         <v>0.0026</v>
       </c>
+      <c r="Q78" s="4" t="n">
+        <v>0.0026</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -7138,6 +7578,10 @@
         <f>SUM(P62:P78)</f>
         <v/>
       </c>
+      <c r="Q79" s="5">
+        <f>SUM(Q62:Q78)</f>
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -7192,6 +7636,9 @@
       <c r="P80" s="4" t="n">
         <v>0.3456</v>
       </c>
+      <c r="Q80" s="4" t="n">
+        <v>0.3688</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -7246,6 +7693,9 @@
       <c r="P81" s="4" t="n">
         <v>0.0941</v>
       </c>
+      <c r="Q81" s="4" t="n">
+        <v>0.0941</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -7300,6 +7750,9 @@
       <c r="P82" s="4" t="n">
         <v>0.0307</v>
       </c>
+      <c r="Q82" s="4" t="n">
+        <v>0.0307</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -7351,6 +7804,9 @@
       <c r="P83" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="Q83" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -7396,6 +7852,9 @@
       <c r="P84" s="4" t="n">
         <v>0.4907</v>
       </c>
+      <c r="Q84" s="4" t="n">
+        <v>0.4907</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -7432,6 +7891,9 @@
       <c r="P85" s="4" t="n">
         <v>0.0044</v>
       </c>
+      <c r="Q85" s="4" t="n">
+        <v>0.0044</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7492,6 +7954,10 @@
         <f>SUM(P78:P83)</f>
         <v/>
       </c>
+      <c r="Q86" s="5">
+        <f>SUM(Q80:Q85)</f>
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -7546,6 +8012,9 @@
       <c r="P87" s="4" t="n">
         <v>0.0072</v>
       </c>
+      <c r="Q87" s="4" t="n">
+        <v>0.0072</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -7600,6 +8069,9 @@
       <c r="P88" s="4" t="n">
         <v>0.0075</v>
       </c>
+      <c r="Q88" s="4" t="n">
+        <v>0.0075</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -7654,6 +8126,9 @@
       <c r="P89" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="Q89" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -7708,6 +8183,9 @@
       <c r="P90" s="4" t="n">
         <v>0.0191</v>
       </c>
+      <c r="Q90" s="4" t="n">
+        <v>0.0191</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -7762,6 +8240,9 @@
       <c r="P91" s="4" t="n">
         <v>0.0151</v>
       </c>
+      <c r="Q91" s="4" t="n">
+        <v>0.0151</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -7816,6 +8297,9 @@
       <c r="P92" s="4" t="n">
         <v>0.3604</v>
       </c>
+      <c r="Q92" s="4" t="n">
+        <v>0.3604</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -7867,6 +8351,9 @@
       <c r="P93" s="4" t="n">
         <v>0.5844</v>
       </c>
+      <c r="Q93" s="4" t="n">
+        <v>0.5844</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -7918,6 +8405,9 @@
       <c r="P94" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="Q94" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -7960,6 +8450,9 @@
       <c r="P95" s="4" t="n">
         <v>0.0062</v>
       </c>
+      <c r="Q95" s="4" t="n">
+        <v>0.0062</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -8018,6 +8511,10 @@
       </c>
       <c r="P96" s="5">
         <f>SUM(P85:P93)</f>
+        <v/>
+      </c>
+      <c r="Q96" s="5">
+        <f>SUM(Q87:Q95)</f>
         <v/>
       </c>
     </row>
@@ -8358,7 +8855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E122"/>
+  <dimension ref="A1:E124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8466,17 +8963,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0</v>
+        <v>674.25</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.17</v>
+        <v>1052.56</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0</v>
+        <v>1561.082684464219</v>
       </c>
     </row>
     <row r="12">
@@ -8487,17 +8984,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>674.25</v>
+        <v>3125.41</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>1052.56</v>
+        <v>2478.809999999999</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>1561.082684464219</v>
+        <v>793.1151432931998</v>
       </c>
     </row>
     <row r="13">
@@ -8508,17 +9005,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>3125.41</v>
+        <v>321.38</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>2478.809999999999</v>
+        <v>437.34</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>793.1151432931998</v>
+        <v>1360.818968199639</v>
       </c>
     </row>
     <row r="14">
@@ -8529,17 +9026,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>321.38</v>
+        <v>14.25</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>437.34</v>
+        <v>52.25</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>1360.818968199639</v>
+        <v>3666.666666666667</v>
       </c>
     </row>
     <row r="15">
@@ -8550,17 +9047,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>14.25</v>
+        <v>21716.48</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>52.25</v>
+        <v>35428.3</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>3666.666666666667</v>
+        <v>1631.401589944595</v>
       </c>
     </row>
     <row r="16">
@@ -8571,38 +9068,38 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>19453.7</v>
+        <v>2290.17</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>31335.91</v>
+        <v>1767.74</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1610.794347604826</v>
+        <v>771.8815633773913</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Hot-Rolled Sheet</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>2290.17</v>
+        <v>1230.35</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>1767.74</v>
+        <v>1361.29</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>771.8815633773913</v>
+        <v>1106.425001015971</v>
       </c>
     </row>
     <row r="18">
@@ -8613,17 +9110,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>1230.35</v>
+        <v>0.23</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>1361.29</v>
+        <v>0.46</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1106.425001015971</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="19">
@@ -8634,17 +9131,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0.23</v>
+        <v>382.7100000000001</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>0.46</v>
+        <v>404.81</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>2000</v>
+        <v>1057.746074050848</v>
       </c>
     </row>
     <row r="20">
@@ -8655,17 +9152,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>382.2400000000001</v>
+        <v>933.4</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>404.07</v>
+        <v>2829.57</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>1057.110715780661</v>
+        <v>3031.465609599315</v>
       </c>
     </row>
     <row r="21">
@@ -8676,17 +9173,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>933.4</v>
+        <v>5298.749999999999</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>2829.57</v>
+        <v>6840.83</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>3031.465609599315</v>
+        <v>1291.027129039868</v>
       </c>
     </row>
     <row r="22">
@@ -8697,17 +9194,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>5298.749999999999</v>
+        <v>310.93</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>6840.83</v>
+        <v>628.1899999999999</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>1291.027129039868</v>
+        <v>2020.358279998713</v>
       </c>
     </row>
     <row r="23">
@@ -8718,17 +9215,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>310.93</v>
+        <v>2.07</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>628.1899999999999</v>
+        <v>6.74</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>2020.358279998713</v>
+        <v>3256.038647342995</v>
       </c>
     </row>
     <row r="24">
@@ -8739,17 +9236,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>2.07</v>
+        <v>16672.35</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>6.74</v>
+        <v>19027.7</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>3256.038647342995</v>
+        <v>1141.272825966345</v>
       </c>
     </row>
     <row r="25">
@@ -8760,17 +9257,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C25" s="6" t="n">
-        <v>16672.35</v>
+        <v>8999.279999999999</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>19027.7</v>
+        <v>10665.01</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>1141.272825966345</v>
+        <v>1185.095918784614</v>
       </c>
     </row>
     <row r="26">
@@ -8781,17 +9278,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>8999.279999999999</v>
+        <v>0.68</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>10665.01</v>
+        <v>13.84</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>1185.095918784614</v>
+        <v>20352.94117647059</v>
       </c>
     </row>
     <row r="27">
@@ -8806,13 +9303,13 @@
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>286.73</v>
+        <v>313.62</v>
       </c>
       <c r="D27" s="6" t="n">
-        <v>592.9499999999999</v>
+        <v>645.9599999999999</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>2067.973354723956</v>
+        <v>2059.690070786301</v>
       </c>
     </row>
     <row r="28">
@@ -8827,13 +9324,13 @@
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>13.42</v>
+        <v>24.22</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>25.28</v>
+        <v>45.67</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>1883.755588673622</v>
+        <v>1885.631709331131</v>
       </c>
     </row>
     <row r="29">
@@ -8911,13 +9408,13 @@
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>11536.66</v>
+        <v>12823.09</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>22004.04</v>
+        <v>24464.32000000001</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>1907.314595385493</v>
+        <v>1907.83344732042</v>
       </c>
     </row>
     <row r="33">
@@ -8974,13 +9471,13 @@
         </is>
       </c>
       <c r="C35" s="6" t="n">
-        <v>44.77</v>
+        <v>46.09999999999999</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>72.66000000000001</v>
+        <v>74.94000000000001</v>
       </c>
       <c r="E35" s="6" t="n">
-        <v>1622.961804779987</v>
+        <v>1625.596529284165</v>
       </c>
     </row>
     <row r="36">
@@ -9054,17 +9551,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="C39" s="6" t="n">
-        <v>438.39</v>
+        <v>41.3</v>
       </c>
       <c r="D39" s="6" t="n">
-        <v>942.6799999999999</v>
+        <v>45.1</v>
       </c>
       <c r="E39" s="6" t="n">
-        <v>2150.322771961039</v>
+        <v>1092.009685230024</v>
       </c>
     </row>
     <row r="40">
@@ -9075,17 +9572,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C40" s="6" t="n">
-        <v>2161.61</v>
+        <v>438.39</v>
       </c>
       <c r="D40" s="6" t="n">
-        <v>1834.44</v>
+        <v>942.6799999999999</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>848.6452227737658</v>
+        <v>2150.322771961039</v>
       </c>
     </row>
     <row r="41">
@@ -9096,17 +9593,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C41" s="6" t="n">
-        <v>5881.17</v>
+        <v>2161.61</v>
       </c>
       <c r="D41" s="6" t="n">
-        <v>5165.24</v>
+        <v>1834.44</v>
       </c>
       <c r="E41" s="6" t="n">
-        <v>878.2674195780771</v>
+        <v>848.6452227737658</v>
       </c>
     </row>
     <row r="42">
@@ -9117,17 +9614,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C42" s="6" t="n">
-        <v>14018.34000000001</v>
+        <v>5881.17</v>
       </c>
       <c r="D42" s="6" t="n">
-        <v>24776.24</v>
+        <v>5165.24</v>
       </c>
       <c r="E42" s="6" t="n">
-        <v>1767.416113462792</v>
+        <v>878.2674195780771</v>
       </c>
     </row>
     <row r="43">
@@ -9138,38 +9635,38 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C43" s="6" t="n">
-        <v>0.4</v>
+        <v>15412</v>
       </c>
       <c r="D43" s="6" t="n">
-        <v>0.64</v>
+        <v>27250.72</v>
       </c>
       <c r="E43" s="6" t="n">
-        <v>1600</v>
+        <v>1768.149493900856</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C44" s="6" t="n">
-        <v>170.56</v>
+        <v>0.4</v>
       </c>
       <c r="D44" s="6" t="n">
-        <v>371.76</v>
+        <v>0.64</v>
       </c>
       <c r="E44" s="6" t="n">
-        <v>2179.643527204503</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="45">
@@ -9180,17 +9677,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C45" s="6" t="n">
-        <v>1427.39</v>
+        <v>170.56</v>
       </c>
       <c r="D45" s="6" t="n">
-        <v>2300.44</v>
+        <v>371.76</v>
       </c>
       <c r="E45" s="6" t="n">
-        <v>1611.640826963899</v>
+        <v>2179.643527204503</v>
       </c>
     </row>
     <row r="46">
@@ -9201,17 +9698,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C46" s="6" t="n">
-        <v>14.96</v>
+        <v>1427.39</v>
       </c>
       <c r="D46" s="6" t="n">
-        <v>45.9</v>
+        <v>2300.44</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>3068.181818181818</v>
+        <v>1611.640826963899</v>
       </c>
     </row>
     <row r="47">
@@ -9222,17 +9719,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C47" s="6" t="n">
-        <v>1037.03</v>
+        <v>14.96</v>
       </c>
       <c r="D47" s="6" t="n">
-        <v>1369.26</v>
+        <v>45.9</v>
       </c>
       <c r="E47" s="6" t="n">
-        <v>1320.366816774828</v>
+        <v>3068.181818181818</v>
       </c>
     </row>
     <row r="48">
@@ -9243,17 +9740,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C48" s="6" t="n">
-        <v>17.7</v>
+        <v>1138.19</v>
       </c>
       <c r="D48" s="6" t="n">
-        <v>48.98</v>
+        <v>1616.86</v>
       </c>
       <c r="E48" s="6" t="n">
-        <v>2767.231638418079</v>
+        <v>1420.553686115675</v>
       </c>
     </row>
     <row r="49">
@@ -9264,17 +9761,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C49" s="6" t="n">
-        <v>4.63</v>
+        <v>17.7</v>
       </c>
       <c r="D49" s="6" t="n">
-        <v>10.26</v>
+        <v>48.98</v>
       </c>
       <c r="E49" s="6" t="n">
-        <v>2215.98272138229</v>
+        <v>2767.231638418079</v>
       </c>
     </row>
     <row r="50">
@@ -9285,17 +9782,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="C50" s="6" t="n">
-        <v>11.28</v>
+        <v>4.63</v>
       </c>
       <c r="D50" s="6" t="n">
-        <v>46.33</v>
+        <v>10.26</v>
       </c>
       <c r="E50" s="6" t="n">
-        <v>4107.269503546099</v>
+        <v>2215.98272138229</v>
       </c>
     </row>
     <row r="51">
@@ -9306,17 +9803,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C51" s="6" t="n">
-        <v>111.46</v>
+        <v>11.28</v>
       </c>
       <c r="D51" s="6" t="n">
-        <v>330.41</v>
+        <v>46.33</v>
       </c>
       <c r="E51" s="6" t="n">
-        <v>2964.3818410192</v>
+        <v>4107.269503546099</v>
       </c>
     </row>
     <row r="52">
@@ -9327,17 +9824,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C52" s="6" t="n">
-        <v>2777.58</v>
+        <v>111.46</v>
       </c>
       <c r="D52" s="6" t="n">
-        <v>5591.32</v>
+        <v>330.41</v>
       </c>
       <c r="E52" s="6" t="n">
-        <v>2013.018526919116</v>
+        <v>2964.3818410192</v>
       </c>
     </row>
     <row r="53">
@@ -9348,17 +9845,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C53" s="6" t="n">
-        <v>13.67</v>
+        <v>2797.02</v>
       </c>
       <c r="D53" s="6" t="n">
-        <v>39.3</v>
+        <v>5628.44</v>
       </c>
       <c r="E53" s="6" t="n">
-        <v>2874.908558888077</v>
+        <v>2012.298803726824</v>
       </c>
     </row>
     <row r="54">
@@ -9369,17 +9866,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C54" s="6" t="n">
-        <v>340.13</v>
+        <v>13.67</v>
       </c>
       <c r="D54" s="6" t="n">
-        <v>471.82</v>
+        <v>39.3</v>
       </c>
       <c r="E54" s="6" t="n">
-        <v>1387.175491723753</v>
+        <v>2874.908558888077</v>
       </c>
     </row>
     <row r="55">
@@ -9390,17 +9887,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="C55" s="6" t="n">
-        <v>98.31</v>
+        <v>340.13</v>
       </c>
       <c r="D55" s="6" t="n">
-        <v>300.11</v>
+        <v>471.82</v>
       </c>
       <c r="E55" s="6" t="n">
-        <v>3052.690468924829</v>
+        <v>1387.175491723753</v>
       </c>
     </row>
     <row r="56">
@@ -9411,17 +9908,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C56" s="6" t="n">
-        <v>893.61</v>
+        <v>122.18</v>
       </c>
       <c r="D56" s="6" t="n">
-        <v>1944.34</v>
+        <v>396.04</v>
       </c>
       <c r="E56" s="6" t="n">
-        <v>2175.826143395889</v>
+        <v>3241.447045342937</v>
       </c>
     </row>
     <row r="57">
@@ -9432,17 +9929,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C57" s="6" t="n">
-        <v>9242.9</v>
+        <v>1253</v>
       </c>
       <c r="D57" s="6" t="n">
-        <v>14292.47</v>
+        <v>2613.01</v>
       </c>
       <c r="E57" s="6" t="n">
-        <v>1546.318796048859</v>
+        <v>2085.403032721468</v>
       </c>
     </row>
     <row r="58">
@@ -9453,17 +9950,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C58" s="6" t="n">
-        <v>53.19</v>
+        <v>9262.59</v>
       </c>
       <c r="D58" s="6" t="n">
-        <v>89.00999999999999</v>
+        <v>14317.28</v>
       </c>
       <c r="E58" s="6" t="n">
-        <v>1673.434856175973</v>
+        <v>1545.710217120697</v>
       </c>
     </row>
     <row r="59">
@@ -9474,17 +9971,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C59" s="6" t="n">
-        <v>1002.95</v>
+        <v>53.19</v>
       </c>
       <c r="D59" s="6" t="n">
-        <v>2328.91</v>
+        <v>89.00999999999999</v>
       </c>
       <c r="E59" s="6" t="n">
-        <v>2322.059923226482</v>
+        <v>1673.434856175973</v>
       </c>
     </row>
     <row r="60">
@@ -9495,17 +9992,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C60" s="6" t="n">
-        <v>648.9700000000001</v>
+        <v>1152.11</v>
       </c>
       <c r="D60" s="6" t="n">
-        <v>1088.52</v>
+        <v>2691.05</v>
       </c>
       <c r="E60" s="6" t="n">
-        <v>1677.304035625683</v>
+        <v>2335.757870342241</v>
       </c>
     </row>
     <row r="61">
@@ -9516,17 +10013,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>New Zealand</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C61" s="6" t="n">
-        <v>489.25</v>
+        <v>648.9700000000001</v>
       </c>
       <c r="D61" s="6" t="n">
-        <v>567.84</v>
+        <v>1088.52</v>
       </c>
       <c r="E61" s="6" t="n">
-        <v>1160.633622892182</v>
+        <v>1677.304035625683</v>
       </c>
     </row>
     <row r="62">
@@ -9537,17 +10034,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>New Zealand</t>
         </is>
       </c>
       <c r="C62" s="6" t="n">
-        <v>996.73</v>
+        <v>489.25</v>
       </c>
       <c r="D62" s="6" t="n">
-        <v>1032.71</v>
+        <v>567.84</v>
       </c>
       <c r="E62" s="6" t="n">
-        <v>1036.098040592738</v>
+        <v>1160.633622892182</v>
       </c>
     </row>
     <row r="63">
@@ -9558,17 +10055,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="C63" s="6" t="n">
-        <v>48.67</v>
+        <v>996.73</v>
       </c>
       <c r="D63" s="6" t="n">
-        <v>57.52</v>
+        <v>1032.71</v>
       </c>
       <c r="E63" s="6" t="n">
-        <v>1181.836860489007</v>
+        <v>1036.098040592738</v>
       </c>
     </row>
     <row r="64">
@@ -9579,17 +10076,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C64" s="6" t="n">
-        <v>63.97</v>
+        <v>48.67</v>
       </c>
       <c r="D64" s="6" t="n">
-        <v>81.75</v>
+        <v>57.52</v>
       </c>
       <c r="E64" s="6" t="n">
-        <v>1277.942785680788</v>
+        <v>1181.836860489007</v>
       </c>
     </row>
     <row r="65">
@@ -9600,17 +10097,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="C65" s="6" t="n">
-        <v>10579.12</v>
+        <v>20</v>
       </c>
       <c r="D65" s="6" t="n">
-        <v>14302.06</v>
+        <v>40.1</v>
       </c>
       <c r="E65" s="6" t="n">
-        <v>1351.913958816991</v>
+        <v>2005</v>
       </c>
     </row>
     <row r="66">
@@ -9621,17 +10118,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="C66" s="6" t="n">
-        <v>2593.2</v>
+        <v>63.97</v>
       </c>
       <c r="D66" s="6" t="n">
-        <v>3265.41</v>
+        <v>81.75</v>
       </c>
       <c r="E66" s="6" t="n">
-        <v>1259.220268394262</v>
+        <v>1277.942785680788</v>
       </c>
     </row>
     <row r="67">
@@ -9642,17 +10139,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C67" s="6" t="n">
-        <v>11334.39</v>
+        <v>10579.12</v>
       </c>
       <c r="D67" s="6" t="n">
-        <v>12765.71</v>
+        <v>14302.06</v>
       </c>
       <c r="E67" s="6" t="n">
-        <v>1126.281167314695</v>
+        <v>1351.913958816991</v>
       </c>
     </row>
     <row r="68">
@@ -9663,17 +10160,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Ukraine</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C68" s="6" t="n">
-        <v>17.65</v>
+        <v>2593.2</v>
       </c>
       <c r="D68" s="6" t="n">
-        <v>68.54000000000001</v>
+        <v>3265.41</v>
       </c>
       <c r="E68" s="6" t="n">
-        <v>3883.28611898017</v>
+        <v>1259.220268394262</v>
       </c>
     </row>
     <row r="69">
@@ -9684,17 +10181,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C69" s="6" t="n">
-        <v>969.2099999999999</v>
+        <v>11334.39</v>
       </c>
       <c r="D69" s="6" t="n">
-        <v>1111.34</v>
+        <v>12765.71</v>
       </c>
       <c r="E69" s="6" t="n">
-        <v>1146.645205889333</v>
+        <v>1126.281167314695</v>
       </c>
     </row>
     <row r="70">
@@ -9705,17 +10202,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Ukraine</t>
         </is>
       </c>
       <c r="C70" s="6" t="n">
-        <v>35915.97</v>
+        <v>17.65</v>
       </c>
       <c r="D70" s="6" t="n">
-        <v>68388.88</v>
+        <v>68.54000000000001</v>
       </c>
       <c r="E70" s="6" t="n">
-        <v>1904.135681146855</v>
+        <v>3883.28611898017</v>
       </c>
     </row>
     <row r="71">
@@ -9726,59 +10223,59 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="C71" s="6" t="n">
-        <v>1189.02</v>
+        <v>969.2099999999999</v>
       </c>
       <c r="D71" s="6" t="n">
-        <v>1275.32</v>
+        <v>1111.34</v>
       </c>
       <c r="E71" s="6" t="n">
-        <v>1072.580780811088</v>
+        <v>1146.645205889333</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Cambodia</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C72" s="6" t="n">
-        <v>6038.5</v>
+        <v>40602.37</v>
       </c>
       <c r="D72" s="6" t="n">
-        <v>4639.469999999999</v>
+        <v>77795.21000000001</v>
       </c>
       <c r="E72" s="6" t="n">
-        <v>768.3149788854846</v>
+        <v>1916.026330482679</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C73" s="6" t="n">
-        <v>18.06</v>
+        <v>1189.02</v>
       </c>
       <c r="D73" s="6" t="n">
-        <v>14.86</v>
+        <v>1275.32</v>
       </c>
       <c r="E73" s="6" t="n">
-        <v>822.8128460686601</v>
+        <v>1072.580780811088</v>
       </c>
     </row>
     <row r="74">
@@ -9789,17 +10286,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Cambodia</t>
         </is>
       </c>
       <c r="C74" s="6" t="n">
-        <v>388.89</v>
+        <v>6038.5</v>
       </c>
       <c r="D74" s="6" t="n">
-        <v>535.6999999999999</v>
+        <v>4639.469999999999</v>
       </c>
       <c r="E74" s="6" t="n">
-        <v>1377.510349970428</v>
+        <v>768.3149788854846</v>
       </c>
     </row>
     <row r="75">
@@ -9810,17 +10307,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C75" s="6" t="n">
-        <v>1311.26</v>
+        <v>18.06</v>
       </c>
       <c r="D75" s="6" t="n">
-        <v>1218.72</v>
+        <v>14.86</v>
       </c>
       <c r="E75" s="6" t="n">
-        <v>929.4266583286305</v>
+        <v>822.8128460686601</v>
       </c>
     </row>
     <row r="76">
@@ -9831,17 +10328,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C76" s="6" t="n">
-        <v>3218.63</v>
+        <v>388.89</v>
       </c>
       <c r="D76" s="6" t="n">
-        <v>2489.5</v>
+        <v>535.6999999999999</v>
       </c>
       <c r="E76" s="6" t="n">
-        <v>773.4657292077685</v>
+        <v>1377.510349970428</v>
       </c>
     </row>
     <row r="77">
@@ -9852,17 +10349,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C77" s="6" t="n">
-        <v>25160.13</v>
+        <v>2577.92</v>
       </c>
       <c r="D77" s="6" t="n">
-        <v>27341.55</v>
+        <v>2016.72</v>
       </c>
       <c r="E77" s="6" t="n">
-        <v>1086.701459809627</v>
+        <v>782.3051142005958</v>
       </c>
     </row>
     <row r="78">
@@ -9873,17 +10370,17 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="C78" s="6" t="n">
-        <v>52.75</v>
+        <v>3218.63</v>
       </c>
       <c r="D78" s="6" t="n">
-        <v>53.87</v>
+        <v>2489.5</v>
       </c>
       <c r="E78" s="6" t="n">
-        <v>1021.232227488152</v>
+        <v>773.4657292077685</v>
       </c>
     </row>
     <row r="79">
@@ -9894,59 +10391,59 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C79" s="6" t="n">
-        <v>1158.09</v>
+        <v>25669.47</v>
       </c>
       <c r="D79" s="6" t="n">
-        <v>2193.55</v>
+        <v>27999.43</v>
       </c>
       <c r="E79" s="6" t="n">
-        <v>1894.11012960996</v>
+        <v>1090.767748613431</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="C80" s="6" t="n">
-        <v>781.04</v>
+        <v>52.75</v>
       </c>
       <c r="D80" s="6" t="n">
-        <v>750.46</v>
+        <v>53.87</v>
       </c>
       <c r="E80" s="6" t="n">
-        <v>960.8470756939465</v>
+        <v>1021.232227488152</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C81" s="6" t="n">
-        <v>204.65</v>
+        <v>1291.6</v>
       </c>
       <c r="D81" s="6" t="n">
-        <v>219.29</v>
+        <v>2373.32</v>
       </c>
       <c r="E81" s="6" t="n">
-        <v>1071.536770095285</v>
+        <v>1837.503871167544</v>
       </c>
     </row>
     <row r="82">
@@ -9957,17 +10454,17 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C82" s="6" t="n">
-        <v>1.12</v>
+        <v>781.04</v>
       </c>
       <c r="D82" s="6" t="n">
-        <v>4.18</v>
+        <v>750.46</v>
       </c>
       <c r="E82" s="6" t="n">
-        <v>3732.142857142857</v>
+        <v>960.8470756939465</v>
       </c>
     </row>
     <row r="83">
@@ -9978,17 +10475,17 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C83" s="6" t="n">
-        <v>19.32</v>
+        <v>204.62</v>
       </c>
       <c r="D83" s="6" t="n">
-        <v>39.73</v>
+        <v>218.88</v>
       </c>
       <c r="E83" s="6" t="n">
-        <v>2056.418219461698</v>
+        <v>1069.690157364872</v>
       </c>
     </row>
     <row r="84">
@@ -9999,17 +10496,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="C84" s="6" t="n">
-        <v>585.71</v>
+        <v>1.12</v>
       </c>
       <c r="D84" s="6" t="n">
-        <v>916.8199999999999</v>
+        <v>4.18</v>
       </c>
       <c r="E84" s="6" t="n">
-        <v>1565.313892540677</v>
+        <v>3732.142857142857</v>
       </c>
     </row>
     <row r="85">
@@ -10020,17 +10517,17 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="C85" s="6" t="n">
-        <v>3.2</v>
+        <v>19.32</v>
       </c>
       <c r="D85" s="6" t="n">
-        <v>4</v>
+        <v>39.73</v>
       </c>
       <c r="E85" s="6" t="n">
-        <v>1250</v>
+        <v>2056.418219461698</v>
       </c>
     </row>
     <row r="86">
@@ -10041,17 +10538,17 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C86" s="6" t="n">
-        <v>40.88</v>
+        <v>585.71</v>
       </c>
       <c r="D86" s="6" t="n">
-        <v>111.35</v>
+        <v>916.8199999999999</v>
       </c>
       <c r="E86" s="6" t="n">
-        <v>2723.825831702544</v>
+        <v>1565.313892540677</v>
       </c>
     </row>
     <row r="87">
@@ -10062,17 +10559,17 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C87" s="6" t="n">
-        <v>8.720000000000001</v>
+        <v>3.2</v>
       </c>
       <c r="D87" s="6" t="n">
-        <v>18.05</v>
+        <v>4</v>
       </c>
       <c r="E87" s="6" t="n">
-        <v>2069.954128440367</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="88">
@@ -10083,17 +10580,17 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C88" s="6" t="n">
-        <v>915.64</v>
+        <v>41.26000000000001</v>
       </c>
       <c r="D88" s="6" t="n">
-        <v>1231.66</v>
+        <v>112.53</v>
       </c>
       <c r="E88" s="6" t="n">
-        <v>1345.135642829059</v>
+        <v>2727.338826951042</v>
       </c>
     </row>
     <row r="89">
@@ -10104,17 +10601,17 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C89" s="6" t="n">
-        <v>1.2</v>
+        <v>9.379999999999999</v>
       </c>
       <c r="D89" s="6" t="n">
-        <v>5.45</v>
+        <v>19.62</v>
       </c>
       <c r="E89" s="6" t="n">
-        <v>4541.666666666666</v>
+        <v>2091.684434968017</v>
       </c>
     </row>
     <row r="90">
@@ -10125,17 +10622,17 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C90" s="6" t="n">
-        <v>25.55</v>
+        <v>926.85</v>
       </c>
       <c r="D90" s="6" t="n">
-        <v>50.78</v>
+        <v>1259.8</v>
       </c>
       <c r="E90" s="6" t="n">
-        <v>1987.47553816047</v>
+        <v>1359.227490964018</v>
       </c>
     </row>
     <row r="91">
@@ -10146,17 +10643,17 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="C91" s="6" t="n">
-        <v>2006.45</v>
+        <v>1.2</v>
       </c>
       <c r="D91" s="6" t="n">
-        <v>1931.12</v>
+        <v>5.45</v>
       </c>
       <c r="E91" s="6" t="n">
-        <v>962.4560791447583</v>
+        <v>4541.666666666666</v>
       </c>
     </row>
     <row r="92">
@@ -10167,17 +10664,17 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C92" s="6" t="n">
-        <v>1277.28</v>
+        <v>25.4</v>
       </c>
       <c r="D92" s="6" t="n">
-        <v>1216.36</v>
+        <v>49.81</v>
       </c>
       <c r="E92" s="6" t="n">
-        <v>952.3048979080546</v>
+        <v>1961.023622047244</v>
       </c>
     </row>
     <row r="93">
@@ -10188,17 +10685,17 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C93" s="6" t="n">
-        <v>10.8</v>
+        <v>2006.45</v>
       </c>
       <c r="D93" s="6" t="n">
-        <v>47.44</v>
+        <v>1931.12</v>
       </c>
       <c r="E93" s="6" t="n">
-        <v>4392.592592592593</v>
+        <v>962.4560791447583</v>
       </c>
     </row>
     <row r="94">
@@ -10209,59 +10706,59 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C94" s="6" t="n">
-        <v>2245.260000000001</v>
+        <v>1277.28</v>
       </c>
       <c r="D94" s="6" t="n">
-        <v>4606.249999999998</v>
+        <v>1216.36</v>
       </c>
       <c r="E94" s="6" t="n">
-        <v>2051.544141881117</v>
+        <v>952.3048979080546</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C95" s="6" t="n">
-        <v>72.08</v>
+        <v>10.8</v>
       </c>
       <c r="D95" s="6" t="n">
-        <v>95.73999999999999</v>
+        <v>47.44</v>
       </c>
       <c r="E95" s="6" t="n">
-        <v>1328.246392896781</v>
+        <v>4392.592592592593</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C96" s="6" t="n">
-        <v>931.79</v>
+        <v>2637.070000000001</v>
       </c>
       <c r="D96" s="6" t="n">
-        <v>1241.13</v>
+        <v>5432.979999999999</v>
       </c>
       <c r="E96" s="6" t="n">
-        <v>1331.984674658453</v>
+        <v>2060.233516743961</v>
       </c>
     </row>
     <row r="97">
@@ -10272,17 +10769,17 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C97" s="6" t="n">
-        <v>5.78</v>
+        <v>72.08</v>
       </c>
       <c r="D97" s="6" t="n">
-        <v>10.29</v>
+        <v>95.73999999999999</v>
       </c>
       <c r="E97" s="6" t="n">
-        <v>1780.276816608997</v>
+        <v>1328.246392896781</v>
       </c>
     </row>
     <row r="98">
@@ -10293,17 +10790,17 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C98" s="6" t="n">
-        <v>6713.799999999999</v>
+        <v>931.79</v>
       </c>
       <c r="D98" s="6" t="n">
-        <v>10090.43</v>
+        <v>1241.13</v>
       </c>
       <c r="E98" s="6" t="n">
-        <v>1502.938723226787</v>
+        <v>1331.984674658453</v>
       </c>
     </row>
     <row r="99">
@@ -10314,17 +10811,17 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C99" s="6" t="n">
-        <v>8103.91</v>
+        <v>5.78</v>
       </c>
       <c r="D99" s="6" t="n">
-        <v>5812.44</v>
+        <v>10.29</v>
       </c>
       <c r="E99" s="6" t="n">
-        <v>717.2389624267792</v>
+        <v>1780.276816608997</v>
       </c>
     </row>
     <row r="100">
@@ -10335,17 +10832,17 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C100" s="6" t="n">
-        <v>256.94</v>
+        <v>7095.829999999999</v>
       </c>
       <c r="D100" s="6" t="n">
-        <v>334.05</v>
+        <v>10565.72</v>
       </c>
       <c r="E100" s="6" t="n">
-        <v>1300.108974857943</v>
+        <v>1489.004105228</v>
       </c>
     </row>
     <row r="101">
@@ -10356,17 +10853,17 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C101" s="6" t="n">
-        <v>506.71</v>
+        <v>8103.91</v>
       </c>
       <c r="D101" s="6" t="n">
-        <v>617.79</v>
+        <v>5812.44</v>
       </c>
       <c r="E101" s="6" t="n">
-        <v>1219.218093189398</v>
+        <v>717.2389624267792</v>
       </c>
     </row>
     <row r="102">
@@ -10377,17 +10874,17 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C102" s="6" t="n">
-        <v>288.96</v>
+        <v>256.94</v>
       </c>
       <c r="D102" s="6" t="n">
-        <v>328.76</v>
+        <v>334.05</v>
       </c>
       <c r="E102" s="6" t="n">
-        <v>1137.735326688815</v>
+        <v>1300.108974857943</v>
       </c>
     </row>
     <row r="103">
@@ -10398,59 +10895,59 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C103" s="6" t="n">
-        <v>6233.420000000001</v>
+        <v>506.71</v>
       </c>
       <c r="D103" s="6" t="n">
-        <v>8790.85</v>
+        <v>617.79</v>
       </c>
       <c r="E103" s="6" t="n">
-        <v>1410.27718331189</v>
+        <v>1219.218093189398</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C104" s="6" t="n">
-        <v>1604.34</v>
+        <v>288.96</v>
       </c>
       <c r="D104" s="6" t="n">
-        <v>1403.65</v>
+        <v>328.76</v>
       </c>
       <c r="E104" s="6" t="n">
-        <v>874.9080618821445</v>
+        <v>1137.735326688815</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C105" s="6" t="n">
-        <v>0.17</v>
+        <v>6756.18</v>
       </c>
       <c r="D105" s="6" t="n">
-        <v>0.63</v>
+        <v>9549.290000000001</v>
       </c>
       <c r="E105" s="6" t="n">
-        <v>3705.882352941176</v>
+        <v>1413.415569152983</v>
       </c>
     </row>
     <row r="106">
@@ -10461,17 +10958,17 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C106" s="6" t="n">
-        <v>564.26</v>
+        <v>1604.34</v>
       </c>
       <c r="D106" s="6" t="n">
-        <v>1869.76</v>
+        <v>1403.65</v>
       </c>
       <c r="E106" s="6" t="n">
-        <v>3313.649735937333</v>
+        <v>874.9080618821445</v>
       </c>
     </row>
     <row r="107">
@@ -10482,17 +10979,17 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C107" s="6" t="n">
-        <v>55.17</v>
+        <v>0.17</v>
       </c>
       <c r="D107" s="6" t="n">
-        <v>81.37</v>
+        <v>0.63</v>
       </c>
       <c r="E107" s="6" t="n">
-        <v>1474.89577669023</v>
+        <v>3705.882352941176</v>
       </c>
     </row>
     <row r="108">
@@ -10503,17 +11000,17 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C108" s="6" t="n">
-        <v>9.529999999999999</v>
+        <v>579.9</v>
       </c>
       <c r="D108" s="6" t="n">
-        <v>39.84</v>
+        <v>1885.65</v>
       </c>
       <c r="E108" s="6" t="n">
-        <v>4180.482686253935</v>
+        <v>3251.68132436627</v>
       </c>
     </row>
     <row r="109">
@@ -10524,17 +11021,17 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C109" s="6" t="n">
-        <v>4717.8</v>
+        <v>55.17</v>
       </c>
       <c r="D109" s="6" t="n">
-        <v>5541.98</v>
+        <v>81.37</v>
       </c>
       <c r="E109" s="6" t="n">
-        <v>1174.695832803425</v>
+        <v>1474.89577669023</v>
       </c>
     </row>
     <row r="110">
@@ -10545,17 +11042,17 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C110" s="6" t="n">
-        <v>53744.44</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="D110" s="6" t="n">
-        <v>53799.49</v>
+        <v>39.84</v>
       </c>
       <c r="E110" s="6" t="n">
-        <v>1001.024292001182</v>
+        <v>4180.482686253935</v>
       </c>
     </row>
     <row r="111">
@@ -10566,17 +11063,17 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C111" s="6" t="n">
-        <v>6022.950000000001</v>
+        <v>4717.8</v>
       </c>
       <c r="D111" s="6" t="n">
-        <v>10125.49</v>
+        <v>5541.98</v>
       </c>
       <c r="E111" s="6" t="n">
-        <v>1681.151263085365</v>
+        <v>1174.695832803425</v>
       </c>
     </row>
     <row r="112">
@@ -10587,17 +11084,17 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C112" s="6" t="n">
-        <v>8309.849999999999</v>
+        <v>53744.44</v>
       </c>
       <c r="D112" s="6" t="n">
-        <v>11572.18</v>
+        <v>53799.49</v>
       </c>
       <c r="E112" s="6" t="n">
-        <v>1392.585907086169</v>
+        <v>1001.024292001182</v>
       </c>
     </row>
     <row r="113">
@@ -10608,17 +11105,17 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Luxembourg</t>
         </is>
       </c>
       <c r="C113" s="6" t="n">
-        <v>0.96</v>
+        <v>6566.25</v>
       </c>
       <c r="D113" s="6" t="n">
-        <v>3.83</v>
+        <v>10907.93</v>
       </c>
       <c r="E113" s="6" t="n">
-        <v>3989.583333333333</v>
+        <v>1661.211498191509</v>
       </c>
     </row>
     <row r="114">
@@ -10629,17 +11126,17 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C114" s="6" t="n">
-        <v>5036.45</v>
+        <v>9464.199999999997</v>
       </c>
       <c r="D114" s="6" t="n">
-        <v>5378</v>
+        <v>13167.46</v>
       </c>
       <c r="E114" s="6" t="n">
-        <v>1067.815624100309</v>
+        <v>1391.291392827709</v>
       </c>
     </row>
     <row r="115">
@@ -10650,17 +11147,17 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C115" s="6" t="n">
-        <v>0.12</v>
+        <v>0.96</v>
       </c>
       <c r="D115" s="6" t="n">
-        <v>0.59</v>
+        <v>3.83</v>
       </c>
       <c r="E115" s="6" t="n">
-        <v>4916.666666666667</v>
+        <v>3989.583333333333</v>
       </c>
     </row>
     <row r="116">
@@ -10671,17 +11168,17 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C116" s="6" t="n">
-        <v>887.71</v>
+        <v>5036.45</v>
       </c>
       <c r="D116" s="6" t="n">
-        <v>852.09</v>
+        <v>5378</v>
       </c>
       <c r="E116" s="6" t="n">
-        <v>959.8742832681844</v>
+        <v>1067.815624100309</v>
       </c>
     </row>
     <row r="117">
@@ -10692,17 +11189,17 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C117" s="6" t="n">
-        <v>6378.700000000001</v>
+        <v>0.12</v>
       </c>
       <c r="D117" s="6" t="n">
-        <v>5627.59</v>
+        <v>0.59</v>
       </c>
       <c r="E117" s="6" t="n">
-        <v>882.2471663505102</v>
+        <v>4916.666666666667</v>
       </c>
     </row>
     <row r="118">
@@ -10713,17 +11210,17 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C118" s="6" t="n">
-        <v>3195.46</v>
+        <v>891.87</v>
       </c>
       <c r="D118" s="6" t="n">
-        <v>4521.78</v>
+        <v>856.11</v>
       </c>
       <c r="E118" s="6" t="n">
-        <v>1415.063871868213</v>
+        <v>959.9044703824549</v>
       </c>
     </row>
     <row r="119">
@@ -10734,17 +11231,17 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C119" s="6" t="n">
-        <v>7469.389999999999</v>
+        <v>6378.700000000001</v>
       </c>
       <c r="D119" s="6" t="n">
-        <v>7839.33</v>
+        <v>5627.59</v>
       </c>
       <c r="E119" s="6" t="n">
-        <v>1049.527471453492</v>
+        <v>882.2471663505102</v>
       </c>
     </row>
     <row r="120">
@@ -10755,17 +11252,17 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C120" s="6" t="n">
-        <v>6316.48</v>
+        <v>3195.46</v>
       </c>
       <c r="D120" s="6" t="n">
-        <v>7401.58</v>
+        <v>4521.78</v>
       </c>
       <c r="E120" s="6" t="n">
-        <v>1171.788717766858</v>
+        <v>1415.063871868213</v>
       </c>
     </row>
     <row r="121">
@@ -10776,17 +11273,17 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="C121" s="6" t="n">
-        <v>13201.82</v>
+        <v>7469.389999999999</v>
       </c>
       <c r="D121" s="6" t="n">
-        <v>32456.15</v>
+        <v>7839.33</v>
       </c>
       <c r="E121" s="6" t="n">
-        <v>2458.460272901767</v>
+        <v>1049.527471453492</v>
       </c>
     </row>
     <row r="122">
@@ -10797,16 +11294,58 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C122" s="6" t="n">
+        <v>6316.48</v>
+      </c>
+      <c r="D122" s="6" t="n">
+        <v>7401.58</v>
+      </c>
+      <c r="E122" s="6" t="n">
+        <v>1171.788717766858</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C123" s="6" t="n">
+        <v>14488.25</v>
+      </c>
+      <c r="D123" s="6" t="n">
+        <v>35891.58000000001</v>
+      </c>
+      <c r="E123" s="6" t="n">
+        <v>2477.288837506256</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
           <t>Vietnam</t>
         </is>
       </c>
-      <c r="C122" s="6" t="n">
+      <c r="C124" s="6" t="n">
         <v>345.42</v>
       </c>
-      <c r="D122" s="6" t="n">
+      <c r="D124" s="6" t="n">
         <v>331.78</v>
       </c>
-      <c r="E122" s="6" t="n">
+      <c r="E124" s="6" t="n">
         <v>960.51184065775</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Weekly TRQ update 2026-06-22
</commit_message>
<xml_diff>
--- a/data/canada_trq_tracker.xlsx
+++ b/data/canada_trq_tracker.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R54"/>
+  <dimension ref="A1:S54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -526,6 +526,11 @@
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
+          <t>June 22 2026</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
           <t>OVER</t>
         </is>
       </c>
@@ -586,6 +591,9 @@
       <c r="Q3" s="4" t="n">
         <v>0.0382</v>
       </c>
+      <c r="R3" s="4" t="n">
+        <v>0.0397</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -643,6 +651,9 @@
       <c r="Q4" s="4" t="n">
         <v>0.0033</v>
       </c>
+      <c r="R4" s="4" t="n">
+        <v>0.0033</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -700,7 +711,10 @@
       <c r="Q5" s="4" t="n">
         <v>0.41</v>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="R5" s="4" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="S5" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -747,6 +761,9 @@
       <c r="Q6" s="4" t="n">
         <v>0.0002</v>
       </c>
+      <c r="R6" s="4" t="n">
+        <v>0.0002</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -811,6 +828,10 @@
         <f>SUM(Q3:Q6)</f>
         <v/>
       </c>
+      <c r="R7" s="5">
+        <f>SUM(R3:R6)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -868,7 +889,10 @@
       <c r="Q8" s="4" t="n">
         <v>0.36</v>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="R8" s="4" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="S8" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -930,6 +954,9 @@
       <c r="Q9" s="4" t="n">
         <v>0.0369</v>
       </c>
+      <c r="R9" s="4" t="n">
+        <v>0.0369</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -972,6 +999,9 @@
       <c r="Q10" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="R10" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1036,6 +1066,10 @@
         <f>SUM(Q8:Q10)</f>
         <v/>
       </c>
+      <c r="R11" s="5">
+        <f>SUM(R8:R10)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1093,6 +1127,9 @@
       <c r="Q12" s="4" t="n">
         <v>0.0063</v>
       </c>
+      <c r="R12" s="4" t="n">
+        <v>0.0063</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1150,6 +1187,9 @@
       <c r="Q13" s="4" t="n">
         <v>0.0113</v>
       </c>
+      <c r="R13" s="4" t="n">
+        <v>0.0113</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1207,6 +1247,9 @@
       <c r="Q14" s="4" t="n">
         <v>0.6692</v>
       </c>
+      <c r="R14" s="4" t="n">
+        <v>0.6692</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1264,6 +1307,9 @@
       <c r="Q15" s="4" t="n">
         <v>0.2512</v>
       </c>
+      <c r="R15" s="4" t="n">
+        <v>0.2512</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1312,6 +1358,9 @@
       <c r="Q16" s="4" t="n">
         <v>0.0552</v>
       </c>
+      <c r="R16" s="4" t="n">
+        <v>0.0552</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1345,6 +1394,9 @@
       <c r="Q17" s="4" t="n">
         <v>0.0067</v>
       </c>
+      <c r="R17" s="4" t="n">
+        <v>0.0067</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1409,6 +1461,10 @@
         <f>SUM(Q12:Q17)</f>
         <v/>
       </c>
+      <c r="R18" s="5">
+        <f>SUM(R12:R17)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1466,6 +1522,9 @@
       <c r="Q19" s="4" t="n">
         <v>0.0092</v>
       </c>
+      <c r="R19" s="4" t="n">
+        <v>0.0092</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1523,6 +1582,9 @@
       <c r="Q20" s="4" t="n">
         <v>0.0005</v>
       </c>
+      <c r="R20" s="4" t="n">
+        <v>0.0005</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1580,6 +1642,9 @@
       <c r="Q21" s="4" t="n">
         <v>0.0532</v>
       </c>
+      <c r="R21" s="4" t="n">
+        <v>0.0532</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1637,6 +1702,9 @@
       <c r="Q22" s="4" t="n">
         <v>0.0119</v>
       </c>
+      <c r="R22" s="4" t="n">
+        <v>0.0119</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1694,6 +1762,9 @@
       <c r="Q23" s="4" t="n">
         <v>0.3695000000000001</v>
       </c>
+      <c r="R23" s="4" t="n">
+        <v>0.3695000000000001</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1751,6 +1822,9 @@
       <c r="Q24" s="4" t="n">
         <v>0.1384</v>
       </c>
+      <c r="R24" s="4" t="n">
+        <v>0.1384</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1808,6 +1882,9 @@
       <c r="Q25" s="4" t="n">
         <v>0.3262</v>
       </c>
+      <c r="R25" s="4" t="n">
+        <v>0.3262</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1865,6 +1942,9 @@
       <c r="Q26" s="4" t="n">
         <v>0.05599999999999999</v>
       </c>
+      <c r="R26" s="4" t="n">
+        <v>0.05599999999999999</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1913,6 +1993,9 @@
       <c r="Q27" s="4" t="n">
         <v>0.0207</v>
       </c>
+      <c r="R27" s="4" t="n">
+        <v>0.0207</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1988,6 +2071,9 @@
       <c r="Q29" s="4" t="n">
         <v>0.0008</v>
       </c>
+      <c r="R29" s="4" t="n">
+        <v>0.0008</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2052,6 +2138,10 @@
         <f>SUM(Q19:Q29)</f>
         <v/>
       </c>
+      <c r="R30" s="5">
+        <f>SUM(R19:R29)</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2109,7 +2199,10 @@
       <c r="Q31" s="4" t="n">
         <v>0.29</v>
       </c>
-      <c r="R31" t="inlineStr">
+      <c r="R31" s="4" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="S31" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -2171,6 +2264,9 @@
       <c r="Q32" s="4" t="n">
         <v>0.1228</v>
       </c>
+      <c r="R32" s="4" t="n">
+        <v>0.1228</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2228,6 +2324,9 @@
       <c r="Q33" s="4" t="n">
         <v>0.2394</v>
       </c>
+      <c r="R33" s="4" t="n">
+        <v>0.2394</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2285,6 +2384,9 @@
       <c r="Q34" s="4" t="n">
         <v>0.1668</v>
       </c>
+      <c r="R34" s="4" t="n">
+        <v>0.1668</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2342,6 +2444,9 @@
       <c r="Q35" s="4" t="n">
         <v>0.0241</v>
       </c>
+      <c r="R35" s="4" t="n">
+        <v>0.0241</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2399,6 +2504,9 @@
       <c r="Q36" s="4" t="n">
         <v>0.1569</v>
       </c>
+      <c r="R36" s="4" t="n">
+        <v>0.1569</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2463,6 +2571,10 @@
         <f>SUM(Q31:Q36)</f>
         <v/>
       </c>
+      <c r="R37" s="5">
+        <f>SUM(R31:R36)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2520,6 +2632,9 @@
       <c r="Q38" s="4" t="n">
         <v>0.0684</v>
       </c>
+      <c r="R38" s="4" t="n">
+        <v>0.0684</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2577,6 +2692,9 @@
       <c r="Q39" s="4" t="n">
         <v>0.3214</v>
       </c>
+      <c r="R39" s="4" t="n">
+        <v>0.3214</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2634,6 +2752,9 @@
       <c r="Q40" s="4" t="n">
         <v>0.3890999999999999</v>
       </c>
+      <c r="R40" s="4" t="n">
+        <v>0.3890999999999999</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2691,6 +2812,9 @@
       <c r="Q41" s="4" t="n">
         <v>0.212</v>
       </c>
+      <c r="R41" s="4" t="n">
+        <v>0.212</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2742,6 +2866,9 @@
       <c r="Q42" s="4" t="n">
         <v>0.0005</v>
       </c>
+      <c r="R42" s="4" t="n">
+        <v>0.0005</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2806,6 +2933,10 @@
         <f>SUM(Q38:Q42)</f>
         <v/>
       </c>
+      <c r="R43" s="5">
+        <f>SUM(R38:R42)</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2863,6 +2994,9 @@
       <c r="Q44" s="4" t="n">
         <v>0.442</v>
       </c>
+      <c r="R44" s="4" t="n">
+        <v>0.442</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2908,7 +3042,10 @@
       <c r="Q45" s="4" t="n">
         <v>0.45</v>
       </c>
-      <c r="R45" t="inlineStr">
+      <c r="R45" s="4" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="S45" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -2955,6 +3092,9 @@
       <c r="Q46" s="4" t="n">
         <v>0.0024</v>
       </c>
+      <c r="R46" s="4" t="n">
+        <v>0.0024</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3019,6 +3159,10 @@
         <f>SUM(Q44:Q46)</f>
         <v/>
       </c>
+      <c r="R47" s="5">
+        <f>SUM(R44:R46)</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3076,6 +3220,9 @@
       <c r="Q48" s="4" t="n">
         <v>0.08810000000000001</v>
       </c>
+      <c r="R48" s="4" t="n">
+        <v>0.08810000000000001</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3133,6 +3280,9 @@
       <c r="Q49" s="4" t="n">
         <v>0.0353</v>
       </c>
+      <c r="R49" s="4" t="n">
+        <v>0.0353</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3190,6 +3340,9 @@
       <c r="Q50" s="4" t="n">
         <v>0.3962</v>
       </c>
+      <c r="R50" s="4" t="n">
+        <v>0.3962</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3247,6 +3400,9 @@
       <c r="Q51" s="4" t="n">
         <v>0.2693</v>
       </c>
+      <c r="R51" s="4" t="n">
+        <v>0.388</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3268,6 +3424,9 @@
       <c r="Q52" s="4" t="n">
         <v>0.0108</v>
       </c>
+      <c r="R52" s="4" t="n">
+        <v>0.0108</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3289,6 +3448,9 @@
       <c r="Q53" s="4" t="n">
         <v>0.04269999999999999</v>
       </c>
+      <c r="R53" s="4" t="n">
+        <v>0.04269999999999999</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3351,6 +3513,10 @@
       </c>
       <c r="Q54" s="5">
         <f>SUM(Q48:Q53)</f>
+        <v/>
+      </c>
+      <c r="R54" s="5">
+        <f>SUM(R48:R53)</f>
         <v/>
       </c>
     </row>
@@ -3365,7 +3531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R96"/>
+  <dimension ref="A1:S96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3458,6 +3624,11 @@
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
+          <t>June 22 2026</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
           <t>OVER</t>
         </is>
       </c>
@@ -3518,6 +3689,9 @@
       <c r="Q3" s="4" t="n">
         <v>0.003</v>
       </c>
+      <c r="R3" s="4" t="n">
+        <v>0.003</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3575,6 +3749,9 @@
       <c r="Q4" s="4" t="n">
         <v>0.1164</v>
       </c>
+      <c r="R4" s="4" t="n">
+        <v>0.1164</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3632,6 +3809,9 @@
       <c r="Q5" s="4" t="n">
         <v>0.115</v>
       </c>
+      <c r="R5" s="4" t="n">
+        <v>0.115</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3689,6 +3869,9 @@
       <c r="Q6" s="4" t="n">
         <v>0.4198</v>
       </c>
+      <c r="R6" s="4" t="n">
+        <v>0.4198</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3746,6 +3929,9 @@
       <c r="Q7" s="4" t="n">
         <v>0.07429999999999999</v>
       </c>
+      <c r="R7" s="4" t="n">
+        <v>0.07429999999999999</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3803,6 +3989,9 @@
       <c r="Q8" s="4" t="n">
         <v>0.0008</v>
       </c>
+      <c r="R8" s="4" t="n">
+        <v>0.0008</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3860,6 +4049,9 @@
       <c r="Q9" s="4" t="n">
         <v>0.0143</v>
       </c>
+      <c r="R9" s="4" t="n">
+        <v>0.0143</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3911,6 +4103,9 @@
       <c r="Q10" s="4" t="n">
         <v>0.014</v>
       </c>
+      <c r="R10" s="4" t="n">
+        <v>0.014</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3968,6 +4163,9 @@
       <c r="Q11" s="4" t="n">
         <v>0.0004</v>
       </c>
+      <c r="R11" s="4" t="n">
+        <v>0.0004</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4022,6 +4220,9 @@
       <c r="Q12" s="4" t="n">
         <v>0.0012</v>
       </c>
+      <c r="R12" s="4" t="n">
+        <v>0.0012</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4076,6 +4277,9 @@
       <c r="Q13" s="4" t="n">
         <v>0.0003</v>
       </c>
+      <c r="R13" s="4" t="n">
+        <v>0.0003</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4124,6 +4328,9 @@
       <c r="Q14" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="R14" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4169,6 +4376,9 @@
       <c r="Q15" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="R15" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4214,6 +4424,9 @@
       <c r="Q16" s="4" t="n">
         <v>0.2405</v>
       </c>
+      <c r="R16" s="4" t="n">
+        <v>0.2405</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4278,6 +4491,10 @@
         <f>SUM(Q3:Q16)</f>
         <v/>
       </c>
+      <c r="R17" s="5">
+        <f>SUM(R3:R16)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4335,6 +4552,9 @@
       <c r="Q18" s="4" t="n">
         <v>0.0338</v>
       </c>
+      <c r="R18" s="4" t="n">
+        <v>0.0338</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4392,6 +4612,9 @@
       <c r="Q19" s="4" t="n">
         <v>0.031</v>
       </c>
+      <c r="R19" s="4" t="n">
+        <v>0.031</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4449,6 +4672,9 @@
       <c r="Q20" s="4" t="n">
         <v>0.0741</v>
       </c>
+      <c r="R20" s="4" t="n">
+        <v>0.0741</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4506,6 +4732,9 @@
       <c r="Q21" s="4" t="n">
         <v>0.154</v>
       </c>
+      <c r="R21" s="4" t="n">
+        <v>0.154</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4563,6 +4792,9 @@
       <c r="Q22" s="4" t="n">
         <v>0.1063</v>
       </c>
+      <c r="R22" s="4" t="n">
+        <v>0.1063</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4620,7 +4852,10 @@
       <c r="Q23" s="4" t="n">
         <v>0.3</v>
       </c>
-      <c r="R23" t="inlineStr">
+      <c r="R23" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="S23" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -4682,6 +4917,9 @@
       <c r="Q24" s="4" t="n">
         <v>0.1668</v>
       </c>
+      <c r="R24" s="4" t="n">
+        <v>0.1668</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4739,6 +4977,9 @@
       <c r="Q25" s="4" t="n">
         <v>0.0005</v>
       </c>
+      <c r="R25" s="4" t="n">
+        <v>0.0005</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4796,6 +5037,9 @@
       <c r="Q26" s="4" t="n">
         <v>0.06900000000000001</v>
       </c>
+      <c r="R26" s="4" t="n">
+        <v>0.06900000000000001</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4850,6 +5094,9 @@
       <c r="Q27" s="4" t="n">
         <v>0.0317</v>
       </c>
+      <c r="R27" s="4" t="n">
+        <v>0.0317</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4904,6 +5151,9 @@
       <c r="Q28" s="4" t="n">
         <v>0.0073</v>
       </c>
+      <c r="R28" s="4" t="n">
+        <v>0.0073</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4958,6 +5208,9 @@
       <c r="Q29" s="4" t="n">
         <v>0.0005999999999999999</v>
       </c>
+      <c r="R29" s="4" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5006,6 +5259,9 @@
       <c r="Q30" s="4" t="n">
         <v>0.0226</v>
       </c>
+      <c r="R30" s="4" t="n">
+        <v>0.0226</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5045,6 +5301,9 @@
       <c r="Q31" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="R31" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5109,6 +5368,10 @@
         <f>SUM(Q18:Q31)</f>
         <v/>
       </c>
+      <c r="R32" s="5">
+        <f>SUM(R18:R31)</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5166,6 +5429,9 @@
       <c r="Q33" s="4" t="n">
         <v>0.258</v>
       </c>
+      <c r="R33" s="4" t="n">
+        <v>0.258</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5220,6 +5486,9 @@
       <c r="Q34" s="4" t="n">
         <v>0.236</v>
       </c>
+      <c r="R34" s="4" t="n">
+        <v>0.236</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5268,6 +5537,9 @@
       <c r="Q35" s="4" t="n">
         <v>0.1992</v>
       </c>
+      <c r="R35" s="4" t="n">
+        <v>0.1992</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5313,6 +5585,9 @@
       <c r="Q36" s="4" t="n">
         <v>0.0011</v>
       </c>
+      <c r="R36" s="4" t="n">
+        <v>0.0011</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5352,6 +5627,9 @@
       <c r="Q37" s="4" t="n">
         <v>0.3057</v>
       </c>
+      <c r="R37" s="4" t="n">
+        <v>0.3057</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5416,6 +5694,10 @@
         <f>SUM(Q33:Q37)</f>
         <v/>
       </c>
+      <c r="R38" s="5">
+        <f>SUM(R33:R37)</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5473,6 +5755,9 @@
       <c r="Q39" s="4" t="n">
         <v>0.166</v>
       </c>
+      <c r="R39" s="4" t="n">
+        <v>0.166</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5530,6 +5815,9 @@
       <c r="Q40" s="4" t="n">
         <v>0.1686</v>
       </c>
+      <c r="R40" s="4" t="n">
+        <v>0.1686</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5587,6 +5875,9 @@
       <c r="Q41" s="4" t="n">
         <v>0.2496</v>
       </c>
+      <c r="R41" s="4" t="n">
+        <v>0.2496</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5644,6 +5935,9 @@
       <c r="Q42" s="4" t="n">
         <v>0.09910000000000001</v>
       </c>
+      <c r="R42" s="4" t="n">
+        <v>0.09910000000000001</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5701,6 +5995,9 @@
       <c r="Q43" s="4" t="n">
         <v>0.0849</v>
       </c>
+      <c r="R43" s="4" t="n">
+        <v>0.0849</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5758,6 +6055,9 @@
       <c r="Q44" s="4" t="n">
         <v>0.0007000000000000001</v>
       </c>
+      <c r="R44" s="4" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5815,6 +6115,9 @@
       <c r="Q45" s="4" t="n">
         <v>0.0906</v>
       </c>
+      <c r="R45" s="4" t="n">
+        <v>0.0906</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5869,6 +6172,9 @@
       <c r="Q46" s="4" t="n">
         <v>0.0014</v>
       </c>
+      <c r="R46" s="4" t="n">
+        <v>0.0014</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5923,6 +6229,9 @@
       <c r="Q47" s="4" t="n">
         <v>0.0354</v>
       </c>
+      <c r="R47" s="4" t="n">
+        <v>0.0354</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5977,6 +6286,9 @@
       <c r="Q48" s="4" t="n">
         <v>0.028</v>
       </c>
+      <c r="R48" s="4" t="n">
+        <v>0.028</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -6028,6 +6340,9 @@
       <c r="Q49" s="4" t="n">
         <v>0.0003</v>
       </c>
+      <c r="R49" s="4" t="n">
+        <v>0.0003</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -6076,6 +6391,9 @@
       <c r="Q50" s="4" t="n">
         <v>0.0014</v>
       </c>
+      <c r="R50" s="4" t="n">
+        <v>0.0014</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -6124,6 +6442,9 @@
       <c r="Q51" s="4" t="n">
         <v>0.0157</v>
       </c>
+      <c r="R51" s="4" t="n">
+        <v>0.0157</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -6172,6 +6493,9 @@
       <c r="Q52" s="4" t="n">
         <v>0.0215</v>
       </c>
+      <c r="R52" s="4" t="n">
+        <v>0.0215</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6217,6 +6541,9 @@
       <c r="Q53" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="R53" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -6262,6 +6589,9 @@
       <c r="Q54" s="4" t="n">
         <v>0.0258</v>
       </c>
+      <c r="R54" s="4" t="n">
+        <v>0.0258</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -6326,6 +6656,10 @@
         <f>SUM(Q39:Q54)</f>
         <v/>
       </c>
+      <c r="R55" s="5">
+        <f>SUM(R39:R54)</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -6383,6 +6717,9 @@
       <c r="Q56" s="4" t="n">
         <v>0.1642</v>
       </c>
+      <c r="R56" s="4" t="n">
+        <v>0.1642</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -6440,6 +6777,9 @@
       <c r="Q57" s="4" t="n">
         <v>0.3234</v>
       </c>
+      <c r="R57" s="4" t="n">
+        <v>0.3234</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -6497,6 +6837,9 @@
       <c r="Q58" s="4" t="n">
         <v>0.0028</v>
       </c>
+      <c r="R58" s="4" t="n">
+        <v>0.0028</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -6554,6 +6897,9 @@
       <c r="Q59" s="4" t="n">
         <v>0.1633</v>
       </c>
+      <c r="R59" s="4" t="n">
+        <v>0.1633</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6611,6 +6957,9 @@
       <c r="Q60" s="4" t="n">
         <v>0.3462</v>
       </c>
+      <c r="R60" s="4" t="n">
+        <v>0.3462</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6675,6 +7024,10 @@
         <f>SUM(Q56:Q60)</f>
         <v/>
       </c>
+      <c r="R61" s="5">
+        <f>SUM(R56:R60)</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -6732,6 +7085,9 @@
       <c r="Q62" s="4" t="n">
         <v>0.004500000000000001</v>
       </c>
+      <c r="R62" s="4" t="n">
+        <v>0.004500000000000001</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -6789,6 +7145,9 @@
       <c r="Q63" s="4" t="n">
         <v>0.0022</v>
       </c>
+      <c r="R63" s="4" t="n">
+        <v>0.0022</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -6846,6 +7205,9 @@
       <c r="Q64" s="4" t="n">
         <v>0.0018</v>
       </c>
+      <c r="R64" s="4" t="n">
+        <v>0.0018</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -6903,6 +7265,9 @@
       <c r="Q65" s="4" t="n">
         <v>0.3186</v>
       </c>
+      <c r="R65" s="4" t="n">
+        <v>0.3186</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -6960,6 +7325,9 @@
       <c r="Q66" s="4" t="n">
         <v>0.0108</v>
       </c>
+      <c r="R66" s="4" t="n">
+        <v>0.0108</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -7017,6 +7385,9 @@
       <c r="Q67" s="4" t="n">
         <v>0.1648</v>
       </c>
+      <c r="R67" s="4" t="n">
+        <v>0.1648</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -7074,6 +7445,9 @@
       <c r="Q68" s="4" t="n">
         <v>0.0015</v>
       </c>
+      <c r="R68" s="4" t="n">
+        <v>0.0015</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -7131,6 +7505,9 @@
       <c r="Q69" s="4" t="n">
         <v>0.2402</v>
       </c>
+      <c r="R69" s="4" t="n">
+        <v>0.2402</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -7188,6 +7565,9 @@
       <c r="Q70" s="4" t="n">
         <v>0.0017</v>
       </c>
+      <c r="R70" s="4" t="n">
+        <v>0.0017</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -7242,6 +7622,9 @@
       <c r="Q71" s="4" t="n">
         <v>0.2399</v>
       </c>
+      <c r="R71" s="4" t="n">
+        <v>0.2399</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -7296,6 +7679,9 @@
       <c r="Q72" s="4" t="n">
         <v>0.0066</v>
       </c>
+      <c r="R72" s="4" t="n">
+        <v>0.0066</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -7347,6 +7733,9 @@
       <c r="Q73" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="R73" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -7395,6 +7784,9 @@
       <c r="Q74" s="4" t="n">
         <v>0.0002</v>
       </c>
+      <c r="R74" s="4" t="n">
+        <v>0.0002</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -7440,6 +7832,9 @@
       <c r="Q75" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="R75" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -7470,6 +7865,9 @@
       <c r="Q76" s="4" t="n">
         <v>0.0019</v>
       </c>
+      <c r="R76" s="4" t="n">
+        <v>0.0019</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -7494,6 +7892,9 @@
       <c r="Q77" s="4" t="n">
         <v>0.0005</v>
       </c>
+      <c r="R77" s="4" t="n">
+        <v>0.0005</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -7518,6 +7919,9 @@
       <c r="Q78" s="4" t="n">
         <v>0.0026</v>
       </c>
+      <c r="R78" s="4" t="n">
+        <v>0.0026</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -7582,6 +7986,10 @@
         <f>SUM(Q62:Q78)</f>
         <v/>
       </c>
+      <c r="R79" s="5">
+        <f>SUM(R62:R78)</f>
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -7639,6 +8047,9 @@
       <c r="Q80" s="4" t="n">
         <v>0.3688</v>
       </c>
+      <c r="R80" s="4" t="n">
+        <v>0.3688</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -7696,6 +8107,9 @@
       <c r="Q81" s="4" t="n">
         <v>0.0941</v>
       </c>
+      <c r="R81" s="4" t="n">
+        <v>0.0941</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -7753,6 +8167,9 @@
       <c r="Q82" s="4" t="n">
         <v>0.0307</v>
       </c>
+      <c r="R82" s="4" t="n">
+        <v>0.0307</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -7807,6 +8224,9 @@
       <c r="Q83" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="R83" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -7855,6 +8275,9 @@
       <c r="Q84" s="4" t="n">
         <v>0.4907</v>
       </c>
+      <c r="R84" s="4" t="n">
+        <v>0.4907</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -7894,6 +8317,9 @@
       <c r="Q85" s="4" t="n">
         <v>0.0044</v>
       </c>
+      <c r="R85" s="4" t="n">
+        <v>0.0044</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7958,6 +8384,10 @@
         <f>SUM(Q80:Q85)</f>
         <v/>
       </c>
+      <c r="R86" s="5">
+        <f>SUM(R80:R85)</f>
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -8015,6 +8445,9 @@
       <c r="Q87" s="4" t="n">
         <v>0.0072</v>
       </c>
+      <c r="R87" s="4" t="n">
+        <v>0.0072</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -8072,6 +8505,9 @@
       <c r="Q88" s="4" t="n">
         <v>0.0075</v>
       </c>
+      <c r="R88" s="4" t="n">
+        <v>0.0075</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -8129,6 +8565,9 @@
       <c r="Q89" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="R89" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -8186,6 +8625,9 @@
       <c r="Q90" s="4" t="n">
         <v>0.0191</v>
       </c>
+      <c r="R90" s="4" t="n">
+        <v>0.0191</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -8243,6 +8685,9 @@
       <c r="Q91" s="4" t="n">
         <v>0.0151</v>
       </c>
+      <c r="R91" s="4" t="n">
+        <v>0.0151</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -8300,6 +8745,9 @@
       <c r="Q92" s="4" t="n">
         <v>0.3604</v>
       </c>
+      <c r="R92" s="4" t="n">
+        <v>0.3604</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -8354,6 +8802,9 @@
       <c r="Q93" s="4" t="n">
         <v>0.5844</v>
       </c>
+      <c r="R93" s="4" t="n">
+        <v>0.5844</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -8408,6 +8859,9 @@
       <c r="Q94" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="R94" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -8453,6 +8907,9 @@
       <c r="Q95" s="4" t="n">
         <v>0.0062</v>
       </c>
+      <c r="R95" s="4" t="n">
+        <v>0.0062</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -8515,6 +8972,10 @@
       </c>
       <c r="Q96" s="5">
         <f>SUM(Q87:Q95)</f>
+        <v/>
+      </c>
+      <c r="R96" s="5">
+        <f>SUM(R87:R95)</f>
         <v/>
       </c>
     </row>
@@ -8855,7 +9316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E124"/>
+  <dimension ref="A1:E126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8963,17 +9424,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>674.25</v>
+        <v>0.6</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>1052.56</v>
+        <v>0.29</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>1561.082684464219</v>
+        <v>483.3333333333334</v>
       </c>
     </row>
     <row r="12">
@@ -8984,17 +9445,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>3125.41</v>
+        <v>674.25</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>2478.809999999999</v>
+        <v>1052.56</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>793.1151432931998</v>
+        <v>1561.082684464219</v>
       </c>
     </row>
     <row r="13">
@@ -9005,17 +9466,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>321.38</v>
+        <v>3125.41</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>437.34</v>
+        <v>2478.809999999999</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>1360.818968199639</v>
+        <v>793.1151432931998</v>
       </c>
     </row>
     <row r="14">
@@ -9026,17 +9487,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>14.25</v>
+        <v>334.15</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>52.25</v>
+        <v>474.3800000000001</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>3666.666666666667</v>
+        <v>1419.661828520126</v>
       </c>
     </row>
     <row r="15">
@@ -9047,17 +9508,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>21716.48</v>
+        <v>14.25</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>35428.3</v>
+        <v>52.25</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>1631.401589944595</v>
+        <v>3666.666666666667</v>
       </c>
     </row>
     <row r="16">
@@ -9068,38 +9529,38 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>2290.17</v>
+        <v>24195.36999999999</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>1767.74</v>
+        <v>39510.46</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>771.8815633773913</v>
+        <v>1632.976061122439</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Steel Plate</t>
+          <t>Hot-Rolled Sheet</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>1230.35</v>
+        <v>2290.17</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>1361.29</v>
+        <v>1767.74</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>1106.425001015971</v>
+        <v>771.8815633773913</v>
       </c>
     </row>
     <row r="18">
@@ -9110,17 +9571,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>0.23</v>
+        <v>1230.35</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>0.46</v>
+        <v>1361.29</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>2000</v>
+        <v>1106.425001015971</v>
       </c>
     </row>
     <row r="19">
@@ -9131,17 +9592,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>382.7100000000001</v>
+        <v>0.23</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>404.81</v>
+        <v>0.46</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>1057.746074050848</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="20">
@@ -9152,17 +9613,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>933.4</v>
+        <v>386.7500000000001</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>2829.57</v>
+        <v>411.76</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>3031.465609599315</v>
+        <v>1064.667097608274</v>
       </c>
     </row>
     <row r="21">
@@ -9173,17 +9634,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>5298.749999999999</v>
+        <v>933.4</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>6840.83</v>
+        <v>2829.57</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>1291.027129039868</v>
+        <v>3031.465609599315</v>
       </c>
     </row>
     <row r="22">
@@ -9194,17 +9655,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>310.93</v>
+        <v>5523.079999999999</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>628.1899999999999</v>
+        <v>7355.33</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>2020.358279998713</v>
+        <v>1331.744244153625</v>
       </c>
     </row>
     <row r="23">
@@ -9215,17 +9676,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>2.07</v>
+        <v>310.93</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>6.74</v>
+        <v>628.1899999999999</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>3256.038647342995</v>
+        <v>2020.358279998713</v>
       </c>
     </row>
     <row r="24">
@@ -9236,17 +9697,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>16672.35</v>
+        <v>2.07</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>19027.7</v>
+        <v>6.74</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>1141.272825966345</v>
+        <v>3256.038647342995</v>
       </c>
     </row>
     <row r="25">
@@ -9257,17 +9718,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C25" s="6" t="n">
-        <v>8999.279999999999</v>
+        <v>16706.3</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>10665.01</v>
+        <v>19071.87</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>1185.095918784614</v>
+        <v>1141.597481189731</v>
       </c>
     </row>
     <row r="26">
@@ -9278,17 +9739,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>0.68</v>
+        <v>8999.279999999999</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>13.84</v>
+        <v>10665.01</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>20352.94117647059</v>
+        <v>1185.095918784614</v>
       </c>
     </row>
     <row r="27">
@@ -9303,13 +9764,13 @@
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>313.62</v>
+        <v>332.66</v>
       </c>
       <c r="D27" s="6" t="n">
-        <v>645.9599999999999</v>
+        <v>691.7199999999999</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>2059.690070786301</v>
+        <v>2079.360307821799</v>
       </c>
     </row>
     <row r="28">
@@ -9408,13 +9869,13 @@
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>12823.09</v>
+        <v>14600.66</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>24464.32000000001</v>
+        <v>27810.02000000001</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>1907.83344732042</v>
+        <v>1904.709787091817</v>
       </c>
     </row>
     <row r="33">
@@ -9471,13 +9932,13 @@
         </is>
       </c>
       <c r="C35" s="6" t="n">
-        <v>46.09999999999999</v>
+        <v>47.69</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>74.94000000000001</v>
+        <v>78.28000000000002</v>
       </c>
       <c r="E35" s="6" t="n">
-        <v>1625.596529284165</v>
+        <v>1641.434262948208</v>
       </c>
     </row>
     <row r="36">
@@ -9509,17 +9970,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C37" s="6" t="n">
-        <v>795.15</v>
+        <v>0.66</v>
       </c>
       <c r="D37" s="6" t="n">
-        <v>1174.87</v>
+        <v>3.77</v>
       </c>
       <c r="E37" s="6" t="n">
-        <v>1477.545117273471</v>
+        <v>5712.121212121212</v>
       </c>
     </row>
     <row r="38">
@@ -9530,17 +9991,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C38" s="6" t="n">
-        <v>0.86</v>
+        <v>795.15</v>
       </c>
       <c r="D38" s="6" t="n">
-        <v>3.13</v>
+        <v>1174.87</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>3639.53488372093</v>
+        <v>1477.545117273471</v>
       </c>
     </row>
     <row r="39">
@@ -9551,17 +10012,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C39" s="6" t="n">
-        <v>41.3</v>
+        <v>56.16</v>
       </c>
       <c r="D39" s="6" t="n">
-        <v>45.1</v>
+        <v>60.02</v>
       </c>
       <c r="E39" s="6" t="n">
-        <v>1092.009685230024</v>
+        <v>1068.732193732194</v>
       </c>
     </row>
     <row r="40">
@@ -9572,17 +10033,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="C40" s="6" t="n">
-        <v>438.39</v>
+        <v>41.3</v>
       </c>
       <c r="D40" s="6" t="n">
-        <v>942.6799999999999</v>
+        <v>45.1</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>2150.322771961039</v>
+        <v>1092.009685230024</v>
       </c>
     </row>
     <row r="41">
@@ -9593,17 +10054,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C41" s="6" t="n">
-        <v>2161.61</v>
+        <v>471.9200000000001</v>
       </c>
       <c r="D41" s="6" t="n">
-        <v>1834.44</v>
+        <v>1019.19</v>
       </c>
       <c r="E41" s="6" t="n">
-        <v>848.6452227737658</v>
+        <v>2159.666892693676</v>
       </c>
     </row>
     <row r="42">
@@ -9614,17 +10075,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C42" s="6" t="n">
-        <v>5881.17</v>
+        <v>2161.61</v>
       </c>
       <c r="D42" s="6" t="n">
-        <v>5165.24</v>
+        <v>1834.44</v>
       </c>
       <c r="E42" s="6" t="n">
-        <v>878.2674195780771</v>
+        <v>848.6452227737658</v>
       </c>
     </row>
     <row r="43">
@@ -9635,17 +10096,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C43" s="6" t="n">
-        <v>15412</v>
+        <v>5881.17</v>
       </c>
       <c r="D43" s="6" t="n">
-        <v>27250.72</v>
+        <v>5165.24</v>
       </c>
       <c r="E43" s="6" t="n">
-        <v>1768.149493900856</v>
+        <v>878.2674195780771</v>
       </c>
     </row>
     <row r="44">
@@ -9656,38 +10117,38 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C44" s="6" t="n">
-        <v>0.4</v>
+        <v>16839.71</v>
       </c>
       <c r="D44" s="6" t="n">
-        <v>0.64</v>
+        <v>29831.54000000001</v>
       </c>
       <c r="E44" s="6" t="n">
-        <v>1600</v>
+        <v>1771.499627962715</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C45" s="6" t="n">
-        <v>170.56</v>
+        <v>0.4</v>
       </c>
       <c r="D45" s="6" t="n">
-        <v>371.76</v>
+        <v>0.64</v>
       </c>
       <c r="E45" s="6" t="n">
-        <v>2179.643527204503</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="46">
@@ -9698,17 +10159,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C46" s="6" t="n">
-        <v>1427.39</v>
+        <v>170.56</v>
       </c>
       <c r="D46" s="6" t="n">
-        <v>2300.44</v>
+        <v>371.76</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>1611.640826963899</v>
+        <v>2179.643527204503</v>
       </c>
     </row>
     <row r="47">
@@ -9719,17 +10180,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C47" s="6" t="n">
-        <v>14.96</v>
+        <v>1631.94</v>
       </c>
       <c r="D47" s="6" t="n">
-        <v>45.9</v>
+        <v>2673.56</v>
       </c>
       <c r="E47" s="6" t="n">
-        <v>3068.181818181818</v>
+        <v>1638.271014865743</v>
       </c>
     </row>
     <row r="48">
@@ -9740,17 +10201,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C48" s="6" t="n">
-        <v>1138.19</v>
+        <v>14.96</v>
       </c>
       <c r="D48" s="6" t="n">
-        <v>1616.86</v>
+        <v>45.9</v>
       </c>
       <c r="E48" s="6" t="n">
-        <v>1420.553686115675</v>
+        <v>3068.181818181818</v>
       </c>
     </row>
     <row r="49">
@@ -9761,17 +10222,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C49" s="6" t="n">
-        <v>17.7</v>
+        <v>1259.09</v>
       </c>
       <c r="D49" s="6" t="n">
-        <v>48.98</v>
+        <v>1728.48</v>
       </c>
       <c r="E49" s="6" t="n">
-        <v>2767.231638418079</v>
+        <v>1372.800991192051</v>
       </c>
     </row>
     <row r="50">
@@ -9782,17 +10243,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C50" s="6" t="n">
-        <v>4.63</v>
+        <v>17.7</v>
       </c>
       <c r="D50" s="6" t="n">
-        <v>10.26</v>
+        <v>48.98</v>
       </c>
       <c r="E50" s="6" t="n">
-        <v>2215.98272138229</v>
+        <v>2767.231638418079</v>
       </c>
     </row>
     <row r="51">
@@ -9803,17 +10264,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="C51" s="6" t="n">
-        <v>11.28</v>
+        <v>4.63</v>
       </c>
       <c r="D51" s="6" t="n">
-        <v>46.33</v>
+        <v>10.26</v>
       </c>
       <c r="E51" s="6" t="n">
-        <v>4107.269503546099</v>
+        <v>2215.98272138229</v>
       </c>
     </row>
     <row r="52">
@@ -9824,17 +10285,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C52" s="6" t="n">
-        <v>111.46</v>
+        <v>23.74</v>
       </c>
       <c r="D52" s="6" t="n">
-        <v>330.41</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="E52" s="6" t="n">
-        <v>2964.3818410192</v>
+        <v>3323.504633529907</v>
       </c>
     </row>
     <row r="53">
@@ -9845,17 +10306,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C53" s="6" t="n">
-        <v>2797.02</v>
+        <v>111.46</v>
       </c>
       <c r="D53" s="6" t="n">
-        <v>5628.44</v>
+        <v>330.41</v>
       </c>
       <c r="E53" s="6" t="n">
-        <v>2012.298803726824</v>
+        <v>2964.3818410192</v>
       </c>
     </row>
     <row r="54">
@@ -9866,17 +10327,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C54" s="6" t="n">
-        <v>13.67</v>
+        <v>3412.5</v>
       </c>
       <c r="D54" s="6" t="n">
-        <v>39.3</v>
+        <v>6849.4</v>
       </c>
       <c r="E54" s="6" t="n">
-        <v>2874.908558888077</v>
+        <v>2007.150183150183</v>
       </c>
     </row>
     <row r="55">
@@ -9887,17 +10348,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C55" s="6" t="n">
-        <v>340.13</v>
+        <v>13.67</v>
       </c>
       <c r="D55" s="6" t="n">
-        <v>471.82</v>
+        <v>39.3</v>
       </c>
       <c r="E55" s="6" t="n">
-        <v>1387.175491723753</v>
+        <v>2874.908558888077</v>
       </c>
     </row>
     <row r="56">
@@ -9908,17 +10369,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="C56" s="6" t="n">
-        <v>122.18</v>
+        <v>340.13</v>
       </c>
       <c r="D56" s="6" t="n">
-        <v>396.04</v>
+        <v>471.82</v>
       </c>
       <c r="E56" s="6" t="n">
-        <v>3241.447045342937</v>
+        <v>1387.175491723753</v>
       </c>
     </row>
     <row r="57">
@@ -9929,17 +10390,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C57" s="6" t="n">
-        <v>1253</v>
+        <v>122.16</v>
       </c>
       <c r="D57" s="6" t="n">
-        <v>2613.01</v>
+        <v>394.13</v>
       </c>
       <c r="E57" s="6" t="n">
-        <v>2085.403032721468</v>
+        <v>3226.342501637197</v>
       </c>
     </row>
     <row r="58">
@@ -9950,17 +10411,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C58" s="6" t="n">
-        <v>9262.59</v>
+        <v>1272.37</v>
       </c>
       <c r="D58" s="6" t="n">
-        <v>14317.28</v>
+        <v>2653.31</v>
       </c>
       <c r="E58" s="6" t="n">
-        <v>1545.710217120697</v>
+        <v>2085.328953056108</v>
       </c>
     </row>
     <row r="59">
@@ -9971,17 +10432,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C59" s="6" t="n">
-        <v>53.19</v>
+        <v>11307.92</v>
       </c>
       <c r="D59" s="6" t="n">
-        <v>89.00999999999999</v>
+        <v>17502.81</v>
       </c>
       <c r="E59" s="6" t="n">
-        <v>1673.434856175973</v>
+        <v>1547.83638370275</v>
       </c>
     </row>
     <row r="60">
@@ -9992,17 +10453,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C60" s="6" t="n">
-        <v>1152.11</v>
+        <v>53.19</v>
       </c>
       <c r="D60" s="6" t="n">
-        <v>2691.05</v>
+        <v>89.00999999999999</v>
       </c>
       <c r="E60" s="6" t="n">
-        <v>2335.757870342241</v>
+        <v>1673.434856175973</v>
       </c>
     </row>
     <row r="61">
@@ -10013,17 +10474,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C61" s="6" t="n">
-        <v>648.9700000000001</v>
+        <v>1152.11</v>
       </c>
       <c r="D61" s="6" t="n">
-        <v>1088.52</v>
+        <v>2691.05</v>
       </c>
       <c r="E61" s="6" t="n">
-        <v>1677.304035625683</v>
+        <v>2335.757870342241</v>
       </c>
     </row>
     <row r="62">
@@ -10034,17 +10495,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>New Zealand</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C62" s="6" t="n">
-        <v>489.25</v>
+        <v>681.9600000000002</v>
       </c>
       <c r="D62" s="6" t="n">
-        <v>567.84</v>
+        <v>1142.74</v>
       </c>
       <c r="E62" s="6" t="n">
-        <v>1160.633622892182</v>
+        <v>1675.670127280192</v>
       </c>
     </row>
     <row r="63">
@@ -10055,17 +10516,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>New Zealand</t>
         </is>
       </c>
       <c r="C63" s="6" t="n">
-        <v>996.73</v>
+        <v>489.25</v>
       </c>
       <c r="D63" s="6" t="n">
-        <v>1032.71</v>
+        <v>567.84</v>
       </c>
       <c r="E63" s="6" t="n">
-        <v>1036.098040592738</v>
+        <v>1160.633622892182</v>
       </c>
     </row>
     <row r="64">
@@ -10076,17 +10537,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="C64" s="6" t="n">
-        <v>48.67</v>
+        <v>996.73</v>
       </c>
       <c r="D64" s="6" t="n">
-        <v>57.52</v>
+        <v>1032.71</v>
       </c>
       <c r="E64" s="6" t="n">
-        <v>1181.836860489007</v>
+        <v>1036.098040592738</v>
       </c>
     </row>
     <row r="65">
@@ -10097,17 +10558,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C65" s="6" t="n">
-        <v>20</v>
+        <v>48.67</v>
       </c>
       <c r="D65" s="6" t="n">
-        <v>40.1</v>
+        <v>57.52</v>
       </c>
       <c r="E65" s="6" t="n">
-        <v>2005</v>
+        <v>1181.836860489007</v>
       </c>
     </row>
     <row r="66">
@@ -10118,17 +10579,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="C66" s="6" t="n">
-        <v>63.97</v>
+        <v>20</v>
       </c>
       <c r="D66" s="6" t="n">
-        <v>81.75</v>
+        <v>40.1</v>
       </c>
       <c r="E66" s="6" t="n">
-        <v>1277.942785680788</v>
+        <v>2005</v>
       </c>
     </row>
     <row r="67">
@@ -10139,17 +10600,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="C67" s="6" t="n">
-        <v>10579.12</v>
+        <v>63.97</v>
       </c>
       <c r="D67" s="6" t="n">
-        <v>14302.06</v>
+        <v>81.75</v>
       </c>
       <c r="E67" s="6" t="n">
-        <v>1351.913958816991</v>
+        <v>1277.942785680788</v>
       </c>
     </row>
     <row r="68">
@@ -10160,17 +10621,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C68" s="6" t="n">
-        <v>2593.2</v>
+        <v>10579.12</v>
       </c>
       <c r="D68" s="6" t="n">
-        <v>3265.41</v>
+        <v>14302.06</v>
       </c>
       <c r="E68" s="6" t="n">
-        <v>1259.220268394262</v>
+        <v>1351.913958816991</v>
       </c>
     </row>
     <row r="69">
@@ -10181,17 +10642,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C69" s="6" t="n">
-        <v>11334.39</v>
+        <v>2593.2</v>
       </c>
       <c r="D69" s="6" t="n">
-        <v>12765.71</v>
+        <v>3265.41</v>
       </c>
       <c r="E69" s="6" t="n">
-        <v>1126.281167314695</v>
+        <v>1259.220268394262</v>
       </c>
     </row>
     <row r="70">
@@ -10202,17 +10663,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Ukraine</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C70" s="6" t="n">
-        <v>17.65</v>
+        <v>11334.39</v>
       </c>
       <c r="D70" s="6" t="n">
-        <v>68.54000000000001</v>
+        <v>12765.71</v>
       </c>
       <c r="E70" s="6" t="n">
-        <v>3883.28611898017</v>
+        <v>1126.281167314695</v>
       </c>
     </row>
     <row r="71">
@@ -10223,17 +10684,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Ukraine</t>
         </is>
       </c>
       <c r="C71" s="6" t="n">
-        <v>969.2099999999999</v>
+        <v>17.65</v>
       </c>
       <c r="D71" s="6" t="n">
-        <v>1111.34</v>
+        <v>68.54000000000001</v>
       </c>
       <c r="E71" s="6" t="n">
-        <v>1146.645205889333</v>
+        <v>3883.28611898017</v>
       </c>
     </row>
     <row r="72">
@@ -10244,17 +10705,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="C72" s="6" t="n">
-        <v>40602.37</v>
+        <v>969.2099999999999</v>
       </c>
       <c r="D72" s="6" t="n">
-        <v>77795.21000000001</v>
+        <v>1111.34</v>
       </c>
       <c r="E72" s="6" t="n">
-        <v>1916.026330482679</v>
+        <v>1146.645205889333</v>
       </c>
     </row>
     <row r="73">
@@ -10265,38 +10726,38 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C73" s="6" t="n">
-        <v>1189.02</v>
+        <v>44749.39999999999</v>
       </c>
       <c r="D73" s="6" t="n">
-        <v>1275.32</v>
+        <v>86060.23</v>
       </c>
       <c r="E73" s="6" t="n">
-        <v>1072.580780811088</v>
+        <v>1923.15941666257</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Cambodia</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C74" s="6" t="n">
-        <v>6038.5</v>
+        <v>1189.02</v>
       </c>
       <c r="D74" s="6" t="n">
-        <v>4639.469999999999</v>
+        <v>1275.32</v>
       </c>
       <c r="E74" s="6" t="n">
-        <v>768.3149788854846</v>
+        <v>1072.580780811088</v>
       </c>
     </row>
     <row r="75">
@@ -10307,17 +10768,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Cambodia</t>
         </is>
       </c>
       <c r="C75" s="6" t="n">
-        <v>18.06</v>
+        <v>6038.5</v>
       </c>
       <c r="D75" s="6" t="n">
-        <v>14.86</v>
+        <v>4639.469999999999</v>
       </c>
       <c r="E75" s="6" t="n">
-        <v>822.8128460686601</v>
+        <v>768.3149788854846</v>
       </c>
     </row>
     <row r="76">
@@ -10328,17 +10789,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C76" s="6" t="n">
-        <v>388.89</v>
+        <v>18.06</v>
       </c>
       <c r="D76" s="6" t="n">
-        <v>535.6999999999999</v>
+        <v>14.86</v>
       </c>
       <c r="E76" s="6" t="n">
-        <v>1377.510349970428</v>
+        <v>822.8128460686601</v>
       </c>
     </row>
     <row r="77">
@@ -10349,17 +10810,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C77" s="6" t="n">
-        <v>2577.92</v>
+        <v>394.41</v>
       </c>
       <c r="D77" s="6" t="n">
-        <v>2016.72</v>
+        <v>557.88</v>
       </c>
       <c r="E77" s="6" t="n">
-        <v>782.3051142005958</v>
+        <v>1414.467178824066</v>
       </c>
     </row>
     <row r="78">
@@ -10370,17 +10831,17 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C78" s="6" t="n">
-        <v>3218.63</v>
+        <v>2577.92</v>
       </c>
       <c r="D78" s="6" t="n">
-        <v>2489.5</v>
+        <v>2016.72</v>
       </c>
       <c r="E78" s="6" t="n">
-        <v>773.4657292077685</v>
+        <v>782.3051142005958</v>
       </c>
     </row>
     <row r="79">
@@ -10391,17 +10852,17 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="C79" s="6" t="n">
-        <v>25669.47</v>
+        <v>3218.63</v>
       </c>
       <c r="D79" s="6" t="n">
-        <v>27999.43</v>
+        <v>2489.5</v>
       </c>
       <c r="E79" s="6" t="n">
-        <v>1090.767748613431</v>
+        <v>773.4657292077685</v>
       </c>
     </row>
     <row r="80">
@@ -10412,17 +10873,17 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C80" s="6" t="n">
-        <v>52.75</v>
+        <v>26154.26</v>
       </c>
       <c r="D80" s="6" t="n">
-        <v>53.87</v>
+        <v>28633.86</v>
       </c>
       <c r="E80" s="6" t="n">
-        <v>1021.232227488152</v>
+        <v>1094.806735116956</v>
       </c>
     </row>
     <row r="81">
@@ -10433,59 +10894,59 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C81" s="6" t="n">
-        <v>1291.6</v>
+        <v>49.88</v>
       </c>
       <c r="D81" s="6" t="n">
-        <v>2373.32</v>
+        <v>70.22</v>
       </c>
       <c r="E81" s="6" t="n">
-        <v>1837.503871167544</v>
+        <v>1407.778668805132</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="C82" s="6" t="n">
-        <v>781.04</v>
+        <v>52.75</v>
       </c>
       <c r="D82" s="6" t="n">
-        <v>750.46</v>
+        <v>53.87</v>
       </c>
       <c r="E82" s="6" t="n">
-        <v>960.8470756939465</v>
+        <v>1021.232227488152</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C83" s="6" t="n">
-        <v>204.62</v>
+        <v>1499.67</v>
       </c>
       <c r="D83" s="6" t="n">
-        <v>218.88</v>
+        <v>2855.9</v>
       </c>
       <c r="E83" s="6" t="n">
-        <v>1069.690157364872</v>
+        <v>1904.352290837317</v>
       </c>
     </row>
     <row r="84">
@@ -10496,17 +10957,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C84" s="6" t="n">
-        <v>1.12</v>
+        <v>800.48</v>
       </c>
       <c r="D84" s="6" t="n">
-        <v>4.18</v>
+        <v>794.91</v>
       </c>
       <c r="E84" s="6" t="n">
-        <v>3732.142857142857</v>
+        <v>993.0416749950029</v>
       </c>
     </row>
     <row r="85">
@@ -10517,17 +10978,17 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C85" s="6" t="n">
-        <v>19.32</v>
+        <v>204.64</v>
       </c>
       <c r="D85" s="6" t="n">
-        <v>39.73</v>
+        <v>218.94</v>
       </c>
       <c r="E85" s="6" t="n">
-        <v>2056.418219461698</v>
+        <v>1069.87881157154</v>
       </c>
     </row>
     <row r="86">
@@ -10538,17 +10999,17 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="C86" s="6" t="n">
-        <v>585.71</v>
+        <v>1.12</v>
       </c>
       <c r="D86" s="6" t="n">
-        <v>916.8199999999999</v>
+        <v>4.18</v>
       </c>
       <c r="E86" s="6" t="n">
-        <v>1565.313892540677</v>
+        <v>3732.142857142857</v>
       </c>
     </row>
     <row r="87">
@@ -10559,17 +11020,17 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="C87" s="6" t="n">
-        <v>3.2</v>
+        <v>19.32</v>
       </c>
       <c r="D87" s="6" t="n">
-        <v>4</v>
+        <v>39.73</v>
       </c>
       <c r="E87" s="6" t="n">
-        <v>1250</v>
+        <v>2056.418219461698</v>
       </c>
     </row>
     <row r="88">
@@ -10580,17 +11041,17 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C88" s="6" t="n">
-        <v>41.26000000000001</v>
+        <v>585.71</v>
       </c>
       <c r="D88" s="6" t="n">
-        <v>112.53</v>
+        <v>916.8199999999999</v>
       </c>
       <c r="E88" s="6" t="n">
-        <v>2727.338826951042</v>
+        <v>1565.313892540677</v>
       </c>
     </row>
     <row r="89">
@@ -10601,17 +11062,17 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C89" s="6" t="n">
-        <v>9.379999999999999</v>
+        <v>5.99</v>
       </c>
       <c r="D89" s="6" t="n">
-        <v>19.62</v>
+        <v>8.460000000000001</v>
       </c>
       <c r="E89" s="6" t="n">
-        <v>2091.684434968017</v>
+        <v>1412.353923205342</v>
       </c>
     </row>
     <row r="90">
@@ -10622,17 +11083,17 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C90" s="6" t="n">
-        <v>926.85</v>
+        <v>41.26000000000001</v>
       </c>
       <c r="D90" s="6" t="n">
-        <v>1259.8</v>
+        <v>112.53</v>
       </c>
       <c r="E90" s="6" t="n">
-        <v>1359.227490964018</v>
+        <v>2727.338826951042</v>
       </c>
     </row>
     <row r="91">
@@ -10643,17 +11104,17 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C91" s="6" t="n">
-        <v>1.2</v>
+        <v>9.379999999999999</v>
       </c>
       <c r="D91" s="6" t="n">
-        <v>5.45</v>
+        <v>19.62</v>
       </c>
       <c r="E91" s="6" t="n">
-        <v>4541.666666666666</v>
+        <v>2091.684434968017</v>
       </c>
     </row>
     <row r="92">
@@ -10664,17 +11125,17 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C92" s="6" t="n">
-        <v>25.4</v>
+        <v>926.85</v>
       </c>
       <c r="D92" s="6" t="n">
-        <v>49.81</v>
+        <v>1259.8</v>
       </c>
       <c r="E92" s="6" t="n">
-        <v>1961.023622047244</v>
+        <v>1359.227490964018</v>
       </c>
     </row>
     <row r="93">
@@ -10685,17 +11146,17 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="C93" s="6" t="n">
-        <v>2006.45</v>
+        <v>1.57</v>
       </c>
       <c r="D93" s="6" t="n">
-        <v>1931.12</v>
+        <v>7.23</v>
       </c>
       <c r="E93" s="6" t="n">
-        <v>962.4560791447583</v>
+        <v>4605.095541401273</v>
       </c>
     </row>
     <row r="94">
@@ -10706,17 +11167,17 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C94" s="6" t="n">
-        <v>1277.28</v>
+        <v>25.4</v>
       </c>
       <c r="D94" s="6" t="n">
-        <v>1216.36</v>
+        <v>49.81</v>
       </c>
       <c r="E94" s="6" t="n">
-        <v>952.3048979080546</v>
+        <v>1961.023622047244</v>
       </c>
     </row>
     <row r="95">
@@ -10727,17 +11188,17 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C95" s="6" t="n">
-        <v>10.8</v>
+        <v>2160.85</v>
       </c>
       <c r="D95" s="6" t="n">
-        <v>47.44</v>
+        <v>2077.93</v>
       </c>
       <c r="E95" s="6" t="n">
-        <v>4392.592592592593</v>
+        <v>961.6262119073514</v>
       </c>
     </row>
     <row r="96">
@@ -10748,59 +11209,59 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C96" s="6" t="n">
-        <v>2637.070000000001</v>
+        <v>1383.67</v>
       </c>
       <c r="D96" s="6" t="n">
-        <v>5432.979999999999</v>
+        <v>1326.04</v>
       </c>
       <c r="E96" s="6" t="n">
-        <v>2060.233516743961</v>
+        <v>958.3498955675847</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C97" s="6" t="n">
-        <v>72.08</v>
+        <v>10.8</v>
       </c>
       <c r="D97" s="6" t="n">
-        <v>95.73999999999999</v>
+        <v>47.44</v>
       </c>
       <c r="E97" s="6" t="n">
-        <v>1328.246392896781</v>
+        <v>4392.592592592593</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C98" s="6" t="n">
-        <v>931.79</v>
+        <v>2847.08</v>
       </c>
       <c r="D98" s="6" t="n">
-        <v>1241.13</v>
+        <v>5859.5</v>
       </c>
       <c r="E98" s="6" t="n">
-        <v>1331.984674658453</v>
+        <v>2058.073534990235</v>
       </c>
     </row>
     <row r="99">
@@ -10811,17 +11272,17 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C99" s="6" t="n">
-        <v>5.78</v>
+        <v>72.08</v>
       </c>
       <c r="D99" s="6" t="n">
-        <v>10.29</v>
+        <v>95.73999999999999</v>
       </c>
       <c r="E99" s="6" t="n">
-        <v>1780.276816608997</v>
+        <v>1328.246392896781</v>
       </c>
     </row>
     <row r="100">
@@ -10832,17 +11293,17 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C100" s="6" t="n">
-        <v>7095.829999999999</v>
+        <v>1147.2</v>
       </c>
       <c r="D100" s="6" t="n">
-        <v>10565.72</v>
+        <v>1518.63</v>
       </c>
       <c r="E100" s="6" t="n">
-        <v>1489.004105228</v>
+        <v>1323.770920502092</v>
       </c>
     </row>
     <row r="101">
@@ -10853,17 +11314,17 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C101" s="6" t="n">
-        <v>8103.91</v>
+        <v>5.78</v>
       </c>
       <c r="D101" s="6" t="n">
-        <v>5812.44</v>
+        <v>10.29</v>
       </c>
       <c r="E101" s="6" t="n">
-        <v>717.2389624267792</v>
+        <v>1780.276816608997</v>
       </c>
     </row>
     <row r="102">
@@ -10874,17 +11335,17 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C102" s="6" t="n">
-        <v>256.94</v>
+        <v>8086.389999999999</v>
       </c>
       <c r="D102" s="6" t="n">
-        <v>334.05</v>
+        <v>11816.42</v>
       </c>
       <c r="E102" s="6" t="n">
-        <v>1300.108974857943</v>
+        <v>1461.272582697595</v>
       </c>
     </row>
     <row r="103">
@@ -10895,17 +11356,17 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C103" s="6" t="n">
-        <v>506.71</v>
+        <v>8103.91</v>
       </c>
       <c r="D103" s="6" t="n">
-        <v>617.79</v>
+        <v>5812.44</v>
       </c>
       <c r="E103" s="6" t="n">
-        <v>1219.218093189398</v>
+        <v>717.2389624267792</v>
       </c>
     </row>
     <row r="104">
@@ -10916,17 +11377,17 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C104" s="6" t="n">
-        <v>288.96</v>
+        <v>256.94</v>
       </c>
       <c r="D104" s="6" t="n">
-        <v>328.76</v>
+        <v>334.05</v>
       </c>
       <c r="E104" s="6" t="n">
-        <v>1137.735326688815</v>
+        <v>1300.108974857943</v>
       </c>
     </row>
     <row r="105">
@@ -10937,59 +11398,59 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C105" s="6" t="n">
-        <v>6756.18</v>
+        <v>506.71</v>
       </c>
       <c r="D105" s="6" t="n">
-        <v>9549.290000000001</v>
+        <v>617.79</v>
       </c>
       <c r="E105" s="6" t="n">
-        <v>1413.415569152983</v>
+        <v>1219.218093189398</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C106" s="6" t="n">
-        <v>1604.34</v>
+        <v>288.96</v>
       </c>
       <c r="D106" s="6" t="n">
-        <v>1403.65</v>
+        <v>328.76</v>
       </c>
       <c r="E106" s="6" t="n">
-        <v>874.9080618821445</v>
+        <v>1137.735326688815</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C107" s="6" t="n">
-        <v>0.17</v>
+        <v>7583.13</v>
       </c>
       <c r="D107" s="6" t="n">
-        <v>0.63</v>
+        <v>10717.53</v>
       </c>
       <c r="E107" s="6" t="n">
-        <v>3705.882352941176</v>
+        <v>1413.338555451377</v>
       </c>
     </row>
     <row r="108">
@@ -11000,17 +11461,17 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C108" s="6" t="n">
-        <v>579.9</v>
+        <v>1650.37</v>
       </c>
       <c r="D108" s="6" t="n">
-        <v>1885.65</v>
+        <v>1440.99</v>
       </c>
       <c r="E108" s="6" t="n">
-        <v>3251.68132436627</v>
+        <v>873.131479607603</v>
       </c>
     </row>
     <row r="109">
@@ -11021,17 +11482,17 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C109" s="6" t="n">
-        <v>55.17</v>
+        <v>0.17</v>
       </c>
       <c r="D109" s="6" t="n">
-        <v>81.37</v>
+        <v>0.63</v>
       </c>
       <c r="E109" s="6" t="n">
-        <v>1474.89577669023</v>
+        <v>3705.882352941176</v>
       </c>
     </row>
     <row r="110">
@@ -11042,17 +11503,17 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C110" s="6" t="n">
-        <v>9.529999999999999</v>
+        <v>579.89</v>
       </c>
       <c r="D110" s="6" t="n">
-        <v>39.84</v>
+        <v>1884.71</v>
       </c>
       <c r="E110" s="6" t="n">
-        <v>4180.482686253935</v>
+        <v>3250.11640138647</v>
       </c>
     </row>
     <row r="111">
@@ -11063,17 +11524,17 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C111" s="6" t="n">
-        <v>4717.8</v>
+        <v>55.17</v>
       </c>
       <c r="D111" s="6" t="n">
-        <v>5541.98</v>
+        <v>81.37</v>
       </c>
       <c r="E111" s="6" t="n">
-        <v>1174.695832803425</v>
+        <v>1474.89577669023</v>
       </c>
     </row>
     <row r="112">
@@ -11084,17 +11545,17 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C112" s="6" t="n">
-        <v>53744.44</v>
+        <v>35.69</v>
       </c>
       <c r="D112" s="6" t="n">
-        <v>53799.49</v>
+        <v>130.5</v>
       </c>
       <c r="E112" s="6" t="n">
-        <v>1001.024292001182</v>
+        <v>3656.486410759317</v>
       </c>
     </row>
     <row r="113">
@@ -11105,17 +11566,17 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C113" s="6" t="n">
-        <v>6566.25</v>
+        <v>4717.8</v>
       </c>
       <c r="D113" s="6" t="n">
-        <v>10907.93</v>
+        <v>5541.98</v>
       </c>
       <c r="E113" s="6" t="n">
-        <v>1661.211498191509</v>
+        <v>1174.695832803425</v>
       </c>
     </row>
     <row r="114">
@@ -11126,17 +11587,17 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C114" s="6" t="n">
-        <v>9464.199999999997</v>
+        <v>65266.67</v>
       </c>
       <c r="D114" s="6" t="n">
-        <v>13167.46</v>
+        <v>64435.03000000001</v>
       </c>
       <c r="E114" s="6" t="n">
-        <v>1391.291392827709</v>
+        <v>987.2578147467921</v>
       </c>
     </row>
     <row r="115">
@@ -11147,17 +11608,17 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Luxembourg</t>
         </is>
       </c>
       <c r="C115" s="6" t="n">
-        <v>0.96</v>
+        <v>6582.36</v>
       </c>
       <c r="D115" s="6" t="n">
-        <v>3.83</v>
+        <v>10977.15</v>
       </c>
       <c r="E115" s="6" t="n">
-        <v>3989.583333333333</v>
+        <v>1667.661750496782</v>
       </c>
     </row>
     <row r="116">
@@ -11168,17 +11629,17 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C116" s="6" t="n">
-        <v>5036.45</v>
+        <v>10501.68</v>
       </c>
       <c r="D116" s="6" t="n">
-        <v>5378</v>
+        <v>14662.98</v>
       </c>
       <c r="E116" s="6" t="n">
-        <v>1067.815624100309</v>
+        <v>1396.250885572594</v>
       </c>
     </row>
     <row r="117">
@@ -11189,17 +11650,17 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C117" s="6" t="n">
-        <v>0.12</v>
+        <v>0.96</v>
       </c>
       <c r="D117" s="6" t="n">
-        <v>0.59</v>
+        <v>3.83</v>
       </c>
       <c r="E117" s="6" t="n">
-        <v>4916.666666666667</v>
+        <v>3989.583333333333</v>
       </c>
     </row>
     <row r="118">
@@ -11210,17 +11671,17 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C118" s="6" t="n">
-        <v>891.87</v>
+        <v>8957.370000000001</v>
       </c>
       <c r="D118" s="6" t="n">
-        <v>856.11</v>
+        <v>9710.829999999998</v>
       </c>
       <c r="E118" s="6" t="n">
-        <v>959.9044703824549</v>
+        <v>1084.116208217367</v>
       </c>
     </row>
     <row r="119">
@@ -11231,17 +11692,17 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C119" s="6" t="n">
-        <v>6378.700000000001</v>
+        <v>0.12</v>
       </c>
       <c r="D119" s="6" t="n">
-        <v>5627.59</v>
+        <v>0.59</v>
       </c>
       <c r="E119" s="6" t="n">
-        <v>882.2471663505102</v>
+        <v>4916.666666666667</v>
       </c>
     </row>
     <row r="120">
@@ -11252,17 +11713,17 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C120" s="6" t="n">
-        <v>3195.46</v>
+        <v>1180.28</v>
       </c>
       <c r="D120" s="6" t="n">
-        <v>4521.78</v>
+        <v>1132.5</v>
       </c>
       <c r="E120" s="6" t="n">
-        <v>1415.063871868213</v>
+        <v>959.5180804554851</v>
       </c>
     </row>
     <row r="121">
@@ -11273,17 +11734,17 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C121" s="6" t="n">
-        <v>7469.389999999999</v>
+        <v>6378.700000000001</v>
       </c>
       <c r="D121" s="6" t="n">
-        <v>7839.33</v>
+        <v>5627.59</v>
       </c>
       <c r="E121" s="6" t="n">
-        <v>1049.527471453492</v>
+        <v>882.2471663505102</v>
       </c>
     </row>
     <row r="122">
@@ -11294,17 +11755,17 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C122" s="6" t="n">
-        <v>6316.48</v>
+        <v>3250.889999999999</v>
       </c>
       <c r="D122" s="6" t="n">
-        <v>7401.58</v>
+        <v>4577.62</v>
       </c>
       <c r="E122" s="6" t="n">
-        <v>1171.788717766858</v>
+        <v>1408.112855248871</v>
       </c>
     </row>
     <row r="123">
@@ -11315,17 +11776,17 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="C123" s="6" t="n">
-        <v>14488.25</v>
+        <v>7469.389999999999</v>
       </c>
       <c r="D123" s="6" t="n">
-        <v>35891.58000000001</v>
+        <v>7839.33</v>
       </c>
       <c r="E123" s="6" t="n">
-        <v>2477.288837506256</v>
+        <v>1049.527471453492</v>
       </c>
     </row>
     <row r="124">
@@ -11336,16 +11797,58 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C124" s="6" t="n">
+        <v>10379.11</v>
+      </c>
+      <c r="D124" s="6" t="n">
+        <v>12309.48</v>
+      </c>
+      <c r="E124" s="6" t="n">
+        <v>1185.986081658254</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C125" s="6" t="n">
+        <v>15626.29</v>
+      </c>
+      <c r="D125" s="6" t="n">
+        <v>38809.40000000001</v>
+      </c>
+      <c r="E125" s="6" t="n">
+        <v>2483.59655426848</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
           <t>Vietnam</t>
         </is>
       </c>
-      <c r="C124" s="6" t="n">
+      <c r="C126" s="6" t="n">
         <v>345.42</v>
       </c>
-      <c r="D124" s="6" t="n">
+      <c r="D126" s="6" t="n">
         <v>331.78</v>
       </c>
-      <c r="E124" s="6" t="n">
+      <c r="E126" s="6" t="n">
         <v>960.51184065775</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Weekly TRQ update 2026-06-30
</commit_message>
<xml_diff>
--- a/data/canada_trq_tracker.xlsx
+++ b/data/canada_trq_tracker.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S54"/>
+  <dimension ref="A1:T54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,6 +531,11 @@
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
+          <t>June 30 2026</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
           <t>OVER</t>
         </is>
       </c>
@@ -594,6 +599,9 @@
       <c r="R3" s="4" t="n">
         <v>0.0397</v>
       </c>
+      <c r="S3" s="4" t="n">
+        <v>0.0401</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -654,6 +662,9 @@
       <c r="R4" s="4" t="n">
         <v>0.0033</v>
       </c>
+      <c r="S4" s="4" t="n">
+        <v>0.0033</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -714,7 +725,10 @@
       <c r="R5" s="4" t="n">
         <v>0.41</v>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="S5" s="4" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="T5" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -764,6 +778,9 @@
       <c r="R6" s="4" t="n">
         <v>0.0002</v>
       </c>
+      <c r="S6" s="4" t="n">
+        <v>0.0002</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -832,6 +849,10 @@
         <f>SUM(R3:R6)</f>
         <v/>
       </c>
+      <c r="S7" s="5">
+        <f>SUM(S3:S6)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -892,7 +913,10 @@
       <c r="R8" s="4" t="n">
         <v>0.36</v>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="S8" s="4" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="T8" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -957,6 +981,9 @@
       <c r="R9" s="4" t="n">
         <v>0.0369</v>
       </c>
+      <c r="S9" s="4" t="n">
+        <v>0.0369</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1002,6 +1029,9 @@
       <c r="R10" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="S10" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1070,6 +1100,10 @@
         <f>SUM(R8:R10)</f>
         <v/>
       </c>
+      <c r="S11" s="5">
+        <f>SUM(S8:S10)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1130,6 +1164,9 @@
       <c r="R12" s="4" t="n">
         <v>0.0063</v>
       </c>
+      <c r="S12" s="4" t="n">
+        <v>0.0063</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1190,6 +1227,9 @@
       <c r="R13" s="4" t="n">
         <v>0.0113</v>
       </c>
+      <c r="S13" s="4" t="n">
+        <v>0.0113</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1250,6 +1290,9 @@
       <c r="R14" s="4" t="n">
         <v>0.6692</v>
       </c>
+      <c r="S14" s="4" t="n">
+        <v>0.6692</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1310,6 +1353,9 @@
       <c r="R15" s="4" t="n">
         <v>0.2512</v>
       </c>
+      <c r="S15" s="4" t="n">
+        <v>0.2512</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1361,6 +1407,9 @@
       <c r="R16" s="4" t="n">
         <v>0.0552</v>
       </c>
+      <c r="S16" s="4" t="n">
+        <v>0.0552</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1397,6 +1446,9 @@
       <c r="R17" s="4" t="n">
         <v>0.0067</v>
       </c>
+      <c r="S17" s="4" t="n">
+        <v>0.0067</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1465,6 +1517,10 @@
         <f>SUM(R12:R17)</f>
         <v/>
       </c>
+      <c r="S18" s="5">
+        <f>SUM(S12:S17)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1525,6 +1581,9 @@
       <c r="R19" s="4" t="n">
         <v>0.0092</v>
       </c>
+      <c r="S19" s="4" t="n">
+        <v>0.0092</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1585,6 +1644,9 @@
       <c r="R20" s="4" t="n">
         <v>0.0005</v>
       </c>
+      <c r="S20" s="4" t="n">
+        <v>0.0005</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1645,6 +1707,9 @@
       <c r="R21" s="4" t="n">
         <v>0.0532</v>
       </c>
+      <c r="S21" s="4" t="n">
+        <v>0.0532</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1705,6 +1770,9 @@
       <c r="R22" s="4" t="n">
         <v>0.0119</v>
       </c>
+      <c r="S22" s="4" t="n">
+        <v>0.0119</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1765,6 +1833,9 @@
       <c r="R23" s="4" t="n">
         <v>0.3695000000000001</v>
       </c>
+      <c r="S23" s="4" t="n">
+        <v>0.3695000000000001</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1825,6 +1896,9 @@
       <c r="R24" s="4" t="n">
         <v>0.1384</v>
       </c>
+      <c r="S24" s="4" t="n">
+        <v>0.1384</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1885,6 +1959,9 @@
       <c r="R25" s="4" t="n">
         <v>0.3262</v>
       </c>
+      <c r="S25" s="4" t="n">
+        <v>0.3262</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1945,6 +2022,9 @@
       <c r="R26" s="4" t="n">
         <v>0.05599999999999999</v>
       </c>
+      <c r="S26" s="4" t="n">
+        <v>0.05599999999999999</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1996,6 +2076,9 @@
       <c r="R27" s="4" t="n">
         <v>0.0207</v>
       </c>
+      <c r="S27" s="4" t="n">
+        <v>0.0207</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2074,6 +2157,9 @@
       <c r="R29" s="4" t="n">
         <v>0.0008</v>
       </c>
+      <c r="S29" s="4" t="n">
+        <v>0.0008</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2142,6 +2228,10 @@
         <f>SUM(R19:R29)</f>
         <v/>
       </c>
+      <c r="S30" s="5">
+        <f>SUM(S19:S29)</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2202,7 +2292,10 @@
       <c r="R31" s="4" t="n">
         <v>0.29</v>
       </c>
-      <c r="S31" t="inlineStr">
+      <c r="S31" s="4" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="T31" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -2267,6 +2360,9 @@
       <c r="R32" s="4" t="n">
         <v>0.1228</v>
       </c>
+      <c r="S32" s="4" t="n">
+        <v>0.1228</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2327,6 +2423,9 @@
       <c r="R33" s="4" t="n">
         <v>0.2394</v>
       </c>
+      <c r="S33" s="4" t="n">
+        <v>0.2394</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2387,6 +2486,9 @@
       <c r="R34" s="4" t="n">
         <v>0.1668</v>
       </c>
+      <c r="S34" s="4" t="n">
+        <v>0.1668</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2447,6 +2549,9 @@
       <c r="R35" s="4" t="n">
         <v>0.0241</v>
       </c>
+      <c r="S35" s="4" t="n">
+        <v>0.0241</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2507,6 +2612,9 @@
       <c r="R36" s="4" t="n">
         <v>0.1569</v>
       </c>
+      <c r="S36" s="4" t="n">
+        <v>0.1569</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2575,6 +2683,10 @@
         <f>SUM(R31:R36)</f>
         <v/>
       </c>
+      <c r="S37" s="5">
+        <f>SUM(S31:S36)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2635,6 +2747,9 @@
       <c r="R38" s="4" t="n">
         <v>0.0684</v>
       </c>
+      <c r="S38" s="4" t="n">
+        <v>0.0684</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2695,6 +2810,9 @@
       <c r="R39" s="4" t="n">
         <v>0.3214</v>
       </c>
+      <c r="S39" s="4" t="n">
+        <v>0.3214</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2755,6 +2873,9 @@
       <c r="R40" s="4" t="n">
         <v>0.3890999999999999</v>
       </c>
+      <c r="S40" s="4" t="n">
+        <v>0.3890999999999999</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2815,6 +2936,9 @@
       <c r="R41" s="4" t="n">
         <v>0.212</v>
       </c>
+      <c r="S41" s="4" t="n">
+        <v>0.212</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2869,6 +2993,9 @@
       <c r="R42" s="4" t="n">
         <v>0.0005</v>
       </c>
+      <c r="S42" s="4" t="n">
+        <v>0.0005</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2937,6 +3064,10 @@
         <f>SUM(R38:R42)</f>
         <v/>
       </c>
+      <c r="S43" s="5">
+        <f>SUM(S38:S42)</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2997,6 +3128,9 @@
       <c r="R44" s="4" t="n">
         <v>0.442</v>
       </c>
+      <c r="S44" s="4" t="n">
+        <v>0.442</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3045,7 +3179,10 @@
       <c r="R45" s="4" t="n">
         <v>0.45</v>
       </c>
-      <c r="S45" t="inlineStr">
+      <c r="S45" s="4" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="T45" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -3095,6 +3232,9 @@
       <c r="R46" s="4" t="n">
         <v>0.0024</v>
       </c>
+      <c r="S46" s="4" t="n">
+        <v>0.0058</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3163,6 +3303,10 @@
         <f>SUM(R44:R46)</f>
         <v/>
       </c>
+      <c r="S47" s="5">
+        <f>SUM(S44:S46)</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3223,6 +3367,9 @@
       <c r="R48" s="4" t="n">
         <v>0.08810000000000001</v>
       </c>
+      <c r="S48" s="4" t="n">
+        <v>0.08810000000000001</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3283,6 +3430,9 @@
       <c r="R49" s="4" t="n">
         <v>0.0353</v>
       </c>
+      <c r="S49" s="4" t="n">
+        <v>0.0353</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3343,6 +3493,9 @@
       <c r="R50" s="4" t="n">
         <v>0.3962</v>
       </c>
+      <c r="S50" s="4" t="n">
+        <v>0.3962</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3403,6 +3556,9 @@
       <c r="R51" s="4" t="n">
         <v>0.388</v>
       </c>
+      <c r="S51" s="4" t="n">
+        <v>0.388</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3427,6 +3583,9 @@
       <c r="R52" s="4" t="n">
         <v>0.0108</v>
       </c>
+      <c r="S52" s="4" t="n">
+        <v>0.0108</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3451,6 +3610,9 @@
       <c r="R53" s="4" t="n">
         <v>0.04269999999999999</v>
       </c>
+      <c r="S53" s="4" t="n">
+        <v>0.04269999999999999</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3517,6 +3679,10 @@
       </c>
       <c r="R54" s="5">
         <f>SUM(R48:R53)</f>
+        <v/>
+      </c>
+      <c r="S54" s="5">
+        <f>SUM(S48:S53)</f>
         <v/>
       </c>
     </row>
@@ -3531,7 +3697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S96"/>
+  <dimension ref="A1:T96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3629,6 +3795,11 @@
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
+          <t>June 30 2026</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
           <t>OVER</t>
         </is>
       </c>
@@ -3692,6 +3863,9 @@
       <c r="R3" s="4" t="n">
         <v>0.003</v>
       </c>
+      <c r="S3" s="4" t="n">
+        <v>0.003</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3752,6 +3926,9 @@
       <c r="R4" s="4" t="n">
         <v>0.1164</v>
       </c>
+      <c r="S4" s="4" t="n">
+        <v>0.1164</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3812,6 +3989,9 @@
       <c r="R5" s="4" t="n">
         <v>0.115</v>
       </c>
+      <c r="S5" s="4" t="n">
+        <v>0.115</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3872,6 +4052,9 @@
       <c r="R6" s="4" t="n">
         <v>0.4198</v>
       </c>
+      <c r="S6" s="4" t="n">
+        <v>0.4198</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3932,6 +4115,9 @@
       <c r="R7" s="4" t="n">
         <v>0.07429999999999999</v>
       </c>
+      <c r="S7" s="4" t="n">
+        <v>0.07429999999999999</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3992,6 +4178,9 @@
       <c r="R8" s="4" t="n">
         <v>0.0008</v>
       </c>
+      <c r="S8" s="4" t="n">
+        <v>0.0008</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4052,6 +4241,9 @@
       <c r="R9" s="4" t="n">
         <v>0.0143</v>
       </c>
+      <c r="S9" s="4" t="n">
+        <v>0.0143</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4106,6 +4298,9 @@
       <c r="R10" s="4" t="n">
         <v>0.014</v>
       </c>
+      <c r="S10" s="4" t="n">
+        <v>0.014</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4166,6 +4361,9 @@
       <c r="R11" s="4" t="n">
         <v>0.0004</v>
       </c>
+      <c r="S11" s="4" t="n">
+        <v>0.0004</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4223,6 +4421,9 @@
       <c r="R12" s="4" t="n">
         <v>0.0012</v>
       </c>
+      <c r="S12" s="4" t="n">
+        <v>0.0012</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4280,6 +4481,9 @@
       <c r="R13" s="4" t="n">
         <v>0.0003</v>
       </c>
+      <c r="S13" s="4" t="n">
+        <v>0.0003</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4331,6 +4535,9 @@
       <c r="R14" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="S14" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4379,6 +4586,9 @@
       <c r="R15" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="S15" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4427,6 +4637,9 @@
       <c r="R16" s="4" t="n">
         <v>0.2405</v>
       </c>
+      <c r="S16" s="4" t="n">
+        <v>0.2405</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4495,6 +4708,10 @@
         <f>SUM(R3:R16)</f>
         <v/>
       </c>
+      <c r="S17" s="5">
+        <f>SUM(S3:S16)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4555,6 +4772,9 @@
       <c r="R18" s="4" t="n">
         <v>0.0338</v>
       </c>
+      <c r="S18" s="4" t="n">
+        <v>0.0338</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4615,6 +4835,9 @@
       <c r="R19" s="4" t="n">
         <v>0.031</v>
       </c>
+      <c r="S19" s="4" t="n">
+        <v>0.031</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4675,6 +4898,9 @@
       <c r="R20" s="4" t="n">
         <v>0.0741</v>
       </c>
+      <c r="S20" s="4" t="n">
+        <v>0.0741</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4735,6 +4961,9 @@
       <c r="R21" s="4" t="n">
         <v>0.154</v>
       </c>
+      <c r="S21" s="4" t="n">
+        <v>0.154</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4795,6 +5024,9 @@
       <c r="R22" s="4" t="n">
         <v>0.1063</v>
       </c>
+      <c r="S22" s="4" t="n">
+        <v>0.1063</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4855,7 +5087,10 @@
       <c r="R23" s="4" t="n">
         <v>0.3</v>
       </c>
-      <c r="S23" t="inlineStr">
+      <c r="S23" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="T23" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -4920,6 +5155,9 @@
       <c r="R24" s="4" t="n">
         <v>0.1668</v>
       </c>
+      <c r="S24" s="4" t="n">
+        <v>0.1668</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4980,6 +5218,9 @@
       <c r="R25" s="4" t="n">
         <v>0.0005</v>
       </c>
+      <c r="S25" s="4" t="n">
+        <v>0.0005</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -5040,6 +5281,9 @@
       <c r="R26" s="4" t="n">
         <v>0.06900000000000001</v>
       </c>
+      <c r="S26" s="4" t="n">
+        <v>0.06900000000000001</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5097,6 +5341,9 @@
       <c r="R27" s="4" t="n">
         <v>0.0317</v>
       </c>
+      <c r="S27" s="4" t="n">
+        <v>0.0317</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5154,6 +5401,9 @@
       <c r="R28" s="4" t="n">
         <v>0.0073</v>
       </c>
+      <c r="S28" s="4" t="n">
+        <v>0.0073</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -5211,6 +5461,9 @@
       <c r="R29" s="4" t="n">
         <v>0.0005999999999999999</v>
       </c>
+      <c r="S29" s="4" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5262,6 +5515,9 @@
       <c r="R30" s="4" t="n">
         <v>0.0226</v>
       </c>
+      <c r="S30" s="4" t="n">
+        <v>0.0226</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5304,6 +5560,9 @@
       <c r="R31" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="S31" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5372,6 +5631,10 @@
         <f>SUM(R18:R31)</f>
         <v/>
       </c>
+      <c r="S32" s="5">
+        <f>SUM(S18:S31)</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5432,6 +5695,9 @@
       <c r="R33" s="4" t="n">
         <v>0.258</v>
       </c>
+      <c r="S33" s="4" t="n">
+        <v>0.258</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5489,6 +5755,9 @@
       <c r="R34" s="4" t="n">
         <v>0.236</v>
       </c>
+      <c r="S34" s="4" t="n">
+        <v>0.236</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5540,6 +5809,9 @@
       <c r="R35" s="4" t="n">
         <v>0.1992</v>
       </c>
+      <c r="S35" s="4" t="n">
+        <v>0.1992</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5588,6 +5860,9 @@
       <c r="R36" s="4" t="n">
         <v>0.0011</v>
       </c>
+      <c r="S36" s="4" t="n">
+        <v>0.0011</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5630,6 +5905,9 @@
       <c r="R37" s="4" t="n">
         <v>0.3057</v>
       </c>
+      <c r="S37" s="4" t="n">
+        <v>0.3057</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5698,6 +5976,10 @@
         <f>SUM(R33:R37)</f>
         <v/>
       </c>
+      <c r="S38" s="5">
+        <f>SUM(S33:S37)</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5758,6 +6040,9 @@
       <c r="R39" s="4" t="n">
         <v>0.166</v>
       </c>
+      <c r="S39" s="4" t="n">
+        <v>0.166</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5818,6 +6103,9 @@
       <c r="R40" s="4" t="n">
         <v>0.1686</v>
       </c>
+      <c r="S40" s="4" t="n">
+        <v>0.1686</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5878,6 +6166,9 @@
       <c r="R41" s="4" t="n">
         <v>0.2496</v>
       </c>
+      <c r="S41" s="4" t="n">
+        <v>0.2496</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5938,6 +6229,9 @@
       <c r="R42" s="4" t="n">
         <v>0.09910000000000001</v>
       </c>
+      <c r="S42" s="4" t="n">
+        <v>0.09910000000000001</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5998,6 +6292,9 @@
       <c r="R43" s="4" t="n">
         <v>0.0849</v>
       </c>
+      <c r="S43" s="4" t="n">
+        <v>0.0849</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -6058,6 +6355,9 @@
       <c r="R44" s="4" t="n">
         <v>0.0007000000000000001</v>
       </c>
+      <c r="S44" s="4" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -6118,6 +6418,9 @@
       <c r="R45" s="4" t="n">
         <v>0.0906</v>
       </c>
+      <c r="S45" s="4" t="n">
+        <v>0.0906</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -6175,6 +6478,9 @@
       <c r="R46" s="4" t="n">
         <v>0.0014</v>
       </c>
+      <c r="S46" s="4" t="n">
+        <v>0.0014</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -6232,6 +6538,9 @@
       <c r="R47" s="4" t="n">
         <v>0.0354</v>
       </c>
+      <c r="S47" s="4" t="n">
+        <v>0.0354</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6289,6 +6598,9 @@
       <c r="R48" s="4" t="n">
         <v>0.028</v>
       </c>
+      <c r="S48" s="4" t="n">
+        <v>0.028</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -6343,6 +6655,9 @@
       <c r="R49" s="4" t="n">
         <v>0.0003</v>
       </c>
+      <c r="S49" s="4" t="n">
+        <v>0.0003</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -6394,6 +6709,9 @@
       <c r="R50" s="4" t="n">
         <v>0.0014</v>
       </c>
+      <c r="S50" s="4" t="n">
+        <v>0.0014</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -6445,6 +6763,9 @@
       <c r="R51" s="4" t="n">
         <v>0.0157</v>
       </c>
+      <c r="S51" s="4" t="n">
+        <v>0.0157</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -6496,6 +6817,9 @@
       <c r="R52" s="4" t="n">
         <v>0.0215</v>
       </c>
+      <c r="S52" s="4" t="n">
+        <v>0.0215</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6544,6 +6868,9 @@
       <c r="R53" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="S53" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -6592,6 +6919,9 @@
       <c r="R54" s="4" t="n">
         <v>0.0258</v>
       </c>
+      <c r="S54" s="4" t="n">
+        <v>0.0258</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -6660,6 +6990,10 @@
         <f>SUM(R39:R54)</f>
         <v/>
       </c>
+      <c r="S55" s="5">
+        <f>SUM(S39:S54)</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -6720,6 +7054,9 @@
       <c r="R56" s="4" t="n">
         <v>0.1642</v>
       </c>
+      <c r="S56" s="4" t="n">
+        <v>0.1642</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -6780,6 +7117,9 @@
       <c r="R57" s="4" t="n">
         <v>0.3234</v>
       </c>
+      <c r="S57" s="4" t="n">
+        <v>0.3234</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -6840,6 +7180,9 @@
       <c r="R58" s="4" t="n">
         <v>0.0028</v>
       </c>
+      <c r="S58" s="4" t="n">
+        <v>0.0028</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -6900,6 +7243,9 @@
       <c r="R59" s="4" t="n">
         <v>0.1633</v>
       </c>
+      <c r="S59" s="4" t="n">
+        <v>0.1633</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6960,6 +7306,9 @@
       <c r="R60" s="4" t="n">
         <v>0.3462</v>
       </c>
+      <c r="S60" s="4" t="n">
+        <v>0.3462</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -7028,6 +7377,10 @@
         <f>SUM(R56:R60)</f>
         <v/>
       </c>
+      <c r="S61" s="5">
+        <f>SUM(S56:S60)</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -7088,6 +7441,9 @@
       <c r="R62" s="4" t="n">
         <v>0.004500000000000001</v>
       </c>
+      <c r="S62" s="4" t="n">
+        <v>0.004500000000000001</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -7148,6 +7504,9 @@
       <c r="R63" s="4" t="n">
         <v>0.0022</v>
       </c>
+      <c r="S63" s="4" t="n">
+        <v>0.0022</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -7208,6 +7567,9 @@
       <c r="R64" s="4" t="n">
         <v>0.0018</v>
       </c>
+      <c r="S64" s="4" t="n">
+        <v>0.0018</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -7268,6 +7630,9 @@
       <c r="R65" s="4" t="n">
         <v>0.3186</v>
       </c>
+      <c r="S65" s="4" t="n">
+        <v>0.3186</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -7328,6 +7693,9 @@
       <c r="R66" s="4" t="n">
         <v>0.0108</v>
       </c>
+      <c r="S66" s="4" t="n">
+        <v>0.0108</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -7388,6 +7756,9 @@
       <c r="R67" s="4" t="n">
         <v>0.1648</v>
       </c>
+      <c r="S67" s="4" t="n">
+        <v>0.1648</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -7448,6 +7819,9 @@
       <c r="R68" s="4" t="n">
         <v>0.0015</v>
       </c>
+      <c r="S68" s="4" t="n">
+        <v>0.0015</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -7508,6 +7882,9 @@
       <c r="R69" s="4" t="n">
         <v>0.2402</v>
       </c>
+      <c r="S69" s="4" t="n">
+        <v>0.2402</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -7568,6 +7945,9 @@
       <c r="R70" s="4" t="n">
         <v>0.0017</v>
       </c>
+      <c r="S70" s="4" t="n">
+        <v>0.0017</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -7625,6 +8005,9 @@
       <c r="R71" s="4" t="n">
         <v>0.2399</v>
       </c>
+      <c r="S71" s="4" t="n">
+        <v>0.2399</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -7682,6 +8065,9 @@
       <c r="R72" s="4" t="n">
         <v>0.0066</v>
       </c>
+      <c r="S72" s="4" t="n">
+        <v>0.0066</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -7736,6 +8122,9 @@
       <c r="R73" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="S73" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -7787,6 +8176,9 @@
       <c r="R74" s="4" t="n">
         <v>0.0002</v>
       </c>
+      <c r="S74" s="4" t="n">
+        <v>0.0002</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -7835,6 +8227,9 @@
       <c r="R75" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="S75" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -7868,6 +8263,9 @@
       <c r="R76" s="4" t="n">
         <v>0.0019</v>
       </c>
+      <c r="S76" s="4" t="n">
+        <v>0.0019</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -7895,6 +8293,9 @@
       <c r="R77" s="4" t="n">
         <v>0.0005</v>
       </c>
+      <c r="S77" s="4" t="n">
+        <v>0.0005</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -7922,6 +8323,9 @@
       <c r="R78" s="4" t="n">
         <v>0.0026</v>
       </c>
+      <c r="S78" s="4" t="n">
+        <v>0.0026</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -7990,6 +8394,10 @@
         <f>SUM(R62:R78)</f>
         <v/>
       </c>
+      <c r="S79" s="5">
+        <f>SUM(S62:S78)</f>
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -8050,6 +8458,9 @@
       <c r="R80" s="4" t="n">
         <v>0.3688</v>
       </c>
+      <c r="S80" s="4" t="n">
+        <v>0.3688</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -8110,6 +8521,9 @@
       <c r="R81" s="4" t="n">
         <v>0.0941</v>
       </c>
+      <c r="S81" s="4" t="n">
+        <v>0.0941</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -8170,6 +8584,9 @@
       <c r="R82" s="4" t="n">
         <v>0.0307</v>
       </c>
+      <c r="S82" s="4" t="n">
+        <v>0.0307</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -8227,6 +8644,9 @@
       <c r="R83" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="S83" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -8278,6 +8698,9 @@
       <c r="R84" s="4" t="n">
         <v>0.4907</v>
       </c>
+      <c r="S84" s="4" t="n">
+        <v>0.4907</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -8320,6 +8743,9 @@
       <c r="R85" s="4" t="n">
         <v>0.0044</v>
       </c>
+      <c r="S85" s="4" t="n">
+        <v>0.0044</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -8388,6 +8814,10 @@
         <f>SUM(R80:R85)</f>
         <v/>
       </c>
+      <c r="S86" s="5">
+        <f>SUM(S80:S85)</f>
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -8448,6 +8878,9 @@
       <c r="R87" s="4" t="n">
         <v>0.0072</v>
       </c>
+      <c r="S87" s="4" t="n">
+        <v>0.0072</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -8508,6 +8941,9 @@
       <c r="R88" s="4" t="n">
         <v>0.0075</v>
       </c>
+      <c r="S88" s="4" t="n">
+        <v>0.0075</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -8568,6 +9004,9 @@
       <c r="R89" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="S89" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -8628,6 +9067,9 @@
       <c r="R90" s="4" t="n">
         <v>0.0191</v>
       </c>
+      <c r="S90" s="4" t="n">
+        <v>0.0191</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -8688,6 +9130,9 @@
       <c r="R91" s="4" t="n">
         <v>0.0151</v>
       </c>
+      <c r="S91" s="4" t="n">
+        <v>0.0151</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -8748,6 +9193,9 @@
       <c r="R92" s="4" t="n">
         <v>0.3604</v>
       </c>
+      <c r="S92" s="4" t="n">
+        <v>0.3604</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -8805,6 +9253,9 @@
       <c r="R93" s="4" t="n">
         <v>0.5844</v>
       </c>
+      <c r="S93" s="4" t="n">
+        <v>0.5844</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -8862,6 +9313,9 @@
       <c r="R94" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="S94" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -8910,6 +9364,9 @@
       <c r="R95" s="4" t="n">
         <v>0.0062</v>
       </c>
+      <c r="S95" s="4" t="n">
+        <v>0.0062</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -8976,6 +9433,10 @@
       </c>
       <c r="R96" s="5">
         <f>SUM(R87:R95)</f>
+        <v/>
+      </c>
+      <c r="S96" s="5">
+        <f>SUM(S87:S95)</f>
         <v/>
       </c>
     </row>
@@ -9316,7 +9777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E126"/>
+  <dimension ref="A1:E129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9431,10 +9892,10 @@
         <v>0.6</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.29</v>
+        <v>0.33</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>483.3333333333334</v>
+        <v>549.9999999999999</v>
       </c>
     </row>
     <row r="12">
@@ -9487,17 +9948,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>334.15</v>
+        <v>96.13</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>474.3800000000001</v>
+        <v>124.07</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>1419.661828520126</v>
+        <v>1290.64808072402</v>
       </c>
     </row>
     <row r="15">
@@ -9508,17 +9969,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>14.25</v>
+        <v>334.15</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>52.25</v>
+        <v>474.3800000000001</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>3666.666666666667</v>
+        <v>1419.661828520126</v>
       </c>
     </row>
     <row r="16">
@@ -9529,17 +9990,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>24195.36999999999</v>
+        <v>14.25</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>39510.46</v>
+        <v>52.25</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1632.976061122439</v>
+        <v>3666.666666666667</v>
       </c>
     </row>
     <row r="17">
@@ -9550,38 +10011,38 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>2290.17</v>
+        <v>25605.86999999999</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>1767.74</v>
+        <v>42000.09</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>771.8815633773913</v>
+        <v>1640.252410872976</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Steel Plate</t>
+          <t>Hot-Rolled Sheet</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>1230.35</v>
+        <v>2290.17</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>1361.29</v>
+        <v>1767.74</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1106.425001015971</v>
+        <v>771.8815633773913</v>
       </c>
     </row>
     <row r="19">
@@ -9592,17 +10053,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0.23</v>
+        <v>1230.35</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>0.46</v>
+        <v>1361.29</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>2000</v>
+        <v>1106.425001015971</v>
       </c>
     </row>
     <row r="20">
@@ -9613,17 +10074,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>386.7500000000001</v>
+        <v>0.23</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>411.76</v>
+        <v>0.46</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>1064.667097608274</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="21">
@@ -9634,17 +10095,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>933.4</v>
+        <v>386.7500000000001</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>2829.57</v>
+        <v>411.76</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>3031.465609599315</v>
+        <v>1064.667097608274</v>
       </c>
     </row>
     <row r="22">
@@ -9655,17 +10116,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>5523.079999999999</v>
+        <v>1310.56</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>7355.33</v>
+        <v>4407.190000000001</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>1331.744244153625</v>
+        <v>3362.829630081798</v>
       </c>
     </row>
     <row r="23">
@@ -9676,17 +10137,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>310.93</v>
+        <v>5523.079999999999</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>628.1899999999999</v>
+        <v>7355.33</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>2020.358279998713</v>
+        <v>1331.744244153625</v>
       </c>
     </row>
     <row r="24">
@@ -9697,17 +10158,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>2.07</v>
+        <v>310.93</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>6.74</v>
+        <v>628.1899999999999</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>3256.038647342995</v>
+        <v>2020.358279998713</v>
       </c>
     </row>
     <row r="25">
@@ -9718,17 +10179,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C25" s="6" t="n">
-        <v>16706.3</v>
+        <v>2.07</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>19071.87</v>
+        <v>6.74</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>1141.597481189731</v>
+        <v>3256.038647342995</v>
       </c>
     </row>
     <row r="26">
@@ -9739,17 +10200,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>8999.279999999999</v>
+        <v>16706.3</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>10665.01</v>
+        <v>19071.87</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>1185.095918784614</v>
+        <v>1141.597481189731</v>
       </c>
     </row>
     <row r="27">
@@ -9760,17 +10221,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>332.66</v>
+        <v>8999.279999999999</v>
       </c>
       <c r="D27" s="6" t="n">
-        <v>691.7199999999999</v>
+        <v>10665.01</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>2079.360307821799</v>
+        <v>1185.095918784614</v>
       </c>
     </row>
     <row r="28">
@@ -9781,17 +10242,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>24.22</v>
+        <v>418.3699999999999</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>45.67</v>
+        <v>887.7199999999998</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>1885.631709331131</v>
+        <v>2121.853861414537</v>
       </c>
     </row>
     <row r="29">
@@ -9802,17 +10263,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>4.109999999999999</v>
+        <v>24.22</v>
       </c>
       <c r="D29" s="6" t="n">
-        <v>9.25</v>
+        <v>45.67</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>2250.608272506083</v>
+        <v>1885.631709331131</v>
       </c>
     </row>
     <row r="30">
@@ -9823,17 +10284,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>20.48</v>
+        <v>4.109999999999999</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>86.87</v>
+        <v>9.25</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>4241.69921875</v>
+        <v>2250.608272506083</v>
       </c>
     </row>
     <row r="31">
@@ -9844,17 +10305,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C31" s="6" t="n">
-        <v>633.6200000000001</v>
+        <v>28.8</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>586.28</v>
+        <v>143.07</v>
       </c>
       <c r="E31" s="6" t="n">
-        <v>925.2864492913732</v>
+        <v>4967.708333333333</v>
       </c>
     </row>
     <row r="32">
@@ -9865,38 +10326,38 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>14600.66</v>
+        <v>633.6200000000001</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>27810.02000000001</v>
+        <v>586.28</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>1904.709787091817</v>
+        <v>925.2864492913732</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Cold-Rolled Sheet</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C33" s="6" t="n">
-        <v>365.06</v>
+        <v>15740.88</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>355.54</v>
+        <v>30498.32</v>
       </c>
       <c r="E33" s="6" t="n">
-        <v>973.9220949980823</v>
+        <v>1937.523188030148</v>
       </c>
     </row>
     <row r="34">
@@ -9907,17 +10368,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C34" s="6" t="n">
-        <v>0.51</v>
+        <v>365.06</v>
       </c>
       <c r="D34" s="6" t="n">
-        <v>0.67</v>
+        <v>355.54</v>
       </c>
       <c r="E34" s="6" t="n">
-        <v>1313.725490196078</v>
+        <v>973.9220949980823</v>
       </c>
     </row>
     <row r="35">
@@ -9928,17 +10389,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C35" s="6" t="n">
-        <v>47.69</v>
+        <v>0.51</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>78.28000000000002</v>
+        <v>0.67</v>
       </c>
       <c r="E35" s="6" t="n">
-        <v>1641.434262948208</v>
+        <v>1313.725490196078</v>
       </c>
     </row>
     <row r="36">
@@ -9949,17 +10410,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C36" s="6" t="n">
-        <v>38.06</v>
+        <v>51.71</v>
       </c>
       <c r="D36" s="6" t="n">
-        <v>89.77</v>
+        <v>89.29000000000001</v>
       </c>
       <c r="E36" s="6" t="n">
-        <v>2358.644245927483</v>
+        <v>1726.745310384839</v>
       </c>
     </row>
     <row r="37">
@@ -9970,17 +10431,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C37" s="6" t="n">
-        <v>0.66</v>
+        <v>39.9</v>
       </c>
       <c r="D37" s="6" t="n">
-        <v>3.77</v>
+        <v>94.75</v>
       </c>
       <c r="E37" s="6" t="n">
-        <v>5712.121212121212</v>
+        <v>2374.68671679198</v>
       </c>
     </row>
     <row r="38">
@@ -10121,13 +10582,13 @@
         </is>
       </c>
       <c r="C44" s="6" t="n">
-        <v>16839.71</v>
+        <v>17716.53</v>
       </c>
       <c r="D44" s="6" t="n">
-        <v>29831.54000000001</v>
+        <v>31422.85000000001</v>
       </c>
       <c r="E44" s="6" t="n">
-        <v>1771.499627962715</v>
+        <v>1773.645855029174</v>
       </c>
     </row>
     <row r="45">
@@ -10226,13 +10687,13 @@
         </is>
       </c>
       <c r="C49" s="6" t="n">
-        <v>1259.09</v>
+        <v>1496.4</v>
       </c>
       <c r="D49" s="6" t="n">
-        <v>1728.48</v>
+        <v>2012.33</v>
       </c>
       <c r="E49" s="6" t="n">
-        <v>1372.800991192051</v>
+        <v>1344.780807270783</v>
       </c>
     </row>
     <row r="50">
@@ -10331,13 +10792,13 @@
         </is>
       </c>
       <c r="C54" s="6" t="n">
-        <v>3412.5</v>
+        <v>3408.78</v>
       </c>
       <c r="D54" s="6" t="n">
-        <v>6849.4</v>
+        <v>6825.16</v>
       </c>
       <c r="E54" s="6" t="n">
-        <v>2007.150183150183</v>
+        <v>2002.229536667077</v>
       </c>
     </row>
     <row r="55">
@@ -10352,13 +10813,13 @@
         </is>
       </c>
       <c r="C55" s="6" t="n">
-        <v>13.67</v>
+        <v>14.67</v>
       </c>
       <c r="D55" s="6" t="n">
-        <v>39.3</v>
+        <v>42.02</v>
       </c>
       <c r="E55" s="6" t="n">
-        <v>2874.908558888077</v>
+        <v>2864.349011588276</v>
       </c>
     </row>
     <row r="56">
@@ -10415,13 +10876,13 @@
         </is>
       </c>
       <c r="C58" s="6" t="n">
-        <v>1272.37</v>
+        <v>1369.53</v>
       </c>
       <c r="D58" s="6" t="n">
-        <v>2653.31</v>
+        <v>2859.07</v>
       </c>
       <c r="E58" s="6" t="n">
-        <v>2085.328953056108</v>
+        <v>2087.628602513271</v>
       </c>
     </row>
     <row r="59">
@@ -10436,13 +10897,13 @@
         </is>
       </c>
       <c r="C59" s="6" t="n">
-        <v>11307.92</v>
+        <v>11896.83</v>
       </c>
       <c r="D59" s="6" t="n">
-        <v>17502.81</v>
+        <v>18283.49</v>
       </c>
       <c r="E59" s="6" t="n">
-        <v>1547.83638370275</v>
+        <v>1536.837123838871</v>
       </c>
     </row>
     <row r="60">
@@ -10478,13 +10939,13 @@
         </is>
       </c>
       <c r="C61" s="6" t="n">
-        <v>1152.11</v>
+        <v>1201.99</v>
       </c>
       <c r="D61" s="6" t="n">
-        <v>2691.05</v>
+        <v>2803.9</v>
       </c>
       <c r="E61" s="6" t="n">
-        <v>2335.757870342241</v>
+        <v>2332.714914433564</v>
       </c>
     </row>
     <row r="62">
@@ -10730,13 +11191,13 @@
         </is>
       </c>
       <c r="C73" s="6" t="n">
-        <v>44749.39999999999</v>
+        <v>49058.38999999999</v>
       </c>
       <c r="D73" s="6" t="n">
-        <v>86060.23</v>
+        <v>95289.64999999999</v>
       </c>
       <c r="E73" s="6" t="n">
-        <v>1923.15941666257</v>
+        <v>1942.372140626711</v>
       </c>
     </row>
     <row r="74">
@@ -10877,13 +11338,13 @@
         </is>
       </c>
       <c r="C80" s="6" t="n">
-        <v>26154.26</v>
+        <v>27783.28</v>
       </c>
       <c r="D80" s="6" t="n">
-        <v>28633.86</v>
+        <v>30880.05</v>
       </c>
       <c r="E80" s="6" t="n">
-        <v>1094.806735116956</v>
+        <v>1111.461641678016</v>
       </c>
     </row>
     <row r="81">
@@ -10940,13 +11401,13 @@
         </is>
       </c>
       <c r="C83" s="6" t="n">
-        <v>1499.67</v>
+        <v>1561.01</v>
       </c>
       <c r="D83" s="6" t="n">
-        <v>2855.9</v>
+        <v>2929.9</v>
       </c>
       <c r="E83" s="6" t="n">
-        <v>1904.352290837317</v>
+        <v>1876.925836477665</v>
       </c>
     </row>
     <row r="84">
@@ -10957,17 +11418,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Afghanistan</t>
         </is>
       </c>
       <c r="C84" s="6" t="n">
-        <v>800.48</v>
+        <v>0.09</v>
       </c>
       <c r="D84" s="6" t="n">
-        <v>794.91</v>
+        <v>0.06</v>
       </c>
       <c r="E84" s="6" t="n">
-        <v>993.0416749950029</v>
+        <v>666.6666666666667</v>
       </c>
     </row>
     <row r="85">
@@ -10978,17 +11439,17 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C85" s="6" t="n">
-        <v>204.64</v>
+        <v>802.0800000000002</v>
       </c>
       <c r="D85" s="6" t="n">
-        <v>218.94</v>
+        <v>799.3</v>
       </c>
       <c r="E85" s="6" t="n">
-        <v>1069.87881157154</v>
+        <v>996.534011569918</v>
       </c>
     </row>
     <row r="86">
@@ -10999,17 +11460,17 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C86" s="6" t="n">
-        <v>1.12</v>
+        <v>499.3899999999999</v>
       </c>
       <c r="D86" s="6" t="n">
-        <v>4.18</v>
+        <v>527.9599999999999</v>
       </c>
       <c r="E86" s="6" t="n">
-        <v>3732.142857142857</v>
+        <v>1057.20979595106</v>
       </c>
     </row>
     <row r="87">
@@ -11020,17 +11481,17 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="C87" s="6" t="n">
-        <v>19.32</v>
+        <v>1.12</v>
       </c>
       <c r="D87" s="6" t="n">
-        <v>39.73</v>
+        <v>4.18</v>
       </c>
       <c r="E87" s="6" t="n">
-        <v>2056.418219461698</v>
+        <v>3732.142857142857</v>
       </c>
     </row>
     <row r="88">
@@ -11041,17 +11502,17 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="C88" s="6" t="n">
-        <v>585.71</v>
+        <v>19.32</v>
       </c>
       <c r="D88" s="6" t="n">
-        <v>916.8199999999999</v>
+        <v>39.73</v>
       </c>
       <c r="E88" s="6" t="n">
-        <v>1565.313892540677</v>
+        <v>2056.418219461698</v>
       </c>
     </row>
     <row r="89">
@@ -11062,17 +11523,17 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C89" s="6" t="n">
-        <v>5.99</v>
+        <v>585.71</v>
       </c>
       <c r="D89" s="6" t="n">
-        <v>8.460000000000001</v>
+        <v>916.8199999999999</v>
       </c>
       <c r="E89" s="6" t="n">
-        <v>1412.353923205342</v>
+        <v>1565.313892540677</v>
       </c>
     </row>
     <row r="90">
@@ -11083,17 +11544,17 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C90" s="6" t="n">
-        <v>41.26000000000001</v>
+        <v>5.99</v>
       </c>
       <c r="D90" s="6" t="n">
-        <v>112.53</v>
+        <v>8.460000000000001</v>
       </c>
       <c r="E90" s="6" t="n">
-        <v>2727.338826951042</v>
+        <v>1412.353923205342</v>
       </c>
     </row>
     <row r="91">
@@ -11104,17 +11565,17 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C91" s="6" t="n">
-        <v>9.379999999999999</v>
+        <v>41.26000000000001</v>
       </c>
       <c r="D91" s="6" t="n">
-        <v>19.62</v>
+        <v>112.53</v>
       </c>
       <c r="E91" s="6" t="n">
-        <v>2091.684434968017</v>
+        <v>2727.338826951042</v>
       </c>
     </row>
     <row r="92">
@@ -11125,17 +11586,17 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C92" s="6" t="n">
-        <v>926.85</v>
+        <v>12.29</v>
       </c>
       <c r="D92" s="6" t="n">
-        <v>1259.8</v>
+        <v>26.13</v>
       </c>
       <c r="E92" s="6" t="n">
-        <v>1359.227490964018</v>
+        <v>2126.118795768918</v>
       </c>
     </row>
     <row r="93">
@@ -11146,17 +11607,17 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C93" s="6" t="n">
-        <v>1.57</v>
+        <v>941.04</v>
       </c>
       <c r="D93" s="6" t="n">
-        <v>7.23</v>
+        <v>1278.49</v>
       </c>
       <c r="E93" s="6" t="n">
-        <v>4605.095541401273</v>
+        <v>1358.592620930035</v>
       </c>
     </row>
     <row r="94">
@@ -11167,17 +11628,17 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="C94" s="6" t="n">
-        <v>25.4</v>
+        <v>1.57</v>
       </c>
       <c r="D94" s="6" t="n">
-        <v>49.81</v>
+        <v>7.23</v>
       </c>
       <c r="E94" s="6" t="n">
-        <v>1961.023622047244</v>
+        <v>4605.095541401273</v>
       </c>
     </row>
     <row r="95">
@@ -11188,17 +11649,17 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C95" s="6" t="n">
-        <v>2160.85</v>
+        <v>25.4</v>
       </c>
       <c r="D95" s="6" t="n">
-        <v>2077.93</v>
+        <v>49.81</v>
       </c>
       <c r="E95" s="6" t="n">
-        <v>961.6262119073514</v>
+        <v>1961.023622047244</v>
       </c>
     </row>
     <row r="96">
@@ -11209,17 +11670,17 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C96" s="6" t="n">
-        <v>1383.67</v>
+        <v>2160.85</v>
       </c>
       <c r="D96" s="6" t="n">
-        <v>1326.04</v>
+        <v>2077.93</v>
       </c>
       <c r="E96" s="6" t="n">
-        <v>958.3498955675847</v>
+        <v>961.6262119073514</v>
       </c>
     </row>
     <row r="97">
@@ -11230,17 +11691,17 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C97" s="6" t="n">
-        <v>10.8</v>
+        <v>1383.67</v>
       </c>
       <c r="D97" s="6" t="n">
-        <v>47.44</v>
+        <v>1326.04</v>
       </c>
       <c r="E97" s="6" t="n">
-        <v>4392.592592592593</v>
+        <v>958.3498955675847</v>
       </c>
     </row>
     <row r="98">
@@ -11251,38 +11712,38 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C98" s="6" t="n">
-        <v>2847.08</v>
+        <v>10.8</v>
       </c>
       <c r="D98" s="6" t="n">
-        <v>5859.5</v>
+        <v>47.44</v>
       </c>
       <c r="E98" s="6" t="n">
-        <v>2058.073534990235</v>
+        <v>4392.592592592593</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C99" s="6" t="n">
-        <v>72.08</v>
+        <v>3067.780000000001</v>
       </c>
       <c r="D99" s="6" t="n">
-        <v>95.73999999999999</v>
+        <v>6286.139999999998</v>
       </c>
       <c r="E99" s="6" t="n">
-        <v>1328.246392896781</v>
+        <v>2049.08435415838</v>
       </c>
     </row>
     <row r="100">
@@ -11293,17 +11754,17 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C100" s="6" t="n">
-        <v>1147.2</v>
+        <v>72.08</v>
       </c>
       <c r="D100" s="6" t="n">
-        <v>1518.63</v>
+        <v>95.73999999999999</v>
       </c>
       <c r="E100" s="6" t="n">
-        <v>1323.770920502092</v>
+        <v>1328.246392896781</v>
       </c>
     </row>
     <row r="101">
@@ -11314,17 +11775,17 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C101" s="6" t="n">
-        <v>5.78</v>
+        <v>1147.2</v>
       </c>
       <c r="D101" s="6" t="n">
-        <v>10.29</v>
+        <v>1518.63</v>
       </c>
       <c r="E101" s="6" t="n">
-        <v>1780.276816608997</v>
+        <v>1323.770920502092</v>
       </c>
     </row>
     <row r="102">
@@ -11335,17 +11796,17 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C102" s="6" t="n">
-        <v>8086.389999999999</v>
+        <v>23.12</v>
       </c>
       <c r="D102" s="6" t="n">
-        <v>11816.42</v>
+        <v>38.08</v>
       </c>
       <c r="E102" s="6" t="n">
-        <v>1461.272582697595</v>
+        <v>1647.058823529412</v>
       </c>
     </row>
     <row r="103">
@@ -11356,17 +11817,17 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C103" s="6" t="n">
-        <v>8103.91</v>
+        <v>8087.369999999999</v>
       </c>
       <c r="D103" s="6" t="n">
-        <v>5812.44</v>
+        <v>11820.87</v>
       </c>
       <c r="E103" s="6" t="n">
-        <v>717.2389624267792</v>
+        <v>1461.645751338198</v>
       </c>
     </row>
     <row r="104">
@@ -11377,17 +11838,17 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C104" s="6" t="n">
-        <v>256.94</v>
+        <v>8103.91</v>
       </c>
       <c r="D104" s="6" t="n">
-        <v>334.05</v>
+        <v>5812.44</v>
       </c>
       <c r="E104" s="6" t="n">
-        <v>1300.108974857943</v>
+        <v>717.2389624267792</v>
       </c>
     </row>
     <row r="105">
@@ -11398,17 +11859,17 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C105" s="6" t="n">
-        <v>506.71</v>
+        <v>256.94</v>
       </c>
       <c r="D105" s="6" t="n">
-        <v>617.79</v>
+        <v>334.05</v>
       </c>
       <c r="E105" s="6" t="n">
-        <v>1219.218093189398</v>
+        <v>1300.108974857943</v>
       </c>
     </row>
     <row r="106">
@@ -11419,17 +11880,17 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C106" s="6" t="n">
-        <v>288.96</v>
+        <v>506.71</v>
       </c>
       <c r="D106" s="6" t="n">
-        <v>328.76</v>
+        <v>617.79</v>
       </c>
       <c r="E106" s="6" t="n">
-        <v>1137.735326688815</v>
+        <v>1219.218093189398</v>
       </c>
     </row>
     <row r="107">
@@ -11440,38 +11901,38 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C107" s="6" t="n">
-        <v>7583.13</v>
+        <v>288.96</v>
       </c>
       <c r="D107" s="6" t="n">
-        <v>10717.53</v>
+        <v>328.76</v>
       </c>
       <c r="E107" s="6" t="n">
-        <v>1413.338555451377</v>
+        <v>1137.735326688815</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C108" s="6" t="n">
-        <v>1650.37</v>
+        <v>8332.24</v>
       </c>
       <c r="D108" s="6" t="n">
-        <v>1440.99</v>
+        <v>11757.15</v>
       </c>
       <c r="E108" s="6" t="n">
-        <v>873.131479607603</v>
+        <v>1411.043128858506</v>
       </c>
     </row>
     <row r="109">
@@ -11482,17 +11943,17 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C109" s="6" t="n">
-        <v>0.17</v>
+        <v>1650.37</v>
       </c>
       <c r="D109" s="6" t="n">
-        <v>0.63</v>
+        <v>1440.99</v>
       </c>
       <c r="E109" s="6" t="n">
-        <v>3705.882352941176</v>
+        <v>873.131479607603</v>
       </c>
     </row>
     <row r="110">
@@ -11503,17 +11964,17 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="C110" s="6" t="n">
-        <v>579.89</v>
+        <v>2.54</v>
       </c>
       <c r="D110" s="6" t="n">
-        <v>1884.71</v>
+        <v>15.79</v>
       </c>
       <c r="E110" s="6" t="n">
-        <v>3250.11640138647</v>
+        <v>6216.535433070866</v>
       </c>
     </row>
     <row r="111">
@@ -11524,17 +11985,17 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C111" s="6" t="n">
-        <v>55.17</v>
+        <v>0.17</v>
       </c>
       <c r="D111" s="6" t="n">
-        <v>81.37</v>
+        <v>0.63</v>
       </c>
       <c r="E111" s="6" t="n">
-        <v>1474.89577669023</v>
+        <v>3705.882352941176</v>
       </c>
     </row>
     <row r="112">
@@ -11545,17 +12006,17 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C112" s="6" t="n">
-        <v>35.69</v>
+        <v>595.5700000000001</v>
       </c>
       <c r="D112" s="6" t="n">
-        <v>130.5</v>
+        <v>1933.18</v>
       </c>
       <c r="E112" s="6" t="n">
-        <v>3656.486410759317</v>
+        <v>3245.932468055812</v>
       </c>
     </row>
     <row r="113">
@@ -11566,17 +12027,17 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C113" s="6" t="n">
-        <v>4717.8</v>
+        <v>109.98</v>
       </c>
       <c r="D113" s="6" t="n">
-        <v>5541.98</v>
+        <v>161.39</v>
       </c>
       <c r="E113" s="6" t="n">
-        <v>1174.695832803425</v>
+        <v>1467.448627023095</v>
       </c>
     </row>
     <row r="114">
@@ -11587,17 +12048,17 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C114" s="6" t="n">
-        <v>65266.67</v>
+        <v>49.54</v>
       </c>
       <c r="D114" s="6" t="n">
-        <v>64435.03000000001</v>
+        <v>200.53</v>
       </c>
       <c r="E114" s="6" t="n">
-        <v>987.2578147467921</v>
+        <v>4047.840129188535</v>
       </c>
     </row>
     <row r="115">
@@ -11608,17 +12069,17 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C115" s="6" t="n">
-        <v>6582.36</v>
+        <v>4717.8</v>
       </c>
       <c r="D115" s="6" t="n">
-        <v>10977.15</v>
+        <v>5541.98</v>
       </c>
       <c r="E115" s="6" t="n">
-        <v>1667.661750496782</v>
+        <v>1174.695832803425</v>
       </c>
     </row>
     <row r="116">
@@ -11629,17 +12090,17 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C116" s="6" t="n">
-        <v>10501.68</v>
+        <v>66405.70999999999</v>
       </c>
       <c r="D116" s="6" t="n">
-        <v>14662.98</v>
+        <v>65757.26000000001</v>
       </c>
       <c r="E116" s="6" t="n">
-        <v>1396.250885572594</v>
+        <v>990.2350264758861</v>
       </c>
     </row>
     <row r="117">
@@ -11650,17 +12111,17 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Luxembourg</t>
         </is>
       </c>
       <c r="C117" s="6" t="n">
-        <v>0.96</v>
+        <v>6582.36</v>
       </c>
       <c r="D117" s="6" t="n">
-        <v>3.83</v>
+        <v>10977.15</v>
       </c>
       <c r="E117" s="6" t="n">
-        <v>3989.583333333333</v>
+        <v>1667.661750496782</v>
       </c>
     </row>
     <row r="118">
@@ -11671,17 +12132,17 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C118" s="6" t="n">
-        <v>8957.370000000001</v>
+        <v>11678.49</v>
       </c>
       <c r="D118" s="6" t="n">
-        <v>9710.829999999998</v>
+        <v>16361.47</v>
       </c>
       <c r="E118" s="6" t="n">
-        <v>1084.116208217367</v>
+        <v>1400.991909056736</v>
       </c>
     </row>
     <row r="119">
@@ -11692,17 +12153,17 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Oman</t>
         </is>
       </c>
       <c r="C119" s="6" t="n">
-        <v>0.12</v>
+        <v>50.34</v>
       </c>
       <c r="D119" s="6" t="n">
-        <v>0.59</v>
+        <v>42.71</v>
       </c>
       <c r="E119" s="6" t="n">
-        <v>4916.666666666667</v>
+        <v>848.4306714342471</v>
       </c>
     </row>
     <row r="120">
@@ -11713,17 +12174,17 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C120" s="6" t="n">
-        <v>1180.28</v>
+        <v>1.82</v>
       </c>
       <c r="D120" s="6" t="n">
-        <v>1132.5</v>
+        <v>7.220000000000001</v>
       </c>
       <c r="E120" s="6" t="n">
-        <v>959.5180804554851</v>
+        <v>3967.032967032968</v>
       </c>
     </row>
     <row r="121">
@@ -11734,17 +12195,17 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C121" s="6" t="n">
-        <v>6378.700000000001</v>
+        <v>8998.390000000001</v>
       </c>
       <c r="D121" s="6" t="n">
-        <v>5627.59</v>
+        <v>9922.479999999998</v>
       </c>
       <c r="E121" s="6" t="n">
-        <v>882.2471663505102</v>
+        <v>1102.695037667849</v>
       </c>
     </row>
     <row r="122">
@@ -11755,17 +12216,17 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C122" s="6" t="n">
-        <v>3250.889999999999</v>
+        <v>0.12</v>
       </c>
       <c r="D122" s="6" t="n">
-        <v>4577.62</v>
+        <v>0.59</v>
       </c>
       <c r="E122" s="6" t="n">
-        <v>1408.112855248871</v>
+        <v>4916.666666666667</v>
       </c>
     </row>
     <row r="123">
@@ -11776,17 +12237,17 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C123" s="6" t="n">
-        <v>7469.389999999999</v>
+        <v>1180.28</v>
       </c>
       <c r="D123" s="6" t="n">
-        <v>7839.33</v>
+        <v>1132.5</v>
       </c>
       <c r="E123" s="6" t="n">
-        <v>1049.527471453492</v>
+        <v>959.5180804554851</v>
       </c>
     </row>
     <row r="124">
@@ -11797,17 +12258,17 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C124" s="6" t="n">
-        <v>10379.11</v>
+        <v>6578.27</v>
       </c>
       <c r="D124" s="6" t="n">
-        <v>12309.48</v>
+        <v>5806.56</v>
       </c>
       <c r="E124" s="6" t="n">
-        <v>1185.986081658254</v>
+        <v>882.6880015566402</v>
       </c>
     </row>
     <row r="125">
@@ -11818,17 +12279,17 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C125" s="6" t="n">
-        <v>15626.29</v>
+        <v>3254.849999999999</v>
       </c>
       <c r="D125" s="6" t="n">
-        <v>38809.40000000001</v>
+        <v>4593.94</v>
       </c>
       <c r="E125" s="6" t="n">
-        <v>2483.59655426848</v>
+        <v>1411.413736424106</v>
       </c>
     </row>
     <row r="126">
@@ -11839,16 +12300,79 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="C126" s="6" t="n">
+        <v>7469.389999999999</v>
+      </c>
+      <c r="D126" s="6" t="n">
+        <v>7839.33</v>
+      </c>
+      <c r="E126" s="6" t="n">
+        <v>1049.527471453492</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C127" s="6" t="n">
+        <v>10917.07</v>
+      </c>
+      <c r="D127" s="6" t="n">
+        <v>12971.43</v>
+      </c>
+      <c r="E127" s="6" t="n">
+        <v>1188.178696298549</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C128" s="6" t="n">
+        <v>17052.90000000001</v>
+      </c>
+      <c r="D128" s="6" t="n">
+        <v>42309.49000000001</v>
+      </c>
+      <c r="E128" s="6" t="n">
+        <v>2481.073013974163</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
           <t>Vietnam</t>
         </is>
       </c>
-      <c r="C126" s="6" t="n">
+      <c r="C129" s="6" t="n">
         <v>345.42</v>
       </c>
-      <c r="D126" s="6" t="n">
+      <c r="D129" s="6" t="n">
         <v>331.78</v>
       </c>
-      <c r="E126" s="6" t="n">
+      <c r="E129" s="6" t="n">
         <v>960.51184065775</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Weekly TRQ update 2026-07-06
</commit_message>
<xml_diff>
--- a/data/canada_trq_tracker.xlsx
+++ b/data/canada_trq_tracker.xlsx
@@ -12390,7 +12390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12421,7 +12421,12 @@
           <t>June 30 2026</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>July 6 2026</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
@@ -12447,6 +12452,9 @@
       <c r="E3" s="4" t="n">
         <v>0.3197</v>
       </c>
+      <c r="F3" s="4" t="n">
+        <v>0.3197</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -12456,33 +12464,37 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E4" s="5">
-        <f>SUM(E3:E3)</f>
-        <v/>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>2366700</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>0.0002</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Steel Plate</t>
+          <t>Hot-Rolled Sheet</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>China</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>5201200</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>0.209</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E5" s="5">
+        <f>SUM(E3:E4)</f>
+        <v/>
+      </c>
+      <c r="F5" s="5">
+        <f>SUM(F3:F4)</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -12493,33 +12505,40 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E6" s="5">
-        <f>SUM(E5:E5)</f>
-        <v/>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>5201200</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>0.209</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>0.2161</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Cold-Rolled Sheet</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>India</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>6168400</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>0</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E7" s="5">
+        <f>SUM(E6:E6)</f>
+        <v/>
+      </c>
+      <c r="F7" s="5">
+        <f>SUM(F6:F6)</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -12530,7 +12549,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
@@ -12540,7 +12559,10 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>0.1099</v>
+        <v>0</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -12551,7 +12573,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
@@ -12561,7 +12583,10 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.5249</v>
+        <v>0.1099</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>0.1099</v>
       </c>
     </row>
     <row r="10">
@@ -12572,18 +12597,26 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E10" s="5">
-        <f>SUM(E7:E9)</f>
-        <v/>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>6168400</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>0.5249</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>0.5249</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -12592,76 +12625,75 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>18732800</v>
+        <v>6168400</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="E11" s="4" t="n">
-        <v>0.0027</v>
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>0.0003</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>18732800</v>
+        <v>6168400</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="E12" s="4" t="n">
-        <v>0.2673</v>
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>18732800</v>
+        <v>6168400</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="E13" s="4" t="n">
-        <v>0.0069</v>
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>0.2191</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Pakistan</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="n">
-        <v>18732800</v>
-      </c>
-      <c r="D14" s="4" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="E14" s="4" t="n">
-        <v>0.2213</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E14" s="5">
+        <f>SUM(E8:E13)</f>
+        <v/>
+      </c>
+      <c r="F14" s="5">
+        <f>SUM(F8:F13)</f>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -12672,7 +12704,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
@@ -12682,7 +12714,10 @@
         <v>0.37</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>0.3697</v>
+        <v>0.0027</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>0.0027</v>
       </c>
     </row>
     <row r="16">
@@ -12693,7 +12728,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
@@ -12703,7 +12738,10 @@
         <v>0.37</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0.0289</v>
+        <v>0.2673</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>0.2673</v>
       </c>
     </row>
     <row r="17">
@@ -12714,39 +12752,50 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E17" s="5">
-        <f>SUM(E11:E16)</f>
-        <v/>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>18732800</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>0.0069</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>0.0069</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>13445100</v>
+        <v>18732800</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>0.29</v>
+        <v>0.37</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>0.2777</v>
+        <v>0.2213</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>0.2488</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -12755,19 +12804,22 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>13445100</v>
+        <v>18732800</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>0.29</v>
+        <v>0.37</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>0.0037</v>
+        <v>0.3697</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>0.3697</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -12776,40 +12828,43 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>13445100</v>
+        <v>18732800</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>0.29</v>
+        <v>0.37</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>0.2899</v>
+        <v>0.0289</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>0.0289</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>13445100</v>
+        <v>18732800</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="E21" s="4" t="n">
-        <v>0.0883</v>
+        <v>0.37</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>0.07539999999999999</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -12818,35 +12873,42 @@
         </is>
       </c>
       <c r="E22" s="5">
-        <f>SUM(E18:E21)</f>
+        <f>SUM(E15:E21)</f>
+        <v/>
+      </c>
+      <c r="F22" s="5">
+        <f>SUM(F15:F21)</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C23" s="3" t="n">
-        <v>5886100</v>
+        <v>13445100</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>0.42</v>
+        <v>0.29</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>0.1023</v>
+        <v>0.2777</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>0.2777</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -12855,61 +12917,70 @@
         </is>
       </c>
       <c r="C24" s="3" t="n">
-        <v>5886100</v>
+        <v>13445100</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>0.42</v>
+        <v>0.29</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>0.1828</v>
+        <v>0.0037</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>0.0037</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C25" s="3" t="n">
-        <v>5886100</v>
+        <v>13445100</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>0.42</v>
+        <v>0.29</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
+        <v>0.2899</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>0.2899</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E26" s="5">
-        <f>SUM(E23:E25)</f>
-        <v/>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>13445100</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>0.0883</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>0.0883</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -12917,35 +12988,43 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E27" s="5" t="n">
-        <v>0</v>
+      <c r="E27" s="5">
+        <f>SUM(E23:E26)</f>
+        <v/>
+      </c>
+      <c r="F27" s="5">
+        <f>SUM(F23:F26)</f>
+        <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C28" s="3" t="n">
-        <v>3753500</v>
+        <v>5886100</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>0.52</v>
+        <v>0.42</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>0.0218</v>
+        <v>0.1023</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>0.147</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -12954,61 +13033,72 @@
         </is>
       </c>
       <c r="C29" s="3" t="n">
-        <v>3753500</v>
+        <v>5886100</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>0.52</v>
+        <v>0.42</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>0.1828</v>
       </c>
+      <c r="F29" s="4" t="n">
+        <v>0.1862</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C30" s="3" t="n">
-        <v>3753500</v>
+        <v>5886100</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>0.52</v>
+        <v>0.42</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>0.3483</v>
+        <v>0.42</v>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>3753500</v>
+        <v>5886100</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="E31" s="4" t="n">
-        <v>0.4306</v>
+        <v>0.42</v>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>0.0009</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -13018,6 +13108,144 @@
       </c>
       <c r="E32" s="5">
         <f>SUM(E28:E31)</f>
+        <v/>
+      </c>
+      <c r="F32" s="5">
+        <f>SUM(F28:F31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="n">
+        <v>3753500</v>
+      </c>
+      <c r="D34" s="4" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>0.0218</v>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>0.0218</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="n">
+        <v>3753500</v>
+      </c>
+      <c r="D35" s="4" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>0.1828</v>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>0.1828</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>3753500</v>
+      </c>
+      <c r="D36" s="4" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>0.3483</v>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>0.3483</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>3753500</v>
+      </c>
+      <c r="D37" s="4" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>0.4306</v>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>0.4306</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E38" s="5">
+        <f>SUM(E34:E37)</f>
+        <v/>
+      </c>
+      <c r="F38" s="5">
+        <f>SUM(F34:F37)</f>
         <v/>
       </c>
     </row>
@@ -13032,7 +13260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13063,7 +13291,12 @@
           <t>June 30 2026</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>July 6 2026</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
@@ -13089,6 +13322,9 @@
       <c r="E3" s="4" t="n">
         <v>0.3165</v>
       </c>
+      <c r="F3" s="4" t="n">
+        <v>0.3165</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -13110,6 +13346,9 @@
       <c r="E4" s="4" t="n">
         <v>0.6835</v>
       </c>
+      <c r="F4" s="4" t="n">
+        <v>0.6835</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -13126,6 +13365,10 @@
         <f>SUM(E3:E4)</f>
         <v/>
       </c>
+      <c r="F5" s="5">
+        <f>SUM(F3:F4)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -13147,6 +13390,9 @@
       <c r="E6" s="4" t="n">
         <v>0.0452</v>
       </c>
+      <c r="F6" s="4" t="n">
+        <v>0.0452</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -13168,6 +13414,9 @@
       <c r="E7" s="4" t="n">
         <v>0.0233</v>
       </c>
+      <c r="F7" s="4" t="n">
+        <v>0.0248</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -13189,6 +13438,9 @@
       <c r="E8" s="4" t="n">
         <v>0.0004</v>
       </c>
+      <c r="F8" s="4" t="n">
+        <v>0.0009</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -13210,6 +13462,9 @@
       <c r="E9" s="4" t="n">
         <v>0.0008</v>
       </c>
+      <c r="F9" s="4" t="n">
+        <v>0.0008</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -13231,6 +13486,9 @@
       <c r="E10" s="4" t="n">
         <v>0.219</v>
       </c>
+      <c r="F10" s="4" t="n">
+        <v>0.2212</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -13252,6 +13510,9 @@
       <c r="E11" s="4" t="n">
         <v>0.044</v>
       </c>
+      <c r="F11" s="4" t="n">
+        <v>0.0518</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -13273,6 +13534,9 @@
       <c r="E12" s="4" t="n">
         <v>0.0053</v>
       </c>
+      <c r="F12" s="4" t="n">
+        <v>0.0053</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -13294,6 +13558,9 @@
       <c r="E13" s="4" t="n">
         <v>0.3287</v>
       </c>
+      <c r="F13" s="4" t="n">
+        <v>0.3287</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -13315,6 +13582,9 @@
       <c r="E14" s="4" t="n">
         <v>0.0005</v>
       </c>
+      <c r="F14" s="4" t="n">
+        <v>0.0005</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -13336,6 +13606,9 @@
       <c r="E15" s="4" t="n">
         <v>0.0011</v>
       </c>
+      <c r="F15" s="4" t="n">
+        <v>0.0229</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -13345,33 +13618,37 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E16" s="5">
-        <f>SUM(E6:E15)</f>
-        <v/>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>38517700</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>0.0002</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Cold-Rolled Sheet</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="n">
-        <v>2785800</v>
-      </c>
-      <c r="D17" s="4" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>0.0068</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E17" s="5">
+        <f>SUM(E6:E16)</f>
+        <v/>
+      </c>
+      <c r="F17" s="5">
+        <f>SUM(F6:F16)</f>
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -13382,7 +13659,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
@@ -13392,7 +13669,10 @@
         <v>0.35</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>0.004500000000000001</v>
+        <v>0.0068</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>0.0068</v>
       </c>
     </row>
     <row r="19">
@@ -13403,7 +13683,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
@@ -13413,7 +13693,10 @@
         <v>0.35</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>0.0175</v>
+        <v>0.004500000000000001</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>0.1068</v>
       </c>
     </row>
     <row r="20">
@@ -13424,54 +13707,61 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E20" s="5">
-        <f>SUM(E17:E19)</f>
-        <v/>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>2785800</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>0.0175</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>0.0175</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>31128200</v>
+        <v>2785800</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E21" s="4" t="n">
-        <v>0.0304</v>
+        <v>0.35</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>0.2056</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Austria</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="n">
-        <v>31128200</v>
-      </c>
-      <c r="D22" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E22" s="4" t="n">
-        <v>0.0003</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E22" s="5">
+        <f>SUM(E18:E21)</f>
+        <v/>
+      </c>
+      <c r="F22" s="5">
+        <f>SUM(F18:F21)</f>
+        <v/>
       </c>
     </row>
     <row r="23">
@@ -13482,7 +13772,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C23" s="3" t="n">
@@ -13492,7 +13782,10 @@
         <v>0.25</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>0.0001</v>
+        <v>0.0304</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>0.0304</v>
       </c>
     </row>
     <row r="24">
@@ -13503,7 +13796,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="C24" s="3" t="n">
@@ -13513,7 +13806,10 @@
         <v>0.25</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>0.0382</v>
+        <v>0.0003</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>0.0609</v>
       </c>
     </row>
     <row r="25">
@@ -13524,7 +13820,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C25" s="3" t="n">
@@ -13534,7 +13830,10 @@
         <v>0.25</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>0</v>
+        <v>0.0001</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>0.0001</v>
       </c>
     </row>
     <row r="26">
@@ -13545,7 +13844,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C26" s="3" t="n">
@@ -13555,7 +13854,10 @@
         <v>0.25</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>0.0213</v>
+        <v>0.0382</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>0.0382</v>
       </c>
     </row>
     <row r="27">
@@ -13566,196 +13868,216 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E27" s="5">
-        <f>SUM(E21:E26)</f>
-        <v/>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>31128200</v>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>0.0341</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C28" s="3" t="n">
-        <v>28710400</v>
+        <v>31128200</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>0.45</v>
+        <v>0.25</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>0.0832</v>
+        <v>0.0213</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>0.0213</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C29" s="3" t="n">
-        <v>28710400</v>
+        <v>31128200</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="E29" s="4" t="n">
-        <v>0.3459</v>
+        <v>0.25</v>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>0.0451</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E30" s="5">
-        <f>SUM(E28:E29)</f>
-        <v/>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>31128200</v>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>0.0146</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>8750300</v>
+        <v>31128200</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="E31" s="4" t="n">
-        <v>0.0025</v>
+        <v>0.25</v>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>0.0195</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="n">
-        <v>8750300</v>
-      </c>
-      <c r="D32" s="4" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="E32" s="4" t="n">
-        <v>0.2277</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E32" s="5">
+        <f>SUM(E23:E31)</f>
+        <v/>
+      </c>
+      <c r="F32" s="5">
+        <f>SUM(F23:F31)</f>
+        <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C33" s="3" t="n">
-        <v>8750300</v>
+        <v>28710400</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>0.58</v>
+        <v>0.45</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>0.1228</v>
+        <v>0.0832</v>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>0.0832</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="C34" s="3" t="n">
-        <v>8750300</v>
+        <v>28710400</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>0.58</v>
+        <v>0.45</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>0.0019</v>
+        <v>0.3459</v>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>0.3459</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C35" s="3" t="n">
-        <v>8750300</v>
+        <v>28710400</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="E35" s="4" t="n">
-        <v>0.0068</v>
+        <v>0.45</v>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>0.0007000000000000001</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="n">
-        <v>8750300</v>
-      </c>
-      <c r="D36" s="4" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="E36" s="4" t="n">
-        <v>0.0191</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E36" s="5">
+        <f>SUM(E33:E35)</f>
+        <v/>
+      </c>
+      <c r="F36" s="5">
+        <f>SUM(F33:F35)</f>
+        <v/>
       </c>
     </row>
     <row r="37">
@@ -13766,18 +14088,26 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E37" s="5">
-        <f>SUM(E31:E36)</f>
-        <v/>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>8750300</v>
+      </c>
+      <c r="D37" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>0.0025</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -13786,19 +14116,22 @@
         </is>
       </c>
       <c r="C38" s="3" t="n">
-        <v>16514800</v>
+        <v>8750300</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>0.59</v>
+        <v>0.58</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>0.0029</v>
+        <v>0.2277</v>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>0.2285</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -13807,217 +14140,455 @@
         </is>
       </c>
       <c r="C39" s="3" t="n">
-        <v>16514800</v>
+        <v>8750300</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>0.59</v>
+        <v>0.58</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>0.0339</v>
+        <v>0.1228</v>
+      </c>
+      <c r="F39" s="4" t="n">
+        <v>0.1253</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Luxembourg</t>
         </is>
       </c>
       <c r="C40" s="3" t="n">
-        <v>16514800</v>
+        <v>8750300</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>0.59</v>
+        <v>0.58</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>0.4926</v>
+        <v>0.0019</v>
+      </c>
+      <c r="F40" s="4" t="n">
+        <v>0.0019</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="C41" s="3" t="n">
-        <v>16514800</v>
+        <v>8750300</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>0.59</v>
+        <v>0.58</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.0068</v>
+      </c>
+      <c r="F41" s="4" t="n">
+        <v>0.0095</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E42" s="5">
-        <f>SUM(E38:E41)</f>
-        <v/>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="n">
+        <v>8750300</v>
+      </c>
+      <c r="D42" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="E42" s="4" t="n">
+        <v>0.0191</v>
+      </c>
+      <c r="F42" s="4" t="n">
+        <v>0.0236</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C43" s="3" t="n">
-        <v>3467600</v>
+        <v>8750300</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="E43" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.58</v>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>0.0017</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C44" s="3" t="n">
-        <v>3467600</v>
+        <v>8750300</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="E44" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.58</v>
+      </c>
+      <c r="F44" s="4" t="n">
+        <v>0.008500000000000001</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="n">
-        <v>3467600</v>
-      </c>
-      <c r="D45" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="E45" s="4" t="n">
-        <v>0.0204</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E45" s="5">
+        <f>SUM(E37:E44)</f>
+        <v/>
+      </c>
+      <c r="F45" s="5">
+        <f>SUM(F37:F44)</f>
+        <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C46" s="3" t="n">
-        <v>3467600</v>
+        <v>16514800</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.59</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
+        <v>0.0029</v>
+      </c>
+      <c r="F46" s="4" t="n">
+        <v>0.0029</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C47" s="3" t="n">
-        <v>3467600</v>
+        <v>16514800</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.59</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.0339</v>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>0.0339</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C48" s="3" t="n">
-        <v>3467600</v>
+        <v>16514800</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.59</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>0.1798</v>
+        <v>0.4926</v>
+      </c>
+      <c r="F48" s="4" t="n">
+        <v>0.4926</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="n">
+        <v>16514800</v>
+      </c>
+      <c r="D49" s="4" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="E49" s="4" t="n">
+        <v>0.008800000000000001</v>
+      </c>
+      <c r="F49" s="4" t="n">
+        <v>0.0146</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E50" s="5">
+        <f>SUM(E46:E49)</f>
+        <v/>
+      </c>
+      <c r="F50" s="5">
+        <f>SUM(F46:F49)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>Structural Steel</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D51" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E51" s="4" t="n">
+        <v>0.0004</v>
+      </c>
+      <c r="F51" s="4" t="n">
+        <v>0.0021</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D52" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E52" s="4" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="F52" s="4" t="n">
+        <v>0.0032</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D53" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E53" s="4" t="n">
+        <v>0.0204</v>
+      </c>
+      <c r="F53" s="4" t="n">
+        <v>0.0204</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Korea, Republic of</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D54" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E54" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="F54" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D55" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E55" s="4" t="n">
+        <v>0.0004</v>
+      </c>
+      <c r="F55" s="4" t="n">
+        <v>0.0004</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D56" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E56" s="4" t="n">
+        <v>0.1798</v>
+      </c>
+      <c r="F56" s="4" t="n">
+        <v>0.1798</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Luxembourg</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D57" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="F57" s="4" t="n">
+        <v>0.0012</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E49" s="5">
-        <f>SUM(E43:E48)</f>
+      <c r="E58" s="5">
+        <f>SUM(E51:E57)</f>
+        <v/>
+      </c>
+      <c r="F58" s="5">
+        <f>SUM(F51:F57)</f>
         <v/>
       </c>
     </row>
@@ -14032,7 +14603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14111,11 +14682,193 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>262.45</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>479.86</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>1828.386359306535</v>
+      </c>
+    </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>B1 data not available for the matching calendar quarter.</t>
-        </is>
+          <t>Cold-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>89.86</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>161.13</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>1793.122635210327</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Korea, Republic of</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>23.06</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>39.55</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>1715.091066782307</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>295.92</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>772.3299999999999</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>2609.92835901595</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>27.64</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>32.04</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>1159.189580318379</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>324.94</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>485.55</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>1494.275866313781</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>34.35</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>123.64</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>3599.417758369723</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Weekly TRQ update 2026-07-13
</commit_message>
<xml_diff>
--- a/data/canada_trq_tracker.xlsx
+++ b/data/canada_trq_tracker.xlsx
@@ -12390,7 +12390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12426,7 +12426,12 @@
           <t>July 6 2026</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>July 13 2026</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
@@ -12455,6 +12460,9 @@
       <c r="F3" s="4" t="n">
         <v>0.3197</v>
       </c>
+      <c r="G3" s="4" t="n">
+        <v>0.3197</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -12476,6 +12484,9 @@
       <c r="F4" s="4" t="n">
         <v>0.0002</v>
       </c>
+      <c r="G4" s="4" t="n">
+        <v>0.005600000000000001</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -12496,6 +12507,10 @@
         <f>SUM(F3:F4)</f>
         <v/>
       </c>
+      <c r="G5" s="5">
+        <f>SUM(G3:G4)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -12520,6 +12535,9 @@
       <c r="F6" s="4" t="n">
         <v>0.2161</v>
       </c>
+      <c r="G6" s="4" t="n">
+        <v>0.2239</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -12529,40 +12547,41 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E7" s="5">
-        <f>SUM(E6:E6)</f>
-        <v/>
-      </c>
-      <c r="F7" s="5">
-        <f>SUM(F6:F6)</f>
-        <v/>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>5201200</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Cold-Rolled Sheet</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>India</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>6168400</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>0</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E8" s="5">
+        <f>SUM(E6:E7)</f>
+        <v/>
+      </c>
+      <c r="F8" s="5">
+        <f>SUM(F6:F7)</f>
+        <v/>
+      </c>
+      <c r="G8" s="5">
+        <f>SUM(G6:G7)</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -12573,7 +12592,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
@@ -12583,10 +12602,13 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.1099</v>
+        <v>0</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>0.1099</v>
+        <v>0</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -12597,7 +12619,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
@@ -12607,10 +12629,13 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>0.5249</v>
+        <v>0.1099</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>0.5249</v>
+        <v>0.1099</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>0.1099</v>
       </c>
     </row>
     <row r="11">
@@ -12621,7 +12646,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
@@ -12630,8 +12655,14 @@
       <c r="D11" s="4" t="n">
         <v>0.5600000000000001</v>
       </c>
+      <c r="E11" s="4" t="n">
+        <v>0.5249</v>
+      </c>
       <c r="F11" s="4" t="n">
-        <v>0.0003</v>
+        <v>0.5249</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>0.5249</v>
       </c>
     </row>
     <row r="12">
@@ -12642,7 +12673,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
@@ -12652,7 +12683,10 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>0</v>
+        <v>0.0003</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>0.0011</v>
       </c>
     </row>
     <row r="13">
@@ -12663,7 +12697,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
@@ -12673,7 +12707,10 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0.2191</v>
+        <v>0</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -12684,88 +12721,86 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E14" s="5">
-        <f>SUM(E8:E13)</f>
-        <v/>
-      </c>
-      <c r="F14" s="5">
-        <f>SUM(F8:F13)</f>
-        <v/>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>6168400</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>0.2191</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>0.2191</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>18732800</v>
+        <v>6168400</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="E15" s="4" t="n">
-        <v>0.0027</v>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>0.0027</v>
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>0.0128</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>18732800</v>
+        <v>6168400</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="E16" s="4" t="n">
-        <v>0.2673</v>
-      </c>
-      <c r="F16" s="4" t="n">
-        <v>0.2673</v>
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Indonesia</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="n">
-        <v>18732800</v>
-      </c>
-      <c r="D17" s="4" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>0.0069</v>
-      </c>
-      <c r="F17" s="4" t="n">
-        <v>0.0069</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E17" s="5">
+        <f>SUM(E9:E16)</f>
+        <v/>
+      </c>
+      <c r="F17" s="5">
+        <f>SUM(F9:F16)</f>
+        <v/>
+      </c>
+      <c r="G17" s="5">
+        <f>SUM(G9:G16)</f>
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -12776,7 +12811,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
@@ -12786,10 +12821,13 @@
         <v>0.37</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>0.2213</v>
+        <v>0.0027</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>0.2488</v>
+        <v>0.0027</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>0.0027</v>
       </c>
     </row>
     <row r="19">
@@ -12800,7 +12838,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
@@ -12810,10 +12848,13 @@
         <v>0.37</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>0.3697</v>
+        <v>0.2673</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>0.3697</v>
+        <v>0.2673</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>0.2673</v>
       </c>
     </row>
     <row r="20">
@@ -12824,7 +12865,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
@@ -12834,10 +12875,13 @@
         <v>0.37</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>0.0289</v>
+        <v>0.0069</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>0.0289</v>
+        <v>0.0069</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>0.0069</v>
       </c>
     </row>
     <row r="21">
@@ -12848,7 +12892,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
@@ -12857,8 +12901,14 @@
       <c r="D21" s="4" t="n">
         <v>0.37</v>
       </c>
+      <c r="E21" s="4" t="n">
+        <v>0.2213</v>
+      </c>
       <c r="F21" s="4" t="n">
-        <v>0.07539999999999999</v>
+        <v>0.2488</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>0.2488</v>
       </c>
     </row>
     <row r="22">
@@ -12869,88 +12919,98 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E22" s="5">
-        <f>SUM(E15:E21)</f>
-        <v/>
-      </c>
-      <c r="F22" s="5">
-        <f>SUM(F15:F21)</f>
-        <v/>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>18732800</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>0.3697</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>0.3697</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>0.3697</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C23" s="3" t="n">
-        <v>13445100</v>
+        <v>18732800</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>0.29</v>
+        <v>0.37</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>0.2777</v>
+        <v>0.0289</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>0.2777</v>
+        <v>0.0289</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>0.0289</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C24" s="3" t="n">
-        <v>13445100</v>
+        <v>18732800</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="E24" s="4" t="n">
-        <v>0.0037</v>
+        <v>0.37</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>0.0037</v>
+        <v>0.07539999999999999</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>0.07539999999999999</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Thailand</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="n">
-        <v>13445100</v>
-      </c>
-      <c r="D25" s="4" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="E25" s="4" t="n">
-        <v>0.2899</v>
-      </c>
-      <c r="F25" s="4" t="n">
-        <v>0.2899</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E25" s="5">
+        <f>SUM(E18:E24)</f>
+        <v/>
+      </c>
+      <c r="F25" s="5">
+        <f>SUM(F18:F24)</f>
+        <v/>
+      </c>
+      <c r="G25" s="5">
+        <f>SUM(G18:G24)</f>
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -12961,7 +13021,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C26" s="3" t="n">
@@ -12971,10 +13031,13 @@
         <v>0.29</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>0.0883</v>
+        <v>0.2777</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>0.0883</v>
+        <v>0.2777</v>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>0.2747</v>
       </c>
     </row>
     <row r="27">
@@ -12985,93 +13048,101 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E27" s="5">
-        <f>SUM(E23:E26)</f>
-        <v/>
-      </c>
-      <c r="F27" s="5">
-        <f>SUM(F23:F26)</f>
-        <v/>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>13445100</v>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>0.0037</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>0.0037</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>0.0037</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C28" s="3" t="n">
-        <v>5886100</v>
+        <v>13445100</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>0.42</v>
+        <v>0.29</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>0.1023</v>
+        <v>0.2899</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>0.147</v>
+        <v>0.2899</v>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>0.2899</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="C29" s="3" t="n">
-        <v>5886100</v>
+        <v>13445100</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>0.42</v>
+        <v>0.29</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>0.1828</v>
+        <v>0.0883</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>0.1862</v>
+        <v>0.0883</v>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>0.0883</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Türkiye</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="n">
-        <v>5886100</v>
-      </c>
-      <c r="D30" s="4" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="E30" s="4" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="F30" s="4" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E30" s="5">
+        <f>SUM(E26:E29)</f>
+        <v/>
+      </c>
+      <c r="F30" s="5">
+        <f>SUM(F26:F29)</f>
+        <v/>
+      </c>
+      <c r="G30" s="5">
+        <f>SUM(G26:G29)</f>
+        <v/>
       </c>
     </row>
     <row r="31">
@@ -13082,7 +13153,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C31" s="3" t="n">
@@ -13091,8 +13162,14 @@
       <c r="D31" s="4" t="n">
         <v>0.42</v>
       </c>
+      <c r="E31" s="4" t="n">
+        <v>0.1023</v>
+      </c>
       <c r="F31" s="4" t="n">
-        <v>0.0009</v>
+        <v>0.147</v>
+      </c>
+      <c r="G31" s="4" t="n">
+        <v>0.1475</v>
       </c>
     </row>
     <row r="32">
@@ -13103,106 +13180,129 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E32" s="5">
-        <f>SUM(E28:E31)</f>
-        <v/>
-      </c>
-      <c r="F32" s="5">
-        <f>SUM(F28:F31)</f>
-        <v/>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>5886100</v>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>0.1828</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>0.1862</v>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F33" s="5" t="n">
-        <v>0</v>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>5886100</v>
+      </c>
+      <c r="D33" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="G33" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C34" s="3" t="n">
-        <v>3753500</v>
+        <v>5886100</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="E34" s="4" t="n">
-        <v>0.0218</v>
+        <v>0.42</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>0.0218</v>
+        <v>0.0009</v>
+      </c>
+      <c r="G34" s="4" t="n">
+        <v>0.0032</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Taiwan</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="n">
-        <v>3753500</v>
-      </c>
-      <c r="D35" s="4" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="E35" s="4" t="n">
-        <v>0.1828</v>
-      </c>
-      <c r="F35" s="4" t="n">
-        <v>0.1828</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E35" s="5">
+        <f>SUM(E31:E34)</f>
+        <v/>
+      </c>
+      <c r="F35" s="5">
+        <f>SUM(F31:F34)</f>
+        <v/>
+      </c>
+      <c r="G35" s="5">
+        <f>SUM(G31:G34)</f>
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Thailand</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="n">
-        <v>3753500</v>
-      </c>
-      <c r="D36" s="4" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="E36" s="4" t="n">
-        <v>0.3483</v>
-      </c>
-      <c r="F36" s="4" t="n">
-        <v>0.3483</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -13213,7 +13313,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C37" s="3" t="n">
@@ -13223,10 +13323,13 @@
         <v>0.52</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>0.4306</v>
+        <v>0.0218</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>0.4306</v>
+        <v>0.0218</v>
+      </c>
+      <c r="G37" s="4" t="n">
+        <v>0.0218</v>
       </c>
     </row>
     <row r="38">
@@ -13237,15 +13340,100 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="n">
+        <v>3753500</v>
+      </c>
+      <c r="D38" s="4" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>0.1828</v>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>0.1828</v>
+      </c>
+      <c r="G38" s="4" t="n">
+        <v>0.1828</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="n">
+        <v>3753500</v>
+      </c>
+      <c r="D39" s="4" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="E39" s="4" t="n">
+        <v>0.3483</v>
+      </c>
+      <c r="F39" s="4" t="n">
+        <v>0.3483</v>
+      </c>
+      <c r="G39" s="4" t="n">
+        <v>0.3483</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="n">
+        <v>3753500</v>
+      </c>
+      <c r="D40" s="4" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="E40" s="4" t="n">
+        <v>0.4306</v>
+      </c>
+      <c r="F40" s="4" t="n">
+        <v>0.4306</v>
+      </c>
+      <c r="G40" s="4" t="n">
+        <v>0.4306</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E38" s="5">
-        <f>SUM(E34:E37)</f>
-        <v/>
-      </c>
-      <c r="F38" s="5">
-        <f>SUM(F34:F37)</f>
+      <c r="E41" s="5">
+        <f>SUM(E37:E40)</f>
+        <v/>
+      </c>
+      <c r="F41" s="5">
+        <f>SUM(F37:F40)</f>
+        <v/>
+      </c>
+      <c r="G41" s="5">
+        <f>SUM(G37:G40)</f>
         <v/>
       </c>
     </row>
@@ -13260,7 +13448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13296,7 +13484,12 @@
           <t>July 6 2026</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>July 13 2026</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
@@ -13325,6 +13518,9 @@
       <c r="F3" s="4" t="n">
         <v>0.3165</v>
       </c>
+      <c r="G3" s="4" t="n">
+        <v>0.3165</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -13349,6 +13545,9 @@
       <c r="F4" s="4" t="n">
         <v>0.6835</v>
       </c>
+      <c r="G4" s="4" t="n">
+        <v>0.6835</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -13369,6 +13568,10 @@
         <f>SUM(F3:F4)</f>
         <v/>
       </c>
+      <c r="G5" s="5">
+        <f>SUM(G3:G4)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -13393,6 +13596,9 @@
       <c r="F6" s="4" t="n">
         <v>0.0452</v>
       </c>
+      <c r="G6" s="4" t="n">
+        <v>0.0452</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -13417,6 +13623,9 @@
       <c r="F7" s="4" t="n">
         <v>0.0248</v>
       </c>
+      <c r="G7" s="4" t="n">
+        <v>0.025</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -13441,6 +13650,9 @@
       <c r="F8" s="4" t="n">
         <v>0.0009</v>
       </c>
+      <c r="G8" s="4" t="n">
+        <v>0.0009</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -13465,6 +13677,9 @@
       <c r="F9" s="4" t="n">
         <v>0.0008</v>
       </c>
+      <c r="G9" s="4" t="n">
+        <v>0.0024</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -13489,6 +13704,9 @@
       <c r="F10" s="4" t="n">
         <v>0.2212</v>
       </c>
+      <c r="G10" s="4" t="n">
+        <v>0.2225</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -13513,6 +13731,9 @@
       <c r="F11" s="4" t="n">
         <v>0.0518</v>
       </c>
+      <c r="G11" s="4" t="n">
+        <v>0.1076</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -13537,6 +13758,9 @@
       <c r="F12" s="4" t="n">
         <v>0.0053</v>
       </c>
+      <c r="G12" s="4" t="n">
+        <v>0.0611</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -13561,6 +13785,9 @@
       <c r="F13" s="4" t="n">
         <v>0.3287</v>
       </c>
+      <c r="G13" s="4" t="n">
+        <v>0.3287</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -13585,6 +13812,9 @@
       <c r="F14" s="4" t="n">
         <v>0.0005</v>
       </c>
+      <c r="G14" s="4" t="n">
+        <v>0.0005</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -13609,6 +13839,9 @@
       <c r="F15" s="4" t="n">
         <v>0.0229</v>
       </c>
+      <c r="G15" s="4" t="n">
+        <v>0.0539</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -13630,6 +13863,9 @@
       <c r="F16" s="4" t="n">
         <v>0.0002</v>
       </c>
+      <c r="G16" s="4" t="n">
+        <v>0.0002</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -13650,6 +13886,10 @@
         <f>SUM(F6:F16)</f>
         <v/>
       </c>
+      <c r="G17" s="5">
+        <f>SUM(G6:G16)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -13674,6 +13914,9 @@
       <c r="F18" s="4" t="n">
         <v>0.0068</v>
       </c>
+      <c r="G18" s="4" t="n">
+        <v>0.0206</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -13698,6 +13941,9 @@
       <c r="F19" s="4" t="n">
         <v>0.1068</v>
       </c>
+      <c r="G19" s="4" t="n">
+        <v>0.1068</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -13722,6 +13968,9 @@
       <c r="F20" s="4" t="n">
         <v>0.0175</v>
       </c>
+      <c r="G20" s="4" t="n">
+        <v>0.0175</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -13743,6 +13992,9 @@
       <c r="F21" s="4" t="n">
         <v>0.2056</v>
       </c>
+      <c r="G21" s="4" t="n">
+        <v>0.2253</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -13763,6 +14015,10 @@
         <f>SUM(F18:F21)</f>
         <v/>
       </c>
+      <c r="G22" s="5">
+        <f>SUM(G18:G21)</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -13787,6 +14043,9 @@
       <c r="F23" s="4" t="n">
         <v>0.0304</v>
       </c>
+      <c r="G23" s="4" t="n">
+        <v>0.0304</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -13811,6 +14070,9 @@
       <c r="F24" s="4" t="n">
         <v>0.0609</v>
       </c>
+      <c r="G24" s="4" t="n">
+        <v>0.0617</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -13835,6 +14097,9 @@
       <c r="F25" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="G25" s="4" t="n">
+        <v>0.2141</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -13859,6 +14124,9 @@
       <c r="F26" s="4" t="n">
         <v>0.0382</v>
       </c>
+      <c r="G26" s="4" t="n">
+        <v>0.0447</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -13883,6 +14151,9 @@
       <c r="F27" s="4" t="n">
         <v>0.0341</v>
       </c>
+      <c r="G27" s="4" t="n">
+        <v>0.0372</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -13907,6 +14178,9 @@
       <c r="F28" s="4" t="n">
         <v>0.0213</v>
       </c>
+      <c r="G28" s="4" t="n">
+        <v>0.0213</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -13928,6 +14202,9 @@
       <c r="F29" s="4" t="n">
         <v>0.0451</v>
       </c>
+      <c r="G29" s="4" t="n">
+        <v>0.0454</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -13949,6 +14226,9 @@
       <c r="F30" s="4" t="n">
         <v>0.0146</v>
       </c>
+      <c r="G30" s="4" t="n">
+        <v>0.0146</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -13970,6 +14250,9 @@
       <c r="F31" s="4" t="n">
         <v>0.0195</v>
       </c>
+      <c r="G31" s="4" t="n">
+        <v>0.021</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -13979,40 +14262,41 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E32" s="5">
-        <f>SUM(E23:E31)</f>
-        <v/>
-      </c>
-      <c r="F32" s="5">
-        <f>SUM(F23:F31)</f>
-        <v/>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>31128200</v>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>0.0014</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="n">
-        <v>28710400</v>
-      </c>
-      <c r="D33" s="4" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="E33" s="4" t="n">
-        <v>0.0832</v>
-      </c>
-      <c r="F33" s="4" t="n">
-        <v>0.0832</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E33" s="5">
+        <f>SUM(E23:E32)</f>
+        <v/>
+      </c>
+      <c r="F33" s="5">
+        <f>SUM(F23:F32)</f>
+        <v/>
+      </c>
+      <c r="G33" s="5">
+        <f>SUM(G23:G32)</f>
+        <v/>
       </c>
     </row>
     <row r="34">
@@ -14023,7 +14307,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C34" s="3" t="n">
@@ -14033,10 +14317,13 @@
         <v>0.45</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>0.3459</v>
+        <v>0.0832</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>0.3459</v>
+        <v>0.0832</v>
+      </c>
+      <c r="G34" s="4" t="n">
+        <v>0.0832</v>
       </c>
     </row>
     <row r="35">
@@ -14047,7 +14334,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="C35" s="3" t="n">
@@ -14056,8 +14343,14 @@
       <c r="D35" s="4" t="n">
         <v>0.45</v>
       </c>
+      <c r="E35" s="4" t="n">
+        <v>0.3459</v>
+      </c>
       <c r="F35" s="4" t="n">
-        <v>0.0007000000000000001</v>
+        <v>0.3459</v>
+      </c>
+      <c r="G35" s="4" t="n">
+        <v>0.3459</v>
       </c>
     </row>
     <row r="36">
@@ -14068,40 +14361,44 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E36" s="5">
-        <f>SUM(E33:E35)</f>
-        <v/>
-      </c>
-      <c r="F36" s="5">
-        <f>SUM(F33:F35)</f>
-        <v/>
+          <t>Czech Republic</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>28710400</v>
+      </c>
+      <c r="D36" s="4" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
+      <c r="G36" s="4" t="n">
+        <v>0.0007000000000000001</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Australia</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="n">
-        <v>8750300</v>
-      </c>
-      <c r="D37" s="4" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="E37" s="4" t="n">
-        <v>0.0025</v>
-      </c>
-      <c r="F37" s="4" t="n">
-        <v>0.0025</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E37" s="5">
+        <f>SUM(E34:E36)</f>
+        <v/>
+      </c>
+      <c r="F37" s="5">
+        <f>SUM(F34:F36)</f>
+        <v/>
+      </c>
+      <c r="G37" s="5">
+        <f>SUM(G34:G36)</f>
+        <v/>
       </c>
     </row>
     <row r="38">
@@ -14112,7 +14409,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C38" s="3" t="n">
@@ -14122,10 +14419,13 @@
         <v>0.58</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>0.2277</v>
+        <v>0.0025</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>0.2285</v>
+        <v>0.0025</v>
+      </c>
+      <c r="G38" s="4" t="n">
+        <v>0.0025</v>
       </c>
     </row>
     <row r="39">
@@ -14136,7 +14436,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C39" s="3" t="n">
@@ -14146,10 +14446,13 @@
         <v>0.58</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>0.1228</v>
+        <v>0.2277</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>0.1253</v>
+        <v>0.2285</v>
+      </c>
+      <c r="G39" s="4" t="n">
+        <v>0.2297</v>
       </c>
     </row>
     <row r="40">
@@ -14160,7 +14463,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C40" s="3" t="n">
@@ -14170,10 +14473,13 @@
         <v>0.58</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>0.0019</v>
+        <v>0.1228</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>0.0019</v>
+        <v>0.1253</v>
+      </c>
+      <c r="G40" s="4" t="n">
+        <v>0.1543</v>
       </c>
     </row>
     <row r="41">
@@ -14184,7 +14490,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Luxembourg</t>
         </is>
       </c>
       <c r="C41" s="3" t="n">
@@ -14194,10 +14500,13 @@
         <v>0.58</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>0.0068</v>
+        <v>0.0019</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>0.0095</v>
+        <v>0.0019</v>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>0.0035</v>
       </c>
     </row>
     <row r="42">
@@ -14208,7 +14517,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="C42" s="3" t="n">
@@ -14218,10 +14527,13 @@
         <v>0.58</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>0.0191</v>
+        <v>0.0068</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>0.0236</v>
+        <v>0.0095</v>
+      </c>
+      <c r="G42" s="4" t="n">
+        <v>0.01</v>
       </c>
     </row>
     <row r="43">
@@ -14232,7 +14544,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C43" s="3" t="n">
@@ -14241,8 +14553,14 @@
       <c r="D43" s="4" t="n">
         <v>0.58</v>
       </c>
+      <c r="E43" s="4" t="n">
+        <v>0.0191</v>
+      </c>
       <c r="F43" s="4" t="n">
-        <v>0.0017</v>
+        <v>0.0236</v>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>0.0294</v>
       </c>
     </row>
     <row r="44">
@@ -14253,7 +14571,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C44" s="3" t="n">
@@ -14263,7 +14581,10 @@
         <v>0.58</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.0017</v>
+      </c>
+      <c r="G44" s="4" t="n">
+        <v>0.0028</v>
       </c>
     </row>
     <row r="45">
@@ -14274,302 +14595,302 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E45" s="5">
-        <f>SUM(E37:E44)</f>
-        <v/>
-      </c>
-      <c r="F45" s="5">
-        <f>SUM(F37:F44)</f>
-        <v/>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="n">
+        <v>8750300</v>
+      </c>
+      <c r="D45" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F45" s="4" t="n">
+        <v>0.008500000000000001</v>
+      </c>
+      <c r="G45" s="4" t="n">
+        <v>0.06950000000000001</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C46" s="3" t="n">
-        <v>16514800</v>
+        <v>8750300</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="E46" s="4" t="n">
-        <v>0.0029</v>
-      </c>
-      <c r="F46" s="4" t="n">
-        <v>0.0029</v>
+        <v>0.58</v>
+      </c>
+      <c r="G46" s="4" t="n">
+        <v>0.0005</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C47" s="3" t="n">
-        <v>16514800</v>
+        <v>8750300</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="E47" s="4" t="n">
-        <v>0.0339</v>
-      </c>
-      <c r="F47" s="4" t="n">
-        <v>0.0339</v>
+        <v>0.58</v>
+      </c>
+      <c r="G47" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C48" s="3" t="n">
-        <v>16514800</v>
+        <v>8750300</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="E48" s="4" t="n">
-        <v>0.4926</v>
-      </c>
-      <c r="F48" s="4" t="n">
-        <v>0.4926</v>
+        <v>0.58</v>
+      </c>
+      <c r="G48" s="4" t="n">
+        <v>0.0022</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="C49" s="3" t="n">
-        <v>16514800</v>
+        <v>8750300</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="E49" s="4" t="n">
-        <v>0.008800000000000001</v>
-      </c>
-      <c r="F49" s="4" t="n">
-        <v>0.0146</v>
+        <v>0.58</v>
+      </c>
+      <c r="G49" s="4" t="n">
+        <v>0.0004</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E50" s="5">
-        <f>SUM(E46:E49)</f>
-        <v/>
-      </c>
-      <c r="F50" s="5">
-        <f>SUM(F46:F49)</f>
-        <v/>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="n">
+        <v>8750300</v>
+      </c>
+      <c r="D50" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="G50" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="C51" s="3" t="n">
-        <v>3467600</v>
-      </c>
-      <c r="D51" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="E51" s="4" t="n">
-        <v>0.0004</v>
-      </c>
-      <c r="F51" s="4" t="n">
-        <v>0.0021</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E51" s="5">
+        <f>SUM(E38:E50)</f>
+        <v/>
+      </c>
+      <c r="F51" s="5">
+        <f>SUM(F38:F50)</f>
+        <v/>
+      </c>
+      <c r="G51" s="5">
+        <f>SUM(G38:G50)</f>
+        <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C52" s="3" t="n">
-        <v>3467600</v>
+        <v>16514800</v>
       </c>
       <c r="D52" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.59</v>
       </c>
       <c r="E52" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.0029</v>
       </c>
       <c r="F52" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.0029</v>
+      </c>
+      <c r="G52" s="4" t="n">
+        <v>0.0029</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C53" s="3" t="n">
-        <v>3467600</v>
+        <v>16514800</v>
       </c>
       <c r="D53" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.59</v>
       </c>
       <c r="E53" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0339</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0339</v>
+      </c>
+      <c r="G53" s="4" t="n">
+        <v>0.0339</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C54" s="3" t="n">
-        <v>3467600</v>
+        <v>16514800</v>
       </c>
       <c r="D54" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.59</v>
       </c>
       <c r="E54" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.4926</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
+        <v>0.4926</v>
+      </c>
+      <c r="G54" s="4" t="n">
+        <v>0.4926</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C55" s="3" t="n">
-        <v>3467600</v>
+        <v>16514800</v>
       </c>
       <c r="D55" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.59</v>
       </c>
       <c r="E55" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.0146</v>
+      </c>
+      <c r="G55" s="4" t="n">
+        <v>0.0161</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C56" s="3" t="n">
-        <v>3467600</v>
+        <v>16514800</v>
       </c>
       <c r="D56" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="E56" s="4" t="n">
-        <v>0.1798</v>
-      </c>
-      <c r="F56" s="4" t="n">
-        <v>0.1798</v>
+        <v>0.59</v>
+      </c>
+      <c r="G56" s="4" t="n">
+        <v>0.0044</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
-        </is>
-      </c>
-      <c r="C57" s="3" t="n">
-        <v>3467600</v>
-      </c>
-      <c r="D57" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="F57" s="4" t="n">
-        <v>0.0012</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E57" s="5">
+        <f>SUM(E52:E56)</f>
+        <v/>
+      </c>
+      <c r="F57" s="5">
+        <f>SUM(F52:F56)</f>
+        <v/>
+      </c>
+      <c r="G57" s="5">
+        <f>SUM(G52:G56)</f>
+        <v/>
       </c>
     </row>
     <row r="58">
@@ -14580,15 +14901,231 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D58" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E58" s="4" t="n">
+        <v>0.0004</v>
+      </c>
+      <c r="F58" s="4" t="n">
+        <v>0.0021</v>
+      </c>
+      <c r="G58" s="4" t="n">
+        <v>0.0021</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D59" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E59" s="4" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="F59" s="4" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="G59" s="4" t="n">
+        <v>0.0032</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D60" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E60" s="4" t="n">
+        <v>0.0204</v>
+      </c>
+      <c r="F60" s="4" t="n">
+        <v>0.0204</v>
+      </c>
+      <c r="G60" s="4" t="n">
+        <v>0.0204</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Korea, Republic of</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D61" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E61" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="F61" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G61" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D62" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E62" s="4" t="n">
+        <v>0.0004</v>
+      </c>
+      <c r="F62" s="4" t="n">
+        <v>0.0004</v>
+      </c>
+      <c r="G62" s="4" t="n">
+        <v>0.0004</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D63" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E63" s="4" t="n">
+        <v>0.1798</v>
+      </c>
+      <c r="F63" s="4" t="n">
+        <v>0.1798</v>
+      </c>
+      <c r="G63" s="4" t="n">
+        <v>0.2828</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Luxembourg</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D64" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="F64" s="4" t="n">
+        <v>0.0012</v>
+      </c>
+      <c r="G64" s="4" t="n">
+        <v>0.0012</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D65" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G65" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E58" s="5">
-        <f>SUM(E51:E57)</f>
-        <v/>
-      </c>
-      <c r="F58" s="5">
-        <f>SUM(F51:F57)</f>
+      <c r="E66" s="5">
+        <f>SUM(E58:E65)</f>
+        <v/>
+      </c>
+      <c r="F66" s="5">
+        <f>SUM(F58:F65)</f>
+        <v/>
+      </c>
+      <c r="G66" s="5">
+        <f>SUM(G58:G65)</f>
         <v/>
       </c>
     </row>
@@ -14603,7 +15140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14690,185 +15227,878 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>262.45</v>
+        <v>0</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>479.86</v>
+        <v>0</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>1828.386359306535</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Cold-Rolled Sheet</t>
+          <t>Hot-Rolled Sheet</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>89.86</v>
+        <v>3989.900000000001</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>161.13</v>
+        <v>3366.49</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>1793.122635210327</v>
+        <v>843.7529762650692</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Hot-Rolled Sheet</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>23.06</v>
+        <v>1329.77</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>39.55</v>
+        <v>2348.59</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>1715.091066782307</v>
+        <v>1766.1625694669</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>295.92</v>
+        <v>81.29000000000001</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>772.3299999999999</v>
+        <v>282.07</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>2609.92835901595</v>
+        <v>3469.922499692459</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>0</v>
+        <v>1.94</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>0.01</v>
+        <v>3.63</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>0</v>
+        <v>1871.134020618557</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>27.64</v>
+        <v>54.64</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>32.04</v>
+        <v>126.5</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>1159.189580318379</v>
+        <v>2315.153733528551</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>0</v>
+        <v>315.28</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>0.06</v>
+        <v>680.3200000000001</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>0</v>
+        <v>2157.82796244608</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>324.94</v>
+        <v>6825.599999999999</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>485.55</v>
+        <v>8274.440000000001</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>1494.275866313781</v>
+        <v>1212.265588373184</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>Steel Plate</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>651.5299999999999</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>1709.37</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>2623.624391816188</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Cold-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>2.57</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>29.25</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>11381.32295719844</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Cold-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>4750</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Cold-Rolled Sheet</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>1555.25</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>2904.179999999999</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>1867.339656003857</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>224.21</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>419.35</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>1870.344766067526</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>338.43</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>454.86</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>1344.029784593564</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>1507.19</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>2785.46</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>1848.114703521122</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>225.99</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>517.6</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>2290.366830390725</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>64.20999999999999</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>115.09</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>1792.399937704408</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Korea, Republic of</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>2939.81</v>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>5150.88</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>1752.113231807498</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>109.42</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>190.06</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <v>1736.976786693475</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Pakistan</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>59.95</v>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>67.52</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>1126.27189324437</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>2657.21</v>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>3880.42</v>
+      </c>
+      <c r="E30" s="6" t="n">
+        <v>1460.336217310638</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>2849.369999999999</v>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>6269.52</v>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v>2200.317965023848</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Coated Steel Sheet</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>650.51</v>
+      </c>
+      <c r="D32" s="6" t="n">
+        <v>1028.35</v>
+      </c>
+      <c r="E32" s="6" t="n">
+        <v>1580.836574380102</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Rebar</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Czechia</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="n">
+        <v>19.72</v>
+      </c>
+      <c r="D33" s="6" t="n">
+        <v>39.63</v>
+      </c>
+      <c r="E33" s="6" t="n">
+        <v>2009.634888438134</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Rebar</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="D34" s="6" t="n">
+        <v>4.48</v>
+      </c>
+      <c r="E34" s="6" t="n">
+        <v>5270.588235294118</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Rebar</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="n">
+        <v>1213.79</v>
+      </c>
+      <c r="D35" s="6" t="n">
+        <v>956.79</v>
+      </c>
+      <c r="E35" s="6" t="n">
+        <v>788.2665040904934</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Rebar</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="n">
+        <v>671.8399999999999</v>
+      </c>
+      <c r="D36" s="6" t="n">
+        <v>1019.13</v>
+      </c>
+      <c r="E36" s="6" t="n">
+        <v>1516.923672302929</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Rebar</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="D37" s="6" t="n">
+        <v>36.38</v>
+      </c>
+      <c r="E37" s="6" t="n">
+        <v>765.8947368421053</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="n">
+        <v>12.05</v>
+      </c>
+      <c r="D38" s="6" t="n">
+        <v>27.27</v>
+      </c>
+      <c r="E38" s="6" t="n">
+        <v>2263.070539419087</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="n">
+        <v>25.53</v>
+      </c>
+      <c r="D39" s="6" t="n">
+        <v>46.35</v>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>1815.51116333725</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="n">
+        <v>128.19</v>
+      </c>
+      <c r="D40" s="6" t="n">
+        <v>122.39</v>
+      </c>
+      <c r="E40" s="6" t="n">
+        <v>954.754661050004</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="n">
+        <v>100.6</v>
+      </c>
+      <c r="D41" s="6" t="n">
+        <v>256.13</v>
+      </c>
+      <c r="E41" s="6" t="n">
+        <v>2546.023856858847</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="D42" s="6" t="n">
+        <v>32.51</v>
+      </c>
+      <c r="E42" s="6" t="n">
+        <v>1438.495575221239</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="n">
+        <v>72.62</v>
+      </c>
+      <c r="D43" s="6" t="n">
+        <v>98.56999999999999</v>
+      </c>
+      <c r="E43" s="6" t="n">
+        <v>1357.339575874415</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="n">
+        <v>427.48</v>
+      </c>
+      <c r="D44" s="6" t="n">
+        <v>680.83</v>
+      </c>
+      <c r="E44" s="6" t="n">
+        <v>1592.659305698512</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>Structural Steel</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="n">
+        <v>70.03</v>
+      </c>
+      <c r="D45" s="6" t="n">
+        <v>58.73</v>
+      </c>
+      <c r="E45" s="6" t="n">
+        <v>838.640582607454</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D46" s="6" t="n">
+        <v>11.03</v>
+      </c>
+      <c r="E46" s="6" t="n">
+        <v>2941.333333333333</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Korea, Republic of</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D47" s="6" t="n">
+        <v>8.73</v>
+      </c>
+      <c r="E47" s="6" t="n">
+        <v>1091.25</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Luxembourg</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="n">
+        <v>500.39</v>
+      </c>
+      <c r="D48" s="6" t="n">
+        <v>879.0699999999999</v>
+      </c>
+      <c r="E48" s="6" t="n">
+        <v>1756.769719618697</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="n">
+        <v>881.6699999999998</v>
+      </c>
+      <c r="D49" s="6" t="n">
+        <v>1396.63</v>
+      </c>
+      <c r="E49" s="6" t="n">
+        <v>1584.073406149693</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="n">
+        <v>97.08</v>
+      </c>
+      <c r="D50" s="6" t="n">
+        <v>94.98999999999999</v>
+      </c>
+      <c r="E50" s="6" t="n">
+        <v>978.4713638236506</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="C18" s="6" t="n">
-        <v>34.35</v>
-      </c>
-      <c r="D18" s="6" t="n">
-        <v>123.64</v>
-      </c>
-      <c r="E18" s="6" t="n">
-        <v>3599.417758369723</v>
+      <c r="C51" s="6" t="n">
+        <v>853.41</v>
+      </c>
+      <c r="D51" s="6" t="n">
+        <v>2047.9</v>
+      </c>
+      <c r="E51" s="6" t="n">
+        <v>2399.667217398437</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Weekly TRQ update 2026-07-20
</commit_message>
<xml_diff>
--- a/data/canada_trq_tracker.xlsx
+++ b/data/canada_trq_tracker.xlsx
@@ -12390,7 +12390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12431,7 +12431,12 @@
           <t>July 13 2026</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>July 20 2026</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
@@ -12463,6 +12468,14 @@
       <c r="G3" s="4" t="n">
         <v>0.3197</v>
       </c>
+      <c r="H3" s="4" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -12487,6 +12500,9 @@
       <c r="G4" s="4" t="n">
         <v>0.005600000000000001</v>
       </c>
+      <c r="H4" s="4" t="n">
+        <v>0.0277</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -12496,47 +12512,45 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E5" s="5">
-        <f>SUM(E3:E4)</f>
-        <v/>
-      </c>
-      <c r="F5" s="5">
-        <f>SUM(F3:F4)</f>
-        <v/>
-      </c>
-      <c r="G5" s="5">
-        <f>SUM(G3:G4)</f>
-        <v/>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>2366700</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>0.0001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Steel Plate</t>
+          <t>Hot-Rolled Sheet</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>China</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>5201200</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>0.209</v>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>0.2161</v>
-      </c>
-      <c r="G6" s="4" t="n">
-        <v>0.2239</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E6" s="5">
+        <f>SUM(E3:E5)</f>
+        <v/>
+      </c>
+      <c r="F6" s="5">
+        <f>SUM(F3:F5)</f>
+        <v/>
+      </c>
+      <c r="G6" s="5">
+        <f>SUM(G3:G5)</f>
+        <v/>
+      </c>
+      <c r="H6" s="5">
+        <f>SUM(H3:H5)</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -12547,7 +12561,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
@@ -12556,8 +12570,17 @@
       <c r="D7" s="4" t="n">
         <v>0.36</v>
       </c>
+      <c r="E7" s="4" t="n">
+        <v>0.209</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>0.2161</v>
+      </c>
       <c r="G7" s="4" t="n">
-        <v>0</v>
+        <v>0.2239</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>0.3212</v>
       </c>
     </row>
     <row r="8">
@@ -12568,47 +12591,48 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E8" s="5">
-        <f>SUM(E6:E7)</f>
-        <v/>
-      </c>
-      <c r="F8" s="5">
-        <f>SUM(F6:F7)</f>
-        <v/>
-      </c>
-      <c r="G8" s="5">
-        <f>SUM(G6:G7)</f>
-        <v/>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>5201200</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Cold-Rolled Sheet</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>India</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>6168400</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>0</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E9" s="5">
+        <f>SUM(E7:E8)</f>
+        <v/>
+      </c>
+      <c r="F9" s="5">
+        <f>SUM(F7:F8)</f>
+        <v/>
+      </c>
+      <c r="G9" s="5">
+        <f>SUM(G7:G8)</f>
+        <v/>
+      </c>
+      <c r="H9" s="5">
+        <f>SUM(H7:H8)</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -12619,7 +12643,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
@@ -12629,13 +12653,16 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>0.1099</v>
+        <v>0</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>0.1099</v>
+        <v>0</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.1099</v>
+        <v>0</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -12646,7 +12673,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
@@ -12656,13 +12683,16 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0.5249</v>
+        <v>0.1099</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>0.5249</v>
+        <v>0.1099</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>0.5249</v>
+        <v>0.1099</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>0.1135</v>
       </c>
     </row>
     <row r="12">
@@ -12673,7 +12703,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
@@ -12682,11 +12712,17 @@
       <c r="D12" s="4" t="n">
         <v>0.5600000000000001</v>
       </c>
+      <c r="E12" s="4" t="n">
+        <v>0.5249</v>
+      </c>
       <c r="F12" s="4" t="n">
-        <v>0.0003</v>
+        <v>0.5249</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.0011</v>
+        <v>0.5249</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>0.5572</v>
       </c>
     </row>
     <row r="13">
@@ -12697,7 +12733,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
@@ -12707,10 +12743,13 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0</v>
+        <v>0.0003</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0</v>
+        <v>0.0011</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>0.0008</v>
       </c>
     </row>
     <row r="14">
@@ -12721,7 +12760,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
@@ -12731,10 +12770,13 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>0.2191</v>
+        <v>0</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.2191</v>
+        <v>0</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -12745,7 +12787,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
@@ -12754,8 +12796,14 @@
       <c r="D15" s="4" t="n">
         <v>0.5600000000000001</v>
       </c>
+      <c r="F15" s="4" t="n">
+        <v>0.2191</v>
+      </c>
       <c r="G15" s="4" t="n">
-        <v>0.0128</v>
+        <v>0.2191</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>0.3156</v>
       </c>
     </row>
     <row r="16">
@@ -12766,7 +12814,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
@@ -12776,7 +12824,10 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0</v>
+        <v>0.0128</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>0.0128</v>
       </c>
     </row>
     <row r="17">
@@ -12787,47 +12838,48 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E17" s="5">
-        <f>SUM(E9:E16)</f>
-        <v/>
-      </c>
-      <c r="F17" s="5">
-        <f>SUM(F9:F16)</f>
-        <v/>
-      </c>
-      <c r="G17" s="5">
-        <f>SUM(G9:G16)</f>
-        <v/>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>6168400</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>China</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="n">
-        <v>18732800</v>
-      </c>
-      <c r="D18" s="4" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="E18" s="4" t="n">
-        <v>0.0027</v>
-      </c>
-      <c r="F18" s="4" t="n">
-        <v>0.0027</v>
-      </c>
-      <c r="G18" s="4" t="n">
-        <v>0.0027</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E18" s="5">
+        <f>SUM(E10:E17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="5">
+        <f>SUM(F10:F17)</f>
+        <v/>
+      </c>
+      <c r="G18" s="5">
+        <f>SUM(G10:G17)</f>
+        <v/>
+      </c>
+      <c r="H18" s="5">
+        <f>SUM(H10:H17)</f>
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -12838,7 +12890,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
@@ -12848,13 +12900,16 @@
         <v>0.37</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>0.2673</v>
+        <v>0.0027</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>0.2673</v>
+        <v>0.0027</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>0.2673</v>
+        <v>0.0027</v>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>0.0027</v>
       </c>
     </row>
     <row r="20">
@@ -12865,7 +12920,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
@@ -12875,13 +12930,16 @@
         <v>0.37</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>0.0069</v>
+        <v>0.2673</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>0.0069</v>
+        <v>0.2673</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.0069</v>
+        <v>0.2673</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>0.2673</v>
       </c>
     </row>
     <row r="21">
@@ -12892,7 +12950,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
@@ -12902,13 +12960,16 @@
         <v>0.37</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>0.2213</v>
+        <v>0.0069</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>0.2488</v>
+        <v>0.0069</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>0.2488</v>
+        <v>0.0069</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>0.0069</v>
       </c>
     </row>
     <row r="22">
@@ -12919,7 +12980,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="C22" s="3" t="n">
@@ -12929,13 +12990,16 @@
         <v>0.37</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>0.3697</v>
+        <v>0.2213</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>0.3697</v>
+        <v>0.2488</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>0.3697</v>
+        <v>0.2488</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>0.2488</v>
       </c>
     </row>
     <row r="23">
@@ -12946,7 +13010,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C23" s="3" t="n">
@@ -12956,13 +13020,16 @@
         <v>0.37</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>0.0289</v>
+        <v>0.3697</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>0.0289</v>
+        <v>0.3697</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.0289</v>
+        <v>0.3697</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>0.3697</v>
       </c>
     </row>
     <row r="24">
@@ -12973,7 +13040,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C24" s="3" t="n">
@@ -12982,11 +13049,17 @@
       <c r="D24" s="4" t="n">
         <v>0.37</v>
       </c>
+      <c r="E24" s="4" t="n">
+        <v>0.0289</v>
+      </c>
       <c r="F24" s="4" t="n">
-        <v>0.07539999999999999</v>
+        <v>0.0289</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>0.07539999999999999</v>
+        <v>0.0289</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>0.0289</v>
       </c>
     </row>
     <row r="25">
@@ -12997,47 +13070,51 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E25" s="5">
-        <f>SUM(E18:E24)</f>
-        <v/>
-      </c>
-      <c r="F25" s="5">
-        <f>SUM(F18:F24)</f>
-        <v/>
-      </c>
-      <c r="G25" s="5">
-        <f>SUM(G18:G24)</f>
-        <v/>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>18732800</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>0.07539999999999999</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>0.07539999999999999</v>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>0.07539999999999999</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>India</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="n">
-        <v>13445100</v>
-      </c>
-      <c r="D26" s="4" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="E26" s="4" t="n">
-        <v>0.2777</v>
-      </c>
-      <c r="F26" s="4" t="n">
-        <v>0.2777</v>
-      </c>
-      <c r="G26" s="4" t="n">
-        <v>0.2747</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E26" s="5">
+        <f>SUM(E19:E25)</f>
+        <v/>
+      </c>
+      <c r="F26" s="5">
+        <f>SUM(F19:F25)</f>
+        <v/>
+      </c>
+      <c r="G26" s="5">
+        <f>SUM(G19:G25)</f>
+        <v/>
+      </c>
+      <c r="H26" s="5">
+        <f>SUM(H19:H25)</f>
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -13048,7 +13125,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C27" s="3" t="n">
@@ -13058,13 +13135,16 @@
         <v>0.29</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>0.0037</v>
+        <v>0.2777</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>0.0037</v>
+        <v>0.2777</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.0037</v>
+        <v>0.2747</v>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>0.2747</v>
       </c>
     </row>
     <row r="28">
@@ -13075,7 +13155,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C28" s="3" t="n">
@@ -13085,13 +13165,16 @@
         <v>0.29</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>0.2899</v>
+        <v>0.0037</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>0.2899</v>
+        <v>0.0037</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.2899</v>
+        <v>0.0037</v>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>0.0037</v>
       </c>
     </row>
     <row r="29">
@@ -13102,7 +13185,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C29" s="3" t="n">
@@ -13112,13 +13195,16 @@
         <v>0.29</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>0.0883</v>
+        <v>0.2899</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>0.0883</v>
+        <v>0.2899</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>0.0883</v>
+        <v>0.2899</v>
+      </c>
+      <c r="H29" s="4" t="n">
+        <v>0.2899</v>
       </c>
     </row>
     <row r="30">
@@ -13129,26 +13215,32 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E30" s="5">
-        <f>SUM(E26:E29)</f>
-        <v/>
-      </c>
-      <c r="F30" s="5">
-        <f>SUM(F26:F29)</f>
-        <v/>
-      </c>
-      <c r="G30" s="5">
-        <f>SUM(G26:G29)</f>
-        <v/>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>13445100</v>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>0.0883</v>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>0.0883</v>
+      </c>
+      <c r="G30" s="4" t="n">
+        <v>0.0883</v>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>0.0883</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -13157,51 +13249,41 @@
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>5886100</v>
+        <v>13445100</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="E31" s="4" t="n">
-        <v>0.1023</v>
-      </c>
-      <c r="F31" s="4" t="n">
-        <v>0.147</v>
-      </c>
-      <c r="G31" s="4" t="n">
-        <v>0.1475</v>
+        <v>0.29</v>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>0.0038</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Taiwan</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="n">
-        <v>5886100</v>
-      </c>
-      <c r="D32" s="4" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="E32" s="4" t="n">
-        <v>0.1828</v>
-      </c>
-      <c r="F32" s="4" t="n">
-        <v>0.1862</v>
-      </c>
-      <c r="G32" s="4" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E32" s="5">
+        <f>SUM(E27:E31)</f>
+        <v/>
+      </c>
+      <c r="F32" s="5">
+        <f>SUM(F27:F31)</f>
+        <v/>
+      </c>
+      <c r="G32" s="5">
+        <f>SUM(G27:G31)</f>
+        <v/>
+      </c>
+      <c r="H32" s="5">
+        <f>SUM(H27:H31)</f>
+        <v/>
       </c>
     </row>
     <row r="33">
@@ -13212,7 +13294,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C33" s="3" t="n">
@@ -13222,18 +13304,16 @@
         <v>0.42</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>0.42</v>
+        <v>0.1023</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>0.42</v>
+        <v>0.147</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
+        <v>0.1475</v>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>0.1559</v>
       </c>
     </row>
     <row r="34">
@@ -13244,7 +13324,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C34" s="3" t="n">
@@ -13253,11 +13333,22 @@
       <c r="D34" s="4" t="n">
         <v>0.42</v>
       </c>
+      <c r="E34" s="4" t="n">
+        <v>0.1828</v>
+      </c>
       <c r="F34" s="4" t="n">
-        <v>0.0009</v>
+        <v>0.1862</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.42</v>
+      </c>
+      <c r="H34" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -13268,95 +13359,110 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E35" s="5">
-        <f>SUM(E31:E34)</f>
-        <v/>
-      </c>
-      <c r="F35" s="5">
-        <f>SUM(F31:F34)</f>
-        <v/>
-      </c>
-      <c r="G35" s="5">
-        <f>SUM(G31:G34)</f>
-        <v/>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="n">
+        <v>5886100</v>
+      </c>
+      <c r="D35" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="G35" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="H35" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F36" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G36" s="5" t="n">
-        <v>0</v>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>5886100</v>
+      </c>
+      <c r="D36" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>0.0009</v>
+      </c>
+      <c r="G36" s="4" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>0.0024</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>India</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="n">
-        <v>3753500</v>
-      </c>
-      <c r="D37" s="4" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="E37" s="4" t="n">
-        <v>0.0218</v>
-      </c>
-      <c r="F37" s="4" t="n">
-        <v>0.0218</v>
-      </c>
-      <c r="G37" s="4" t="n">
-        <v>0.0218</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E37" s="5">
+        <f>SUM(E33:E36)</f>
+        <v/>
+      </c>
+      <c r="F37" s="5">
+        <f>SUM(F33:F36)</f>
+        <v/>
+      </c>
+      <c r="G37" s="5">
+        <f>SUM(G33:G36)</f>
+        <v/>
+      </c>
+      <c r="H37" s="5">
+        <f>SUM(H33:H36)</f>
+        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Taiwan</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="n">
-        <v>3753500</v>
-      </c>
-      <c r="D38" s="4" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="E38" s="4" t="n">
-        <v>0.1828</v>
-      </c>
-      <c r="F38" s="4" t="n">
-        <v>0.1828</v>
-      </c>
-      <c r="G38" s="4" t="n">
-        <v>0.1828</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -13367,7 +13473,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C39" s="3" t="n">
@@ -13377,13 +13483,16 @@
         <v>0.52</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>0.3483</v>
+        <v>0.0218</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>0.3483</v>
+        <v>0.0218</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>0.3483</v>
+        <v>0.0218</v>
+      </c>
+      <c r="H39" s="4" t="n">
+        <v>0.0218</v>
       </c>
     </row>
     <row r="40">
@@ -13394,7 +13503,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C40" s="3" t="n">
@@ -13404,13 +13513,16 @@
         <v>0.52</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>0.4306</v>
+        <v>0.1828</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>0.4306</v>
+        <v>0.1828</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>0.4306</v>
+        <v>0.1828</v>
+      </c>
+      <c r="H40" s="4" t="n">
+        <v>0.1983</v>
       </c>
     </row>
     <row r="41">
@@ -13421,19 +13533,83 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="n">
+        <v>3753500</v>
+      </c>
+      <c r="D41" s="4" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="E41" s="4" t="n">
+        <v>0.3483</v>
+      </c>
+      <c r="F41" s="4" t="n">
+        <v>0.3483</v>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>0.3483</v>
+      </c>
+      <c r="H41" s="4" t="n">
+        <v>0.3483</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="n">
+        <v>3753500</v>
+      </c>
+      <c r="D42" s="4" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="E42" s="4" t="n">
+        <v>0.4306</v>
+      </c>
+      <c r="F42" s="4" t="n">
+        <v>0.4306</v>
+      </c>
+      <c r="G42" s="4" t="n">
+        <v>0.4306</v>
+      </c>
+      <c r="H42" s="4" t="n">
+        <v>0.4306</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E41" s="5">
-        <f>SUM(E37:E40)</f>
-        <v/>
-      </c>
-      <c r="F41" s="5">
-        <f>SUM(F37:F40)</f>
-        <v/>
-      </c>
-      <c r="G41" s="5">
-        <f>SUM(G37:G40)</f>
+      <c r="E43" s="5">
+        <f>SUM(E39:E42)</f>
+        <v/>
+      </c>
+      <c r="F43" s="5">
+        <f>SUM(F39:F42)</f>
+        <v/>
+      </c>
+      <c r="G43" s="5">
+        <f>SUM(G39:G42)</f>
+        <v/>
+      </c>
+      <c r="H43" s="5">
+        <f>SUM(H39:H42)</f>
         <v/>
       </c>
     </row>
@@ -13448,7 +13624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:I68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13489,7 +13665,12 @@
           <t>July 13 2026</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>July 20 2026</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
@@ -13521,6 +13702,9 @@
       <c r="G3" s="4" t="n">
         <v>0.3165</v>
       </c>
+      <c r="H3" s="4" t="n">
+        <v>0.3165</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -13548,6 +13732,9 @@
       <c r="G4" s="4" t="n">
         <v>0.6835</v>
       </c>
+      <c r="H4" s="4" t="n">
+        <v>0.6835</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -13572,6 +13759,10 @@
         <f>SUM(G3:G4)</f>
         <v/>
       </c>
+      <c r="H5" s="5">
+        <f>SUM(H3:H4)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -13599,6 +13790,9 @@
       <c r="G6" s="4" t="n">
         <v>0.0452</v>
       </c>
+      <c r="H6" s="4" t="n">
+        <v>0.0452</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -13626,6 +13820,9 @@
       <c r="G7" s="4" t="n">
         <v>0.025</v>
       </c>
+      <c r="H7" s="4" t="n">
+        <v>0.0261</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -13653,6 +13850,9 @@
       <c r="G8" s="4" t="n">
         <v>0.0009</v>
       </c>
+      <c r="H8" s="4" t="n">
+        <v>0.0009</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -13680,6 +13880,9 @@
       <c r="G9" s="4" t="n">
         <v>0.0024</v>
       </c>
+      <c r="H9" s="4" t="n">
+        <v>0.0128</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -13707,6 +13910,9 @@
       <c r="G10" s="4" t="n">
         <v>0.2225</v>
       </c>
+      <c r="H10" s="4" t="n">
+        <v>0.2225</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -13734,6 +13940,9 @@
       <c r="G11" s="4" t="n">
         <v>0.1076</v>
       </c>
+      <c r="H11" s="4" t="n">
+        <v>0.2191</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -13761,6 +13970,9 @@
       <c r="G12" s="4" t="n">
         <v>0.0611</v>
       </c>
+      <c r="H12" s="4" t="n">
+        <v>0.0785</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -13788,6 +14000,14 @@
       <c r="G13" s="4" t="n">
         <v>0.3287</v>
       </c>
+      <c r="H13" s="4" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -13815,6 +14035,9 @@
       <c r="G14" s="4" t="n">
         <v>0.0005</v>
       </c>
+      <c r="H14" s="4" t="n">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -13842,6 +14065,9 @@
       <c r="G15" s="4" t="n">
         <v>0.0539</v>
       </c>
+      <c r="H15" s="4" t="n">
+        <v>0.0626</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -13866,6 +14092,9 @@
       <c r="G16" s="4" t="n">
         <v>0.0002</v>
       </c>
+      <c r="H16" s="4" t="n">
+        <v>0.0013</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -13890,6 +14119,10 @@
         <f>SUM(G6:G16)</f>
         <v/>
       </c>
+      <c r="H17" s="5">
+        <f>SUM(H6:H16)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -13917,6 +14150,9 @@
       <c r="G18" s="4" t="n">
         <v>0.0206</v>
       </c>
+      <c r="H18" s="4" t="n">
+        <v>0.0206</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -13944,6 +14180,9 @@
       <c r="G19" s="4" t="n">
         <v>0.1068</v>
       </c>
+      <c r="H19" s="4" t="n">
+        <v>0.1118</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -13971,6 +14210,9 @@
       <c r="G20" s="4" t="n">
         <v>0.0175</v>
       </c>
+      <c r="H20" s="4" t="n">
+        <v>0.0175</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -13995,6 +14237,9 @@
       <c r="G21" s="4" t="n">
         <v>0.2253</v>
       </c>
+      <c r="H21" s="4" t="n">
+        <v>0.2381</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -14019,6 +14264,10 @@
         <f>SUM(G18:G21)</f>
         <v/>
       </c>
+      <c r="H22" s="5">
+        <f>SUM(H18:H21)</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -14046,6 +14295,9 @@
       <c r="G23" s="4" t="n">
         <v>0.0304</v>
       </c>
+      <c r="H23" s="4" t="n">
+        <v>0.0304</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -14073,6 +14325,9 @@
       <c r="G24" s="4" t="n">
         <v>0.0617</v>
       </c>
+      <c r="H24" s="4" t="n">
+        <v>0.0616</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -14100,6 +14355,14 @@
       <c r="G25" s="4" t="n">
         <v>0.2141</v>
       </c>
+      <c r="H25" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -14127,6 +14390,9 @@
       <c r="G26" s="4" t="n">
         <v>0.0447</v>
       </c>
+      <c r="H26" s="4" t="n">
+        <v>0.0447</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -14154,6 +14420,9 @@
       <c r="G27" s="4" t="n">
         <v>0.0372</v>
       </c>
+      <c r="H27" s="4" t="n">
+        <v>0.0372</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -14181,6 +14450,9 @@
       <c r="G28" s="4" t="n">
         <v>0.0213</v>
       </c>
+      <c r="H28" s="4" t="n">
+        <v>0.0213</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -14205,6 +14477,9 @@
       <c r="G29" s="4" t="n">
         <v>0.0454</v>
       </c>
+      <c r="H29" s="4" t="n">
+        <v>0.0454</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -14229,6 +14504,9 @@
       <c r="G30" s="4" t="n">
         <v>0.0146</v>
       </c>
+      <c r="H30" s="4" t="n">
+        <v>0.0146</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -14253,6 +14531,9 @@
       <c r="G31" s="4" t="n">
         <v>0.021</v>
       </c>
+      <c r="H31" s="4" t="n">
+        <v>0.021</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -14274,6 +14555,9 @@
       <c r="G32" s="4" t="n">
         <v>0.0014</v>
       </c>
+      <c r="H32" s="4" t="n">
+        <v>0.0014</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -14298,6 +14582,10 @@
         <f>SUM(G23:G32)</f>
         <v/>
       </c>
+      <c r="H33" s="5">
+        <f>SUM(H23:H32)</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -14325,6 +14613,9 @@
       <c r="G34" s="4" t="n">
         <v>0.0832</v>
       </c>
+      <c r="H34" s="4" t="n">
+        <v>0.0832</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -14352,6 +14643,9 @@
       <c r="G35" s="4" t="n">
         <v>0.3459</v>
       </c>
+      <c r="H35" s="4" t="n">
+        <v>0.3459</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -14376,6 +14670,9 @@
       <c r="G36" s="4" t="n">
         <v>0.0007000000000000001</v>
       </c>
+      <c r="H36" s="4" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -14400,6 +14697,10 @@
         <f>SUM(G34:G36)</f>
         <v/>
       </c>
+      <c r="H37" s="5">
+        <f>SUM(H34:H36)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -14427,6 +14728,9 @@
       <c r="G38" s="4" t="n">
         <v>0.0025</v>
       </c>
+      <c r="H38" s="4" t="n">
+        <v>0.0025</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -14454,6 +14758,9 @@
       <c r="G39" s="4" t="n">
         <v>0.2297</v>
       </c>
+      <c r="H39" s="4" t="n">
+        <v>0.2419</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -14481,6 +14788,9 @@
       <c r="G40" s="4" t="n">
         <v>0.1543</v>
       </c>
+      <c r="H40" s="4" t="n">
+        <v>0.1545</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -14508,6 +14818,9 @@
       <c r="G41" s="4" t="n">
         <v>0.0035</v>
       </c>
+      <c r="H41" s="4" t="n">
+        <v>0.0035</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -14535,6 +14848,9 @@
       <c r="G42" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="H42" s="4" t="n">
+        <v>0.0104</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -14562,6 +14878,9 @@
       <c r="G43" s="4" t="n">
         <v>0.0294</v>
       </c>
+      <c r="H43" s="4" t="n">
+        <v>0.03759999999999999</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -14586,6 +14905,9 @@
       <c r="G44" s="4" t="n">
         <v>0.0028</v>
       </c>
+      <c r="H44" s="4" t="n">
+        <v>0.006500000000000001</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -14610,6 +14932,9 @@
       <c r="G45" s="4" t="n">
         <v>0.06950000000000001</v>
       </c>
+      <c r="H45" s="4" t="n">
+        <v>0.1435</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -14631,6 +14956,9 @@
       <c r="G46" s="4" t="n">
         <v>0.0005</v>
       </c>
+      <c r="H46" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -14652,6 +14980,9 @@
       <c r="G47" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="H47" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -14673,6 +15004,9 @@
       <c r="G48" s="4" t="n">
         <v>0.0022</v>
       </c>
+      <c r="H48" s="4" t="n">
+        <v>0.0022</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -14694,6 +15028,9 @@
       <c r="G49" s="4" t="n">
         <v>0.0004</v>
       </c>
+      <c r="H49" s="4" t="n">
+        <v>0.0004</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -14715,6 +15052,9 @@
       <c r="G50" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="H50" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -14724,74 +15064,66 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E51" s="5">
-        <f>SUM(E38:E50)</f>
-        <v/>
-      </c>
-      <c r="F51" s="5">
-        <f>SUM(F38:F50)</f>
-        <v/>
-      </c>
-      <c r="G51" s="5">
-        <f>SUM(G38:G50)</f>
-        <v/>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="n">
+        <v>8750300</v>
+      </c>
+      <c r="D51" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="H51" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C52" s="3" t="n">
-        <v>16514800</v>
+        <v>8750300</v>
       </c>
       <c r="D52" s="4" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="E52" s="4" t="n">
-        <v>0.0029</v>
-      </c>
-      <c r="F52" s="4" t="n">
-        <v>0.0029</v>
-      </c>
-      <c r="G52" s="4" t="n">
-        <v>0.0029</v>
+        <v>0.58</v>
+      </c>
+      <c r="H52" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="n">
-        <v>16514800</v>
-      </c>
-      <c r="D53" s="4" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="E53" s="4" t="n">
-        <v>0.0339</v>
-      </c>
-      <c r="F53" s="4" t="n">
-        <v>0.0339</v>
-      </c>
-      <c r="G53" s="4" t="n">
-        <v>0.0339</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E53" s="5">
+        <f>SUM(E38:E52)</f>
+        <v/>
+      </c>
+      <c r="F53" s="5">
+        <f>SUM(F38:F52)</f>
+        <v/>
+      </c>
+      <c r="G53" s="5">
+        <f>SUM(G38:G52)</f>
+        <v/>
+      </c>
+      <c r="H53" s="5">
+        <f>SUM(H38:H52)</f>
+        <v/>
       </c>
     </row>
     <row r="54">
@@ -14802,7 +15134,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C54" s="3" t="n">
@@ -14812,13 +15144,16 @@
         <v>0.59</v>
       </c>
       <c r="E54" s="4" t="n">
-        <v>0.4926</v>
+        <v>0.0029</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>0.4926</v>
+        <v>0.0029</v>
       </c>
       <c r="G54" s="4" t="n">
-        <v>0.4926</v>
+        <v>0.0029</v>
+      </c>
+      <c r="H54" s="4" t="n">
+        <v>0.0325</v>
       </c>
     </row>
     <row r="55">
@@ -14829,7 +15164,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C55" s="3" t="n">
@@ -14839,13 +15174,16 @@
         <v>0.59</v>
       </c>
       <c r="E55" s="4" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.0339</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>0.0146</v>
+        <v>0.0339</v>
       </c>
       <c r="G55" s="4" t="n">
-        <v>0.0161</v>
+        <v>0.0339</v>
+      </c>
+      <c r="H55" s="4" t="n">
+        <v>0.0339</v>
       </c>
     </row>
     <row r="56">
@@ -14856,7 +15194,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C56" s="3" t="n">
@@ -14865,8 +15203,17 @@
       <c r="D56" s="4" t="n">
         <v>0.59</v>
       </c>
+      <c r="E56" s="4" t="n">
+        <v>0.4926</v>
+      </c>
+      <c r="F56" s="4" t="n">
+        <v>0.4926</v>
+      </c>
       <c r="G56" s="4" t="n">
-        <v>0.0044</v>
+        <v>0.4926</v>
+      </c>
+      <c r="H56" s="4" t="n">
+        <v>0.4926</v>
       </c>
     </row>
     <row r="57">
@@ -14877,74 +15224,78 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E57" s="5">
-        <f>SUM(E52:E56)</f>
-        <v/>
-      </c>
-      <c r="F57" s="5">
-        <f>SUM(F52:F56)</f>
-        <v/>
-      </c>
-      <c r="G57" s="5">
-        <f>SUM(G52:G56)</f>
-        <v/>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="n">
+        <v>16514800</v>
+      </c>
+      <c r="D57" s="4" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="E57" s="4" t="n">
+        <v>0.008800000000000001</v>
+      </c>
+      <c r="F57" s="4" t="n">
+        <v>0.0146</v>
+      </c>
+      <c r="G57" s="4" t="n">
+        <v>0.0161</v>
+      </c>
+      <c r="H57" s="4" t="n">
+        <v>0.0161</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C58" s="3" t="n">
-        <v>3467600</v>
+        <v>16514800</v>
       </c>
       <c r="D58" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="E58" s="4" t="n">
-        <v>0.0004</v>
-      </c>
-      <c r="F58" s="4" t="n">
-        <v>0.0021</v>
+        <v>0.59</v>
       </c>
       <c r="G58" s="4" t="n">
-        <v>0.0021</v>
+        <v>0.0044</v>
+      </c>
+      <c r="H58" s="4" t="n">
+        <v>0.0044</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="C59" s="3" t="n">
-        <v>3467600</v>
-      </c>
-      <c r="D59" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="E59" s="4" t="n">
-        <v>0.0032</v>
-      </c>
-      <c r="F59" s="4" t="n">
-        <v>0.0032</v>
-      </c>
-      <c r="G59" s="4" t="n">
-        <v>0.0032</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E59" s="5">
+        <f>SUM(E54:E58)</f>
+        <v/>
+      </c>
+      <c r="F59" s="5">
+        <f>SUM(F54:F58)</f>
+        <v/>
+      </c>
+      <c r="G59" s="5">
+        <f>SUM(G54:G58)</f>
+        <v/>
+      </c>
+      <c r="H59" s="5">
+        <f>SUM(H54:H58)</f>
+        <v/>
       </c>
     </row>
     <row r="60">
@@ -14955,7 +15306,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C60" s="3" t="n">
@@ -14965,13 +15316,16 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E60" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0004</v>
       </c>
       <c r="F60" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0021</v>
       </c>
       <c r="G60" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0021</v>
+      </c>
+      <c r="H60" s="4" t="n">
+        <v>0.0021</v>
       </c>
     </row>
     <row r="61">
@@ -14982,7 +15336,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C61" s="3" t="n">
@@ -14992,18 +15346,16 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E61" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.0032</v>
       </c>
       <c r="F61" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.0032</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
+        <v>0.0032</v>
+      </c>
+      <c r="H61" s="4" t="n">
+        <v>0.0032</v>
       </c>
     </row>
     <row r="62">
@@ -15014,7 +15366,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C62" s="3" t="n">
@@ -15024,13 +15376,16 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E62" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.0204</v>
       </c>
       <c r="F62" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.0204</v>
       </c>
       <c r="G62" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.0204</v>
+      </c>
+      <c r="H62" s="4" t="n">
+        <v>0.0204</v>
       </c>
     </row>
     <row r="63">
@@ -15041,7 +15396,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C63" s="3" t="n">
@@ -15051,13 +15406,21 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E63" s="4" t="n">
-        <v>0.1798</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="F63" s="4" t="n">
-        <v>0.1798</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>0.2828</v>
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="H63" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
       </c>
     </row>
     <row r="64">
@@ -15068,7 +15431,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C64" s="3" t="n">
@@ -15077,11 +15440,17 @@
       <c r="D64" s="4" t="n">
         <v>0.6899999999999999</v>
       </c>
+      <c r="E64" s="4" t="n">
+        <v>0.0004</v>
+      </c>
       <c r="F64" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.0004</v>
       </c>
       <c r="G64" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.0004</v>
+      </c>
+      <c r="H64" s="4" t="n">
+        <v>0.0004</v>
       </c>
     </row>
     <row r="65">
@@ -15092,7 +15461,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C65" s="3" t="n">
@@ -15101,8 +15470,17 @@
       <c r="D65" s="4" t="n">
         <v>0.6899999999999999</v>
       </c>
+      <c r="E65" s="4" t="n">
+        <v>0.1798</v>
+      </c>
+      <c r="F65" s="4" t="n">
+        <v>0.1798</v>
+      </c>
       <c r="G65" s="4" t="n">
-        <v>0</v>
+        <v>0.2828</v>
+      </c>
+      <c r="H65" s="4" t="n">
+        <v>0.2828</v>
       </c>
     </row>
     <row r="66">
@@ -15113,19 +15491,74 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
+          <t>Luxembourg</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D66" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="F66" s="4" t="n">
+        <v>0.0012</v>
+      </c>
+      <c r="G66" s="4" t="n">
+        <v>0.0012</v>
+      </c>
+      <c r="H66" s="4" t="n">
+        <v>0.0012</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D67" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G67" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E66" s="5">
-        <f>SUM(E58:E65)</f>
-        <v/>
-      </c>
-      <c r="F66" s="5">
-        <f>SUM(F58:F65)</f>
-        <v/>
-      </c>
-      <c r="G66" s="5">
-        <f>SUM(G58:G65)</f>
+      <c r="E68" s="5">
+        <f>SUM(E60:E67)</f>
+        <v/>
+      </c>
+      <c r="F68" s="5">
+        <f>SUM(F60:F67)</f>
+        <v/>
+      </c>
+      <c r="G68" s="5">
+        <f>SUM(G60:G67)</f>
+        <v/>
+      </c>
+      <c r="H68" s="5">
+        <f>SUM(H60:H67)</f>
         <v/>
       </c>
     </row>
@@ -15140,7 +15573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15227,17 +15660,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0</v>
+        <v>28.79</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0</v>
+        <v>37.4</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0</v>
+        <v>1299.062174366099</v>
       </c>
     </row>
     <row r="11">
@@ -15248,17 +15681,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>3989.900000000001</v>
+        <v>0</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>3366.49</v>
+        <v>0</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>843.7529762650692</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -15269,101 +15702,101 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>1329.77</v>
+        <v>1552.69</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>2348.59</v>
+        <v>2269.02</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>1766.1625694669</v>
+        <v>1461.347725560157</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Steel Plate</t>
+          <t>Hot-Rolled Sheet</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>81.29000000000001</v>
+        <v>3989.900000000001</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>282.07</v>
+        <v>3366.49</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>3469.922499692459</v>
+        <v>843.7529762650692</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Steel Plate</t>
+          <t>Hot-Rolled Sheet</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>1.94</v>
+        <v>0.02</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>3.63</v>
+        <v>0.09</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>1871.134020618557</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Steel Plate</t>
+          <t>Hot-Rolled Sheet</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>54.64</v>
+        <v>41.91</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>126.5</v>
+        <v>31.74</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>2315.153733528551</v>
+        <v>757.3371510379385</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Steel Plate</t>
+          <t>Hot-Rolled Sheet</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>315.28</v>
+        <v>2604.53</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>680.3200000000001</v>
+        <v>4528.89</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>2157.82796244608</v>
+        <v>1738.851155486787</v>
       </c>
     </row>
     <row r="17">
@@ -15374,17 +15807,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>6825.599999999999</v>
+        <v>81.29000000000001</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>8274.440000000001</v>
+        <v>282.07</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>1212.265588373184</v>
+        <v>3469.922499692459</v>
       </c>
     </row>
     <row r="18">
@@ -15395,269 +15828,269 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>651.5299999999999</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>1709.37</v>
+        <v>15.27</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>2623.624391816188</v>
+        <v>1844.202898550725</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Cold-Rolled Sheet</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>2.57</v>
+        <v>54.64</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>29.25</v>
+        <v>126.5</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>11381.32295719844</v>
+        <v>2315.153733528551</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Cold-Rolled Sheet</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>0.04</v>
+        <v>315.28</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>0.19</v>
+        <v>680.3200000000001</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>4750</v>
+        <v>2157.82796244608</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Cold-Rolled Sheet</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>1555.25</v>
+        <v>7463.45</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>2904.179999999999</v>
+        <v>8994.029999999999</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>1867.339656003857</v>
+        <v>1205.076740649431</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>224.21</v>
+        <v>16.61</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>419.35</v>
+        <v>25.17</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>1870.344766067526</v>
+        <v>1515.352197471403</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>338.43</v>
+        <v>25.68</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>454.86</v>
+        <v>34.82</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>1344.029784593564</v>
+        <v>1355.919003115265</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>1507.19</v>
+        <v>1724.58</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>2785.46</v>
+        <v>3694.98</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>1848.114703521122</v>
+        <v>2142.539052986815</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C25" s="6" t="n">
-        <v>225.99</v>
+        <v>7.15</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>517.6</v>
+        <v>16.26</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>2290.366830390725</v>
+        <v>2274.125874125874</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>64.20999999999999</v>
+        <v>0</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>115.09</v>
+        <v>0.03</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>1792.399937704408</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>2939.81</v>
+        <v>154.64</v>
       </c>
       <c r="D27" s="6" t="n">
-        <v>5150.88</v>
+        <v>180.58</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>1752.113231807498</v>
+        <v>1167.744438696327</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>109.42</v>
+        <v>1425.92</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>190.06</v>
+        <v>1699.87</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>1736.976786693475</v>
+        <v>1192.121577648115</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>59.95</v>
+        <v>0.04</v>
       </c>
       <c r="D29" s="6" t="n">
-        <v>67.52</v>
+        <v>0.19</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>1126.27189324437</v>
+        <v>4750</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>2657.21</v>
+        <v>2462.55</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>3880.42</v>
+        <v>4557.640000000001</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>1460.336217310638</v>
+        <v>1850.780694808228</v>
       </c>
     </row>
     <row r="31">
@@ -15668,17 +16101,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C31" s="6" t="n">
-        <v>2849.369999999999</v>
+        <v>1099.45</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>6269.52</v>
+        <v>1768.94</v>
       </c>
       <c r="E31" s="6" t="n">
-        <v>2200.317965023848</v>
+        <v>1608.931738596571</v>
       </c>
     </row>
     <row r="32">
@@ -15689,44 +16122,44 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>650.51</v>
+        <v>566.6999999999999</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>1028.35</v>
+        <v>781.8299999999999</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>1580.836574380102</v>
+        <v>1379.618845950238</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C33" s="6" t="n">
-        <v>19.72</v>
+        <v>40.24</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>39.63</v>
+        <v>88.01000000000001</v>
       </c>
       <c r="E33" s="6" t="n">
-        <v>2009.634888438134</v>
+        <v>2187.127236580517</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -15735,370 +16168,727 @@
         </is>
       </c>
       <c r="C34" s="6" t="n">
-        <v>0.85</v>
+        <v>2897.2</v>
       </c>
       <c r="D34" s="6" t="n">
-        <v>4.48</v>
+        <v>5530.73</v>
       </c>
       <c r="E34" s="6" t="n">
-        <v>5270.588235294118</v>
+        <v>1908.991440011045</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C35" s="6" t="n">
-        <v>1213.79</v>
+        <v>246.5</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>956.79</v>
+        <v>602.38</v>
       </c>
       <c r="E35" s="6" t="n">
-        <v>788.2665040904934</v>
+        <v>2443.732251521298</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C36" s="6" t="n">
-        <v>671.8399999999999</v>
+        <v>267.58</v>
       </c>
       <c r="D36" s="6" t="n">
-        <v>1019.13</v>
+        <v>474.55</v>
       </c>
       <c r="E36" s="6" t="n">
-        <v>1516.923672302929</v>
+        <v>1773.488302563719</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C37" s="6" t="n">
-        <v>47.5</v>
+        <v>5178.2</v>
       </c>
       <c r="D37" s="6" t="n">
-        <v>36.38</v>
+        <v>8867.09</v>
       </c>
       <c r="E37" s="6" t="n">
-        <v>765.8947368421053</v>
+        <v>1712.388474759569</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C38" s="6" t="n">
-        <v>12.05</v>
+        <v>87.97</v>
       </c>
       <c r="D38" s="6" t="n">
-        <v>27.27</v>
+        <v>180.34</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>2263.070539419087</v>
+        <v>2050.017051267478</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C39" s="6" t="n">
-        <v>25.53</v>
+        <v>284.88</v>
       </c>
       <c r="D39" s="6" t="n">
-        <v>46.35</v>
+        <v>577.25</v>
       </c>
       <c r="E39" s="6" t="n">
-        <v>1815.51116333725</v>
+        <v>2026.291771974165</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="C40" s="6" t="n">
-        <v>128.19</v>
+        <v>1922.54</v>
       </c>
       <c r="D40" s="6" t="n">
-        <v>122.39</v>
+        <v>2374.78</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>954.754661050004</v>
+        <v>1235.230476348996</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C41" s="6" t="n">
-        <v>100.6</v>
+        <v>0.12</v>
       </c>
       <c r="D41" s="6" t="n">
-        <v>256.13</v>
+        <v>0.25</v>
       </c>
       <c r="E41" s="6" t="n">
-        <v>2546.023856858847</v>
+        <v>2083.333333333333</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C42" s="6" t="n">
-        <v>22.6</v>
+        <v>2785.19</v>
       </c>
       <c r="D42" s="6" t="n">
-        <v>32.51</v>
+        <v>4035.09</v>
       </c>
       <c r="E42" s="6" t="n">
-        <v>1438.495575221239</v>
+        <v>1448.766511440871</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C43" s="6" t="n">
-        <v>72.62</v>
+        <v>6358.75</v>
       </c>
       <c r="D43" s="6" t="n">
-        <v>98.56999999999999</v>
+        <v>13217.57</v>
       </c>
       <c r="E43" s="6" t="n">
-        <v>1357.339575874415</v>
+        <v>2078.642815018675</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C44" s="6" t="n">
-        <v>427.48</v>
+        <v>799.97</v>
       </c>
       <c r="D44" s="6" t="n">
-        <v>680.83</v>
+        <v>1173.88</v>
       </c>
       <c r="E44" s="6" t="n">
-        <v>1592.659305698512</v>
+        <v>1467.405027688538</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="C45" s="6" t="n">
-        <v>70.03</v>
+        <v>19.72</v>
       </c>
       <c r="D45" s="6" t="n">
-        <v>58.73</v>
+        <v>39.63</v>
       </c>
       <c r="E45" s="6" t="n">
-        <v>838.640582607454</v>
+        <v>2009.634888438134</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C46" s="6" t="n">
-        <v>3.75</v>
+        <v>1213.79</v>
       </c>
       <c r="D46" s="6" t="n">
-        <v>11.03</v>
+        <v>956.79</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>2941.333333333333</v>
+        <v>788.2665040904934</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C47" s="6" t="n">
-        <v>8</v>
+        <v>1175.59</v>
       </c>
       <c r="D47" s="6" t="n">
-        <v>8.73</v>
+        <v>1819.18</v>
       </c>
       <c r="E47" s="6" t="n">
-        <v>1091.25</v>
+        <v>1547.461274764161</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C48" s="6" t="n">
-        <v>500.39</v>
+        <v>100.42</v>
       </c>
       <c r="D48" s="6" t="n">
-        <v>879.0699999999999</v>
+        <v>161.19</v>
       </c>
       <c r="E48" s="6" t="n">
-        <v>1756.769719618697</v>
+        <v>1605.158334993029</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C49" s="6" t="n">
-        <v>881.6699999999998</v>
+        <v>18.95</v>
       </c>
       <c r="D49" s="6" t="n">
-        <v>1396.63</v>
+        <v>43.36</v>
       </c>
       <c r="E49" s="6" t="n">
-        <v>1584.073406149693</v>
+        <v>2288.126649076517</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C50" s="6" t="n">
-        <v>97.08</v>
+        <v>25.53</v>
       </c>
       <c r="D50" s="6" t="n">
-        <v>94.98999999999999</v>
+        <v>46.35</v>
       </c>
       <c r="E50" s="6" t="n">
-        <v>978.4713638236506</v>
+        <v>1815.51116333725</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="n">
+        <v>6.84</v>
+      </c>
+      <c r="D51" s="6" t="n">
+        <v>30.16</v>
+      </c>
+      <c r="E51" s="6" t="n">
+        <v>4409.356725146199</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D52" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E52" s="6" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="n">
+        <v>229.71</v>
+      </c>
+      <c r="D53" s="6" t="n">
+        <v>344.33</v>
+      </c>
+      <c r="E53" s="6" t="n">
+        <v>1498.976970963388</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Slovenia</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D54" s="6" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="E54" s="6" t="n">
+        <v>114000</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="n">
+        <v>238.1</v>
+      </c>
+      <c r="D55" s="6" t="n">
+        <v>256.29</v>
+      </c>
+      <c r="E55" s="6" t="n">
+        <v>1076.396472070558</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Hot-Rolled Bar</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="n">
+        <v>529.3099999999999</v>
+      </c>
+      <c r="D56" s="6" t="n">
+        <v>1075.13</v>
+      </c>
+      <c r="E56" s="6" t="n">
+        <v>2031.191551264855</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="D57" s="6" t="n">
+        <v>32.51</v>
+      </c>
+      <c r="E57" s="6" t="n">
+        <v>1438.495575221239</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="n">
+        <v>72.62</v>
+      </c>
+      <c r="D58" s="6" t="n">
+        <v>98.56999999999999</v>
+      </c>
+      <c r="E58" s="6" t="n">
+        <v>1357.339575874415</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Wire Rod</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="n">
+        <v>887.39</v>
+      </c>
+      <c r="D59" s="6" t="n">
+        <v>1419.21</v>
+      </c>
+      <c r="E59" s="6" t="n">
+        <v>1599.308083255389</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t>Structural Steel</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="n">
+        <v>70.04000000000001</v>
+      </c>
+      <c r="D60" s="6" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="E60" s="6" t="n">
+        <v>839.5202741290691</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D61" s="6" t="n">
+        <v>11.03</v>
+      </c>
+      <c r="E61" s="6" t="n">
+        <v>2941.333333333333</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Korea, Republic of</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D62" s="6" t="n">
+        <v>8.73</v>
+      </c>
+      <c r="E62" s="6" t="n">
+        <v>1091.25</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Luxembourg</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="n">
+        <v>3325.32</v>
+      </c>
+      <c r="D63" s="6" t="n">
+        <v>5482.570000000001</v>
+      </c>
+      <c r="E63" s="6" t="n">
+        <v>1648.734557877137</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="n">
+        <v>2311.129999999999</v>
+      </c>
+      <c r="D64" s="6" t="n">
+        <v>3533.67</v>
+      </c>
+      <c r="E64" s="6" t="n">
+        <v>1528.979330457396</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="n">
+        <v>6037.94</v>
+      </c>
+      <c r="D65" s="6" t="n">
+        <v>6900.929999999999</v>
+      </c>
+      <c r="E65" s="6" t="n">
+        <v>1142.927886000854</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="n">
+        <v>436.41</v>
+      </c>
+      <c r="D66" s="6" t="n">
+        <v>496.74</v>
+      </c>
+      <c r="E66" s="6" t="n">
+        <v>1138.241561834055</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="C51" s="6" t="n">
-        <v>853.41</v>
-      </c>
-      <c r="D51" s="6" t="n">
-        <v>2047.9</v>
-      </c>
-      <c r="E51" s="6" t="n">
-        <v>2399.667217398437</v>
+      <c r="C67" s="6" t="n">
+        <v>1447.37</v>
+      </c>
+      <c r="D67" s="6" t="n">
+        <v>3666.469999999999</v>
+      </c>
+      <c r="E67" s="6" t="n">
+        <v>2533.194691060337</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="n">
+        <v>307.36</v>
+      </c>
+      <c r="D68" s="6" t="n">
+        <v>258.04</v>
+      </c>
+      <c r="E68" s="6" t="n">
+        <v>839.5366996356065</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Weekly TRQ update 2026-07-27
</commit_message>
<xml_diff>
--- a/data/canada_trq_tracker.xlsx
+++ b/data/canada_trq_tracker.xlsx
@@ -12390,7 +12390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12436,7 +12436,12 @@
           <t>July 20 2026</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>July 27 2026</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
@@ -12471,7 +12476,10 @@
       <c r="H3" s="4" t="n">
         <v>0.41</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="4" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -12503,6 +12511,9 @@
       <c r="H4" s="4" t="n">
         <v>0.0277</v>
       </c>
+      <c r="I4" s="4" t="n">
+        <v>0.0301</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -12524,6 +12535,9 @@
       <c r="H5" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="I5" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -12552,6 +12566,10 @@
         <f>SUM(H3:H5)</f>
         <v/>
       </c>
+      <c r="I6" s="5">
+        <f>SUM(I3:I5)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -12582,6 +12600,9 @@
       <c r="H7" s="4" t="n">
         <v>0.3212</v>
       </c>
+      <c r="I7" s="4" t="n">
+        <v>0.3564</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -12606,6 +12627,9 @@
       <c r="H8" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="I8" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -12634,6 +12658,10 @@
         <f>SUM(H7:H8)</f>
         <v/>
       </c>
+      <c r="I9" s="5">
+        <f>SUM(I7:I8)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -12664,6 +12692,9 @@
       <c r="H10" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="I10" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -12694,6 +12725,9 @@
       <c r="H11" s="4" t="n">
         <v>0.1135</v>
       </c>
+      <c r="I11" s="4" t="n">
+        <v>0.1135</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -12724,6 +12758,9 @@
       <c r="H12" s="4" t="n">
         <v>0.5572</v>
       </c>
+      <c r="I12" s="4" t="n">
+        <v>0.5572</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -12751,6 +12788,9 @@
       <c r="H13" s="4" t="n">
         <v>0.0008</v>
       </c>
+      <c r="I13" s="4" t="n">
+        <v>0.0008</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -12778,6 +12818,9 @@
       <c r="H14" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="I14" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -12805,6 +12848,9 @@
       <c r="H15" s="4" t="n">
         <v>0.3156</v>
       </c>
+      <c r="I15" s="4" t="n">
+        <v>0.3156</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -12829,6 +12875,9 @@
       <c r="H16" s="4" t="n">
         <v>0.0128</v>
       </c>
+      <c r="I16" s="4" t="n">
+        <v>0.0128</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -12853,6 +12902,9 @@
       <c r="H17" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="I17" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -12881,6 +12933,10 @@
         <f>SUM(H10:H17)</f>
         <v/>
       </c>
+      <c r="I18" s="5">
+        <f>SUM(I10:I17)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -12911,6 +12967,9 @@
       <c r="H19" s="4" t="n">
         <v>0.0027</v>
       </c>
+      <c r="I19" s="4" t="n">
+        <v>0.0027</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -12941,6 +13000,9 @@
       <c r="H20" s="4" t="n">
         <v>0.2673</v>
       </c>
+      <c r="I20" s="4" t="n">
+        <v>0.2673</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -12971,6 +13033,9 @@
       <c r="H21" s="4" t="n">
         <v>0.0069</v>
       </c>
+      <c r="I21" s="4" t="n">
+        <v>0.0069</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -13001,6 +13066,9 @@
       <c r="H22" s="4" t="n">
         <v>0.2488</v>
       </c>
+      <c r="I22" s="4" t="n">
+        <v>0.2488</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -13031,6 +13099,9 @@
       <c r="H23" s="4" t="n">
         <v>0.3697</v>
       </c>
+      <c r="I23" s="4" t="n">
+        <v>0.3697</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -13061,6 +13132,9 @@
       <c r="H24" s="4" t="n">
         <v>0.0289</v>
       </c>
+      <c r="I24" s="4" t="n">
+        <v>0.0289</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -13088,6 +13162,9 @@
       <c r="H25" s="4" t="n">
         <v>0.07539999999999999</v>
       </c>
+      <c r="I25" s="4" t="n">
+        <v>0.07539999999999999</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -13116,6 +13193,10 @@
         <f>SUM(H19:H25)</f>
         <v/>
       </c>
+      <c r="I26" s="5">
+        <f>SUM(I19:I25)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -13146,6 +13227,9 @@
       <c r="H27" s="4" t="n">
         <v>0.2747</v>
       </c>
+      <c r="I27" s="4" t="n">
+        <v>0.2747</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -13176,6 +13260,9 @@
       <c r="H28" s="4" t="n">
         <v>0.0037</v>
       </c>
+      <c r="I28" s="4" t="n">
+        <v>0.0037</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -13206,6 +13293,9 @@
       <c r="H29" s="4" t="n">
         <v>0.2899</v>
       </c>
+      <c r="I29" s="4" t="n">
+        <v>0.2899</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -13236,6 +13326,9 @@
       <c r="H30" s="4" t="n">
         <v>0.0883</v>
       </c>
+      <c r="I30" s="4" t="n">
+        <v>0.0883</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -13257,6 +13350,9 @@
       <c r="H31" s="4" t="n">
         <v>0.0038</v>
       </c>
+      <c r="I31" s="4" t="n">
+        <v>0.0038</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -13285,6 +13381,10 @@
         <f>SUM(H27:H31)</f>
         <v/>
       </c>
+      <c r="I32" s="5">
+        <f>SUM(I27:I31)</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -13315,6 +13415,9 @@
       <c r="H33" s="4" t="n">
         <v>0.1559</v>
       </c>
+      <c r="I33" s="4" t="n">
+        <v>0.1576</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -13345,7 +13448,10 @@
       <c r="H34" s="4" t="n">
         <v>0.42</v>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="I34" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="J34" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -13380,7 +13486,10 @@
       <c r="H35" s="4" t="n">
         <v>0.42</v>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="I35" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="J35" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -13412,6 +13521,9 @@
       <c r="H36" s="4" t="n">
         <v>0.0024</v>
       </c>
+      <c r="I36" s="4" t="n">
+        <v>0.0024</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -13440,6 +13552,10 @@
         <f>SUM(H33:H36)</f>
         <v/>
       </c>
+      <c r="I37" s="5">
+        <f>SUM(I33:I36)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -13449,50 +13565,49 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F38" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H38" s="5" t="n">
-        <v>0</v>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="n">
+        <v>1571700</v>
+      </c>
+      <c r="D38" s="4" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="I38" s="4" t="n">
+        <v>0.0397</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>India</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="n">
-        <v>3753500</v>
-      </c>
-      <c r="D39" s="4" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="E39" s="4" t="n">
-        <v>0.0218</v>
-      </c>
-      <c r="F39" s="4" t="n">
-        <v>0.0218</v>
-      </c>
-      <c r="G39" s="4" t="n">
-        <v>0.0218</v>
-      </c>
-      <c r="H39" s="4" t="n">
-        <v>0.0218</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E39" s="5">
+        <f>SUM(E38:E38)</f>
+        <v/>
+      </c>
+      <c r="F39" s="5">
+        <f>SUM(F38:F38)</f>
+        <v/>
+      </c>
+      <c r="G39" s="5">
+        <f>SUM(G38:G38)</f>
+        <v/>
+      </c>
+      <c r="H39" s="5">
+        <f>SUM(H38:H38)</f>
+        <v/>
+      </c>
+      <c r="I39" s="5">
+        <f>SUM(I38:I38)</f>
+        <v/>
       </c>
     </row>
     <row r="40">
@@ -13503,7 +13618,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C40" s="3" t="n">
@@ -13513,16 +13628,19 @@
         <v>0.52</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>0.1828</v>
+        <v>0.0218</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>0.1828</v>
+        <v>0.0218</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>0.1828</v>
+        <v>0.0218</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>0.1983</v>
+        <v>0.0218</v>
+      </c>
+      <c r="I40" s="4" t="n">
+        <v>0.0218</v>
       </c>
     </row>
     <row r="41">
@@ -13533,7 +13651,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C41" s="3" t="n">
@@ -13543,16 +13661,19 @@
         <v>0.52</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>0.3483</v>
+        <v>0.1828</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>0.3483</v>
+        <v>0.1828</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>0.3483</v>
+        <v>0.1828</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>0.3483</v>
+        <v>0.1983</v>
+      </c>
+      <c r="I41" s="4" t="n">
+        <v>0.1993</v>
       </c>
     </row>
     <row r="42">
@@ -13563,7 +13684,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C42" s="3" t="n">
@@ -13573,16 +13694,19 @@
         <v>0.52</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>0.4306</v>
+        <v>0.3483</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>0.4306</v>
+        <v>0.3483</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>0.4306</v>
+        <v>0.3483</v>
       </c>
       <c r="H42" s="4" t="n">
-        <v>0.4306</v>
+        <v>0.3483</v>
+      </c>
+      <c r="I42" s="4" t="n">
+        <v>0.3483</v>
       </c>
     </row>
     <row r="43">
@@ -13593,23 +13717,60 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="n">
+        <v>3753500</v>
+      </c>
+      <c r="D43" s="4" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="E43" s="4" t="n">
+        <v>0.4306</v>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>0.4306</v>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>0.4306</v>
+      </c>
+      <c r="H43" s="4" t="n">
+        <v>0.4306</v>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>0.4306</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E43" s="5">
-        <f>SUM(E39:E42)</f>
-        <v/>
-      </c>
-      <c r="F43" s="5">
-        <f>SUM(F39:F42)</f>
-        <v/>
-      </c>
-      <c r="G43" s="5">
-        <f>SUM(G39:G42)</f>
-        <v/>
-      </c>
-      <c r="H43" s="5">
-        <f>SUM(H39:H42)</f>
+      <c r="E44" s="5">
+        <f>SUM(E40:E43)</f>
+        <v/>
+      </c>
+      <c r="F44" s="5">
+        <f>SUM(F40:F43)</f>
+        <v/>
+      </c>
+      <c r="G44" s="5">
+        <f>SUM(G40:G43)</f>
+        <v/>
+      </c>
+      <c r="H44" s="5">
+        <f>SUM(H40:H43)</f>
+        <v/>
+      </c>
+      <c r="I44" s="5">
+        <f>SUM(I40:I43)</f>
         <v/>
       </c>
     </row>
@@ -13624,7 +13785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I68"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13670,7 +13831,12 @@
           <t>July 20 2026</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>July 27 2026</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
@@ -13705,6 +13871,9 @@
       <c r="H3" s="4" t="n">
         <v>0.3165</v>
       </c>
+      <c r="I3" s="4" t="n">
+        <v>0.3165</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -13735,6 +13904,9 @@
       <c r="H4" s="4" t="n">
         <v>0.6835</v>
       </c>
+      <c r="I4" s="4" t="n">
+        <v>0.6835</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -13763,6 +13935,10 @@
         <f>SUM(H3:H4)</f>
         <v/>
       </c>
+      <c r="I5" s="5">
+        <f>SUM(I3:I4)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -13793,6 +13969,9 @@
       <c r="H6" s="4" t="n">
         <v>0.0452</v>
       </c>
+      <c r="I6" s="4" t="n">
+        <v>0.0452</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -13823,6 +14002,9 @@
       <c r="H7" s="4" t="n">
         <v>0.0261</v>
       </c>
+      <c r="I7" s="4" t="n">
+        <v>0.0261</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -13853,6 +14035,9 @@
       <c r="H8" s="4" t="n">
         <v>0.0009</v>
       </c>
+      <c r="I8" s="4" t="n">
+        <v>0.0009</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -13883,6 +14068,9 @@
       <c r="H9" s="4" t="n">
         <v>0.0128</v>
       </c>
+      <c r="I9" s="4" t="n">
+        <v>0.0128</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -13913,6 +14101,9 @@
       <c r="H10" s="4" t="n">
         <v>0.2225</v>
       </c>
+      <c r="I10" s="4" t="n">
+        <v>0.2225</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -13943,6 +14134,9 @@
       <c r="H11" s="4" t="n">
         <v>0.2191</v>
       </c>
+      <c r="I11" s="4" t="n">
+        <v>0.2191</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -13973,6 +14167,9 @@
       <c r="H12" s="4" t="n">
         <v>0.0785</v>
       </c>
+      <c r="I12" s="4" t="n">
+        <v>0.0785</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -14003,7 +14200,10 @@
       <c r="H13" s="4" t="n">
         <v>0.33</v>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I13" s="4" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J13" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -14038,6 +14238,9 @@
       <c r="H14" s="4" t="n">
         <v>0.001</v>
       </c>
+      <c r="I14" s="4" t="n">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -14068,6 +14271,9 @@
       <c r="H15" s="4" t="n">
         <v>0.0626</v>
       </c>
+      <c r="I15" s="4" t="n">
+        <v>0.0622</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -14095,6 +14301,9 @@
       <c r="H16" s="4" t="n">
         <v>0.0013</v>
       </c>
+      <c r="I16" s="4" t="n">
+        <v>0.0013</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -14123,6 +14332,10 @@
         <f>SUM(H6:H16)</f>
         <v/>
       </c>
+      <c r="I17" s="5">
+        <f>SUM(I6:I16)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -14153,6 +14366,9 @@
       <c r="H18" s="4" t="n">
         <v>0.0206</v>
       </c>
+      <c r="I18" s="4" t="n">
+        <v>0.0206</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -14183,6 +14399,9 @@
       <c r="H19" s="4" t="n">
         <v>0.1118</v>
       </c>
+      <c r="I19" s="4" t="n">
+        <v>0.1124</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -14213,6 +14432,9 @@
       <c r="H20" s="4" t="n">
         <v>0.0175</v>
       </c>
+      <c r="I20" s="4" t="n">
+        <v>0.0175</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -14240,6 +14462,9 @@
       <c r="H21" s="4" t="n">
         <v>0.2381</v>
       </c>
+      <c r="I21" s="4" t="n">
+        <v>0.3055</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -14268,6 +14493,10 @@
         <f>SUM(H18:H21)</f>
         <v/>
       </c>
+      <c r="I22" s="5">
+        <f>SUM(I18:I21)</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -14298,6 +14527,9 @@
       <c r="H23" s="4" t="n">
         <v>0.0304</v>
       </c>
+      <c r="I23" s="4" t="n">
+        <v>0.0304</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -14328,6 +14560,9 @@
       <c r="H24" s="4" t="n">
         <v>0.0616</v>
       </c>
+      <c r="I24" s="4" t="n">
+        <v>0.0793</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -14358,7 +14593,10 @@
       <c r="H25" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="I25" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J25" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -14393,6 +14631,9 @@
       <c r="H26" s="4" t="n">
         <v>0.0447</v>
       </c>
+      <c r="I26" s="4" t="n">
+        <v>0.0447</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -14423,6 +14664,9 @@
       <c r="H27" s="4" t="n">
         <v>0.0372</v>
       </c>
+      <c r="I27" s="4" t="n">
+        <v>0.039</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -14453,6 +14697,9 @@
       <c r="H28" s="4" t="n">
         <v>0.0213</v>
       </c>
+      <c r="I28" s="4" t="n">
+        <v>0.0213</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -14480,6 +14727,9 @@
       <c r="H29" s="4" t="n">
         <v>0.0454</v>
       </c>
+      <c r="I29" s="4" t="n">
+        <v>0.0454</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -14507,6 +14757,9 @@
       <c r="H30" s="4" t="n">
         <v>0.0146</v>
       </c>
+      <c r="I30" s="4" t="n">
+        <v>0.0152</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -14534,6 +14787,9 @@
       <c r="H31" s="4" t="n">
         <v>0.021</v>
       </c>
+      <c r="I31" s="4" t="n">
+        <v>0.021</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -14558,6 +14814,9 @@
       <c r="H32" s="4" t="n">
         <v>0.0014</v>
       </c>
+      <c r="I32" s="4" t="n">
+        <v>0.0014</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -14586,6 +14845,10 @@
         <f>SUM(H23:H32)</f>
         <v/>
       </c>
+      <c r="I33" s="5">
+        <f>SUM(I23:I32)</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -14616,6 +14879,9 @@
       <c r="H34" s="4" t="n">
         <v>0.0832</v>
       </c>
+      <c r="I34" s="4" t="n">
+        <v>0.08349999999999999</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -14646,6 +14912,9 @@
       <c r="H35" s="4" t="n">
         <v>0.3459</v>
       </c>
+      <c r="I35" s="4" t="n">
+        <v>0.3459</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -14673,6 +14942,9 @@
       <c r="H36" s="4" t="n">
         <v>0.0007000000000000001</v>
       </c>
+      <c r="I36" s="4" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -14701,6 +14973,10 @@
         <f>SUM(H34:H36)</f>
         <v/>
       </c>
+      <c r="I37" s="5">
+        <f>SUM(I34:I36)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -14731,6 +15007,9 @@
       <c r="H38" s="4" t="n">
         <v>0.0025</v>
       </c>
+      <c r="I38" s="4" t="n">
+        <v>0.0025</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -14761,6 +15040,9 @@
       <c r="H39" s="4" t="n">
         <v>0.2419</v>
       </c>
+      <c r="I39" s="4" t="n">
+        <v>0.2441</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -14791,6 +15073,9 @@
       <c r="H40" s="4" t="n">
         <v>0.1545</v>
       </c>
+      <c r="I40" s="4" t="n">
+        <v>0.1549</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -14821,6 +15106,9 @@
       <c r="H41" s="4" t="n">
         <v>0.0035</v>
       </c>
+      <c r="I41" s="4" t="n">
+        <v>0.0035</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -14851,6 +15139,9 @@
       <c r="H42" s="4" t="n">
         <v>0.0104</v>
       </c>
+      <c r="I42" s="4" t="n">
+        <v>0.0105</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -14881,6 +15172,9 @@
       <c r="H43" s="4" t="n">
         <v>0.03759999999999999</v>
       </c>
+      <c r="I43" s="4" t="n">
+        <v>0.0546</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -14908,6 +15202,9 @@
       <c r="H44" s="4" t="n">
         <v>0.006500000000000001</v>
       </c>
+      <c r="I44" s="4" t="n">
+        <v>0.0066</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -14935,6 +15232,9 @@
       <c r="H45" s="4" t="n">
         <v>0.1435</v>
       </c>
+      <c r="I45" s="4" t="n">
+        <v>0.2085</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -14959,6 +15259,9 @@
       <c r="H46" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="I46" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -14983,6 +15286,9 @@
       <c r="H47" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="I47" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -15007,6 +15313,9 @@
       <c r="H48" s="4" t="n">
         <v>0.0022</v>
       </c>
+      <c r="I48" s="4" t="n">
+        <v>0.0022</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -15031,6 +15340,9 @@
       <c r="H49" s="4" t="n">
         <v>0.0004</v>
       </c>
+      <c r="I49" s="4" t="n">
+        <v>0.0004</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -15055,6 +15367,9 @@
       <c r="H50" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="I50" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -15076,6 +15391,9 @@
       <c r="H51" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="I51" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -15097,6 +15415,9 @@
       <c r="H52" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="I52" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -15106,54 +15427,49 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E53" s="5">
-        <f>SUM(E38:E52)</f>
-        <v/>
-      </c>
-      <c r="F53" s="5">
-        <f>SUM(F38:F52)</f>
-        <v/>
-      </c>
-      <c r="G53" s="5">
-        <f>SUM(G38:G52)</f>
-        <v/>
-      </c>
-      <c r="H53" s="5">
-        <f>SUM(H38:H52)</f>
-        <v/>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="n">
+        <v>8750300</v>
+      </c>
+      <c r="D53" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="I53" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="C54" s="3" t="n">
-        <v>16514800</v>
-      </c>
-      <c r="D54" s="4" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="E54" s="4" t="n">
-        <v>0.0029</v>
-      </c>
-      <c r="F54" s="4" t="n">
-        <v>0.0029</v>
-      </c>
-      <c r="G54" s="4" t="n">
-        <v>0.0029</v>
-      </c>
-      <c r="H54" s="4" t="n">
-        <v>0.0325</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E54" s="5">
+        <f>SUM(E38:E53)</f>
+        <v/>
+      </c>
+      <c r="F54" s="5">
+        <f>SUM(F38:F53)</f>
+        <v/>
+      </c>
+      <c r="G54" s="5">
+        <f>SUM(G38:G53)</f>
+        <v/>
+      </c>
+      <c r="H54" s="5">
+        <f>SUM(H38:H53)</f>
+        <v/>
+      </c>
+      <c r="I54" s="5">
+        <f>SUM(I38:I53)</f>
+        <v/>
       </c>
     </row>
     <row r="55">
@@ -15164,7 +15480,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C55" s="3" t="n">
@@ -15174,16 +15490,19 @@
         <v>0.59</v>
       </c>
       <c r="E55" s="4" t="n">
-        <v>0.0339</v>
+        <v>0.0029</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>0.0339</v>
+        <v>0.0029</v>
       </c>
       <c r="G55" s="4" t="n">
-        <v>0.0339</v>
+        <v>0.0029</v>
       </c>
       <c r="H55" s="4" t="n">
-        <v>0.0339</v>
+        <v>0.0325</v>
+      </c>
+      <c r="I55" s="4" t="n">
+        <v>0.0898</v>
       </c>
     </row>
     <row r="56">
@@ -15194,7 +15513,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C56" s="3" t="n">
@@ -15204,16 +15523,19 @@
         <v>0.59</v>
       </c>
       <c r="E56" s="4" t="n">
-        <v>0.4926</v>
+        <v>0.0339</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>0.4926</v>
+        <v>0.0339</v>
       </c>
       <c r="G56" s="4" t="n">
-        <v>0.4926</v>
+        <v>0.0339</v>
       </c>
       <c r="H56" s="4" t="n">
-        <v>0.4926</v>
+        <v>0.0339</v>
+      </c>
+      <c r="I56" s="4" t="n">
+        <v>0.04269999999999999</v>
       </c>
     </row>
     <row r="57">
@@ -15224,7 +15546,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C57" s="3" t="n">
@@ -15234,16 +15556,19 @@
         <v>0.59</v>
       </c>
       <c r="E57" s="4" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.4926</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>0.0146</v>
+        <v>0.4926</v>
       </c>
       <c r="G57" s="4" t="n">
-        <v>0.0161</v>
+        <v>0.4926</v>
       </c>
       <c r="H57" s="4" t="n">
-        <v>0.0161</v>
+        <v>0.4926</v>
+      </c>
+      <c r="I57" s="4" t="n">
+        <v>0.4926</v>
       </c>
     </row>
     <row r="58">
@@ -15254,7 +15579,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C58" s="3" t="n">
@@ -15263,11 +15588,20 @@
       <c r="D58" s="4" t="n">
         <v>0.59</v>
       </c>
+      <c r="E58" s="4" t="n">
+        <v>0.008800000000000001</v>
+      </c>
+      <c r="F58" s="4" t="n">
+        <v>0.0146</v>
+      </c>
       <c r="G58" s="4" t="n">
-        <v>0.0044</v>
+        <v>0.0161</v>
       </c>
       <c r="H58" s="4" t="n">
-        <v>0.0044</v>
+        <v>0.0161</v>
+      </c>
+      <c r="I58" s="4" t="n">
+        <v>0.0161</v>
       </c>
     </row>
     <row r="59">
@@ -15278,54 +15612,55 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E59" s="5">
-        <f>SUM(E54:E58)</f>
-        <v/>
-      </c>
-      <c r="F59" s="5">
-        <f>SUM(F54:F58)</f>
-        <v/>
-      </c>
-      <c r="G59" s="5">
-        <f>SUM(G54:G58)</f>
-        <v/>
-      </c>
-      <c r="H59" s="5">
-        <f>SUM(H54:H58)</f>
-        <v/>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="n">
+        <v>16514800</v>
+      </c>
+      <c r="D59" s="4" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="G59" s="4" t="n">
+        <v>0.0044</v>
+      </c>
+      <c r="H59" s="4" t="n">
+        <v>0.0044</v>
+      </c>
+      <c r="I59" s="4" t="n">
+        <v>0.0044</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="C60" s="3" t="n">
-        <v>3467600</v>
-      </c>
-      <c r="D60" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="E60" s="4" t="n">
-        <v>0.0004</v>
-      </c>
-      <c r="F60" s="4" t="n">
-        <v>0.0021</v>
-      </c>
-      <c r="G60" s="4" t="n">
-        <v>0.0021</v>
-      </c>
-      <c r="H60" s="4" t="n">
-        <v>0.0021</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E60" s="5">
+        <f>SUM(E55:E59)</f>
+        <v/>
+      </c>
+      <c r="F60" s="5">
+        <f>SUM(F55:F59)</f>
+        <v/>
+      </c>
+      <c r="G60" s="5">
+        <f>SUM(G55:G59)</f>
+        <v/>
+      </c>
+      <c r="H60" s="5">
+        <f>SUM(H55:H59)</f>
+        <v/>
+      </c>
+      <c r="I60" s="5">
+        <f>SUM(I55:I59)</f>
+        <v/>
       </c>
     </row>
     <row r="61">
@@ -15336,7 +15671,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C61" s="3" t="n">
@@ -15346,16 +15681,19 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E61" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.0004</v>
       </c>
       <c r="F61" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.0021</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.0021</v>
       </c>
       <c r="H61" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.0021</v>
+      </c>
+      <c r="I61" s="4" t="n">
+        <v>0.0021</v>
       </c>
     </row>
     <row r="62">
@@ -15366,7 +15704,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C62" s="3" t="n">
@@ -15376,16 +15714,19 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E62" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0032</v>
       </c>
       <c r="F62" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0032</v>
       </c>
       <c r="G62" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0032</v>
       </c>
       <c r="H62" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0032</v>
+      </c>
+      <c r="I62" s="4" t="n">
+        <v>0.0032</v>
       </c>
     </row>
     <row r="63">
@@ -15396,7 +15737,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C63" s="3" t="n">
@@ -15406,21 +15747,19 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E63" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.0204</v>
       </c>
       <c r="F63" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.0204</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.0204</v>
       </c>
       <c r="H63" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
+        <v>0.0204</v>
+      </c>
+      <c r="I63" s="4" t="n">
+        <v>0.0204</v>
       </c>
     </row>
     <row r="64">
@@ -15431,7 +15770,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C64" s="3" t="n">
@@ -15441,16 +15780,24 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E64" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G64" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H64" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="I64" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
       </c>
     </row>
     <row r="65">
@@ -15461,7 +15808,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C65" s="3" t="n">
@@ -15471,16 +15818,19 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E65" s="4" t="n">
-        <v>0.1798</v>
+        <v>0.0004</v>
       </c>
       <c r="F65" s="4" t="n">
-        <v>0.1798</v>
+        <v>0.0004</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>0.2828</v>
+        <v>0.0004</v>
       </c>
       <c r="H65" s="4" t="n">
-        <v>0.2828</v>
+        <v>0.0004</v>
+      </c>
+      <c r="I65" s="4" t="n">
+        <v>0.0004</v>
       </c>
     </row>
     <row r="66">
@@ -15491,7 +15841,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C66" s="3" t="n">
@@ -15500,14 +15850,20 @@
       <c r="D66" s="4" t="n">
         <v>0.6899999999999999</v>
       </c>
+      <c r="E66" s="4" t="n">
+        <v>0.1798</v>
+      </c>
       <c r="F66" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.1798</v>
       </c>
       <c r="G66" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.2828</v>
       </c>
       <c r="H66" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.2828</v>
+      </c>
+      <c r="I66" s="4" t="n">
+        <v>0.2828</v>
       </c>
     </row>
     <row r="67">
@@ -15518,7 +15874,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Luxembourg</t>
         </is>
       </c>
       <c r="C67" s="3" t="n">
@@ -15527,11 +15883,17 @@
       <c r="D67" s="4" t="n">
         <v>0.6899999999999999</v>
       </c>
+      <c r="F67" s="4" t="n">
+        <v>0.0012</v>
+      </c>
       <c r="G67" s="4" t="n">
-        <v>0</v>
+        <v>0.0012</v>
       </c>
       <c r="H67" s="4" t="n">
-        <v>0</v>
+        <v>0.0012</v>
+      </c>
+      <c r="I67" s="4" t="n">
+        <v>0.0012</v>
       </c>
     </row>
     <row r="68">
@@ -15542,23 +15904,54 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D68" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G68" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E68" s="5">
-        <f>SUM(E60:E67)</f>
-        <v/>
-      </c>
-      <c r="F68" s="5">
-        <f>SUM(F60:F67)</f>
-        <v/>
-      </c>
-      <c r="G68" s="5">
-        <f>SUM(G60:G67)</f>
-        <v/>
-      </c>
-      <c r="H68" s="5">
-        <f>SUM(H60:H67)</f>
+      <c r="E69" s="5">
+        <f>SUM(E61:E68)</f>
+        <v/>
+      </c>
+      <c r="F69" s="5">
+        <f>SUM(F61:F68)</f>
+        <v/>
+      </c>
+      <c r="G69" s="5">
+        <f>SUM(G61:G68)</f>
+        <v/>
+      </c>
+      <c r="H69" s="5">
+        <f>SUM(H61:H68)</f>
+        <v/>
+      </c>
+      <c r="I69" s="5">
+        <f>SUM(I61:I68)</f>
         <v/>
       </c>
     </row>
@@ -15573,7 +15966,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15702,17 +16095,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>1552.69</v>
+        <v>39.64</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>2269.02</v>
+        <v>48.29</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>1461.347725560157</v>
+        <v>1218.213925327952</v>
       </c>
     </row>
     <row r="13">
@@ -15723,17 +16116,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>3989.900000000001</v>
+        <v>1552.69</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>3366.49</v>
+        <v>2269.02</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>843.7529762650692</v>
+        <v>1461.347725560157</v>
       </c>
     </row>
     <row r="14">
@@ -15744,17 +16137,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>0.02</v>
+        <v>4071.71</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>0.09</v>
+        <v>3434.38</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>4500</v>
+        <v>843.4736265598482</v>
       </c>
     </row>
     <row r="15">
@@ -15765,17 +16158,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>41.91</v>
+        <v>0.02</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>31.74</v>
+        <v>0.09</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>757.3371510379385</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="16">
@@ -15786,38 +16179,38 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>2604.53</v>
+        <v>41.91</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>4528.89</v>
+        <v>31.74</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1738.851155486787</v>
+        <v>757.3371510379385</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Steel Plate</t>
+          <t>Hot-Rolled Sheet</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>81.29000000000001</v>
+        <v>4262.799999999999</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>282.07</v>
+        <v>7312.120000000001</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>3469.922499692459</v>
+        <v>1715.332645209722</v>
       </c>
     </row>
     <row r="18">
@@ -15828,17 +16221,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>8.279999999999999</v>
+        <v>81.29000000000001</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>15.27</v>
+        <v>282.07</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1844.202898550725</v>
+        <v>3469.922499692459</v>
       </c>
     </row>
     <row r="19">
@@ -15849,17 +16242,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>54.64</v>
+        <v>54.23</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>126.5</v>
+        <v>57.19</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>2315.153733528551</v>
+        <v>1054.582334501199</v>
       </c>
     </row>
     <row r="20">
@@ -15870,17 +16263,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>315.28</v>
+        <v>354.8699999999999</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>680.3200000000001</v>
+        <v>1531.98</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>2157.82796244608</v>
+        <v>4317.017499365965</v>
       </c>
     </row>
     <row r="21">
@@ -15891,17 +16284,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>7463.45</v>
+        <v>54.64</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>8994.029999999999</v>
+        <v>126.5</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>1205.076740649431</v>
+        <v>2315.153733528551</v>
       </c>
     </row>
     <row r="22">
@@ -15912,17 +16305,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>16.61</v>
+        <v>1507.27</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>25.17</v>
+        <v>3411.48</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>1515.352197471403</v>
+        <v>2263.350295567483</v>
       </c>
     </row>
     <row r="23">
@@ -15933,17 +16326,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>25.68</v>
+        <v>8243.16</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>34.82</v>
+        <v>9949.52</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>1355.919003115265</v>
+        <v>1207.003139572688</v>
       </c>
     </row>
     <row r="24">
@@ -15954,59 +16347,59 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>1724.58</v>
+        <v>32.77</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>3694.98</v>
+        <v>72.72999999999999</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>2142.539052986815</v>
+        <v>2219.407995117485</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Cold-Rolled Sheet</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C25" s="6" t="n">
-        <v>7.15</v>
+        <v>25.68</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>16.26</v>
+        <v>34.82</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>2274.125874125874</v>
+        <v>1355.919003115265</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Cold-Rolled Sheet</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>0</v>
+        <v>2600.28</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>0.03</v>
+        <v>5688.669999999999</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>0</v>
+        <v>2187.714399987693</v>
       </c>
     </row>
     <row r="27">
@@ -16017,17 +16410,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>154.64</v>
+        <v>8.709999999999999</v>
       </c>
       <c r="D27" s="6" t="n">
-        <v>180.58</v>
+        <v>20.06</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>1167.744438696327</v>
+        <v>2303.099885189438</v>
       </c>
     </row>
     <row r="28">
@@ -16038,17 +16431,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>1425.92</v>
+        <v>741.5</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>1699.87</v>
+        <v>1138.12</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>1192.121577648115</v>
+        <v>1534.888739042481</v>
       </c>
     </row>
     <row r="29">
@@ -16059,17 +16452,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>0.04</v>
+        <v>230.06</v>
       </c>
       <c r="D29" s="6" t="n">
-        <v>0.19</v>
+        <v>299.02</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>4750</v>
+        <v>1299.747891854299</v>
       </c>
     </row>
     <row r="30">
@@ -16080,80 +16473,80 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>2462.55</v>
+        <v>1425.92</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>4557.640000000001</v>
+        <v>1699.87</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>1850.780694808228</v>
+        <v>1192.121577648115</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C31" s="6" t="n">
-        <v>1099.45</v>
+        <v>0.04</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>1768.94</v>
+        <v>0.19</v>
       </c>
       <c r="E31" s="6" t="n">
-        <v>1608.931738596571</v>
+        <v>4750</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>566.6999999999999</v>
+        <v>1520.24</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>781.8299999999999</v>
+        <v>1562.54</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>1379.618845950238</v>
+        <v>1027.824554017787</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C33" s="6" t="n">
-        <v>40.24</v>
+        <v>3460.769999999999</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>88.01000000000001</v>
+        <v>6425.440000000001</v>
       </c>
       <c r="E33" s="6" t="n">
-        <v>2187.127236580517</v>
+        <v>1856.650398610715</v>
       </c>
     </row>
     <row r="34">
@@ -16164,17 +16557,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="C34" s="6" t="n">
-        <v>2897.2</v>
+        <v>6.44</v>
       </c>
       <c r="D34" s="6" t="n">
-        <v>5530.73</v>
+        <v>38.19</v>
       </c>
       <c r="E34" s="6" t="n">
-        <v>1908.991440011045</v>
+        <v>5930.124223602485</v>
       </c>
     </row>
     <row r="35">
@@ -16185,17 +16578,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C35" s="6" t="n">
-        <v>246.5</v>
+        <v>1110.32</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>602.38</v>
+        <v>1790.26</v>
       </c>
       <c r="E35" s="6" t="n">
-        <v>2443.732251521298</v>
+        <v>1612.382015995388</v>
       </c>
     </row>
     <row r="36">
@@ -16206,17 +16599,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C36" s="6" t="n">
-        <v>267.58</v>
+        <v>582.0599999999999</v>
       </c>
       <c r="D36" s="6" t="n">
-        <v>474.55</v>
+        <v>728.85</v>
       </c>
       <c r="E36" s="6" t="n">
-        <v>1773.488302563719</v>
+        <v>1252.190495825173</v>
       </c>
     </row>
     <row r="37">
@@ -16227,17 +16620,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C37" s="6" t="n">
-        <v>5178.2</v>
+        <v>40.24</v>
       </c>
       <c r="D37" s="6" t="n">
-        <v>8867.09</v>
+        <v>88.01000000000001</v>
       </c>
       <c r="E37" s="6" t="n">
-        <v>1712.388474759569</v>
+        <v>2187.127236580517</v>
       </c>
     </row>
     <row r="38">
@@ -16248,17 +16641,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C38" s="6" t="n">
-        <v>87.97</v>
+        <v>2907.21</v>
       </c>
       <c r="D38" s="6" t="n">
-        <v>180.34</v>
+        <v>5548.78</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>2050.017051267478</v>
+        <v>1908.627171755738</v>
       </c>
     </row>
     <row r="39">
@@ -16269,17 +16662,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C39" s="6" t="n">
-        <v>284.88</v>
+        <v>246.5</v>
       </c>
       <c r="D39" s="6" t="n">
-        <v>577.25</v>
+        <v>602.38</v>
       </c>
       <c r="E39" s="6" t="n">
-        <v>2026.291771974165</v>
+        <v>2443.732251521298</v>
       </c>
     </row>
     <row r="40">
@@ -16290,17 +16683,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C40" s="6" t="n">
-        <v>1922.54</v>
+        <v>409.57</v>
       </c>
       <c r="D40" s="6" t="n">
-        <v>2374.78</v>
+        <v>751.4299999999999</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>1235.230476348996</v>
+        <v>1834.680274434163</v>
       </c>
     </row>
     <row r="41">
@@ -16311,17 +16704,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C41" s="6" t="n">
-        <v>0.12</v>
+        <v>9983.290000000001</v>
       </c>
       <c r="D41" s="6" t="n">
-        <v>0.25</v>
+        <v>15988.71</v>
       </c>
       <c r="E41" s="6" t="n">
-        <v>2083.333333333333</v>
+        <v>1601.547185346714</v>
       </c>
     </row>
     <row r="42">
@@ -16332,17 +16725,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C42" s="6" t="n">
-        <v>2785.19</v>
+        <v>87.97</v>
       </c>
       <c r="D42" s="6" t="n">
-        <v>4035.09</v>
+        <v>180.34</v>
       </c>
       <c r="E42" s="6" t="n">
-        <v>1448.766511440871</v>
+        <v>2050.017051267478</v>
       </c>
     </row>
     <row r="43">
@@ -16353,17 +16746,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C43" s="6" t="n">
-        <v>6358.75</v>
+        <v>284.88</v>
       </c>
       <c r="D43" s="6" t="n">
-        <v>13217.57</v>
+        <v>577.25</v>
       </c>
       <c r="E43" s="6" t="n">
-        <v>2078.642815018675</v>
+        <v>2026.291771974165</v>
       </c>
     </row>
     <row r="44">
@@ -16374,248 +16767,248 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="C44" s="6" t="n">
-        <v>799.97</v>
+        <v>3311.71</v>
       </c>
       <c r="D44" s="6" t="n">
-        <v>1173.88</v>
+        <v>4170.44</v>
       </c>
       <c r="E44" s="6" t="n">
-        <v>1467.405027688538</v>
+        <v>1259.301086145828</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C45" s="6" t="n">
-        <v>19.72</v>
+        <v>0.12</v>
       </c>
       <c r="D45" s="6" t="n">
-        <v>39.63</v>
+        <v>0.25</v>
       </c>
       <c r="E45" s="6" t="n">
-        <v>2009.634888438134</v>
+        <v>2083.333333333333</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C46" s="6" t="n">
-        <v>1213.79</v>
+        <v>3666.65</v>
       </c>
       <c r="D46" s="6" t="n">
-        <v>956.79</v>
+        <v>5877.52</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>788.2665040904934</v>
+        <v>1602.967286214938</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C47" s="6" t="n">
-        <v>1175.59</v>
+        <v>23.05</v>
       </c>
       <c r="D47" s="6" t="n">
-        <v>1819.18</v>
+        <v>29.59</v>
       </c>
       <c r="E47" s="6" t="n">
-        <v>1547.461274764161</v>
+        <v>1283.731019522776</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C48" s="6" t="n">
-        <v>100.42</v>
+        <v>1412.89</v>
       </c>
       <c r="D48" s="6" t="n">
-        <v>161.19</v>
+        <v>1664.87</v>
       </c>
       <c r="E48" s="6" t="n">
-        <v>1605.158334993029</v>
+        <v>1178.343678559548</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C49" s="6" t="n">
-        <v>18.95</v>
+        <v>0.63</v>
       </c>
       <c r="D49" s="6" t="n">
-        <v>43.36</v>
+        <v>1.37</v>
       </c>
       <c r="E49" s="6" t="n">
-        <v>2288.126649076517</v>
+        <v>2174.603174603174</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C50" s="6" t="n">
-        <v>25.53</v>
+        <v>9998.359999999999</v>
       </c>
       <c r="D50" s="6" t="n">
-        <v>46.35</v>
+        <v>20823.45</v>
       </c>
       <c r="E50" s="6" t="n">
-        <v>1815.51116333725</v>
+        <v>2082.686560595938</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C51" s="6" t="n">
-        <v>6.84</v>
+        <v>1147.37</v>
       </c>
       <c r="D51" s="6" t="n">
-        <v>30.16</v>
+        <v>1533.44</v>
       </c>
       <c r="E51" s="6" t="n">
-        <v>4409.356725146199</v>
+        <v>1336.482564473535</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="C52" s="6" t="n">
-        <v>0.01</v>
+        <v>19.72</v>
       </c>
       <c r="D52" s="6" t="n">
-        <v>0.01</v>
+        <v>39.63</v>
       </c>
       <c r="E52" s="6" t="n">
-        <v>1000</v>
+        <v>2009.634888438134</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C53" s="6" t="n">
-        <v>229.71</v>
+        <v>1721.39</v>
       </c>
       <c r="D53" s="6" t="n">
-        <v>344.33</v>
+        <v>1312.5</v>
       </c>
       <c r="E53" s="6" t="n">
-        <v>1498.976970963388</v>
+        <v>762.465217062955</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C54" s="6" t="n">
-        <v>0.01</v>
+        <v>2348.38</v>
       </c>
       <c r="D54" s="6" t="n">
-        <v>1.14</v>
+        <v>3384.33</v>
       </c>
       <c r="E54" s="6" t="n">
-        <v>114000</v>
+        <v>1441.133888041969</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C55" s="6" t="n">
-        <v>238.1</v>
+        <v>212.86</v>
       </c>
       <c r="D55" s="6" t="n">
-        <v>256.29</v>
+        <v>318.99</v>
       </c>
       <c r="E55" s="6" t="n">
-        <v>1076.396472070558</v>
+        <v>1498.590622944658</v>
       </c>
     </row>
     <row r="56">
@@ -16626,227 +17019,227 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C56" s="6" t="n">
-        <v>529.3099999999999</v>
+        <v>60.87</v>
       </c>
       <c r="D56" s="6" t="n">
-        <v>1075.13</v>
+        <v>132.23</v>
       </c>
       <c r="E56" s="6" t="n">
-        <v>2031.191551264855</v>
+        <v>2172.334483325119</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C57" s="6" t="n">
-        <v>22.6</v>
+        <v>25.53</v>
       </c>
       <c r="D57" s="6" t="n">
-        <v>32.51</v>
+        <v>46.35</v>
       </c>
       <c r="E57" s="6" t="n">
-        <v>1438.495575221239</v>
+        <v>1815.51116333725</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C58" s="6" t="n">
-        <v>72.62</v>
+        <v>112.54</v>
       </c>
       <c r="D58" s="6" t="n">
-        <v>98.56999999999999</v>
+        <v>228.5</v>
       </c>
       <c r="E58" s="6" t="n">
-        <v>1357.339575874415</v>
+        <v>2030.389194952905</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C59" s="6" t="n">
-        <v>887.39</v>
+        <v>0.01</v>
       </c>
       <c r="D59" s="6" t="n">
-        <v>1419.21</v>
+        <v>0.01</v>
       </c>
       <c r="E59" s="6" t="n">
-        <v>1599.308083255389</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C60" s="6" t="n">
-        <v>70.04000000000001</v>
+        <v>273.6</v>
       </c>
       <c r="D60" s="6" t="n">
-        <v>58.8</v>
+        <v>410.07</v>
       </c>
       <c r="E60" s="6" t="n">
-        <v>839.5202741290691</v>
+        <v>1498.793859649123</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C61" s="6" t="n">
-        <v>3.75</v>
+        <v>48.36</v>
       </c>
       <c r="D61" s="6" t="n">
-        <v>11.03</v>
+        <v>97.23999999999999</v>
       </c>
       <c r="E61" s="6" t="n">
-        <v>2941.333333333333</v>
+        <v>2010.752688172043</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C62" s="6" t="n">
-        <v>8</v>
+        <v>278.34</v>
       </c>
       <c r="D62" s="6" t="n">
-        <v>8.73</v>
+        <v>281.93</v>
       </c>
       <c r="E62" s="6" t="n">
-        <v>1091.25</v>
+        <v>1012.897894661206</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C63" s="6" t="n">
-        <v>3325.32</v>
+        <v>1037.32</v>
       </c>
       <c r="D63" s="6" t="n">
-        <v>5482.570000000001</v>
+        <v>2204.18</v>
       </c>
       <c r="E63" s="6" t="n">
-        <v>1648.734557877137</v>
+        <v>2124.879497165774</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C64" s="6" t="n">
-        <v>2311.129999999999</v>
+        <v>968.02</v>
       </c>
       <c r="D64" s="6" t="n">
-        <v>3533.67</v>
+        <v>1201.9</v>
       </c>
       <c r="E64" s="6" t="n">
-        <v>1528.979330457396</v>
+        <v>1241.60657837648</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C65" s="6" t="n">
-        <v>6037.94</v>
+        <v>72.62</v>
       </c>
       <c r="D65" s="6" t="n">
-        <v>6900.929999999999</v>
+        <v>98.56999999999999</v>
       </c>
       <c r="E65" s="6" t="n">
-        <v>1142.927886000854</v>
+        <v>1357.339575874415</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C66" s="6" t="n">
-        <v>436.41</v>
+        <v>2059.47</v>
       </c>
       <c r="D66" s="6" t="n">
-        <v>496.74</v>
+        <v>3323.92</v>
       </c>
       <c r="E66" s="6" t="n">
-        <v>1138.241561834055</v>
+        <v>1613.968642417709</v>
       </c>
     </row>
     <row r="67">
@@ -16857,17 +17250,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C67" s="6" t="n">
-        <v>1447.37</v>
+        <v>70.03</v>
       </c>
       <c r="D67" s="6" t="n">
-        <v>3666.469999999999</v>
+        <v>58.73</v>
       </c>
       <c r="E67" s="6" t="n">
-        <v>2533.194691060337</v>
+        <v>838.640582607454</v>
       </c>
     </row>
     <row r="68">
@@ -16878,17 +17271,227 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="D68" s="6" t="n">
+        <v>64.56999999999999</v>
+      </c>
+      <c r="E68" s="6" t="n">
+        <v>2646.311475409836</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="n">
+        <v>54.89</v>
+      </c>
+      <c r="D69" s="6" t="n">
+        <v>80.14</v>
+      </c>
+      <c r="E69" s="6" t="n">
+        <v>1460.010930952815</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Korea, Republic of</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="n">
+        <v>22943.82</v>
+      </c>
+      <c r="D70" s="6" t="n">
+        <v>23796.01</v>
+      </c>
+      <c r="E70" s="6" t="n">
+        <v>1037.142463635088</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Luxembourg</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="n">
+        <v>3325.32</v>
+      </c>
+      <c r="D71" s="6" t="n">
+        <v>5482.570000000001</v>
+      </c>
+      <c r="E71" s="6" t="n">
+        <v>1648.734557877137</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="n">
+        <v>2674.93</v>
+      </c>
+      <c r="D72" s="6" t="n">
+        <v>4081.2</v>
+      </c>
+      <c r="E72" s="6" t="n">
+        <v>1525.722168430576</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D73" s="6" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="E73" s="6" t="n">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="n">
+        <v>6088.31</v>
+      </c>
+      <c r="D74" s="6" t="n">
+        <v>7011.77</v>
+      </c>
+      <c r="E74" s="6" t="n">
+        <v>1151.677559125603</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="n">
+        <v>103.74</v>
+      </c>
+      <c r="D75" s="6" t="n">
+        <v>101.29</v>
+      </c>
+      <c r="E75" s="6" t="n">
+        <v>976.3832658569498</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="n">
+        <v>621.55</v>
+      </c>
+      <c r="D76" s="6" t="n">
+        <v>930.3099999999999</v>
+      </c>
+      <c r="E76" s="6" t="n">
+        <v>1496.758104738155</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="n">
+        <v>2380.89</v>
+      </c>
+      <c r="D77" s="6" t="n">
+        <v>6171.320000000001</v>
+      </c>
+      <c r="E77" s="6" t="n">
+        <v>2592.022310984548</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
           <t>Vietnam</t>
         </is>
       </c>
-      <c r="C68" s="6" t="n">
-        <v>307.36</v>
-      </c>
-      <c r="D68" s="6" t="n">
-        <v>258.04</v>
-      </c>
-      <c r="E68" s="6" t="n">
-        <v>839.5366996356065</v>
+      <c r="C78" s="6" t="n">
+        <v>403.97</v>
+      </c>
+      <c r="D78" s="6" t="n">
+        <v>338.95</v>
+      </c>
+      <c r="E78" s="6" t="n">
+        <v>839.0474540188627</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Weekly TRQ update 2026-08-02
</commit_message>
<xml_diff>
--- a/data/canada_trq_tracker.xlsx
+++ b/data/canada_trq_tracker.xlsx
@@ -12390,7 +12390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12441,7 +12441,12 @@
           <t>July 27 2026</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="1" t="inlineStr">
+        <is>
+          <t>August 2 2026</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
@@ -12479,11 +12484,6 @@
       <c r="I3" s="4" t="n">
         <v>0.41</v>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -12570,6 +12570,10 @@
         <f>SUM(I3:I5)</f>
         <v/>
       </c>
+      <c r="J6" s="5">
+        <f>SUM(J3:J5)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -12662,6 +12666,10 @@
         <f>SUM(I7:I8)</f>
         <v/>
       </c>
+      <c r="J9" s="5">
+        <f>SUM(J7:J8)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -12937,6 +12945,10 @@
         <f>SUM(I10:I17)</f>
         <v/>
       </c>
+      <c r="J18" s="5">
+        <f>SUM(J10:J17)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -13197,6 +13209,10 @@
         <f>SUM(I19:I25)</f>
         <v/>
       </c>
+      <c r="J26" s="5">
+        <f>SUM(J19:J25)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -13385,6 +13401,10 @@
         <f>SUM(I27:I31)</f>
         <v/>
       </c>
+      <c r="J32" s="5">
+        <f>SUM(J27:J31)</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -13451,11 +13471,6 @@
       <c r="I34" s="4" t="n">
         <v>0.42</v>
       </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -13489,11 +13504,6 @@
       <c r="I35" s="4" t="n">
         <v>0.42</v>
       </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -13556,6 +13566,10 @@
         <f>SUM(I33:I36)</f>
         <v/>
       </c>
+      <c r="J37" s="5">
+        <f>SUM(J33:J36)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -13609,6 +13623,10 @@
         <f>SUM(I38:I38)</f>
         <v/>
       </c>
+      <c r="J39" s="5">
+        <f>SUM(J38:J38)</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -13771,6 +13789,10 @@
       </c>
       <c r="I44" s="5">
         <f>SUM(I40:I43)</f>
+        <v/>
+      </c>
+      <c r="J44" s="5">
+        <f>SUM(J40:J43)</f>
         <v/>
       </c>
     </row>
@@ -13785,7 +13807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:K69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13836,7 +13858,12 @@
           <t>July 27 2026</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="1" t="inlineStr">
+        <is>
+          <t>August 2 2026</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
@@ -13939,6 +13966,10 @@
         <f>SUM(I3:I4)</f>
         <v/>
       </c>
+      <c r="J5" s="5">
+        <f>SUM(J3:J4)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -14203,11 +14234,6 @@
       <c r="I13" s="4" t="n">
         <v>0.33</v>
       </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -14336,6 +14362,10 @@
         <f>SUM(I6:I16)</f>
         <v/>
       </c>
+      <c r="J17" s="5">
+        <f>SUM(J6:J16)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -14497,6 +14527,10 @@
         <f>SUM(I18:I21)</f>
         <v/>
       </c>
+      <c r="J22" s="5">
+        <f>SUM(J18:J21)</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -14596,11 +14630,6 @@
       <c r="I25" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -14849,6 +14878,10 @@
         <f>SUM(I23:I32)</f>
         <v/>
       </c>
+      <c r="J33" s="5">
+        <f>SUM(J23:J32)</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -14977,6 +15010,10 @@
         <f>SUM(I34:I36)</f>
         <v/>
       </c>
+      <c r="J37" s="5">
+        <f>SUM(J34:J36)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -15471,6 +15508,10 @@
         <f>SUM(I38:I53)</f>
         <v/>
       </c>
+      <c r="J54" s="5">
+        <f>SUM(J38:J53)</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -15662,6 +15703,10 @@
         <f>SUM(I55:I59)</f>
         <v/>
       </c>
+      <c r="J60" s="5">
+        <f>SUM(J55:J59)</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -15794,11 +15839,6 @@
       <c r="I64" s="4" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -15952,6 +15992,10 @@
       </c>
       <c r="I69" s="5">
         <f>SUM(I61:I68)</f>
+        <v/>
+      </c>
+      <c r="J69" s="5">
+        <f>SUM(J61:J68)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Weekly TRQ update 2026-08-03
</commit_message>
<xml_diff>
--- a/data/canada_trq_tracker.xlsx
+++ b/data/canada_trq_tracker.xlsx
@@ -12390,7 +12390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12446,7 +12446,12 @@
           <t>August 2 2026</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="1" t="inlineStr">
+        <is>
+          <t>August 3 2026</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
@@ -12484,6 +12489,14 @@
       <c r="I3" s="4" t="n">
         <v>0.41</v>
       </c>
+      <c r="K3" s="4" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -12514,6 +12527,9 @@
       <c r="I4" s="4" t="n">
         <v>0.0301</v>
       </c>
+      <c r="K4" s="4" t="n">
+        <v>0.0333</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -12538,6 +12554,9 @@
       <c r="I5" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="K5" s="4" t="n">
+        <v>0.0003</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -12574,6 +12593,10 @@
         <f>SUM(J3:J5)</f>
         <v/>
       </c>
+      <c r="K6" s="5">
+        <f>SUM(K3:K5)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -12607,6 +12630,9 @@
       <c r="I7" s="4" t="n">
         <v>0.3564</v>
       </c>
+      <c r="K7" s="4" t="n">
+        <v>0.3567</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -12634,6 +12660,9 @@
       <c r="I8" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="K8" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -12670,6 +12699,10 @@
         <f>SUM(J7:J8)</f>
         <v/>
       </c>
+      <c r="K9" s="5">
+        <f>SUM(K7:K8)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -12703,6 +12736,9 @@
       <c r="I10" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="K10" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -12736,6 +12772,9 @@
       <c r="I11" s="4" t="n">
         <v>0.1135</v>
       </c>
+      <c r="K11" s="4" t="n">
+        <v>0.1135</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -12769,6 +12808,9 @@
       <c r="I12" s="4" t="n">
         <v>0.5572</v>
       </c>
+      <c r="K12" s="4" t="n">
+        <v>0.5572</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -12799,6 +12841,9 @@
       <c r="I13" s="4" t="n">
         <v>0.0008</v>
       </c>
+      <c r="K13" s="4" t="n">
+        <v>0.0008</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -12829,6 +12874,9 @@
       <c r="I14" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="K14" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -12859,6 +12907,9 @@
       <c r="I15" s="4" t="n">
         <v>0.3156</v>
       </c>
+      <c r="K15" s="4" t="n">
+        <v>0.3156</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -12886,6 +12937,9 @@
       <c r="I16" s="4" t="n">
         <v>0.0128</v>
       </c>
+      <c r="K16" s="4" t="n">
+        <v>0.0128</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -12913,6 +12967,9 @@
       <c r="I17" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="K17" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -12949,6 +13006,10 @@
         <f>SUM(J10:J17)</f>
         <v/>
       </c>
+      <c r="K18" s="5">
+        <f>SUM(K10:K17)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -12982,6 +13043,9 @@
       <c r="I19" s="4" t="n">
         <v>0.0027</v>
       </c>
+      <c r="K19" s="4" t="n">
+        <v>0.0027</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -13015,6 +13079,9 @@
       <c r="I20" s="4" t="n">
         <v>0.2673</v>
       </c>
+      <c r="K20" s="4" t="n">
+        <v>0.2673</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -13048,6 +13115,9 @@
       <c r="I21" s="4" t="n">
         <v>0.0069</v>
       </c>
+      <c r="K21" s="4" t="n">
+        <v>0.0069</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -13081,6 +13151,9 @@
       <c r="I22" s="4" t="n">
         <v>0.2488</v>
       </c>
+      <c r="K22" s="4" t="n">
+        <v>0.2488</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -13114,6 +13187,9 @@
       <c r="I23" s="4" t="n">
         <v>0.3697</v>
       </c>
+      <c r="K23" s="4" t="n">
+        <v>0.3697</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -13147,6 +13223,9 @@
       <c r="I24" s="4" t="n">
         <v>0.0289</v>
       </c>
+      <c r="K24" s="4" t="n">
+        <v>0.0289</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -13177,6 +13256,9 @@
       <c r="I25" s="4" t="n">
         <v>0.07539999999999999</v>
       </c>
+      <c r="K25" s="4" t="n">
+        <v>0.07539999999999999</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -13213,6 +13295,10 @@
         <f>SUM(J19:J25)</f>
         <v/>
       </c>
+      <c r="K26" s="5">
+        <f>SUM(K19:K25)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -13246,6 +13332,9 @@
       <c r="I27" s="4" t="n">
         <v>0.2747</v>
       </c>
+      <c r="K27" s="4" t="n">
+        <v>0.2747</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -13279,6 +13368,9 @@
       <c r="I28" s="4" t="n">
         <v>0.0037</v>
       </c>
+      <c r="K28" s="4" t="n">
+        <v>0.0037</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -13312,6 +13404,9 @@
       <c r="I29" s="4" t="n">
         <v>0.2899</v>
       </c>
+      <c r="K29" s="4" t="n">
+        <v>0.2899</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -13345,6 +13440,9 @@
       <c r="I30" s="4" t="n">
         <v>0.0883</v>
       </c>
+      <c r="K30" s="4" t="n">
+        <v>0.0883</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -13369,6 +13467,9 @@
       <c r="I31" s="4" t="n">
         <v>0.0038</v>
       </c>
+      <c r="K31" s="4" t="n">
+        <v>0.0038</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -13405,6 +13506,10 @@
         <f>SUM(J27:J31)</f>
         <v/>
       </c>
+      <c r="K32" s="5">
+        <f>SUM(K27:K31)</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -13438,6 +13543,9 @@
       <c r="I33" s="4" t="n">
         <v>0.1576</v>
       </c>
+      <c r="K33" s="4" t="n">
+        <v>0.1576</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -13471,6 +13579,14 @@
       <c r="I34" s="4" t="n">
         <v>0.42</v>
       </c>
+      <c r="K34" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -13504,6 +13620,14 @@
       <c r="I35" s="4" t="n">
         <v>0.42</v>
       </c>
+      <c r="K35" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -13534,6 +13658,9 @@
       <c r="I36" s="4" t="n">
         <v>0.0024</v>
       </c>
+      <c r="K36" s="4" t="n">
+        <v>0.0024</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -13570,6 +13697,10 @@
         <f>SUM(J33:J36)</f>
         <v/>
       </c>
+      <c r="K37" s="5">
+        <f>SUM(K33:K36)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -13591,6 +13722,9 @@
       <c r="I38" s="4" t="n">
         <v>0.0397</v>
       </c>
+      <c r="K38" s="4" t="n">
+        <v>0.2893</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -13600,65 +13734,57 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E39" s="5">
-        <f>SUM(E38:E38)</f>
-        <v/>
-      </c>
-      <c r="F39" s="5">
-        <f>SUM(F38:F38)</f>
-        <v/>
-      </c>
-      <c r="G39" s="5">
-        <f>SUM(G38:G38)</f>
-        <v/>
-      </c>
-      <c r="H39" s="5">
-        <f>SUM(H38:H38)</f>
-        <v/>
-      </c>
-      <c r="I39" s="5">
-        <f>SUM(I38:I38)</f>
-        <v/>
-      </c>
-      <c r="J39" s="5">
-        <f>SUM(J38:J38)</f>
-        <v/>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="n">
+        <v>1571700</v>
+      </c>
+      <c r="D39" s="4" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="K39" s="4" t="n">
+        <v>0.0924</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>India</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="n">
-        <v>3753500</v>
-      </c>
-      <c r="D40" s="4" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="E40" s="4" t="n">
-        <v>0.0218</v>
-      </c>
-      <c r="F40" s="4" t="n">
-        <v>0.0218</v>
-      </c>
-      <c r="G40" s="4" t="n">
-        <v>0.0218</v>
-      </c>
-      <c r="H40" s="4" t="n">
-        <v>0.0218</v>
-      </c>
-      <c r="I40" s="4" t="n">
-        <v>0.0218</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E40" s="5">
+        <f>SUM(E38:E39)</f>
+        <v/>
+      </c>
+      <c r="F40" s="5">
+        <f>SUM(F38:F39)</f>
+        <v/>
+      </c>
+      <c r="G40" s="5">
+        <f>SUM(G38:G39)</f>
+        <v/>
+      </c>
+      <c r="H40" s="5">
+        <f>SUM(H38:H39)</f>
+        <v/>
+      </c>
+      <c r="I40" s="5">
+        <f>SUM(I38:I39)</f>
+        <v/>
+      </c>
+      <c r="J40" s="5">
+        <f>SUM(J38:J39)</f>
+        <v/>
+      </c>
+      <c r="K40" s="5">
+        <f>SUM(K38:K39)</f>
+        <v/>
       </c>
     </row>
     <row r="41">
@@ -13669,7 +13795,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C41" s="3" t="n">
@@ -13679,19 +13805,22 @@
         <v>0.52</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>0.1828</v>
+        <v>0.0218</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>0.1828</v>
+        <v>0.0218</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>0.1828</v>
+        <v>0.0218</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>0.1983</v>
+        <v>0.0218</v>
       </c>
       <c r="I41" s="4" t="n">
-        <v>0.1993</v>
+        <v>0.0218</v>
+      </c>
+      <c r="K41" s="4" t="n">
+        <v>0.0146</v>
       </c>
     </row>
     <row r="42">
@@ -13702,7 +13831,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C42" s="3" t="n">
@@ -13712,19 +13841,22 @@
         <v>0.52</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>0.3483</v>
+        <v>0.1828</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>0.3483</v>
+        <v>0.1828</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>0.3483</v>
+        <v>0.1828</v>
       </c>
       <c r="H42" s="4" t="n">
-        <v>0.3483</v>
+        <v>0.1983</v>
       </c>
       <c r="I42" s="4" t="n">
-        <v>0.3483</v>
+        <v>0.1993</v>
+      </c>
+      <c r="K42" s="4" t="n">
+        <v>0.1993</v>
       </c>
     </row>
     <row r="43">
@@ -13735,7 +13867,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C43" s="3" t="n">
@@ -13745,19 +13877,22 @@
         <v>0.52</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>0.4306</v>
+        <v>0.3483</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>0.4306</v>
+        <v>0.3483</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>0.4306</v>
+        <v>0.3483</v>
       </c>
       <c r="H43" s="4" t="n">
-        <v>0.4306</v>
+        <v>0.3483</v>
       </c>
       <c r="I43" s="4" t="n">
-        <v>0.4306</v>
+        <v>0.3483</v>
+      </c>
+      <c r="K43" s="4" t="n">
+        <v>0.3483</v>
       </c>
     </row>
     <row r="44">
@@ -13768,31 +13903,71 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="n">
+        <v>3753500</v>
+      </c>
+      <c r="D44" s="4" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="E44" s="4" t="n">
+        <v>0.4306</v>
+      </c>
+      <c r="F44" s="4" t="n">
+        <v>0.4306</v>
+      </c>
+      <c r="G44" s="4" t="n">
+        <v>0.4306</v>
+      </c>
+      <c r="H44" s="4" t="n">
+        <v>0.4306</v>
+      </c>
+      <c r="I44" s="4" t="n">
+        <v>0.4306</v>
+      </c>
+      <c r="K44" s="4" t="n">
+        <v>0.4306</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E44" s="5">
-        <f>SUM(E40:E43)</f>
-        <v/>
-      </c>
-      <c r="F44" s="5">
-        <f>SUM(F40:F43)</f>
-        <v/>
-      </c>
-      <c r="G44" s="5">
-        <f>SUM(G40:G43)</f>
-        <v/>
-      </c>
-      <c r="H44" s="5">
-        <f>SUM(H40:H43)</f>
-        <v/>
-      </c>
-      <c r="I44" s="5">
-        <f>SUM(I40:I43)</f>
-        <v/>
-      </c>
-      <c r="J44" s="5">
-        <f>SUM(J40:J43)</f>
+      <c r="E45" s="5">
+        <f>SUM(E41:E44)</f>
+        <v/>
+      </c>
+      <c r="F45" s="5">
+        <f>SUM(F41:F44)</f>
+        <v/>
+      </c>
+      <c r="G45" s="5">
+        <f>SUM(G41:G44)</f>
+        <v/>
+      </c>
+      <c r="H45" s="5">
+        <f>SUM(H41:H44)</f>
+        <v/>
+      </c>
+      <c r="I45" s="5">
+        <f>SUM(I41:I44)</f>
+        <v/>
+      </c>
+      <c r="J45" s="5">
+        <f>SUM(J41:J44)</f>
+        <v/>
+      </c>
+      <c r="K45" s="5">
+        <f>SUM(K41:K44)</f>
         <v/>
       </c>
     </row>
@@ -13807,7 +13982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K69"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13863,7 +14038,12 @@
           <t>August 2 2026</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="1" t="inlineStr">
+        <is>
+          <t>August 3 2026</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
@@ -13901,6 +14081,9 @@
       <c r="I3" s="4" t="n">
         <v>0.3165</v>
       </c>
+      <c r="K3" s="4" t="n">
+        <v>0.3165</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -13934,6 +14117,9 @@
       <c r="I4" s="4" t="n">
         <v>0.6835</v>
       </c>
+      <c r="K4" s="4" t="n">
+        <v>0.6835</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -13970,6 +14156,10 @@
         <f>SUM(J3:J4)</f>
         <v/>
       </c>
+      <c r="K5" s="5">
+        <f>SUM(K3:K4)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -14003,6 +14193,9 @@
       <c r="I6" s="4" t="n">
         <v>0.0452</v>
       </c>
+      <c r="K6" s="4" t="n">
+        <v>0.0452</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -14036,6 +14229,9 @@
       <c r="I7" s="4" t="n">
         <v>0.0261</v>
       </c>
+      <c r="K7" s="4" t="n">
+        <v>0.0261</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -14069,6 +14265,9 @@
       <c r="I8" s="4" t="n">
         <v>0.0009</v>
       </c>
+      <c r="K8" s="4" t="n">
+        <v>0.0009</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -14102,6 +14301,9 @@
       <c r="I9" s="4" t="n">
         <v>0.0128</v>
       </c>
+      <c r="K9" s="4" t="n">
+        <v>0.0128</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -14135,6 +14337,9 @@
       <c r="I10" s="4" t="n">
         <v>0.2225</v>
       </c>
+      <c r="K10" s="4" t="n">
+        <v>0.2225</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -14168,6 +14373,9 @@
       <c r="I11" s="4" t="n">
         <v>0.2191</v>
       </c>
+      <c r="K11" s="4" t="n">
+        <v>0.2191</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -14201,6 +14409,9 @@
       <c r="I12" s="4" t="n">
         <v>0.0785</v>
       </c>
+      <c r="K12" s="4" t="n">
+        <v>0.0785</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -14234,6 +14445,14 @@
       <c r="I13" s="4" t="n">
         <v>0.33</v>
       </c>
+      <c r="K13" s="4" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -14267,6 +14486,9 @@
       <c r="I14" s="4" t="n">
         <v>0.001</v>
       </c>
+      <c r="K14" s="4" t="n">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -14300,6 +14522,9 @@
       <c r="I15" s="4" t="n">
         <v>0.0622</v>
       </c>
+      <c r="K15" s="4" t="n">
+        <v>0.0622</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -14330,6 +14555,9 @@
       <c r="I16" s="4" t="n">
         <v>0.0013</v>
       </c>
+      <c r="K16" s="4" t="n">
+        <v>0.0013</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -14366,6 +14594,10 @@
         <f>SUM(J6:J16)</f>
         <v/>
       </c>
+      <c r="K17" s="5">
+        <f>SUM(K6:K16)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -14399,6 +14631,9 @@
       <c r="I18" s="4" t="n">
         <v>0.0206</v>
       </c>
+      <c r="K18" s="4" t="n">
+        <v>0.0206</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -14432,6 +14667,9 @@
       <c r="I19" s="4" t="n">
         <v>0.1124</v>
       </c>
+      <c r="K19" s="4" t="n">
+        <v>0.1972</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -14465,6 +14703,9 @@
       <c r="I20" s="4" t="n">
         <v>0.0175</v>
       </c>
+      <c r="K20" s="4" t="n">
+        <v>0.0175</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -14495,6 +14736,9 @@
       <c r="I21" s="4" t="n">
         <v>0.3055</v>
       </c>
+      <c r="K21" s="4" t="n">
+        <v>0.3255</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -14531,6 +14775,10 @@
         <f>SUM(J18:J21)</f>
         <v/>
       </c>
+      <c r="K22" s="5">
+        <f>SUM(K18:K21)</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -14564,6 +14812,9 @@
       <c r="I23" s="4" t="n">
         <v>0.0304</v>
       </c>
+      <c r="K23" s="4" t="n">
+        <v>0.0304</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -14597,6 +14848,9 @@
       <c r="I24" s="4" t="n">
         <v>0.0793</v>
       </c>
+      <c r="K24" s="4" t="n">
+        <v>0.0793</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -14630,6 +14884,14 @@
       <c r="I25" s="4" t="n">
         <v>0.25</v>
       </c>
+      <c r="K25" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -14663,6 +14925,9 @@
       <c r="I26" s="4" t="n">
         <v>0.0447</v>
       </c>
+      <c r="K26" s="4" t="n">
+        <v>0.0482</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -14696,6 +14961,9 @@
       <c r="I27" s="4" t="n">
         <v>0.039</v>
       </c>
+      <c r="K27" s="4" t="n">
+        <v>0.039</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -14729,6 +14997,9 @@
       <c r="I28" s="4" t="n">
         <v>0.0213</v>
       </c>
+      <c r="K28" s="4" t="n">
+        <v>0.0256</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -14759,6 +15030,9 @@
       <c r="I29" s="4" t="n">
         <v>0.0454</v>
       </c>
+      <c r="K29" s="4" t="n">
+        <v>0.096</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -14789,6 +15063,9 @@
       <c r="I30" s="4" t="n">
         <v>0.0152</v>
       </c>
+      <c r="K30" s="4" t="n">
+        <v>0.0157</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -14819,6 +15096,9 @@
       <c r="I31" s="4" t="n">
         <v>0.021</v>
       </c>
+      <c r="K31" s="4" t="n">
+        <v>0.0369</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -14846,6 +15126,9 @@
       <c r="I32" s="4" t="n">
         <v>0.0014</v>
       </c>
+      <c r="K32" s="4" t="n">
+        <v>0.0014</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -14855,65 +15138,57 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E33" s="5">
-        <f>SUM(E23:E32)</f>
-        <v/>
-      </c>
-      <c r="F33" s="5">
-        <f>SUM(F23:F32)</f>
-        <v/>
-      </c>
-      <c r="G33" s="5">
-        <f>SUM(G23:G32)</f>
-        <v/>
-      </c>
-      <c r="H33" s="5">
-        <f>SUM(H23:H32)</f>
-        <v/>
-      </c>
-      <c r="I33" s="5">
-        <f>SUM(I23:I32)</f>
-        <v/>
-      </c>
-      <c r="J33" s="5">
-        <f>SUM(J23:J32)</f>
-        <v/>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>31128200</v>
+      </c>
+      <c r="D33" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K33" s="4" t="n">
+        <v>0.0063</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="n">
-        <v>28710400</v>
-      </c>
-      <c r="D34" s="4" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="E34" s="4" t="n">
-        <v>0.0832</v>
-      </c>
-      <c r="F34" s="4" t="n">
-        <v>0.0832</v>
-      </c>
-      <c r="G34" s="4" t="n">
-        <v>0.0832</v>
-      </c>
-      <c r="H34" s="4" t="n">
-        <v>0.0832</v>
-      </c>
-      <c r="I34" s="4" t="n">
-        <v>0.08349999999999999</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E34" s="5">
+        <f>SUM(E23:E33)</f>
+        <v/>
+      </c>
+      <c r="F34" s="5">
+        <f>SUM(F23:F33)</f>
+        <v/>
+      </c>
+      <c r="G34" s="5">
+        <f>SUM(G23:G33)</f>
+        <v/>
+      </c>
+      <c r="H34" s="5">
+        <f>SUM(H23:H33)</f>
+        <v/>
+      </c>
+      <c r="I34" s="5">
+        <f>SUM(I23:I33)</f>
+        <v/>
+      </c>
+      <c r="J34" s="5">
+        <f>SUM(J23:J33)</f>
+        <v/>
+      </c>
+      <c r="K34" s="5">
+        <f>SUM(K23:K33)</f>
+        <v/>
       </c>
     </row>
     <row r="35">
@@ -14924,7 +15199,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C35" s="3" t="n">
@@ -14934,19 +15209,22 @@
         <v>0.45</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>0.3459</v>
+        <v>0.0832</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>0.3459</v>
+        <v>0.0832</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.3459</v>
+        <v>0.0832</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>0.3459</v>
+        <v>0.0832</v>
       </c>
       <c r="I35" s="4" t="n">
-        <v>0.3459</v>
+        <v>0.08349999999999999</v>
+      </c>
+      <c r="K35" s="4" t="n">
+        <v>0.08349999999999999</v>
       </c>
     </row>
     <row r="36">
@@ -14957,7 +15235,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="C36" s="3" t="n">
@@ -14966,17 +15244,23 @@
       <c r="D36" s="4" t="n">
         <v>0.45</v>
       </c>
+      <c r="E36" s="4" t="n">
+        <v>0.3459</v>
+      </c>
       <c r="F36" s="4" t="n">
-        <v>0.0007000000000000001</v>
+        <v>0.3459</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.0007000000000000001</v>
+        <v>0.3459</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>0.0007000000000000001</v>
+        <v>0.3459</v>
       </c>
       <c r="I36" s="4" t="n">
-        <v>0.0007000000000000001</v>
+        <v>0.3459</v>
+      </c>
+      <c r="K36" s="4" t="n">
+        <v>0.3459</v>
       </c>
     </row>
     <row r="37">
@@ -14987,98 +15271,90 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E37" s="5">
-        <f>SUM(E34:E36)</f>
-        <v/>
-      </c>
-      <c r="F37" s="5">
-        <f>SUM(F34:F36)</f>
-        <v/>
-      </c>
-      <c r="G37" s="5">
-        <f>SUM(G34:G36)</f>
-        <v/>
-      </c>
-      <c r="H37" s="5">
-        <f>SUM(H34:H36)</f>
-        <v/>
-      </c>
-      <c r="I37" s="5">
-        <f>SUM(I34:I36)</f>
-        <v/>
-      </c>
-      <c r="J37" s="5">
-        <f>SUM(J34:J36)</f>
-        <v/>
+          <t>Czech Republic</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>28710400</v>
+      </c>
+      <c r="D37" s="4" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
+      <c r="G37" s="4" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
+      <c r="H37" s="4" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
+      <c r="I37" s="4" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
+      <c r="K37" s="4" t="n">
+        <v>0.0007000000000000001</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C38" s="3" t="n">
-        <v>8750300</v>
+        <v>28710400</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="E38" s="4" t="n">
-        <v>0.0025</v>
-      </c>
-      <c r="F38" s="4" t="n">
-        <v>0.0025</v>
-      </c>
-      <c r="G38" s="4" t="n">
-        <v>0.0025</v>
-      </c>
-      <c r="H38" s="4" t="n">
-        <v>0.0025</v>
-      </c>
-      <c r="I38" s="4" t="n">
-        <v>0.0025</v>
+        <v>0.45</v>
+      </c>
+      <c r="K38" s="4" t="n">
+        <v>0.4389</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="n">
-        <v>8750300</v>
-      </c>
-      <c r="D39" s="4" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="E39" s="4" t="n">
-        <v>0.2277</v>
-      </c>
-      <c r="F39" s="4" t="n">
-        <v>0.2285</v>
-      </c>
-      <c r="G39" s="4" t="n">
-        <v>0.2297</v>
-      </c>
-      <c r="H39" s="4" t="n">
-        <v>0.2419</v>
-      </c>
-      <c r="I39" s="4" t="n">
-        <v>0.2441</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E39" s="5">
+        <f>SUM(E35:E38)</f>
+        <v/>
+      </c>
+      <c r="F39" s="5">
+        <f>SUM(F35:F38)</f>
+        <v/>
+      </c>
+      <c r="G39" s="5">
+        <f>SUM(G35:G38)</f>
+        <v/>
+      </c>
+      <c r="H39" s="5">
+        <f>SUM(H35:H38)</f>
+        <v/>
+      </c>
+      <c r="I39" s="5">
+        <f>SUM(I35:I38)</f>
+        <v/>
+      </c>
+      <c r="J39" s="5">
+        <f>SUM(J35:J38)</f>
+        <v/>
+      </c>
+      <c r="K39" s="5">
+        <f>SUM(K35:K38)</f>
+        <v/>
       </c>
     </row>
     <row r="40">
@@ -15089,7 +15365,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C40" s="3" t="n">
@@ -15099,19 +15375,22 @@
         <v>0.58</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>0.1228</v>
+        <v>0.0025</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>0.1253</v>
+        <v>0.0025</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>0.1543</v>
+        <v>0.0025</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>0.1545</v>
+        <v>0.0025</v>
       </c>
       <c r="I40" s="4" t="n">
-        <v>0.1549</v>
+        <v>0.0025</v>
+      </c>
+      <c r="K40" s="4" t="n">
+        <v>0.0025</v>
       </c>
     </row>
     <row r="41">
@@ -15122,7 +15401,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C41" s="3" t="n">
@@ -15132,19 +15411,22 @@
         <v>0.58</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>0.0019</v>
+        <v>0.2277</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>0.0019</v>
+        <v>0.2285</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>0.0035</v>
+        <v>0.2297</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>0.0035</v>
+        <v>0.2419</v>
       </c>
       <c r="I41" s="4" t="n">
-        <v>0.0035</v>
+        <v>0.2441</v>
+      </c>
+      <c r="K41" s="4" t="n">
+        <v>0.2444</v>
       </c>
     </row>
     <row r="42">
@@ -15155,7 +15437,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C42" s="3" t="n">
@@ -15165,19 +15447,22 @@
         <v>0.58</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>0.0068</v>
+        <v>0.1228</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>0.0095</v>
+        <v>0.1253</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>0.01</v>
+        <v>0.1543</v>
       </c>
       <c r="H42" s="4" t="n">
-        <v>0.0104</v>
+        <v>0.1545</v>
       </c>
       <c r="I42" s="4" t="n">
-        <v>0.0105</v>
+        <v>0.1549</v>
+      </c>
+      <c r="K42" s="4" t="n">
+        <v>0.155</v>
       </c>
     </row>
     <row r="43">
@@ -15188,7 +15473,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Luxembourg</t>
         </is>
       </c>
       <c r="C43" s="3" t="n">
@@ -15198,19 +15483,22 @@
         <v>0.58</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>0.0191</v>
+        <v>0.0019</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>0.0236</v>
+        <v>0.0019</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>0.0294</v>
+        <v>0.0035</v>
       </c>
       <c r="H43" s="4" t="n">
-        <v>0.03759999999999999</v>
+        <v>0.0035</v>
       </c>
       <c r="I43" s="4" t="n">
-        <v>0.0546</v>
+        <v>0.0035</v>
+      </c>
+      <c r="K43" s="4" t="n">
+        <v>0.016</v>
       </c>
     </row>
     <row r="44">
@@ -15221,7 +15509,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="C44" s="3" t="n">
@@ -15230,17 +15518,23 @@
       <c r="D44" s="4" t="n">
         <v>0.58</v>
       </c>
+      <c r="E44" s="4" t="n">
+        <v>0.0068</v>
+      </c>
       <c r="F44" s="4" t="n">
-        <v>0.0017</v>
+        <v>0.0095</v>
       </c>
       <c r="G44" s="4" t="n">
-        <v>0.0028</v>
+        <v>0.01</v>
       </c>
       <c r="H44" s="4" t="n">
-        <v>0.006500000000000001</v>
+        <v>0.0104</v>
       </c>
       <c r="I44" s="4" t="n">
-        <v>0.0066</v>
+        <v>0.0105</v>
+      </c>
+      <c r="K44" s="4" t="n">
+        <v>0.0133</v>
       </c>
     </row>
     <row r="45">
@@ -15251,7 +15545,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C45" s="3" t="n">
@@ -15260,17 +15554,23 @@
       <c r="D45" s="4" t="n">
         <v>0.58</v>
       </c>
+      <c r="E45" s="4" t="n">
+        <v>0.0191</v>
+      </c>
       <c r="F45" s="4" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.0236</v>
       </c>
       <c r="G45" s="4" t="n">
-        <v>0.06950000000000001</v>
+        <v>0.0294</v>
       </c>
       <c r="H45" s="4" t="n">
-        <v>0.1435</v>
+        <v>0.03759999999999999</v>
       </c>
       <c r="I45" s="4" t="n">
-        <v>0.2085</v>
+        <v>0.0546</v>
+      </c>
+      <c r="K45" s="4" t="n">
+        <v>0.0708</v>
       </c>
     </row>
     <row r="46">
@@ -15281,7 +15581,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C46" s="3" t="n">
@@ -15290,14 +15590,20 @@
       <c r="D46" s="4" t="n">
         <v>0.58</v>
       </c>
+      <c r="F46" s="4" t="n">
+        <v>0.0017</v>
+      </c>
       <c r="G46" s="4" t="n">
-        <v>0.0005</v>
+        <v>0.0028</v>
       </c>
       <c r="H46" s="4" t="n">
-        <v>0.0001</v>
+        <v>0.006500000000000001</v>
       </c>
       <c r="I46" s="4" t="n">
-        <v>0.0001</v>
+        <v>0.0066</v>
+      </c>
+      <c r="K46" s="4" t="n">
+        <v>0.0066</v>
       </c>
     </row>
     <row r="47">
@@ -15308,7 +15614,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C47" s="3" t="n">
@@ -15317,14 +15623,20 @@
       <c r="D47" s="4" t="n">
         <v>0.58</v>
       </c>
+      <c r="F47" s="4" t="n">
+        <v>0.008500000000000001</v>
+      </c>
       <c r="G47" s="4" t="n">
-        <v>0</v>
+        <v>0.06950000000000001</v>
       </c>
       <c r="H47" s="4" t="n">
-        <v>0</v>
+        <v>0.1435</v>
       </c>
       <c r="I47" s="4" t="n">
-        <v>0</v>
+        <v>0.2085</v>
+      </c>
+      <c r="K47" s="4" t="n">
+        <v>0.29</v>
       </c>
     </row>
     <row r="48">
@@ -15335,7 +15647,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C48" s="3" t="n">
@@ -15345,13 +15657,16 @@
         <v>0.58</v>
       </c>
       <c r="G48" s="4" t="n">
-        <v>0.0022</v>
+        <v>0.0005</v>
       </c>
       <c r="H48" s="4" t="n">
-        <v>0.0022</v>
+        <v>0.0001</v>
       </c>
       <c r="I48" s="4" t="n">
-        <v>0.0022</v>
+        <v>0.0001</v>
+      </c>
+      <c r="K48" s="4" t="n">
+        <v>0.0001</v>
       </c>
     </row>
     <row r="49">
@@ -15362,7 +15677,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C49" s="3" t="n">
@@ -15372,13 +15687,16 @@
         <v>0.58</v>
       </c>
       <c r="G49" s="4" t="n">
-        <v>0.0004</v>
+        <v>0</v>
       </c>
       <c r="H49" s="4" t="n">
-        <v>0.0004</v>
+        <v>0</v>
       </c>
       <c r="I49" s="4" t="n">
-        <v>0.0004</v>
+        <v>0</v>
+      </c>
+      <c r="K49" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -15389,7 +15707,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C50" s="3" t="n">
@@ -15399,13 +15717,16 @@
         <v>0.58</v>
       </c>
       <c r="G50" s="4" t="n">
-        <v>0</v>
+        <v>0.0022</v>
       </c>
       <c r="H50" s="4" t="n">
-        <v>0</v>
+        <v>0.0022</v>
       </c>
       <c r="I50" s="4" t="n">
-        <v>0</v>
+        <v>0.0022</v>
+      </c>
+      <c r="K50" s="4" t="n">
+        <v>0.0022</v>
       </c>
     </row>
     <row r="51">
@@ -15416,7 +15737,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="C51" s="3" t="n">
@@ -15425,11 +15746,17 @@
       <c r="D51" s="4" t="n">
         <v>0.58</v>
       </c>
+      <c r="G51" s="4" t="n">
+        <v>0.0004</v>
+      </c>
       <c r="H51" s="4" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
       <c r="I51" s="4" t="n">
-        <v>0</v>
+        <v>0.0004</v>
+      </c>
+      <c r="K51" s="4" t="n">
+        <v>0.0004</v>
       </c>
     </row>
     <row r="52">
@@ -15440,7 +15767,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C52" s="3" t="n">
@@ -15449,12 +15776,18 @@
       <c r="D52" s="4" t="n">
         <v>0.58</v>
       </c>
+      <c r="G52" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="H52" s="4" t="n">
         <v>0</v>
       </c>
       <c r="I52" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="K52" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -15464,7 +15797,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C53" s="3" t="n">
@@ -15473,9 +15806,15 @@
       <c r="D53" s="4" t="n">
         <v>0.58</v>
       </c>
+      <c r="H53" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="I53" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="K53" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -15485,131 +15824,108 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E54" s="5">
-        <f>SUM(E38:E53)</f>
-        <v/>
-      </c>
-      <c r="F54" s="5">
-        <f>SUM(F38:F53)</f>
-        <v/>
-      </c>
-      <c r="G54" s="5">
-        <f>SUM(G38:G53)</f>
-        <v/>
-      </c>
-      <c r="H54" s="5">
-        <f>SUM(H38:H53)</f>
-        <v/>
-      </c>
-      <c r="I54" s="5">
-        <f>SUM(I38:I53)</f>
-        <v/>
-      </c>
-      <c r="J54" s="5">
-        <f>SUM(J38:J53)</f>
-        <v/>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="n">
+        <v>8750300</v>
+      </c>
+      <c r="D54" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="H54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="C55" s="3" t="n">
-        <v>16514800</v>
+        <v>8750300</v>
       </c>
       <c r="D55" s="4" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="E55" s="4" t="n">
-        <v>0.0029</v>
-      </c>
-      <c r="F55" s="4" t="n">
-        <v>0.0029</v>
-      </c>
-      <c r="G55" s="4" t="n">
-        <v>0.0029</v>
-      </c>
-      <c r="H55" s="4" t="n">
-        <v>0.0325</v>
+        <v>0.58</v>
       </c>
       <c r="I55" s="4" t="n">
-        <v>0.0898</v>
+        <v>0</v>
+      </c>
+      <c r="K55" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C56" s="3" t="n">
-        <v>16514800</v>
+        <v>8750300</v>
       </c>
       <c r="D56" s="4" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="E56" s="4" t="n">
-        <v>0.0339</v>
-      </c>
-      <c r="F56" s="4" t="n">
-        <v>0.0339</v>
-      </c>
-      <c r="G56" s="4" t="n">
-        <v>0.0339</v>
-      </c>
-      <c r="H56" s="4" t="n">
-        <v>0.0339</v>
-      </c>
-      <c r="I56" s="4" t="n">
-        <v>0.04269999999999999</v>
+        <v>0.58</v>
+      </c>
+      <c r="K56" s="4" t="n">
+        <v>0.0001</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Malaysia</t>
-        </is>
-      </c>
-      <c r="C57" s="3" t="n">
-        <v>16514800</v>
-      </c>
-      <c r="D57" s="4" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="E57" s="4" t="n">
-        <v>0.4926</v>
-      </c>
-      <c r="F57" s="4" t="n">
-        <v>0.4926</v>
-      </c>
-      <c r="G57" s="4" t="n">
-        <v>0.4926</v>
-      </c>
-      <c r="H57" s="4" t="n">
-        <v>0.4926</v>
-      </c>
-      <c r="I57" s="4" t="n">
-        <v>0.4926</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E57" s="5">
+        <f>SUM(E40:E56)</f>
+        <v/>
+      </c>
+      <c r="F57" s="5">
+        <f>SUM(F40:F56)</f>
+        <v/>
+      </c>
+      <c r="G57" s="5">
+        <f>SUM(G40:G56)</f>
+        <v/>
+      </c>
+      <c r="H57" s="5">
+        <f>SUM(H40:H56)</f>
+        <v/>
+      </c>
+      <c r="I57" s="5">
+        <f>SUM(I40:I56)</f>
+        <v/>
+      </c>
+      <c r="J57" s="5">
+        <f>SUM(J40:J56)</f>
+        <v/>
+      </c>
+      <c r="K57" s="5">
+        <f>SUM(K40:K56)</f>
+        <v/>
       </c>
     </row>
     <row r="58">
@@ -15620,7 +15936,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C58" s="3" t="n">
@@ -15630,19 +15946,22 @@
         <v>0.59</v>
       </c>
       <c r="E58" s="4" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.0029</v>
       </c>
       <c r="F58" s="4" t="n">
-        <v>0.0146</v>
+        <v>0.0029</v>
       </c>
       <c r="G58" s="4" t="n">
-        <v>0.0161</v>
+        <v>0.0029</v>
       </c>
       <c r="H58" s="4" t="n">
-        <v>0.0161</v>
+        <v>0.0325</v>
       </c>
       <c r="I58" s="4" t="n">
-        <v>0.0161</v>
+        <v>0.0898</v>
+      </c>
+      <c r="K58" s="4" t="n">
+        <v>0.1142</v>
       </c>
     </row>
     <row r="59">
@@ -15653,7 +15972,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C59" s="3" t="n">
@@ -15662,14 +15981,23 @@
       <c r="D59" s="4" t="n">
         <v>0.59</v>
       </c>
+      <c r="E59" s="4" t="n">
+        <v>0.0339</v>
+      </c>
+      <c r="F59" s="4" t="n">
+        <v>0.0339</v>
+      </c>
       <c r="G59" s="4" t="n">
-        <v>0.0044</v>
+        <v>0.0339</v>
       </c>
       <c r="H59" s="4" t="n">
-        <v>0.0044</v>
+        <v>0.0339</v>
       </c>
       <c r="I59" s="4" t="n">
-        <v>0.0044</v>
+        <v>0.04269999999999999</v>
+      </c>
+      <c r="K59" s="4" t="n">
+        <v>0.04269999999999999</v>
       </c>
     </row>
     <row r="60">
@@ -15680,131 +16008,138 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E60" s="5">
-        <f>SUM(E55:E59)</f>
-        <v/>
-      </c>
-      <c r="F60" s="5">
-        <f>SUM(F55:F59)</f>
-        <v/>
-      </c>
-      <c r="G60" s="5">
-        <f>SUM(G55:G59)</f>
-        <v/>
-      </c>
-      <c r="H60" s="5">
-        <f>SUM(H55:H59)</f>
-        <v/>
-      </c>
-      <c r="I60" s="5">
-        <f>SUM(I55:I59)</f>
-        <v/>
-      </c>
-      <c r="J60" s="5">
-        <f>SUM(J55:J59)</f>
-        <v/>
+          <t>Malaysia</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="n">
+        <v>16514800</v>
+      </c>
+      <c r="D60" s="4" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="E60" s="4" t="n">
+        <v>0.4926</v>
+      </c>
+      <c r="F60" s="4" t="n">
+        <v>0.4926</v>
+      </c>
+      <c r="G60" s="4" t="n">
+        <v>0.4926</v>
+      </c>
+      <c r="H60" s="4" t="n">
+        <v>0.4926</v>
+      </c>
+      <c r="I60" s="4" t="n">
+        <v>0.4926</v>
+      </c>
+      <c r="K60" s="4" t="n">
+        <v>0.4926</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C61" s="3" t="n">
-        <v>3467600</v>
+        <v>16514800</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.59</v>
       </c>
       <c r="E61" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="F61" s="4" t="n">
-        <v>0.0021</v>
+        <v>0.0146</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0.0021</v>
+        <v>0.0161</v>
       </c>
       <c r="H61" s="4" t="n">
-        <v>0.0021</v>
+        <v>0.0161</v>
       </c>
       <c r="I61" s="4" t="n">
-        <v>0.0021</v>
+        <v>0.0161</v>
+      </c>
+      <c r="K61" s="4" t="n">
+        <v>0.0161</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C62" s="3" t="n">
-        <v>3467600</v>
+        <v>16514800</v>
       </c>
       <c r="D62" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="E62" s="4" t="n">
-        <v>0.0032</v>
-      </c>
-      <c r="F62" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.59</v>
       </c>
       <c r="G62" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.0044</v>
       </c>
       <c r="H62" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.0044</v>
       </c>
       <c r="I62" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.0044</v>
+      </c>
+      <c r="K62" s="4" t="n">
+        <v>0.0044</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="C63" s="3" t="n">
-        <v>3467600</v>
-      </c>
-      <c r="D63" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="E63" s="4" t="n">
-        <v>0.0204</v>
-      </c>
-      <c r="F63" s="4" t="n">
-        <v>0.0204</v>
-      </c>
-      <c r="G63" s="4" t="n">
-        <v>0.0204</v>
-      </c>
-      <c r="H63" s="4" t="n">
-        <v>0.0204</v>
-      </c>
-      <c r="I63" s="4" t="n">
-        <v>0.0204</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E63" s="5">
+        <f>SUM(E58:E62)</f>
+        <v/>
+      </c>
+      <c r="F63" s="5">
+        <f>SUM(F58:F62)</f>
+        <v/>
+      </c>
+      <c r="G63" s="5">
+        <f>SUM(G58:G62)</f>
+        <v/>
+      </c>
+      <c r="H63" s="5">
+        <f>SUM(H58:H62)</f>
+        <v/>
+      </c>
+      <c r="I63" s="5">
+        <f>SUM(I58:I62)</f>
+        <v/>
+      </c>
+      <c r="J63" s="5">
+        <f>SUM(J58:J62)</f>
+        <v/>
+      </c>
+      <c r="K63" s="5">
+        <f>SUM(K58:K62)</f>
+        <v/>
       </c>
     </row>
     <row r="64">
@@ -15815,7 +16150,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C64" s="3" t="n">
@@ -15825,19 +16160,22 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E64" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.0004</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.0021</v>
       </c>
       <c r="G64" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.0021</v>
       </c>
       <c r="H64" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.0021</v>
       </c>
       <c r="I64" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.0021</v>
+      </c>
+      <c r="K64" s="4" t="n">
+        <v>0.0021</v>
       </c>
     </row>
     <row r="65">
@@ -15848,7 +16186,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C65" s="3" t="n">
@@ -15858,19 +16196,22 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E65" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.0032</v>
       </c>
       <c r="F65" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.0032</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.0032</v>
       </c>
       <c r="H65" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.0032</v>
       </c>
       <c r="I65" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.0032</v>
+      </c>
+      <c r="K65" s="4" t="n">
+        <v>0.0032</v>
       </c>
     </row>
     <row r="66">
@@ -15881,7 +16222,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C66" s="3" t="n">
@@ -15891,19 +16232,22 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E66" s="4" t="n">
-        <v>0.1798</v>
+        <v>0.0204</v>
       </c>
       <c r="F66" s="4" t="n">
-        <v>0.1798</v>
+        <v>0.0204</v>
       </c>
       <c r="G66" s="4" t="n">
-        <v>0.2828</v>
+        <v>0.0204</v>
       </c>
       <c r="H66" s="4" t="n">
-        <v>0.2828</v>
+        <v>0.0204</v>
       </c>
       <c r="I66" s="4" t="n">
-        <v>0.2828</v>
+        <v>0.0204</v>
+      </c>
+      <c r="K66" s="4" t="n">
+        <v>0.0204</v>
       </c>
     </row>
     <row r="67">
@@ -15914,7 +16258,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C67" s="3" t="n">
@@ -15923,17 +16267,28 @@
       <c r="D67" s="4" t="n">
         <v>0.6899999999999999</v>
       </c>
+      <c r="E67" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
       <c r="F67" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H67" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="I67" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="K67" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
       </c>
     </row>
     <row r="68">
@@ -15944,7 +16299,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C68" s="3" t="n">
@@ -15953,14 +16308,23 @@
       <c r="D68" s="4" t="n">
         <v>0.6899999999999999</v>
       </c>
+      <c r="E68" s="4" t="n">
+        <v>0.0004</v>
+      </c>
+      <c r="F68" s="4" t="n">
+        <v>0.0004</v>
+      </c>
       <c r="G68" s="4" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
       <c r="H68" s="4" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
       <c r="I68" s="4" t="n">
-        <v>0</v>
+        <v>0.0004</v>
+      </c>
+      <c r="K68" s="4" t="n">
+        <v>0.0004</v>
       </c>
     </row>
     <row r="69">
@@ -15971,31 +16335,134 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D69" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E69" s="4" t="n">
+        <v>0.1798</v>
+      </c>
+      <c r="F69" s="4" t="n">
+        <v>0.1798</v>
+      </c>
+      <c r="G69" s="4" t="n">
+        <v>0.2828</v>
+      </c>
+      <c r="H69" s="4" t="n">
+        <v>0.2828</v>
+      </c>
+      <c r="I69" s="4" t="n">
+        <v>0.2828</v>
+      </c>
+      <c r="K69" s="4" t="n">
+        <v>0.2828</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Luxembourg</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D70" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="F70" s="4" t="n">
+        <v>0.0012</v>
+      </c>
+      <c r="G70" s="4" t="n">
+        <v>0.0012</v>
+      </c>
+      <c r="H70" s="4" t="n">
+        <v>0.0012</v>
+      </c>
+      <c r="I70" s="4" t="n">
+        <v>0.0012</v>
+      </c>
+      <c r="K70" s="4" t="n">
+        <v>0.0012</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D71" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G71" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I71" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K71" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E69" s="5">
-        <f>SUM(E61:E68)</f>
-        <v/>
-      </c>
-      <c r="F69" s="5">
-        <f>SUM(F61:F68)</f>
-        <v/>
-      </c>
-      <c r="G69" s="5">
-        <f>SUM(G61:G68)</f>
-        <v/>
-      </c>
-      <c r="H69" s="5">
-        <f>SUM(H61:H68)</f>
-        <v/>
-      </c>
-      <c r="I69" s="5">
-        <f>SUM(I61:I68)</f>
-        <v/>
-      </c>
-      <c r="J69" s="5">
-        <f>SUM(J61:J68)</f>
+      <c r="E72" s="5">
+        <f>SUM(E64:E71)</f>
+        <v/>
+      </c>
+      <c r="F72" s="5">
+        <f>SUM(F64:F71)</f>
+        <v/>
+      </c>
+      <c r="G72" s="5">
+        <f>SUM(G64:G71)</f>
+        <v/>
+      </c>
+      <c r="H72" s="5">
+        <f>SUM(H64:H71)</f>
+        <v/>
+      </c>
+      <c r="I72" s="5">
+        <f>SUM(I64:I71)</f>
+        <v/>
+      </c>
+      <c r="J72" s="5">
+        <f>SUM(J64:J71)</f>
+        <v/>
+      </c>
+      <c r="K72" s="5">
+        <f>SUM(K64:K71)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Weekly TRQ update 2026-08-10
</commit_message>
<xml_diff>
--- a/data/canada_trq_tracker.xlsx
+++ b/data/canada_trq_tracker.xlsx
@@ -12390,7 +12390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:M45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12451,7 +12451,12 @@
           <t>August 3 2026</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L2" s="1" t="inlineStr">
+        <is>
+          <t>August 10 2026</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
@@ -12492,7 +12497,10 @@
       <c r="K3" s="4" t="n">
         <v>0.41</v>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" s="4" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="M3" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -12530,6 +12538,9 @@
       <c r="K4" s="4" t="n">
         <v>0.0333</v>
       </c>
+      <c r="L4" s="4" t="n">
+        <v>0.036</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -12557,6 +12568,9 @@
       <c r="K5" s="4" t="n">
         <v>0.0003</v>
       </c>
+      <c r="L5" s="4" t="n">
+        <v>0.0003</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -12597,6 +12611,10 @@
         <f>SUM(K3:K5)</f>
         <v/>
       </c>
+      <c r="L6" s="5">
+        <f>SUM(L3:L5)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -12633,6 +12651,9 @@
       <c r="K7" s="4" t="n">
         <v>0.3567</v>
       </c>
+      <c r="L7" s="4" t="n">
+        <v>0.3468</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -12663,6 +12684,9 @@
       <c r="K8" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L8" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -12703,6 +12727,10 @@
         <f>SUM(K7:K8)</f>
         <v/>
       </c>
+      <c r="L9" s="5">
+        <f>SUM(L7:L8)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -12739,6 +12767,9 @@
       <c r="K10" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L10" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -12775,6 +12806,9 @@
       <c r="K11" s="4" t="n">
         <v>0.1135</v>
       </c>
+      <c r="L11" s="4" t="n">
+        <v>0.1135</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -12811,6 +12845,9 @@
       <c r="K12" s="4" t="n">
         <v>0.5572</v>
       </c>
+      <c r="L12" s="4" t="n">
+        <v>0.5572</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -12844,6 +12881,9 @@
       <c r="K13" s="4" t="n">
         <v>0.0008</v>
       </c>
+      <c r="L13" s="4" t="n">
+        <v>0.0008</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -12877,6 +12917,9 @@
       <c r="K14" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L14" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -12910,6 +12953,9 @@
       <c r="K15" s="4" t="n">
         <v>0.3156</v>
       </c>
+      <c r="L15" s="4" t="n">
+        <v>0.3156</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -12940,6 +12986,9 @@
       <c r="K16" s="4" t="n">
         <v>0.0128</v>
       </c>
+      <c r="L16" s="4" t="n">
+        <v>0.0128</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -12970,6 +13019,9 @@
       <c r="K17" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L17" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -13010,6 +13062,10 @@
         <f>SUM(K10:K17)</f>
         <v/>
       </c>
+      <c r="L18" s="5">
+        <f>SUM(L10:L17)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -13046,6 +13102,9 @@
       <c r="K19" s="4" t="n">
         <v>0.0027</v>
       </c>
+      <c r="L19" s="4" t="n">
+        <v>0.0027</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -13082,6 +13141,9 @@
       <c r="K20" s="4" t="n">
         <v>0.2673</v>
       </c>
+      <c r="L20" s="4" t="n">
+        <v>0.2673</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -13118,6 +13180,9 @@
       <c r="K21" s="4" t="n">
         <v>0.0069</v>
       </c>
+      <c r="L21" s="4" t="n">
+        <v>0.0069</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -13154,6 +13219,9 @@
       <c r="K22" s="4" t="n">
         <v>0.2488</v>
       </c>
+      <c r="L22" s="4" t="n">
+        <v>0.2488</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -13190,6 +13258,9 @@
       <c r="K23" s="4" t="n">
         <v>0.3697</v>
       </c>
+      <c r="L23" s="4" t="n">
+        <v>0.3697</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -13226,6 +13297,9 @@
       <c r="K24" s="4" t="n">
         <v>0.0289</v>
       </c>
+      <c r="L24" s="4" t="n">
+        <v>0.0289</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -13259,6 +13333,9 @@
       <c r="K25" s="4" t="n">
         <v>0.07539999999999999</v>
       </c>
+      <c r="L25" s="4" t="n">
+        <v>0.07539999999999999</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -13299,6 +13376,10 @@
         <f>SUM(K19:K25)</f>
         <v/>
       </c>
+      <c r="L26" s="5">
+        <f>SUM(L19:L25)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -13335,6 +13416,9 @@
       <c r="K27" s="4" t="n">
         <v>0.2747</v>
       </c>
+      <c r="L27" s="4" t="n">
+        <v>0.2747</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -13371,6 +13455,9 @@
       <c r="K28" s="4" t="n">
         <v>0.0037</v>
       </c>
+      <c r="L28" s="4" t="n">
+        <v>0.0037</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -13407,6 +13494,9 @@
       <c r="K29" s="4" t="n">
         <v>0.2899</v>
       </c>
+      <c r="L29" s="4" t="n">
+        <v>0.2899</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -13443,6 +13533,9 @@
       <c r="K30" s="4" t="n">
         <v>0.0883</v>
       </c>
+      <c r="L30" s="4" t="n">
+        <v>0.0883</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -13470,6 +13563,9 @@
       <c r="K31" s="4" t="n">
         <v>0.0038</v>
       </c>
+      <c r="L31" s="4" t="n">
+        <v>0.0038</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -13510,6 +13606,10 @@
         <f>SUM(K27:K31)</f>
         <v/>
       </c>
+      <c r="L32" s="5">
+        <f>SUM(L27:L31)</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -13546,6 +13646,9 @@
       <c r="K33" s="4" t="n">
         <v>0.1576</v>
       </c>
+      <c r="L33" s="4" t="n">
+        <v>0.1576</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -13582,7 +13685,10 @@
       <c r="K34" s="4" t="n">
         <v>0.42</v>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="L34" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="M34" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -13623,7 +13729,10 @@
       <c r="K35" s="4" t="n">
         <v>0.42</v>
       </c>
-      <c r="L35" t="inlineStr">
+      <c r="L35" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="M35" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -13661,6 +13770,9 @@
       <c r="K36" s="4" t="n">
         <v>0.0024</v>
       </c>
+      <c r="L36" s="4" t="n">
+        <v>0.0024</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -13701,6 +13813,10 @@
         <f>SUM(K33:K36)</f>
         <v/>
       </c>
+      <c r="L37" s="5">
+        <f>SUM(L33:L36)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -13725,6 +13841,9 @@
       <c r="K38" s="4" t="n">
         <v>0.2893</v>
       </c>
+      <c r="L38" s="4" t="n">
+        <v>0.2893</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -13746,6 +13865,9 @@
       <c r="K39" s="4" t="n">
         <v>0.0924</v>
       </c>
+      <c r="L39" s="4" t="n">
+        <v>0.1692</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -13786,6 +13908,10 @@
         <f>SUM(K38:K39)</f>
         <v/>
       </c>
+      <c r="L40" s="5">
+        <f>SUM(L38:L39)</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -13822,6 +13948,9 @@
       <c r="K41" s="4" t="n">
         <v>0.0146</v>
       </c>
+      <c r="L41" s="4" t="n">
+        <v>0.0146</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -13858,6 +13987,9 @@
       <c r="K42" s="4" t="n">
         <v>0.1993</v>
       </c>
+      <c r="L42" s="4" t="n">
+        <v>0.1993</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -13894,6 +14026,9 @@
       <c r="K43" s="4" t="n">
         <v>0.3483</v>
       </c>
+      <c r="L43" s="4" t="n">
+        <v>0.3483</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -13930,6 +14065,9 @@
       <c r="K44" s="4" t="n">
         <v>0.4306</v>
       </c>
+      <c r="L44" s="4" t="n">
+        <v>0.4306</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -13968,6 +14106,10 @@
       </c>
       <c r="K45" s="5">
         <f>SUM(K41:K44)</f>
+        <v/>
+      </c>
+      <c r="L45" s="5">
+        <f>SUM(L41:L44)</f>
         <v/>
       </c>
     </row>
@@ -13982,7 +14124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L72"/>
+  <dimension ref="A1:M73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14043,7 +14185,12 @@
           <t>August 3 2026</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L2" s="1" t="inlineStr">
+        <is>
+          <t>August 10 2026</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
@@ -14084,6 +14231,9 @@
       <c r="K3" s="4" t="n">
         <v>0.3165</v>
       </c>
+      <c r="L3" s="4" t="n">
+        <v>0.3165</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -14120,6 +14270,9 @@
       <c r="K4" s="4" t="n">
         <v>0.6835</v>
       </c>
+      <c r="L4" s="4" t="n">
+        <v>0.6835</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -14160,6 +14313,10 @@
         <f>SUM(K3:K4)</f>
         <v/>
       </c>
+      <c r="L5" s="5">
+        <f>SUM(L3:L4)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -14196,6 +14353,9 @@
       <c r="K6" s="4" t="n">
         <v>0.0452</v>
       </c>
+      <c r="L6" s="4" t="n">
+        <v>0.0452</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -14232,6 +14392,9 @@
       <c r="K7" s="4" t="n">
         <v>0.0261</v>
       </c>
+      <c r="L7" s="4" t="n">
+        <v>0.0261</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -14268,6 +14431,9 @@
       <c r="K8" s="4" t="n">
         <v>0.0009</v>
       </c>
+      <c r="L8" s="4" t="n">
+        <v>0.0009</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -14304,6 +14470,9 @@
       <c r="K9" s="4" t="n">
         <v>0.0128</v>
       </c>
+      <c r="L9" s="4" t="n">
+        <v>0.0128</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -14340,6 +14509,9 @@
       <c r="K10" s="4" t="n">
         <v>0.2225</v>
       </c>
+      <c r="L10" s="4" t="n">
+        <v>0.2225</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -14376,6 +14548,9 @@
       <c r="K11" s="4" t="n">
         <v>0.2191</v>
       </c>
+      <c r="L11" s="4" t="n">
+        <v>0.2191</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -14412,6 +14587,9 @@
       <c r="K12" s="4" t="n">
         <v>0.0785</v>
       </c>
+      <c r="L12" s="4" t="n">
+        <v>0.0785</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -14448,7 +14626,10 @@
       <c r="K13" s="4" t="n">
         <v>0.33</v>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="L13" s="4" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="M13" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -14489,6 +14670,9 @@
       <c r="K14" s="4" t="n">
         <v>0.001</v>
       </c>
+      <c r="L14" s="4" t="n">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -14525,6 +14709,9 @@
       <c r="K15" s="4" t="n">
         <v>0.0622</v>
       </c>
+      <c r="L15" s="4" t="n">
+        <v>0.0622</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -14558,6 +14745,9 @@
       <c r="K16" s="4" t="n">
         <v>0.0013</v>
       </c>
+      <c r="L16" s="4" t="n">
+        <v>0.0013</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -14598,6 +14788,10 @@
         <f>SUM(K6:K16)</f>
         <v/>
       </c>
+      <c r="L17" s="5">
+        <f>SUM(L6:L16)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -14634,6 +14828,9 @@
       <c r="K18" s="4" t="n">
         <v>0.0206</v>
       </c>
+      <c r="L18" s="4" t="n">
+        <v>0.0206</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -14670,6 +14867,9 @@
       <c r="K19" s="4" t="n">
         <v>0.1972</v>
       </c>
+      <c r="L19" s="4" t="n">
+        <v>0.1972</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -14706,6 +14906,9 @@
       <c r="K20" s="4" t="n">
         <v>0.0175</v>
       </c>
+      <c r="L20" s="4" t="n">
+        <v>0.0175</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -14739,6 +14942,9 @@
       <c r="K21" s="4" t="n">
         <v>0.3255</v>
       </c>
+      <c r="L21" s="4" t="n">
+        <v>0.3255</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -14748,72 +14954,61 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E22" s="5">
-        <f>SUM(E18:E21)</f>
-        <v/>
-      </c>
-      <c r="F22" s="5">
-        <f>SUM(F18:F21)</f>
-        <v/>
-      </c>
-      <c r="G22" s="5">
-        <f>SUM(G18:G21)</f>
-        <v/>
-      </c>
-      <c r="H22" s="5">
-        <f>SUM(H18:H21)</f>
-        <v/>
-      </c>
-      <c r="I22" s="5">
-        <f>SUM(I18:I21)</f>
-        <v/>
-      </c>
-      <c r="J22" s="5">
-        <f>SUM(J18:J21)</f>
-        <v/>
-      </c>
-      <c r="K22" s="5">
-        <f>SUM(K18:K21)</f>
-        <v/>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>2785800</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>0.0043</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Australia</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="n">
-        <v>31128200</v>
-      </c>
-      <c r="D23" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E23" s="4" t="n">
-        <v>0.0304</v>
-      </c>
-      <c r="F23" s="4" t="n">
-        <v>0.0304</v>
-      </c>
-      <c r="G23" s="4" t="n">
-        <v>0.0304</v>
-      </c>
-      <c r="H23" s="4" t="n">
-        <v>0.0304</v>
-      </c>
-      <c r="I23" s="4" t="n">
-        <v>0.0304</v>
-      </c>
-      <c r="K23" s="4" t="n">
-        <v>0.0304</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E23" s="5">
+        <f>SUM(E18:E22)</f>
+        <v/>
+      </c>
+      <c r="F23" s="5">
+        <f>SUM(F18:F22)</f>
+        <v/>
+      </c>
+      <c r="G23" s="5">
+        <f>SUM(G18:G22)</f>
+        <v/>
+      </c>
+      <c r="H23" s="5">
+        <f>SUM(H18:H22)</f>
+        <v/>
+      </c>
+      <c r="I23" s="5">
+        <f>SUM(I18:I22)</f>
+        <v/>
+      </c>
+      <c r="J23" s="5">
+        <f>SUM(J18:J22)</f>
+        <v/>
+      </c>
+      <c r="K23" s="5">
+        <f>SUM(K18:K22)</f>
+        <v/>
+      </c>
+      <c r="L23" s="5">
+        <f>SUM(L18:L22)</f>
+        <v/>
       </c>
     </row>
     <row r="24">
@@ -14824,7 +15019,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C24" s="3" t="n">
@@ -14834,22 +15029,25 @@
         <v>0.25</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>0.0003</v>
+        <v>0.0304</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>0.0609</v>
+        <v>0.0304</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>0.0617</v>
+        <v>0.0304</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>0.0616</v>
+        <v>0.0304</v>
       </c>
       <c r="I24" s="4" t="n">
-        <v>0.0793</v>
+        <v>0.0304</v>
       </c>
       <c r="K24" s="4" t="n">
-        <v>0.0793</v>
+        <v>0.0304</v>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>0.0304</v>
       </c>
     </row>
     <row r="25">
@@ -14860,7 +15058,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="C25" s="3" t="n">
@@ -14870,27 +15068,25 @@
         <v>0.25</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>0.0001</v>
+        <v>0.0003</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>0.0001</v>
+        <v>0.0609</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.2141</v>
+        <v>0.0617</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>0.25</v>
+        <v>0.0616</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>0.25</v>
+        <v>0.0793</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
+        <v>0.0793</v>
+      </c>
+      <c r="L25" s="4" t="n">
+        <v>0.0793</v>
       </c>
     </row>
     <row r="26">
@@ -14901,7 +15097,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C26" s="3" t="n">
@@ -14911,22 +15107,30 @@
         <v>0.25</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>0.0382</v>
+        <v>0.0001</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>0.0382</v>
+        <v>0.0001</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>0.0447</v>
+        <v>0.2141</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>0.0447</v>
+        <v>0.25</v>
       </c>
       <c r="I26" s="4" t="n">
-        <v>0.0447</v>
+        <v>0.25</v>
       </c>
       <c r="K26" s="4" t="n">
-        <v>0.0482</v>
+        <v>0.25</v>
+      </c>
+      <c r="L26" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -14937,7 +15141,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C27" s="3" t="n">
@@ -14947,22 +15151,25 @@
         <v>0.25</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>0</v>
+        <v>0.0382</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>0.0341</v>
+        <v>0.0382</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.0372</v>
+        <v>0.0447</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>0.0372</v>
+        <v>0.0447</v>
       </c>
       <c r="I27" s="4" t="n">
-        <v>0.039</v>
+        <v>0.0447</v>
       </c>
       <c r="K27" s="4" t="n">
-        <v>0.039</v>
+        <v>0.0482</v>
+      </c>
+      <c r="L27" s="4" t="n">
+        <v>0.0482</v>
       </c>
     </row>
     <row r="28">
@@ -14973,7 +15180,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C28" s="3" t="n">
@@ -14983,22 +15190,25 @@
         <v>0.25</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>0.0213</v>
+        <v>0</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>0.0213</v>
+        <v>0.0341</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.0213</v>
+        <v>0.0372</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>0.0213</v>
+        <v>0.0372</v>
       </c>
       <c r="I28" s="4" t="n">
-        <v>0.0213</v>
+        <v>0.039</v>
       </c>
       <c r="K28" s="4" t="n">
-        <v>0.0256</v>
+        <v>0.039</v>
+      </c>
+      <c r="L28" s="4" t="n">
+        <v>0.039</v>
       </c>
     </row>
     <row r="29">
@@ -15009,7 +15219,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C29" s="3" t="n">
@@ -15018,20 +15228,26 @@
       <c r="D29" s="4" t="n">
         <v>0.25</v>
       </c>
+      <c r="E29" s="4" t="n">
+        <v>0.0213</v>
+      </c>
       <c r="F29" s="4" t="n">
-        <v>0.0451</v>
+        <v>0.0213</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>0.0454</v>
+        <v>0.0213</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>0.0454</v>
+        <v>0.0213</v>
       </c>
       <c r="I29" s="4" t="n">
-        <v>0.0454</v>
+        <v>0.0213</v>
       </c>
       <c r="K29" s="4" t="n">
-        <v>0.096</v>
+        <v>0.0256</v>
+      </c>
+      <c r="L29" s="4" t="n">
+        <v>0.0256</v>
       </c>
     </row>
     <row r="30">
@@ -15042,7 +15258,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C30" s="3" t="n">
@@ -15052,19 +15268,22 @@
         <v>0.25</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>0.0146</v>
+        <v>0.0451</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>0.0146</v>
+        <v>0.0454</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>0.0146</v>
+        <v>0.0454</v>
       </c>
       <c r="I30" s="4" t="n">
-        <v>0.0152</v>
+        <v>0.0454</v>
       </c>
       <c r="K30" s="4" t="n">
-        <v>0.0157</v>
+        <v>0.096</v>
+      </c>
+      <c r="L30" s="4" t="n">
+        <v>0.1027</v>
       </c>
     </row>
     <row r="31">
@@ -15075,7 +15294,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C31" s="3" t="n">
@@ -15085,19 +15304,22 @@
         <v>0.25</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>0.0195</v>
+        <v>0.0146</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.021</v>
+        <v>0.0146</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>0.021</v>
+        <v>0.0146</v>
       </c>
       <c r="I31" s="4" t="n">
-        <v>0.021</v>
+        <v>0.0152</v>
       </c>
       <c r="K31" s="4" t="n">
-        <v>0.0369</v>
+        <v>0.0157</v>
+      </c>
+      <c r="L31" s="4" t="n">
+        <v>0.0157</v>
       </c>
     </row>
     <row r="32">
@@ -15108,7 +15330,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C32" s="3" t="n">
@@ -15117,17 +15339,23 @@
       <c r="D32" s="4" t="n">
         <v>0.25</v>
       </c>
+      <c r="F32" s="4" t="n">
+        <v>0.0195</v>
+      </c>
       <c r="G32" s="4" t="n">
-        <v>0.0014</v>
+        <v>0.021</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>0.0014</v>
+        <v>0.021</v>
       </c>
       <c r="I32" s="4" t="n">
-        <v>0.0014</v>
+        <v>0.021</v>
       </c>
       <c r="K32" s="4" t="n">
-        <v>0.0014</v>
+        <v>0.0369</v>
+      </c>
+      <c r="L32" s="4" t="n">
+        <v>0.0369</v>
       </c>
     </row>
     <row r="33">
@@ -15138,7 +15366,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C33" s="3" t="n">
@@ -15147,8 +15375,20 @@
       <c r="D33" s="4" t="n">
         <v>0.25</v>
       </c>
+      <c r="G33" s="4" t="n">
+        <v>0.0014</v>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>0.0014</v>
+      </c>
+      <c r="I33" s="4" t="n">
+        <v>0.0014</v>
+      </c>
       <c r="K33" s="4" t="n">
-        <v>0.0063</v>
+        <v>0.0014</v>
+      </c>
+      <c r="L33" s="4" t="n">
+        <v>0.0014</v>
       </c>
     </row>
     <row r="34">
@@ -15159,72 +15399,64 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E34" s="5">
-        <f>SUM(E23:E33)</f>
-        <v/>
-      </c>
-      <c r="F34" s="5">
-        <f>SUM(F23:F33)</f>
-        <v/>
-      </c>
-      <c r="G34" s="5">
-        <f>SUM(G23:G33)</f>
-        <v/>
-      </c>
-      <c r="H34" s="5">
-        <f>SUM(H23:H33)</f>
-        <v/>
-      </c>
-      <c r="I34" s="5">
-        <f>SUM(I23:I33)</f>
-        <v/>
-      </c>
-      <c r="J34" s="5">
-        <f>SUM(J23:J33)</f>
-        <v/>
-      </c>
-      <c r="K34" s="5">
-        <f>SUM(K23:K33)</f>
-        <v/>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="n">
+        <v>31128200</v>
+      </c>
+      <c r="D34" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K34" s="4" t="n">
+        <v>0.0063</v>
+      </c>
+      <c r="L34" s="4" t="n">
+        <v>0.0063</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="n">
-        <v>28710400</v>
-      </c>
-      <c r="D35" s="4" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="E35" s="4" t="n">
-        <v>0.0832</v>
-      </c>
-      <c r="F35" s="4" t="n">
-        <v>0.0832</v>
-      </c>
-      <c r="G35" s="4" t="n">
-        <v>0.0832</v>
-      </c>
-      <c r="H35" s="4" t="n">
-        <v>0.0832</v>
-      </c>
-      <c r="I35" s="4" t="n">
-        <v>0.08349999999999999</v>
-      </c>
-      <c r="K35" s="4" t="n">
-        <v>0.08349999999999999</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E35" s="5">
+        <f>SUM(E24:E34)</f>
+        <v/>
+      </c>
+      <c r="F35" s="5">
+        <f>SUM(F24:F34)</f>
+        <v/>
+      </c>
+      <c r="G35" s="5">
+        <f>SUM(G24:G34)</f>
+        <v/>
+      </c>
+      <c r="H35" s="5">
+        <f>SUM(H24:H34)</f>
+        <v/>
+      </c>
+      <c r="I35" s="5">
+        <f>SUM(I24:I34)</f>
+        <v/>
+      </c>
+      <c r="J35" s="5">
+        <f>SUM(J24:J34)</f>
+        <v/>
+      </c>
+      <c r="K35" s="5">
+        <f>SUM(K24:K34)</f>
+        <v/>
+      </c>
+      <c r="L35" s="5">
+        <f>SUM(L24:L34)</f>
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -15235,7 +15467,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C36" s="3" t="n">
@@ -15245,22 +15477,25 @@
         <v>0.45</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>0.3459</v>
+        <v>0.0832</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>0.3459</v>
+        <v>0.0832</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.3459</v>
+        <v>0.0832</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>0.3459</v>
+        <v>0.0832</v>
       </c>
       <c r="I36" s="4" t="n">
-        <v>0.3459</v>
+        <v>0.08349999999999999</v>
       </c>
       <c r="K36" s="4" t="n">
-        <v>0.3459</v>
+        <v>0.08349999999999999</v>
+      </c>
+      <c r="L36" s="4" t="n">
+        <v>0.08349999999999999</v>
       </c>
     </row>
     <row r="37">
@@ -15271,7 +15506,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="C37" s="3" t="n">
@@ -15280,20 +15515,26 @@
       <c r="D37" s="4" t="n">
         <v>0.45</v>
       </c>
+      <c r="E37" s="4" t="n">
+        <v>0.3459</v>
+      </c>
       <c r="F37" s="4" t="n">
-        <v>0.0007000000000000001</v>
+        <v>0.3459</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>0.0007000000000000001</v>
+        <v>0.3459</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>0.0007000000000000001</v>
+        <v>0.3459</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>0.0007000000000000001</v>
+        <v>0.3459</v>
       </c>
       <c r="K37" s="4" t="n">
-        <v>0.0007000000000000001</v>
+        <v>0.3459</v>
+      </c>
+      <c r="L37" s="4" t="n">
+        <v>0.3459</v>
       </c>
     </row>
     <row r="38">
@@ -15304,7 +15545,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C38" s="3" t="n">
@@ -15313,8 +15554,23 @@
       <c r="D38" s="4" t="n">
         <v>0.45</v>
       </c>
+      <c r="F38" s="4" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
+      <c r="G38" s="4" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
+      <c r="H38" s="4" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
+      <c r="I38" s="4" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
       <c r="K38" s="4" t="n">
-        <v>0.4389</v>
+        <v>0.0007000000000000001</v>
+      </c>
+      <c r="L38" s="4" t="n">
+        <v>0.0007000000000000001</v>
       </c>
     </row>
     <row r="39">
@@ -15325,72 +15581,64 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E39" s="5">
-        <f>SUM(E35:E38)</f>
-        <v/>
-      </c>
-      <c r="F39" s="5">
-        <f>SUM(F35:F38)</f>
-        <v/>
-      </c>
-      <c r="G39" s="5">
-        <f>SUM(G35:G38)</f>
-        <v/>
-      </c>
-      <c r="H39" s="5">
-        <f>SUM(H35:H38)</f>
-        <v/>
-      </c>
-      <c r="I39" s="5">
-        <f>SUM(I35:I38)</f>
-        <v/>
-      </c>
-      <c r="J39" s="5">
-        <f>SUM(J35:J38)</f>
-        <v/>
-      </c>
-      <c r="K39" s="5">
-        <f>SUM(K35:K38)</f>
-        <v/>
+          <t>Malaysia</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="n">
+        <v>28710400</v>
+      </c>
+      <c r="D39" s="4" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="K39" s="4" t="n">
+        <v>0.4389</v>
+      </c>
+      <c r="L39" s="4" t="n">
+        <v>0.4389</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Australia</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="n">
-        <v>8750300</v>
-      </c>
-      <c r="D40" s="4" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="E40" s="4" t="n">
-        <v>0.0025</v>
-      </c>
-      <c r="F40" s="4" t="n">
-        <v>0.0025</v>
-      </c>
-      <c r="G40" s="4" t="n">
-        <v>0.0025</v>
-      </c>
-      <c r="H40" s="4" t="n">
-        <v>0.0025</v>
-      </c>
-      <c r="I40" s="4" t="n">
-        <v>0.0025</v>
-      </c>
-      <c r="K40" s="4" t="n">
-        <v>0.0025</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E40" s="5">
+        <f>SUM(E36:E39)</f>
+        <v/>
+      </c>
+      <c r="F40" s="5">
+        <f>SUM(F36:F39)</f>
+        <v/>
+      </c>
+      <c r="G40" s="5">
+        <f>SUM(G36:G39)</f>
+        <v/>
+      </c>
+      <c r="H40" s="5">
+        <f>SUM(H36:H39)</f>
+        <v/>
+      </c>
+      <c r="I40" s="5">
+        <f>SUM(I36:I39)</f>
+        <v/>
+      </c>
+      <c r="J40" s="5">
+        <f>SUM(J36:J39)</f>
+        <v/>
+      </c>
+      <c r="K40" s="5">
+        <f>SUM(K36:K39)</f>
+        <v/>
+      </c>
+      <c r="L40" s="5">
+        <f>SUM(L36:L39)</f>
+        <v/>
       </c>
     </row>
     <row r="41">
@@ -15401,7 +15649,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C41" s="3" t="n">
@@ -15411,22 +15659,25 @@
         <v>0.58</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>0.2277</v>
+        <v>0.0025</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>0.2285</v>
+        <v>0.0025</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>0.2297</v>
+        <v>0.0025</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>0.2419</v>
+        <v>0.0025</v>
       </c>
       <c r="I41" s="4" t="n">
-        <v>0.2441</v>
+        <v>0.0025</v>
       </c>
       <c r="K41" s="4" t="n">
-        <v>0.2444</v>
+        <v>0.0025</v>
+      </c>
+      <c r="L41" s="4" t="n">
+        <v>0.0025</v>
       </c>
     </row>
     <row r="42">
@@ -15437,7 +15688,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C42" s="3" t="n">
@@ -15447,22 +15698,25 @@
         <v>0.58</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>0.1228</v>
+        <v>0.2277</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>0.1253</v>
+        <v>0.2285</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>0.1543</v>
+        <v>0.2297</v>
       </c>
       <c r="H42" s="4" t="n">
-        <v>0.1545</v>
+        <v>0.2419</v>
       </c>
       <c r="I42" s="4" t="n">
-        <v>0.1549</v>
+        <v>0.2441</v>
       </c>
       <c r="K42" s="4" t="n">
-        <v>0.155</v>
+        <v>0.2444</v>
+      </c>
+      <c r="L42" s="4" t="n">
+        <v>0.4215</v>
       </c>
     </row>
     <row r="43">
@@ -15473,7 +15727,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C43" s="3" t="n">
@@ -15483,22 +15737,25 @@
         <v>0.58</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>0.0019</v>
+        <v>0.1228</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>0.0019</v>
+        <v>0.1253</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>0.0035</v>
+        <v>0.1543</v>
       </c>
       <c r="H43" s="4" t="n">
-        <v>0.0035</v>
+        <v>0.1545</v>
       </c>
       <c r="I43" s="4" t="n">
-        <v>0.0035</v>
+        <v>0.1549</v>
       </c>
       <c r="K43" s="4" t="n">
-        <v>0.016</v>
+        <v>0.155</v>
+      </c>
+      <c r="L43" s="4" t="n">
+        <v>0.1712</v>
       </c>
     </row>
     <row r="44">
@@ -15509,7 +15766,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Luxembourg</t>
         </is>
       </c>
       <c r="C44" s="3" t="n">
@@ -15519,22 +15776,25 @@
         <v>0.58</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>0.0068</v>
+        <v>0.0019</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>0.0095</v>
+        <v>0.0019</v>
       </c>
       <c r="G44" s="4" t="n">
-        <v>0.01</v>
+        <v>0.0035</v>
       </c>
       <c r="H44" s="4" t="n">
-        <v>0.0104</v>
+        <v>0.0035</v>
       </c>
       <c r="I44" s="4" t="n">
-        <v>0.0105</v>
+        <v>0.0035</v>
       </c>
       <c r="K44" s="4" t="n">
-        <v>0.0133</v>
+        <v>0.016</v>
+      </c>
+      <c r="L44" s="4" t="n">
+        <v>0.016</v>
       </c>
     </row>
     <row r="45">
@@ -15545,7 +15805,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="C45" s="3" t="n">
@@ -15555,22 +15815,25 @@
         <v>0.58</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>0.0191</v>
+        <v>0.0068</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>0.0236</v>
+        <v>0.0095</v>
       </c>
       <c r="G45" s="4" t="n">
-        <v>0.0294</v>
+        <v>0.01</v>
       </c>
       <c r="H45" s="4" t="n">
-        <v>0.03759999999999999</v>
+        <v>0.0104</v>
       </c>
       <c r="I45" s="4" t="n">
-        <v>0.0546</v>
+        <v>0.0105</v>
       </c>
       <c r="K45" s="4" t="n">
-        <v>0.0708</v>
+        <v>0.0133</v>
+      </c>
+      <c r="L45" s="4" t="n">
+        <v>0.0133</v>
       </c>
     </row>
     <row r="46">
@@ -15581,7 +15844,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C46" s="3" t="n">
@@ -15590,20 +15853,26 @@
       <c r="D46" s="4" t="n">
         <v>0.58</v>
       </c>
+      <c r="E46" s="4" t="n">
+        <v>0.0191</v>
+      </c>
       <c r="F46" s="4" t="n">
-        <v>0.0017</v>
+        <v>0.0236</v>
       </c>
       <c r="G46" s="4" t="n">
-        <v>0.0028</v>
+        <v>0.0294</v>
       </c>
       <c r="H46" s="4" t="n">
-        <v>0.006500000000000001</v>
+        <v>0.03759999999999999</v>
       </c>
       <c r="I46" s="4" t="n">
-        <v>0.0066</v>
+        <v>0.0546</v>
       </c>
       <c r="K46" s="4" t="n">
-        <v>0.0066</v>
+        <v>0.0708</v>
+      </c>
+      <c r="L46" s="4" t="n">
+        <v>0.0708</v>
       </c>
     </row>
     <row r="47">
@@ -15614,7 +15883,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C47" s="3" t="n">
@@ -15624,19 +15893,22 @@
         <v>0.58</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.0017</v>
       </c>
       <c r="G47" s="4" t="n">
-        <v>0.06950000000000001</v>
+        <v>0.0028</v>
       </c>
       <c r="H47" s="4" t="n">
-        <v>0.1435</v>
+        <v>0.006500000000000001</v>
       </c>
       <c r="I47" s="4" t="n">
-        <v>0.2085</v>
+        <v>0.0066</v>
       </c>
       <c r="K47" s="4" t="n">
-        <v>0.29</v>
+        <v>0.0066</v>
+      </c>
+      <c r="L47" s="4" t="n">
+        <v>0.0072</v>
       </c>
     </row>
     <row r="48">
@@ -15647,7 +15919,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C48" s="3" t="n">
@@ -15656,17 +15928,23 @@
       <c r="D48" s="4" t="n">
         <v>0.58</v>
       </c>
+      <c r="F48" s="4" t="n">
+        <v>0.008500000000000001</v>
+      </c>
       <c r="G48" s="4" t="n">
-        <v>0.0005</v>
+        <v>0.06950000000000001</v>
       </c>
       <c r="H48" s="4" t="n">
-        <v>0.0001</v>
+        <v>0.1435</v>
       </c>
       <c r="I48" s="4" t="n">
-        <v>0.0001</v>
+        <v>0.2085</v>
       </c>
       <c r="K48" s="4" t="n">
-        <v>0.0001</v>
+        <v>0.29</v>
+      </c>
+      <c r="L48" s="4" t="n">
+        <v>0.2946</v>
       </c>
     </row>
     <row r="49">
@@ -15677,7 +15955,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C49" s="3" t="n">
@@ -15687,16 +15965,19 @@
         <v>0.58</v>
       </c>
       <c r="G49" s="4" t="n">
-        <v>0</v>
+        <v>0.0005</v>
       </c>
       <c r="H49" s="4" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="I49" s="4" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="K49" s="4" t="n">
-        <v>0</v>
+        <v>0.0001</v>
+      </c>
+      <c r="L49" s="4" t="n">
+        <v>0.0001</v>
       </c>
     </row>
     <row r="50">
@@ -15707,7 +15988,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C50" s="3" t="n">
@@ -15717,16 +15998,19 @@
         <v>0.58</v>
       </c>
       <c r="G50" s="4" t="n">
-        <v>0.0022</v>
+        <v>0</v>
       </c>
       <c r="H50" s="4" t="n">
-        <v>0.0022</v>
+        <v>0</v>
       </c>
       <c r="I50" s="4" t="n">
-        <v>0.0022</v>
+        <v>0</v>
       </c>
       <c r="K50" s="4" t="n">
-        <v>0.0022</v>
+        <v>0</v>
+      </c>
+      <c r="L50" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -15737,7 +16021,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C51" s="3" t="n">
@@ -15747,16 +16031,19 @@
         <v>0.58</v>
       </c>
       <c r="G51" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.0022</v>
       </c>
       <c r="H51" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.0022</v>
       </c>
       <c r="I51" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.0022</v>
       </c>
       <c r="K51" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.0022</v>
+      </c>
+      <c r="L51" s="4" t="n">
+        <v>0.0022</v>
       </c>
     </row>
     <row r="52">
@@ -15767,7 +16054,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="C52" s="3" t="n">
@@ -15777,16 +16064,19 @@
         <v>0.58</v>
       </c>
       <c r="G52" s="4" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
       <c r="H52" s="4" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
       <c r="I52" s="4" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
       <c r="K52" s="4" t="n">
-        <v>0</v>
+        <v>0.0004</v>
+      </c>
+      <c r="L52" s="4" t="n">
+        <v>0.0004</v>
       </c>
     </row>
     <row r="53">
@@ -15797,7 +16087,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C53" s="3" t="n">
@@ -15806,6 +16096,9 @@
       <c r="D53" s="4" t="n">
         <v>0.58</v>
       </c>
+      <c r="G53" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="H53" s="4" t="n">
         <v>0</v>
       </c>
@@ -15815,6 +16108,9 @@
       <c r="K53" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L53" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -15824,7 +16120,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C54" s="3" t="n">
@@ -15842,6 +16138,9 @@
       <c r="K54" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L54" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -15851,7 +16150,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C55" s="3" t="n">
@@ -15860,12 +16159,18 @@
       <c r="D55" s="4" t="n">
         <v>0.58</v>
       </c>
+      <c r="H55" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="I55" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K55" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L55" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -15875,7 +16180,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="C56" s="3" t="n">
@@ -15884,8 +16189,14 @@
       <c r="D56" s="4" t="n">
         <v>0.58</v>
       </c>
+      <c r="I56" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K56" s="4" t="n">
-        <v>0.0001</v>
+        <v>0</v>
+      </c>
+      <c r="L56" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -15896,72 +16207,64 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E57" s="5">
-        <f>SUM(E40:E56)</f>
-        <v/>
-      </c>
-      <c r="F57" s="5">
-        <f>SUM(F40:F56)</f>
-        <v/>
-      </c>
-      <c r="G57" s="5">
-        <f>SUM(G40:G56)</f>
-        <v/>
-      </c>
-      <c r="H57" s="5">
-        <f>SUM(H40:H56)</f>
-        <v/>
-      </c>
-      <c r="I57" s="5">
-        <f>SUM(I40:I56)</f>
-        <v/>
-      </c>
-      <c r="J57" s="5">
-        <f>SUM(J40:J56)</f>
-        <v/>
-      </c>
-      <c r="K57" s="5">
-        <f>SUM(K40:K56)</f>
-        <v/>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="n">
+        <v>8750300</v>
+      </c>
+      <c r="D57" s="4" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="K57" s="4" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="L57" s="4" t="n">
+        <v>0.0001</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="C58" s="3" t="n">
-        <v>16514800</v>
-      </c>
-      <c r="D58" s="4" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="E58" s="4" t="n">
-        <v>0.0029</v>
-      </c>
-      <c r="F58" s="4" t="n">
-        <v>0.0029</v>
-      </c>
-      <c r="G58" s="4" t="n">
-        <v>0.0029</v>
-      </c>
-      <c r="H58" s="4" t="n">
-        <v>0.0325</v>
-      </c>
-      <c r="I58" s="4" t="n">
-        <v>0.0898</v>
-      </c>
-      <c r="K58" s="4" t="n">
-        <v>0.1142</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E58" s="5">
+        <f>SUM(E41:E57)</f>
+        <v/>
+      </c>
+      <c r="F58" s="5">
+        <f>SUM(F41:F57)</f>
+        <v/>
+      </c>
+      <c r="G58" s="5">
+        <f>SUM(G41:G57)</f>
+        <v/>
+      </c>
+      <c r="H58" s="5">
+        <f>SUM(H41:H57)</f>
+        <v/>
+      </c>
+      <c r="I58" s="5">
+        <f>SUM(I41:I57)</f>
+        <v/>
+      </c>
+      <c r="J58" s="5">
+        <f>SUM(J41:J57)</f>
+        <v/>
+      </c>
+      <c r="K58" s="5">
+        <f>SUM(K41:K57)</f>
+        <v/>
+      </c>
+      <c r="L58" s="5">
+        <f>SUM(L41:L57)</f>
+        <v/>
       </c>
     </row>
     <row r="59">
@@ -15972,7 +16275,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C59" s="3" t="n">
@@ -15982,22 +16285,25 @@
         <v>0.59</v>
       </c>
       <c r="E59" s="4" t="n">
-        <v>0.0339</v>
+        <v>0.0029</v>
       </c>
       <c r="F59" s="4" t="n">
-        <v>0.0339</v>
+        <v>0.0029</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>0.0339</v>
+        <v>0.0029</v>
       </c>
       <c r="H59" s="4" t="n">
-        <v>0.0339</v>
+        <v>0.0325</v>
       </c>
       <c r="I59" s="4" t="n">
-        <v>0.04269999999999999</v>
+        <v>0.0898</v>
       </c>
       <c r="K59" s="4" t="n">
-        <v>0.04269999999999999</v>
+        <v>0.1142</v>
+      </c>
+      <c r="L59" s="4" t="n">
+        <v>0.1433</v>
       </c>
     </row>
     <row r="60">
@@ -16008,7 +16314,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C60" s="3" t="n">
@@ -16018,22 +16324,25 @@
         <v>0.59</v>
       </c>
       <c r="E60" s="4" t="n">
-        <v>0.4926</v>
+        <v>0.0339</v>
       </c>
       <c r="F60" s="4" t="n">
-        <v>0.4926</v>
+        <v>0.0339</v>
       </c>
       <c r="G60" s="4" t="n">
-        <v>0.4926</v>
+        <v>0.0339</v>
       </c>
       <c r="H60" s="4" t="n">
-        <v>0.4926</v>
+        <v>0.0339</v>
       </c>
       <c r="I60" s="4" t="n">
-        <v>0.4926</v>
+        <v>0.04269999999999999</v>
       </c>
       <c r="K60" s="4" t="n">
-        <v>0.4926</v>
+        <v>0.04269999999999999</v>
+      </c>
+      <c r="L60" s="4" t="n">
+        <v>0.04269999999999999</v>
       </c>
     </row>
     <row r="61">
@@ -16044,7 +16353,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C61" s="3" t="n">
@@ -16054,22 +16363,25 @@
         <v>0.59</v>
       </c>
       <c r="E61" s="4" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.4926</v>
       </c>
       <c r="F61" s="4" t="n">
-        <v>0.0146</v>
+        <v>0.4926</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>0.0161</v>
+        <v>0.4926</v>
       </c>
       <c r="H61" s="4" t="n">
-        <v>0.0161</v>
+        <v>0.4926</v>
       </c>
       <c r="I61" s="4" t="n">
-        <v>0.0161</v>
+        <v>0.4926</v>
       </c>
       <c r="K61" s="4" t="n">
-        <v>0.0161</v>
+        <v>0.4926</v>
+      </c>
+      <c r="L61" s="4" t="n">
+        <v>0.4926</v>
       </c>
     </row>
     <row r="62">
@@ -16080,7 +16392,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C62" s="3" t="n">
@@ -16089,17 +16401,26 @@
       <c r="D62" s="4" t="n">
         <v>0.59</v>
       </c>
+      <c r="E62" s="4" t="n">
+        <v>0.008800000000000001</v>
+      </c>
+      <c r="F62" s="4" t="n">
+        <v>0.0146</v>
+      </c>
       <c r="G62" s="4" t="n">
-        <v>0.0044</v>
+        <v>0.0161</v>
       </c>
       <c r="H62" s="4" t="n">
-        <v>0.0044</v>
+        <v>0.0161</v>
       </c>
       <c r="I62" s="4" t="n">
-        <v>0.0044</v>
+        <v>0.0161</v>
       </c>
       <c r="K62" s="4" t="n">
-        <v>0.0044</v>
+        <v>0.0161</v>
+      </c>
+      <c r="L62" s="4" t="n">
+        <v>0.0161</v>
       </c>
     </row>
     <row r="63">
@@ -16110,72 +16431,73 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E63" s="5">
-        <f>SUM(E58:E62)</f>
-        <v/>
-      </c>
-      <c r="F63" s="5">
-        <f>SUM(F58:F62)</f>
-        <v/>
-      </c>
-      <c r="G63" s="5">
-        <f>SUM(G58:G62)</f>
-        <v/>
-      </c>
-      <c r="H63" s="5">
-        <f>SUM(H58:H62)</f>
-        <v/>
-      </c>
-      <c r="I63" s="5">
-        <f>SUM(I58:I62)</f>
-        <v/>
-      </c>
-      <c r="J63" s="5">
-        <f>SUM(J58:J62)</f>
-        <v/>
-      </c>
-      <c r="K63" s="5">
-        <f>SUM(K58:K62)</f>
-        <v/>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="n">
+        <v>16514800</v>
+      </c>
+      <c r="D63" s="4" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="G63" s="4" t="n">
+        <v>0.0044</v>
+      </c>
+      <c r="H63" s="4" t="n">
+        <v>0.0044</v>
+      </c>
+      <c r="I63" s="4" t="n">
+        <v>0.0044</v>
+      </c>
+      <c r="K63" s="4" t="n">
+        <v>0.0044</v>
+      </c>
+      <c r="L63" s="4" t="n">
+        <v>0.0044</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="n">
-        <v>3467600</v>
-      </c>
-      <c r="D64" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="E64" s="4" t="n">
-        <v>0.0004</v>
-      </c>
-      <c r="F64" s="4" t="n">
-        <v>0.0021</v>
-      </c>
-      <c r="G64" s="4" t="n">
-        <v>0.0021</v>
-      </c>
-      <c r="H64" s="4" t="n">
-        <v>0.0021</v>
-      </c>
-      <c r="I64" s="4" t="n">
-        <v>0.0021</v>
-      </c>
-      <c r="K64" s="4" t="n">
-        <v>0.0021</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E64" s="5">
+        <f>SUM(E59:E63)</f>
+        <v/>
+      </c>
+      <c r="F64" s="5">
+        <f>SUM(F59:F63)</f>
+        <v/>
+      </c>
+      <c r="G64" s="5">
+        <f>SUM(G59:G63)</f>
+        <v/>
+      </c>
+      <c r="H64" s="5">
+        <f>SUM(H59:H63)</f>
+        <v/>
+      </c>
+      <c r="I64" s="5">
+        <f>SUM(I59:I63)</f>
+        <v/>
+      </c>
+      <c r="J64" s="5">
+        <f>SUM(J59:J63)</f>
+        <v/>
+      </c>
+      <c r="K64" s="5">
+        <f>SUM(K59:K63)</f>
+        <v/>
+      </c>
+      <c r="L64" s="5">
+        <f>SUM(L59:L63)</f>
+        <v/>
       </c>
     </row>
     <row r="65">
@@ -16186,7 +16508,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C65" s="3" t="n">
@@ -16196,22 +16518,25 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E65" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.0004</v>
       </c>
       <c r="F65" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.0021</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.0021</v>
       </c>
       <c r="H65" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.0021</v>
       </c>
       <c r="I65" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.0021</v>
       </c>
       <c r="K65" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.0021</v>
+      </c>
+      <c r="L65" s="4" t="n">
+        <v>0.0021</v>
       </c>
     </row>
     <row r="66">
@@ -16222,7 +16547,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C66" s="3" t="n">
@@ -16232,22 +16557,25 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E66" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0032</v>
       </c>
       <c r="F66" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0032</v>
       </c>
       <c r="G66" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0032</v>
       </c>
       <c r="H66" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0032</v>
       </c>
       <c r="I66" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0032</v>
       </c>
       <c r="K66" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0032</v>
+      </c>
+      <c r="L66" s="4" t="n">
+        <v>0.0032</v>
       </c>
     </row>
     <row r="67">
@@ -16258,7 +16586,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C67" s="3" t="n">
@@ -16268,27 +16596,25 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E67" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.0204</v>
       </c>
       <c r="F67" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.0204</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.0204</v>
       </c>
       <c r="H67" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.0204</v>
       </c>
       <c r="I67" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.0204</v>
       </c>
       <c r="K67" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="L67" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
+        <v>0.0204</v>
+      </c>
+      <c r="L67" s="4" t="n">
+        <v>0.0204</v>
       </c>
     </row>
     <row r="68">
@@ -16299,7 +16625,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C68" s="3" t="n">
@@ -16309,22 +16635,30 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E68" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="F68" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G68" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H68" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="I68" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="K68" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="L68" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
       </c>
     </row>
     <row r="69">
@@ -16335,7 +16669,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C69" s="3" t="n">
@@ -16345,22 +16679,25 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E69" s="4" t="n">
-        <v>0.1798</v>
+        <v>0.0004</v>
       </c>
       <c r="F69" s="4" t="n">
-        <v>0.1798</v>
+        <v>0.0004</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>0.2828</v>
+        <v>0.0004</v>
       </c>
       <c r="H69" s="4" t="n">
-        <v>0.2828</v>
+        <v>0.0004</v>
       </c>
       <c r="I69" s="4" t="n">
-        <v>0.2828</v>
+        <v>0.0004</v>
       </c>
       <c r="K69" s="4" t="n">
-        <v>0.2828</v>
+        <v>0.0004</v>
+      </c>
+      <c r="L69" s="4" t="n">
+        <v>0.0004</v>
       </c>
     </row>
     <row r="70">
@@ -16371,7 +16708,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C70" s="3" t="n">
@@ -16380,20 +16717,26 @@
       <c r="D70" s="4" t="n">
         <v>0.6899999999999999</v>
       </c>
+      <c r="E70" s="4" t="n">
+        <v>0.1798</v>
+      </c>
       <c r="F70" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.1798</v>
       </c>
       <c r="G70" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.2828</v>
       </c>
       <c r="H70" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.2828</v>
       </c>
       <c r="I70" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.2828</v>
       </c>
       <c r="K70" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.2828</v>
+      </c>
+      <c r="L70" s="4" t="n">
+        <v>0.2828</v>
       </c>
     </row>
     <row r="71">
@@ -16404,7 +16747,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Luxembourg</t>
         </is>
       </c>
       <c r="C71" s="3" t="n">
@@ -16413,17 +16756,23 @@
       <c r="D71" s="4" t="n">
         <v>0.6899999999999999</v>
       </c>
+      <c r="F71" s="4" t="n">
+        <v>0.0012</v>
+      </c>
       <c r="G71" s="4" t="n">
-        <v>0</v>
+        <v>0.0012</v>
       </c>
       <c r="H71" s="4" t="n">
-        <v>0</v>
+        <v>0.0012</v>
       </c>
       <c r="I71" s="4" t="n">
-        <v>0</v>
+        <v>0.0012</v>
       </c>
       <c r="K71" s="4" t="n">
-        <v>0</v>
+        <v>0.0012</v>
+      </c>
+      <c r="L71" s="4" t="n">
+        <v>0.0012</v>
       </c>
     </row>
     <row r="72">
@@ -16434,35 +16783,72 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D72" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G72" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I72" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K72" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L72" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E72" s="5">
-        <f>SUM(E64:E71)</f>
-        <v/>
-      </c>
-      <c r="F72" s="5">
-        <f>SUM(F64:F71)</f>
-        <v/>
-      </c>
-      <c r="G72" s="5">
-        <f>SUM(G64:G71)</f>
-        <v/>
-      </c>
-      <c r="H72" s="5">
-        <f>SUM(H64:H71)</f>
-        <v/>
-      </c>
-      <c r="I72" s="5">
-        <f>SUM(I64:I71)</f>
-        <v/>
-      </c>
-      <c r="J72" s="5">
-        <f>SUM(J64:J71)</f>
-        <v/>
-      </c>
-      <c r="K72" s="5">
-        <f>SUM(K64:K71)</f>
+      <c r="E73" s="5">
+        <f>SUM(E65:E72)</f>
+        <v/>
+      </c>
+      <c r="F73" s="5">
+        <f>SUM(F65:F72)</f>
+        <v/>
+      </c>
+      <c r="G73" s="5">
+        <f>SUM(G65:G72)</f>
+        <v/>
+      </c>
+      <c r="H73" s="5">
+        <f>SUM(H65:H72)</f>
+        <v/>
+      </c>
+      <c r="I73" s="5">
+        <f>SUM(I65:I72)</f>
+        <v/>
+      </c>
+      <c r="J73" s="5">
+        <f>SUM(J65:J72)</f>
+        <v/>
+      </c>
+      <c r="K73" s="5">
+        <f>SUM(K65:K72)</f>
+        <v/>
+      </c>
+      <c r="L73" s="5">
+        <f>SUM(L65:L72)</f>
         <v/>
       </c>
     </row>
@@ -16477,7 +16863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E78"/>
+  <dimension ref="A1:E90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16589,13 +16975,13 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0</v>
+        <v>8.27</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0</v>
+        <v>295.3571428571428</v>
       </c>
     </row>
     <row r="12">
@@ -16715,13 +17101,13 @@
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>4262.799999999999</v>
+        <v>5813.71</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>7312.120000000001</v>
+        <v>9938.76</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>1715.332645209722</v>
+        <v>1709.538315464652</v>
       </c>
     </row>
     <row r="18">
@@ -16757,13 +17143,13 @@
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>54.23</v>
+        <v>127.72</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>57.19</v>
+        <v>125.6</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>1054.582334501199</v>
+        <v>983.401190103351</v>
       </c>
     </row>
     <row r="20">
@@ -16778,13 +17164,13 @@
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>354.8699999999999</v>
+        <v>399.2</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>1531.98</v>
+        <v>1721.69</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>4317.017499365965</v>
+        <v>4312.850701402806</v>
       </c>
     </row>
     <row r="21">
@@ -16841,13 +17227,13 @@
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>8243.16</v>
+        <v>8807.609999999999</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>9949.52</v>
+        <v>11940</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>1207.003139572688</v>
+        <v>1355.645856253853</v>
       </c>
     </row>
     <row r="24">
@@ -16862,13 +17248,13 @@
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>32.77</v>
+        <v>43.15</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>72.72999999999999</v>
+        <v>98.15000000000001</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>2219.407995117485</v>
+        <v>2274.623406720742</v>
       </c>
     </row>
     <row r="25">
@@ -16904,13 +17290,13 @@
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>2600.28</v>
+        <v>3540.700000000001</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>5688.669999999999</v>
+        <v>7802.979999999999</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>2187.714399987693</v>
+        <v>2203.79585957579</v>
       </c>
     </row>
     <row r="27">
@@ -16925,13 +17311,13 @@
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>8.709999999999999</v>
+        <v>13.38</v>
       </c>
       <c r="D27" s="6" t="n">
-        <v>20.06</v>
+        <v>32.54</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>2303.099885189438</v>
+        <v>2431.988041853513</v>
       </c>
     </row>
     <row r="28">
@@ -16946,13 +17332,13 @@
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>741.5</v>
+        <v>1477.26</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>1138.12</v>
+        <v>2260.03</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>1534.888739042481</v>
+        <v>1529.879642039993</v>
       </c>
     </row>
     <row r="29">
@@ -16963,17 +17349,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>230.06</v>
+        <v>645.8000000000001</v>
       </c>
       <c r="D29" s="6" t="n">
-        <v>299.02</v>
+        <v>786.75</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>1299.747891854299</v>
+        <v>1218.256426138123</v>
       </c>
     </row>
     <row r="30">
@@ -16984,17 +17370,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>1425.92</v>
+        <v>424.12</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>1699.87</v>
+        <v>761.33</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>1192.121577648115</v>
+        <v>1795.081580684712</v>
       </c>
     </row>
     <row r="31">
@@ -17005,17 +17391,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C31" s="6" t="n">
-        <v>0.04</v>
+        <v>2851.83</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>0.19</v>
+        <v>3001.82</v>
       </c>
       <c r="E31" s="6" t="n">
-        <v>4750</v>
+        <v>1052.594299099175</v>
       </c>
     </row>
     <row r="32">
@@ -17026,17 +17412,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>1520.24</v>
+        <v>0.04</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>1562.54</v>
+        <v>0.19</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>1027.824554017787</v>
+        <v>4750</v>
       </c>
     </row>
     <row r="33">
@@ -17047,38 +17433,38 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C33" s="6" t="n">
-        <v>3460.769999999999</v>
+        <v>1641.42</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>6425.440000000001</v>
+        <v>1690.42</v>
       </c>
       <c r="E33" s="6" t="n">
-        <v>1856.650398610715</v>
+        <v>1029.852201142913</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C34" s="6" t="n">
-        <v>6.44</v>
+        <v>4452.63</v>
       </c>
       <c r="D34" s="6" t="n">
-        <v>38.19</v>
+        <v>8263.219999999999</v>
       </c>
       <c r="E34" s="6" t="n">
-        <v>5930.124223602485</v>
+        <v>1855.80656825292</v>
       </c>
     </row>
     <row r="35">
@@ -17114,13 +17500,13 @@
         </is>
       </c>
       <c r="C36" s="6" t="n">
-        <v>582.0599999999999</v>
+        <v>824.96</v>
       </c>
       <c r="D36" s="6" t="n">
-        <v>728.85</v>
+        <v>1032.88</v>
       </c>
       <c r="E36" s="6" t="n">
-        <v>1252.190495825173</v>
+        <v>1252.036462373933</v>
       </c>
     </row>
     <row r="37">
@@ -17198,13 +17584,13 @@
         </is>
       </c>
       <c r="C40" s="6" t="n">
-        <v>409.57</v>
+        <v>447.02</v>
       </c>
       <c r="D40" s="6" t="n">
-        <v>751.4299999999999</v>
+        <v>827.6900000000001</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>1834.680274434163</v>
+        <v>1851.572636571071</v>
       </c>
     </row>
     <row r="41">
@@ -17219,13 +17605,13 @@
         </is>
       </c>
       <c r="C41" s="6" t="n">
-        <v>9983.290000000001</v>
+        <v>14339.53</v>
       </c>
       <c r="D41" s="6" t="n">
-        <v>15988.71</v>
+        <v>23370.68</v>
       </c>
       <c r="E41" s="6" t="n">
-        <v>1601.547185346714</v>
+        <v>1629.807950469785</v>
       </c>
     </row>
     <row r="42">
@@ -17240,13 +17626,13 @@
         </is>
       </c>
       <c r="C42" s="6" t="n">
-        <v>87.97</v>
+        <v>160.98</v>
       </c>
       <c r="D42" s="6" t="n">
-        <v>180.34</v>
+        <v>274.8</v>
       </c>
       <c r="E42" s="6" t="n">
-        <v>2050.017051267478</v>
+        <v>1707.044353335818</v>
       </c>
     </row>
     <row r="43">
@@ -17282,13 +17668,13 @@
         </is>
       </c>
       <c r="C44" s="6" t="n">
-        <v>3311.71</v>
+        <v>3609.36</v>
       </c>
       <c r="D44" s="6" t="n">
-        <v>4170.44</v>
+        <v>4508.49</v>
       </c>
       <c r="E44" s="6" t="n">
-        <v>1259.301086145828</v>
+        <v>1249.110645654631</v>
       </c>
     </row>
     <row r="45">
@@ -17299,17 +17685,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="C45" s="6" t="n">
-        <v>0.12</v>
+        <v>144.18</v>
       </c>
       <c r="D45" s="6" t="n">
-        <v>0.25</v>
+        <v>204.36</v>
       </c>
       <c r="E45" s="6" t="n">
-        <v>2083.333333333333</v>
+        <v>1417.394923012901</v>
       </c>
     </row>
     <row r="46">
@@ -17320,17 +17706,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C46" s="6" t="n">
-        <v>3666.65</v>
+        <v>0.12</v>
       </c>
       <c r="D46" s="6" t="n">
-        <v>5877.52</v>
+        <v>0.25</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>1602.967286214938</v>
+        <v>2083.333333333333</v>
       </c>
     </row>
     <row r="47">
@@ -17341,17 +17727,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C47" s="6" t="n">
-        <v>23.05</v>
+        <v>5138.799999999999</v>
       </c>
       <c r="D47" s="6" t="n">
-        <v>29.59</v>
+        <v>8197.349999999999</v>
       </c>
       <c r="E47" s="6" t="n">
-        <v>1283.731019522776</v>
+        <v>1595.187592434031</v>
       </c>
     </row>
     <row r="48">
@@ -17362,17 +17748,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C48" s="6" t="n">
-        <v>1412.89</v>
+        <v>542.15</v>
       </c>
       <c r="D48" s="6" t="n">
-        <v>1664.87</v>
+        <v>737.62</v>
       </c>
       <c r="E48" s="6" t="n">
-        <v>1178.343678559548</v>
+        <v>1360.545974361339</v>
       </c>
     </row>
     <row r="49">
@@ -17383,17 +17769,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C49" s="6" t="n">
-        <v>0.63</v>
+        <v>1412.89</v>
       </c>
       <c r="D49" s="6" t="n">
-        <v>1.37</v>
+        <v>1664.87</v>
       </c>
       <c r="E49" s="6" t="n">
-        <v>2174.603174603174</v>
+        <v>1178.343678559548</v>
       </c>
     </row>
     <row r="50">
@@ -17404,17 +17790,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="C50" s="6" t="n">
-        <v>9998.359999999999</v>
+        <v>0.33</v>
       </c>
       <c r="D50" s="6" t="n">
-        <v>20823.45</v>
+        <v>1.37</v>
       </c>
       <c r="E50" s="6" t="n">
-        <v>2082.686560595938</v>
+        <v>4151.515151515151</v>
       </c>
     </row>
     <row r="51">
@@ -17425,59 +17811,59 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C51" s="6" t="n">
-        <v>1147.37</v>
+        <v>0.63</v>
       </c>
       <c r="D51" s="6" t="n">
-        <v>1533.44</v>
+        <v>1.37</v>
       </c>
       <c r="E51" s="6" t="n">
-        <v>1336.482564473535</v>
+        <v>2174.603174603174</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C52" s="6" t="n">
-        <v>19.72</v>
+        <v>14911.05</v>
       </c>
       <c r="D52" s="6" t="n">
-        <v>39.63</v>
+        <v>31301.04</v>
       </c>
       <c r="E52" s="6" t="n">
-        <v>2009.634888438134</v>
+        <v>2099.184162081141</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C53" s="6" t="n">
-        <v>1721.39</v>
+        <v>1281.18</v>
       </c>
       <c r="D53" s="6" t="n">
-        <v>1312.5</v>
+        <v>1691.49</v>
       </c>
       <c r="E53" s="6" t="n">
-        <v>762.465217062955</v>
+        <v>1320.259448321079</v>
       </c>
     </row>
     <row r="54">
@@ -17488,17 +17874,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C54" s="6" t="n">
-        <v>2348.38</v>
+        <v>25.53</v>
       </c>
       <c r="D54" s="6" t="n">
-        <v>3384.33</v>
+        <v>42.55</v>
       </c>
       <c r="E54" s="6" t="n">
-        <v>1441.133888041969</v>
+        <v>1666.666666666667</v>
       </c>
     </row>
     <row r="55">
@@ -17509,101 +17895,101 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="C55" s="6" t="n">
-        <v>212.86</v>
+        <v>19.72</v>
       </c>
       <c r="D55" s="6" t="n">
-        <v>318.99</v>
+        <v>39.63</v>
       </c>
       <c r="E55" s="6" t="n">
-        <v>1498.590622944658</v>
+        <v>2009.634888438134</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C56" s="6" t="n">
-        <v>60.87</v>
+        <v>7.25</v>
       </c>
       <c r="D56" s="6" t="n">
-        <v>132.23</v>
+        <v>19.82</v>
       </c>
       <c r="E56" s="6" t="n">
-        <v>2172.334483325119</v>
+        <v>2733.793103448276</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C57" s="6" t="n">
-        <v>25.53</v>
+        <v>1721.39</v>
       </c>
       <c r="D57" s="6" t="n">
-        <v>46.35</v>
+        <v>1312.5</v>
       </c>
       <c r="E57" s="6" t="n">
-        <v>1815.51116333725</v>
+        <v>762.465217062955</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C58" s="6" t="n">
-        <v>112.54</v>
+        <v>5026.549999999999</v>
       </c>
       <c r="D58" s="6" t="n">
-        <v>228.5</v>
+        <v>6984.03</v>
       </c>
       <c r="E58" s="6" t="n">
-        <v>2030.389194952905</v>
+        <v>1389.428136594682</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C59" s="6" t="n">
-        <v>0.01</v>
+        <v>228.32</v>
       </c>
       <c r="D59" s="6" t="n">
-        <v>0.01</v>
+        <v>339.98</v>
       </c>
       <c r="E59" s="6" t="n">
-        <v>1000</v>
+        <v>1489.050455501051</v>
       </c>
     </row>
     <row r="60">
@@ -17614,17 +18000,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C60" s="6" t="n">
-        <v>273.6</v>
+        <v>86.63</v>
       </c>
       <c r="D60" s="6" t="n">
-        <v>410.07</v>
+        <v>188.27</v>
       </c>
       <c r="E60" s="6" t="n">
-        <v>1498.793859649123</v>
+        <v>2173.265612374466</v>
       </c>
     </row>
     <row r="61">
@@ -17635,17 +18021,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C61" s="6" t="n">
-        <v>48.36</v>
+        <v>25.8</v>
       </c>
       <c r="D61" s="6" t="n">
-        <v>97.23999999999999</v>
+        <v>47.1</v>
       </c>
       <c r="E61" s="6" t="n">
-        <v>2010.752688172043</v>
+        <v>1825.581395348837</v>
       </c>
     </row>
     <row r="62">
@@ -17656,17 +18042,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C62" s="6" t="n">
-        <v>278.34</v>
+        <v>112.54</v>
       </c>
       <c r="D62" s="6" t="n">
-        <v>281.93</v>
+        <v>228.5</v>
       </c>
       <c r="E62" s="6" t="n">
-        <v>1012.897894661206</v>
+        <v>2030.389194952905</v>
       </c>
     </row>
     <row r="63">
@@ -17677,248 +18063,248 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C63" s="6" t="n">
-        <v>1037.32</v>
+        <v>0.01</v>
       </c>
       <c r="D63" s="6" t="n">
-        <v>2204.18</v>
+        <v>0.01</v>
       </c>
       <c r="E63" s="6" t="n">
-        <v>2124.879497165774</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C64" s="6" t="n">
-        <v>968.02</v>
+        <v>273.96</v>
       </c>
       <c r="D64" s="6" t="n">
-        <v>1201.9</v>
+        <v>412.03</v>
       </c>
       <c r="E64" s="6" t="n">
-        <v>1241.60657837648</v>
+        <v>1503.978683019419</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="C65" s="6" t="n">
-        <v>72.62</v>
+        <v>0</v>
       </c>
       <c r="D65" s="6" t="n">
-        <v>98.56999999999999</v>
+        <v>1.29</v>
       </c>
       <c r="E65" s="6" t="n">
-        <v>1357.339575874415</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C66" s="6" t="n">
-        <v>2059.47</v>
+        <v>61.92</v>
       </c>
       <c r="D66" s="6" t="n">
-        <v>3323.92</v>
+        <v>127.05</v>
       </c>
       <c r="E66" s="6" t="n">
-        <v>1613.968642417709</v>
+        <v>2051.841085271318</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C67" s="6" t="n">
-        <v>70.03</v>
+        <v>278.34</v>
       </c>
       <c r="D67" s="6" t="n">
-        <v>58.73</v>
+        <v>281.93</v>
       </c>
       <c r="E67" s="6" t="n">
-        <v>838.640582607454</v>
+        <v>1012.897894661206</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C68" s="6" t="n">
-        <v>24.4</v>
+        <v>1389.84</v>
       </c>
       <c r="D68" s="6" t="n">
-        <v>64.56999999999999</v>
+        <v>3032.35</v>
       </c>
       <c r="E68" s="6" t="n">
-        <v>2646.311475409836</v>
+        <v>2181.797904794797</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C69" s="6" t="n">
-        <v>54.89</v>
+        <v>145.18</v>
       </c>
       <c r="D69" s="6" t="n">
-        <v>80.14</v>
+        <v>179.39</v>
       </c>
       <c r="E69" s="6" t="n">
-        <v>1460.010930952815</v>
+        <v>1235.638517702163</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C70" s="6" t="n">
-        <v>22943.82</v>
+        <v>1378.34</v>
       </c>
       <c r="D70" s="6" t="n">
-        <v>23796.01</v>
+        <v>1751.17</v>
       </c>
       <c r="E70" s="6" t="n">
-        <v>1037.142463635088</v>
+        <v>1270.492041150949</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C71" s="6" t="n">
-        <v>3325.32</v>
+        <v>76.91</v>
       </c>
       <c r="D71" s="6" t="n">
-        <v>5482.570000000001</v>
+        <v>229.62</v>
       </c>
       <c r="E71" s="6" t="n">
-        <v>1648.734557877137</v>
+        <v>2985.567546482902</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C72" s="6" t="n">
-        <v>2674.93</v>
+        <v>169.23</v>
       </c>
       <c r="D72" s="6" t="n">
-        <v>4081.2</v>
+        <v>230.99</v>
       </c>
       <c r="E72" s="6" t="n">
-        <v>1525.722168430576</v>
+        <v>1364.94711339597</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C73" s="6" t="n">
-        <v>2</v>
+        <v>93.3</v>
       </c>
       <c r="D73" s="6" t="n">
-        <v>3.57</v>
+        <v>138.03</v>
       </c>
       <c r="E73" s="6" t="n">
-        <v>1785</v>
+        <v>1479.421221864952</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C74" s="6" t="n">
-        <v>6088.31</v>
+        <v>3006.56</v>
       </c>
       <c r="D74" s="6" t="n">
-        <v>7011.77</v>
+        <v>4648.9</v>
       </c>
       <c r="E74" s="6" t="n">
-        <v>1151.677559125603</v>
+        <v>1546.252195199829</v>
       </c>
     </row>
     <row r="75">
@@ -17929,17 +18315,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C75" s="6" t="n">
-        <v>103.74</v>
+        <v>74.12</v>
       </c>
       <c r="D75" s="6" t="n">
-        <v>101.29</v>
+        <v>65.39</v>
       </c>
       <c r="E75" s="6" t="n">
-        <v>976.3832658569498</v>
+        <v>882.2180248246087</v>
       </c>
     </row>
     <row r="76">
@@ -17950,17 +18336,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C76" s="6" t="n">
-        <v>621.55</v>
+        <v>99.94</v>
       </c>
       <c r="D76" s="6" t="n">
-        <v>930.3099999999999</v>
+        <v>281.04</v>
       </c>
       <c r="E76" s="6" t="n">
-        <v>1496.758104738155</v>
+        <v>2812.087252351411</v>
       </c>
     </row>
     <row r="77">
@@ -17971,17 +18357,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C77" s="6" t="n">
-        <v>2380.89</v>
+        <v>55.54</v>
       </c>
       <c r="D77" s="6" t="n">
-        <v>6171.320000000001</v>
+        <v>81.45</v>
       </c>
       <c r="E77" s="6" t="n">
-        <v>2592.022310984548</v>
+        <v>1466.510622974433</v>
       </c>
     </row>
     <row r="78">
@@ -17992,17 +18378,269 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="D78" s="6" t="n">
+        <v>28.52</v>
+      </c>
+      <c r="E78" s="6" t="n">
+        <v>6004.210526315789</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Korea, Republic of</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="n">
+        <v>23499.35</v>
+      </c>
+      <c r="D79" s="6" t="n">
+        <v>24530.11</v>
+      </c>
+      <c r="E79" s="6" t="n">
+        <v>1043.863340900919</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Luxembourg</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="n">
+        <v>4817.210000000001</v>
+      </c>
+      <c r="D80" s="6" t="n">
+        <v>8156.56</v>
+      </c>
+      <c r="E80" s="6" t="n">
+        <v>1693.2124611549</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="n">
+        <v>3325.159999999999</v>
+      </c>
+      <c r="D81" s="6" t="n">
+        <v>5062.68</v>
+      </c>
+      <c r="E81" s="6" t="n">
+        <v>1522.537261364867</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D82" s="6" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="E82" s="6" t="n">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="n">
+        <v>6088.31</v>
+      </c>
+      <c r="D83" s="6" t="n">
+        <v>7011.77</v>
+      </c>
+      <c r="E83" s="6" t="n">
+        <v>1151.677559125603</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D84" s="6" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="E84" s="6" t="n">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="D85" s="6" t="n">
+        <v>12.48</v>
+      </c>
+      <c r="E85" s="6" t="n">
+        <v>8210.526315789473</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="C86" s="6" t="n">
+        <v>350.4399999999999</v>
+      </c>
+      <c r="D86" s="6" t="n">
+        <v>340.99</v>
+      </c>
+      <c r="E86" s="6" t="n">
+        <v>973.0339002396988</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="n">
+        <v>628.9299999999999</v>
+      </c>
+      <c r="D87" s="6" t="n">
+        <v>972.9</v>
+      </c>
+      <c r="E87" s="6" t="n">
+        <v>1546.913010986915</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C88" s="6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D88" s="6" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="E88" s="6" t="n">
+        <v>4925</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C89" s="6" t="n">
+        <v>2966.21</v>
+      </c>
+      <c r="D89" s="6" t="n">
+        <v>7558.589999999999</v>
+      </c>
+      <c r="E89" s="6" t="n">
+        <v>2548.231581715387</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
           <t>Vietnam</t>
         </is>
       </c>
-      <c r="C78" s="6" t="n">
-        <v>403.97</v>
-      </c>
-      <c r="D78" s="6" t="n">
-        <v>338.95</v>
-      </c>
-      <c r="E78" s="6" t="n">
-        <v>839.0474540188627</v>
+      <c r="C90" s="6" t="n">
+        <v>446.88</v>
+      </c>
+      <c r="D90" s="6" t="n">
+        <v>374.9</v>
+      </c>
+      <c r="E90" s="6" t="n">
+        <v>838.9276763336914</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Weekly TRQ update 2026-08-17
</commit_message>
<xml_diff>
--- a/data/canada_trq_tracker.xlsx
+++ b/data/canada_trq_tracker.xlsx
@@ -12390,7 +12390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M45"/>
+  <dimension ref="A1:N45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12456,7 +12456,12 @@
           <t>August 10 2026</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="M2" s="1" t="inlineStr">
+        <is>
+          <t>August 17 2026</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
@@ -12500,7 +12505,10 @@
       <c r="L3" s="4" t="n">
         <v>0.41</v>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M3" s="4" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="N3" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -12541,6 +12549,9 @@
       <c r="L4" s="4" t="n">
         <v>0.036</v>
       </c>
+      <c r="M4" s="4" t="n">
+        <v>0.0373</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -12571,6 +12582,9 @@
       <c r="L5" s="4" t="n">
         <v>0.0003</v>
       </c>
+      <c r="M5" s="4" t="n">
+        <v>0.0003</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -12615,6 +12629,10 @@
         <f>SUM(L3:L5)</f>
         <v/>
       </c>
+      <c r="M6" s="5">
+        <f>SUM(M3:M5)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -12654,6 +12672,9 @@
       <c r="L7" s="4" t="n">
         <v>0.3468</v>
       </c>
+      <c r="M7" s="4" t="n">
+        <v>0.3402000000000001</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -12687,6 +12708,9 @@
       <c r="L8" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="M8" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -12731,6 +12755,10 @@
         <f>SUM(L7:L8)</f>
         <v/>
       </c>
+      <c r="M9" s="5">
+        <f>SUM(M7:M8)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -12770,6 +12798,9 @@
       <c r="L10" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="M10" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -12809,6 +12840,9 @@
       <c r="L11" s="4" t="n">
         <v>0.1135</v>
       </c>
+      <c r="M11" s="4" t="n">
+        <v>0.1135</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -12848,6 +12882,9 @@
       <c r="L12" s="4" t="n">
         <v>0.5572</v>
       </c>
+      <c r="M12" s="4" t="n">
+        <v>0.5572</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -12884,6 +12921,9 @@
       <c r="L13" s="4" t="n">
         <v>0.0008</v>
       </c>
+      <c r="M13" s="4" t="n">
+        <v>0.0008</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -12920,6 +12960,9 @@
       <c r="L14" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="M14" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -12956,6 +12999,9 @@
       <c r="L15" s="4" t="n">
         <v>0.3156</v>
       </c>
+      <c r="M15" s="4" t="n">
+        <v>0.3156</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -12989,6 +13035,9 @@
       <c r="L16" s="4" t="n">
         <v>0.0128</v>
       </c>
+      <c r="M16" s="4" t="n">
+        <v>0.0128</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -13022,6 +13071,9 @@
       <c r="L17" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="M17" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -13066,6 +13118,10 @@
         <f>SUM(L10:L17)</f>
         <v/>
       </c>
+      <c r="M18" s="5">
+        <f>SUM(M10:M17)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -13105,6 +13161,9 @@
       <c r="L19" s="4" t="n">
         <v>0.0027</v>
       </c>
+      <c r="M19" s="4" t="n">
+        <v>0.0027</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -13144,6 +13203,9 @@
       <c r="L20" s="4" t="n">
         <v>0.2673</v>
       </c>
+      <c r="M20" s="4" t="n">
+        <v>0.2673</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -13183,6 +13245,9 @@
       <c r="L21" s="4" t="n">
         <v>0.0069</v>
       </c>
+      <c r="M21" s="4" t="n">
+        <v>0.0069</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -13222,6 +13287,9 @@
       <c r="L22" s="4" t="n">
         <v>0.2488</v>
       </c>
+      <c r="M22" s="4" t="n">
+        <v>0.2488</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -13261,6 +13329,9 @@
       <c r="L23" s="4" t="n">
         <v>0.3697</v>
       </c>
+      <c r="M23" s="4" t="n">
+        <v>0.3697</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -13300,6 +13371,9 @@
       <c r="L24" s="4" t="n">
         <v>0.0289</v>
       </c>
+      <c r="M24" s="4" t="n">
+        <v>0.0289</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -13336,6 +13410,9 @@
       <c r="L25" s="4" t="n">
         <v>0.07539999999999999</v>
       </c>
+      <c r="M25" s="4" t="n">
+        <v>0.07539999999999999</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -13380,6 +13457,10 @@
         <f>SUM(L19:L25)</f>
         <v/>
       </c>
+      <c r="M26" s="5">
+        <f>SUM(M19:M25)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -13419,6 +13500,9 @@
       <c r="L27" s="4" t="n">
         <v>0.2747</v>
       </c>
+      <c r="M27" s="4" t="n">
+        <v>0.2747</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -13458,6 +13542,9 @@
       <c r="L28" s="4" t="n">
         <v>0.0037</v>
       </c>
+      <c r="M28" s="4" t="n">
+        <v>0.0037</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -13497,6 +13584,9 @@
       <c r="L29" s="4" t="n">
         <v>0.2899</v>
       </c>
+      <c r="M29" s="4" t="n">
+        <v>0.2899</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -13536,6 +13626,9 @@
       <c r="L30" s="4" t="n">
         <v>0.0883</v>
       </c>
+      <c r="M30" s="4" t="n">
+        <v>0.0883</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -13566,6 +13659,9 @@
       <c r="L31" s="4" t="n">
         <v>0.0038</v>
       </c>
+      <c r="M31" s="4" t="n">
+        <v>0.0038</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -13610,6 +13706,10 @@
         <f>SUM(L27:L31)</f>
         <v/>
       </c>
+      <c r="M32" s="5">
+        <f>SUM(M27:M31)</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -13649,6 +13749,9 @@
       <c r="L33" s="4" t="n">
         <v>0.1576</v>
       </c>
+      <c r="M33" s="4" t="n">
+        <v>0.1576</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -13688,7 +13791,10 @@
       <c r="L34" s="4" t="n">
         <v>0.42</v>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="M34" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="N34" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -13732,7 +13838,10 @@
       <c r="L35" s="4" t="n">
         <v>0.42</v>
       </c>
-      <c r="M35" t="inlineStr">
+      <c r="M35" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="N35" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -13773,6 +13882,9 @@
       <c r="L36" s="4" t="n">
         <v>0.0024</v>
       </c>
+      <c r="M36" s="4" t="n">
+        <v>0.0024</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -13817,6 +13929,10 @@
         <f>SUM(L33:L36)</f>
         <v/>
       </c>
+      <c r="M37" s="5">
+        <f>SUM(M33:M36)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -13844,6 +13960,9 @@
       <c r="L38" s="4" t="n">
         <v>0.2893</v>
       </c>
+      <c r="M38" s="4" t="n">
+        <v>0.2893</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -13868,6 +13987,9 @@
       <c r="L39" s="4" t="n">
         <v>0.1692</v>
       </c>
+      <c r="M39" s="4" t="n">
+        <v>0.1692</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -13912,6 +14034,10 @@
         <f>SUM(L38:L39)</f>
         <v/>
       </c>
+      <c r="M40" s="5">
+        <f>SUM(M38:M39)</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -13951,6 +14077,9 @@
       <c r="L41" s="4" t="n">
         <v>0.0146</v>
       </c>
+      <c r="M41" s="4" t="n">
+        <v>0.0146</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -13990,6 +14119,9 @@
       <c r="L42" s="4" t="n">
         <v>0.1993</v>
       </c>
+      <c r="M42" s="4" t="n">
+        <v>0.2009</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -14029,6 +14161,9 @@
       <c r="L43" s="4" t="n">
         <v>0.3483</v>
       </c>
+      <c r="M43" s="4" t="n">
+        <v>0.3483</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -14068,6 +14203,9 @@
       <c r="L44" s="4" t="n">
         <v>0.4306</v>
       </c>
+      <c r="M44" s="4" t="n">
+        <v>0.4306</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -14110,6 +14248,10 @@
       </c>
       <c r="L45" s="5">
         <f>SUM(L41:L44)</f>
+        <v/>
+      </c>
+      <c r="M45" s="5">
+        <f>SUM(M41:M44)</f>
         <v/>
       </c>
     </row>
@@ -14124,7 +14266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M73"/>
+  <dimension ref="A1:N74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14190,7 +14332,12 @@
           <t>August 10 2026</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="M2" s="1" t="inlineStr">
+        <is>
+          <t>August 17 2026</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
@@ -14234,6 +14381,9 @@
       <c r="L3" s="4" t="n">
         <v>0.3165</v>
       </c>
+      <c r="M3" s="4" t="n">
+        <v>0.3165</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -14273,6 +14423,9 @@
       <c r="L4" s="4" t="n">
         <v>0.6835</v>
       </c>
+      <c r="M4" s="4" t="n">
+        <v>0.6835</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -14317,6 +14470,10 @@
         <f>SUM(L3:L4)</f>
         <v/>
       </c>
+      <c r="M5" s="5">
+        <f>SUM(M3:M4)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -14356,6 +14513,9 @@
       <c r="L6" s="4" t="n">
         <v>0.0452</v>
       </c>
+      <c r="M6" s="4" t="n">
+        <v>0.0452</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -14395,6 +14555,9 @@
       <c r="L7" s="4" t="n">
         <v>0.0261</v>
       </c>
+      <c r="M7" s="4" t="n">
+        <v>0.0261</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -14434,6 +14597,9 @@
       <c r="L8" s="4" t="n">
         <v>0.0009</v>
       </c>
+      <c r="M8" s="4" t="n">
+        <v>0.0009</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -14473,6 +14639,9 @@
       <c r="L9" s="4" t="n">
         <v>0.0128</v>
       </c>
+      <c r="M9" s="4" t="n">
+        <v>0.0142</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -14512,6 +14681,9 @@
       <c r="L10" s="4" t="n">
         <v>0.2225</v>
       </c>
+      <c r="M10" s="4" t="n">
+        <v>0.2225</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -14551,6 +14723,9 @@
       <c r="L11" s="4" t="n">
         <v>0.2191</v>
       </c>
+      <c r="M11" s="4" t="n">
+        <v>0.2087</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -14590,6 +14765,9 @@
       <c r="L12" s="4" t="n">
         <v>0.0785</v>
       </c>
+      <c r="M12" s="4" t="n">
+        <v>0.08310000000000001</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -14629,7 +14807,10 @@
       <c r="L13" s="4" t="n">
         <v>0.33</v>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="M13" s="4" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="N13" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -14673,6 +14854,9 @@
       <c r="L14" s="4" t="n">
         <v>0.001</v>
       </c>
+      <c r="M14" s="4" t="n">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -14712,6 +14896,9 @@
       <c r="L15" s="4" t="n">
         <v>0.0622</v>
       </c>
+      <c r="M15" s="4" t="n">
+        <v>0.06370000000000001</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -14748,6 +14935,9 @@
       <c r="L16" s="4" t="n">
         <v>0.0013</v>
       </c>
+      <c r="M16" s="4" t="n">
+        <v>0.0013</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -14792,6 +14982,10 @@
         <f>SUM(L6:L16)</f>
         <v/>
       </c>
+      <c r="M17" s="5">
+        <f>SUM(M6:M16)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -14831,6 +15025,9 @@
       <c r="L18" s="4" t="n">
         <v>0.0206</v>
       </c>
+      <c r="M18" s="4" t="n">
+        <v>0.0206</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -14870,6 +15067,9 @@
       <c r="L19" s="4" t="n">
         <v>0.1972</v>
       </c>
+      <c r="M19" s="4" t="n">
+        <v>0.1997</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -14909,6 +15109,9 @@
       <c r="L20" s="4" t="n">
         <v>0.0175</v>
       </c>
+      <c r="M20" s="4" t="n">
+        <v>0.0175</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -14945,6 +15148,9 @@
       <c r="L21" s="4" t="n">
         <v>0.3255</v>
       </c>
+      <c r="M21" s="4" t="n">
+        <v>0.3255</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -14966,6 +15172,9 @@
       <c r="L22" s="4" t="n">
         <v>0.0043</v>
       </c>
+      <c r="M22" s="4" t="n">
+        <v>0.0043</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -15010,6 +15219,10 @@
         <f>SUM(L18:L22)</f>
         <v/>
       </c>
+      <c r="M23" s="5">
+        <f>SUM(M18:M22)</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -15049,6 +15262,9 @@
       <c r="L24" s="4" t="n">
         <v>0.0304</v>
       </c>
+      <c r="M24" s="4" t="n">
+        <v>0.2387</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -15088,6 +15304,9 @@
       <c r="L25" s="4" t="n">
         <v>0.0793</v>
       </c>
+      <c r="M25" s="4" t="n">
+        <v>0.0795</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -15127,7 +15346,10 @@
       <c r="L26" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="M26" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N26" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -15171,6 +15393,9 @@
       <c r="L27" s="4" t="n">
         <v>0.0482</v>
       </c>
+      <c r="M27" s="4" t="n">
+        <v>0.0482</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -15210,6 +15435,9 @@
       <c r="L28" s="4" t="n">
         <v>0.039</v>
       </c>
+      <c r="M28" s="4" t="n">
+        <v>0.04269999999999999</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -15249,6 +15477,9 @@
       <c r="L29" s="4" t="n">
         <v>0.0256</v>
       </c>
+      <c r="M29" s="4" t="n">
+        <v>0.0294</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -15285,6 +15516,9 @@
       <c r="L30" s="4" t="n">
         <v>0.1027</v>
       </c>
+      <c r="M30" s="4" t="n">
+        <v>0.1027</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -15321,6 +15555,9 @@
       <c r="L31" s="4" t="n">
         <v>0.0157</v>
       </c>
+      <c r="M31" s="4" t="n">
+        <v>0.0157</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -15357,6 +15594,9 @@
       <c r="L32" s="4" t="n">
         <v>0.0369</v>
       </c>
+      <c r="M32" s="4" t="n">
+        <v>0.0369</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -15390,6 +15630,9 @@
       <c r="L33" s="4" t="n">
         <v>0.0014</v>
       </c>
+      <c r="M33" s="4" t="n">
+        <v>0.0014</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -15414,6 +15657,9 @@
       <c r="L34" s="4" t="n">
         <v>0.0063</v>
       </c>
+      <c r="M34" s="4" t="n">
+        <v>0.0063</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -15458,6 +15704,10 @@
         <f>SUM(L24:L34)</f>
         <v/>
       </c>
+      <c r="M35" s="5">
+        <f>SUM(M24:M34)</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -15497,6 +15747,9 @@
       <c r="L36" s="4" t="n">
         <v>0.08349999999999999</v>
       </c>
+      <c r="M36" s="4" t="n">
+        <v>0.08349999999999999</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -15536,6 +15789,9 @@
       <c r="L37" s="4" t="n">
         <v>0.3459</v>
       </c>
+      <c r="M37" s="4" t="n">
+        <v>0.3459</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -15572,6 +15828,9 @@
       <c r="L38" s="4" t="n">
         <v>0.0007000000000000001</v>
       </c>
+      <c r="M38" s="4" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -15596,6 +15855,9 @@
       <c r="L39" s="4" t="n">
         <v>0.4389</v>
       </c>
+      <c r="M39" s="4" t="n">
+        <v>0.4389</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -15640,6 +15902,10 @@
         <f>SUM(L36:L39)</f>
         <v/>
       </c>
+      <c r="M40" s="5">
+        <f>SUM(M36:M39)</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -15679,6 +15945,9 @@
       <c r="L41" s="4" t="n">
         <v>0.0025</v>
       </c>
+      <c r="M41" s="4" t="n">
+        <v>0.0025</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -15718,6 +15987,9 @@
       <c r="L42" s="4" t="n">
         <v>0.4215</v>
       </c>
+      <c r="M42" s="4" t="n">
+        <v>0.4215</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -15757,6 +16029,9 @@
       <c r="L43" s="4" t="n">
         <v>0.1712</v>
       </c>
+      <c r="M43" s="4" t="n">
+        <v>0.1712</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -15796,6 +16071,9 @@
       <c r="L44" s="4" t="n">
         <v>0.016</v>
       </c>
+      <c r="M44" s="4" t="n">
+        <v>0.016</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -15835,6 +16113,9 @@
       <c r="L45" s="4" t="n">
         <v>0.0133</v>
       </c>
+      <c r="M45" s="4" t="n">
+        <v>0.0133</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -15874,6 +16155,9 @@
       <c r="L46" s="4" t="n">
         <v>0.0708</v>
       </c>
+      <c r="M46" s="4" t="n">
+        <v>0.0708</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -15910,6 +16194,9 @@
       <c r="L47" s="4" t="n">
         <v>0.0072</v>
       </c>
+      <c r="M47" s="4" t="n">
+        <v>0.0072</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -15946,6 +16233,9 @@
       <c r="L48" s="4" t="n">
         <v>0.2946</v>
       </c>
+      <c r="M48" s="4" t="n">
+        <v>0.2946</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -15979,6 +16269,9 @@
       <c r="L49" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="M49" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -16012,6 +16305,9 @@
       <c r="L50" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="M50" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -16045,6 +16341,9 @@
       <c r="L51" s="4" t="n">
         <v>0.0022</v>
       </c>
+      <c r="M51" s="4" t="n">
+        <v>0.0022</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -16078,6 +16377,9 @@
       <c r="L52" s="4" t="n">
         <v>0.0004</v>
       </c>
+      <c r="M52" s="4" t="n">
+        <v>0.0004</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -16111,6 +16413,9 @@
       <c r="L53" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="M53" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -16141,6 +16446,9 @@
       <c r="L54" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="M54" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -16171,6 +16479,9 @@
       <c r="L55" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="M55" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -16198,6 +16509,9 @@
       <c r="L56" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="M56" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -16222,6 +16536,9 @@
       <c r="L57" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="M57" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -16266,6 +16583,10 @@
         <f>SUM(L41:L57)</f>
         <v/>
       </c>
+      <c r="M58" s="5">
+        <f>SUM(M41:M57)</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -16305,6 +16626,9 @@
       <c r="L59" s="4" t="n">
         <v>0.1433</v>
       </c>
+      <c r="M59" s="4" t="n">
+        <v>0.1433</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -16344,6 +16668,9 @@
       <c r="L60" s="4" t="n">
         <v>0.04269999999999999</v>
       </c>
+      <c r="M60" s="4" t="n">
+        <v>0.04269999999999999</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -16383,6 +16710,9 @@
       <c r="L61" s="4" t="n">
         <v>0.4926</v>
       </c>
+      <c r="M61" s="4" t="n">
+        <v>0.4926</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -16422,6 +16752,9 @@
       <c r="L62" s="4" t="n">
         <v>0.0161</v>
       </c>
+      <c r="M62" s="4" t="n">
+        <v>0.0161</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -16455,6 +16788,9 @@
       <c r="L63" s="4" t="n">
         <v>0.0044</v>
       </c>
+      <c r="M63" s="4" t="n">
+        <v>0.0044</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -16464,79 +16800,65 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E64" s="5">
-        <f>SUM(E59:E63)</f>
-        <v/>
-      </c>
-      <c r="F64" s="5">
-        <f>SUM(F59:F63)</f>
-        <v/>
-      </c>
-      <c r="G64" s="5">
-        <f>SUM(G59:G63)</f>
-        <v/>
-      </c>
-      <c r="H64" s="5">
-        <f>SUM(H59:H63)</f>
-        <v/>
-      </c>
-      <c r="I64" s="5">
-        <f>SUM(I59:I63)</f>
-        <v/>
-      </c>
-      <c r="J64" s="5">
-        <f>SUM(J59:J63)</f>
-        <v/>
-      </c>
-      <c r="K64" s="5">
-        <f>SUM(K59:K63)</f>
-        <v/>
-      </c>
-      <c r="L64" s="5">
-        <f>SUM(L59:L63)</f>
-        <v/>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="n">
+        <v>16514800</v>
+      </c>
+      <c r="D64" s="4" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="M64" s="4" t="n">
+        <v>0.0022</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="C65" s="3" t="n">
-        <v>3467600</v>
-      </c>
-      <c r="D65" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="E65" s="4" t="n">
-        <v>0.0004</v>
-      </c>
-      <c r="F65" s="4" t="n">
-        <v>0.0021</v>
-      </c>
-      <c r="G65" s="4" t="n">
-        <v>0.0021</v>
-      </c>
-      <c r="H65" s="4" t="n">
-        <v>0.0021</v>
-      </c>
-      <c r="I65" s="4" t="n">
-        <v>0.0021</v>
-      </c>
-      <c r="K65" s="4" t="n">
-        <v>0.0021</v>
-      </c>
-      <c r="L65" s="4" t="n">
-        <v>0.0021</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E65" s="5">
+        <f>SUM(E59:E64)</f>
+        <v/>
+      </c>
+      <c r="F65" s="5">
+        <f>SUM(F59:F64)</f>
+        <v/>
+      </c>
+      <c r="G65" s="5">
+        <f>SUM(G59:G64)</f>
+        <v/>
+      </c>
+      <c r="H65" s="5">
+        <f>SUM(H59:H64)</f>
+        <v/>
+      </c>
+      <c r="I65" s="5">
+        <f>SUM(I59:I64)</f>
+        <v/>
+      </c>
+      <c r="J65" s="5">
+        <f>SUM(J59:J64)</f>
+        <v/>
+      </c>
+      <c r="K65" s="5">
+        <f>SUM(K59:K64)</f>
+        <v/>
+      </c>
+      <c r="L65" s="5">
+        <f>SUM(L59:L64)</f>
+        <v/>
+      </c>
+      <c r="M65" s="5">
+        <f>SUM(M59:M64)</f>
+        <v/>
       </c>
     </row>
     <row r="66">
@@ -16547,7 +16869,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C66" s="3" t="n">
@@ -16557,25 +16879,28 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E66" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.0004</v>
       </c>
       <c r="F66" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.0021</v>
       </c>
       <c r="G66" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.0021</v>
       </c>
       <c r="H66" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.0021</v>
       </c>
       <c r="I66" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.0021</v>
       </c>
       <c r="K66" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.0021</v>
       </c>
       <c r="L66" s="4" t="n">
-        <v>0.0032</v>
+        <v>0.0021</v>
+      </c>
+      <c r="M66" s="4" t="n">
+        <v>0.0021</v>
       </c>
     </row>
     <row r="67">
@@ -16586,7 +16911,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C67" s="3" t="n">
@@ -16596,25 +16921,28 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E67" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0032</v>
       </c>
       <c r="F67" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0032</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0032</v>
       </c>
       <c r="H67" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0032</v>
       </c>
       <c r="I67" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0032</v>
       </c>
       <c r="K67" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0032</v>
       </c>
       <c r="L67" s="4" t="n">
-        <v>0.0204</v>
+        <v>0.0032</v>
+      </c>
+      <c r="M67" s="4" t="n">
+        <v>0.0032</v>
       </c>
     </row>
     <row r="68">
@@ -16625,7 +16953,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C68" s="3" t="n">
@@ -16635,30 +16963,28 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E68" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.0204</v>
       </c>
       <c r="F68" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.0204</v>
       </c>
       <c r="G68" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.0204</v>
       </c>
       <c r="H68" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.0204</v>
       </c>
       <c r="I68" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.0204</v>
       </c>
       <c r="K68" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.0204</v>
       </c>
       <c r="L68" s="4" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="M68" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
+        <v>0.0204</v>
+      </c>
+      <c r="M68" s="4" t="n">
+        <v>0.0204</v>
       </c>
     </row>
     <row r="69">
@@ -16669,7 +16995,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C69" s="3" t="n">
@@ -16679,25 +17005,33 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E69" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="F69" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H69" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="I69" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="K69" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="L69" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="M69" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
       </c>
     </row>
     <row r="70">
@@ -16708,7 +17042,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C70" s="3" t="n">
@@ -16718,25 +17052,28 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E70" s="4" t="n">
-        <v>0.1798</v>
+        <v>0.0004</v>
       </c>
       <c r="F70" s="4" t="n">
-        <v>0.1798</v>
+        <v>0.0004</v>
       </c>
       <c r="G70" s="4" t="n">
-        <v>0.2828</v>
+        <v>0.0004</v>
       </c>
       <c r="H70" s="4" t="n">
-        <v>0.2828</v>
+        <v>0.0004</v>
       </c>
       <c r="I70" s="4" t="n">
-        <v>0.2828</v>
+        <v>0.0004</v>
       </c>
       <c r="K70" s="4" t="n">
-        <v>0.2828</v>
+        <v>0.0004</v>
       </c>
       <c r="L70" s="4" t="n">
-        <v>0.2828</v>
+        <v>0.0004</v>
+      </c>
+      <c r="M70" s="4" t="n">
+        <v>0.0004</v>
       </c>
     </row>
     <row r="71">
@@ -16747,7 +17084,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C71" s="3" t="n">
@@ -16756,23 +17093,29 @@
       <c r="D71" s="4" t="n">
         <v>0.6899999999999999</v>
       </c>
+      <c r="E71" s="4" t="n">
+        <v>0.1798</v>
+      </c>
       <c r="F71" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.1798</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.2828</v>
       </c>
       <c r="H71" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.2828</v>
       </c>
       <c r="I71" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.2828</v>
       </c>
       <c r="K71" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.2828</v>
       </c>
       <c r="L71" s="4" t="n">
-        <v>0.0012</v>
+        <v>0.2828</v>
+      </c>
+      <c r="M71" s="4" t="n">
+        <v>0.2828</v>
       </c>
     </row>
     <row r="72">
@@ -16783,7 +17126,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Luxembourg</t>
         </is>
       </c>
       <c r="C72" s="3" t="n">
@@ -16792,20 +17135,26 @@
       <c r="D72" s="4" t="n">
         <v>0.6899999999999999</v>
       </c>
+      <c r="F72" s="4" t="n">
+        <v>0.0012</v>
+      </c>
       <c r="G72" s="4" t="n">
-        <v>0</v>
+        <v>0.0012</v>
       </c>
       <c r="H72" s="4" t="n">
-        <v>0</v>
+        <v>0.0012</v>
       </c>
       <c r="I72" s="4" t="n">
-        <v>0</v>
+        <v>0.0012</v>
       </c>
       <c r="K72" s="4" t="n">
-        <v>0</v>
+        <v>0.0012</v>
       </c>
       <c r="L72" s="4" t="n">
-        <v>0</v>
+        <v>0.0012</v>
+      </c>
+      <c r="M72" s="4" t="n">
+        <v>0.0012</v>
       </c>
     </row>
     <row r="73">
@@ -16816,39 +17165,79 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="n">
+        <v>3467600</v>
+      </c>
+      <c r="D73" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G73" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I73" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K73" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L73" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M73" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E73" s="5">
-        <f>SUM(E65:E72)</f>
-        <v/>
-      </c>
-      <c r="F73" s="5">
-        <f>SUM(F65:F72)</f>
-        <v/>
-      </c>
-      <c r="G73" s="5">
-        <f>SUM(G65:G72)</f>
-        <v/>
-      </c>
-      <c r="H73" s="5">
-        <f>SUM(H65:H72)</f>
-        <v/>
-      </c>
-      <c r="I73" s="5">
-        <f>SUM(I65:I72)</f>
-        <v/>
-      </c>
-      <c r="J73" s="5">
-        <f>SUM(J65:J72)</f>
-        <v/>
-      </c>
-      <c r="K73" s="5">
-        <f>SUM(K65:K72)</f>
-        <v/>
-      </c>
-      <c r="L73" s="5">
-        <f>SUM(L65:L72)</f>
+      <c r="E74" s="5">
+        <f>SUM(E66:E73)</f>
+        <v/>
+      </c>
+      <c r="F74" s="5">
+        <f>SUM(F66:F73)</f>
+        <v/>
+      </c>
+      <c r="G74" s="5">
+        <f>SUM(G66:G73)</f>
+        <v/>
+      </c>
+      <c r="H74" s="5">
+        <f>SUM(H66:H73)</f>
+        <v/>
+      </c>
+      <c r="I74" s="5">
+        <f>SUM(I66:I73)</f>
+        <v/>
+      </c>
+      <c r="J74" s="5">
+        <f>SUM(J66:J73)</f>
+        <v/>
+      </c>
+      <c r="K74" s="5">
+        <f>SUM(K66:K73)</f>
+        <v/>
+      </c>
+      <c r="L74" s="5">
+        <f>SUM(L66:L73)</f>
+        <v/>
+      </c>
+      <c r="M74" s="5">
+        <f>SUM(M66:M73)</f>
         <v/>
       </c>
     </row>
@@ -16863,7 +17252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E90"/>
+  <dimension ref="A1:E94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17101,13 +17490,13 @@
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>5813.71</v>
+        <v>7095.56</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>9938.76</v>
+        <v>12210.83</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>1709.538315464652</v>
+        <v>1720.911386839093</v>
       </c>
     </row>
     <row r="18">
@@ -17139,17 +17528,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>127.72</v>
+        <v>0.29</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>125.6</v>
+        <v>0.51</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>983.401190103351</v>
+        <v>1758.620689655173</v>
       </c>
     </row>
     <row r="20">
@@ -17160,17 +17549,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>399.2</v>
+        <v>129.67</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>1721.69</v>
+        <v>129.37</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>4312.850701402806</v>
+        <v>997.6864347960208</v>
       </c>
     </row>
     <row r="21">
@@ -17181,17 +17570,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>54.64</v>
+        <v>703.4300000000001</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>126.5</v>
+        <v>3059.44</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>2315.153733528551</v>
+        <v>4349.316918527784</v>
       </c>
     </row>
     <row r="22">
@@ -17202,17 +17591,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>1507.27</v>
+        <v>191.71</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>3411.48</v>
+        <v>387.08</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>2263.350295567483</v>
+        <v>2019.09133587189</v>
       </c>
     </row>
     <row r="23">
@@ -17223,17 +17612,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>8807.609999999999</v>
+        <v>1507.27</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>11940</v>
+        <v>3411.48</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>1355.645856253853</v>
+        <v>2263.350295567483</v>
       </c>
     </row>
     <row r="24">
@@ -17244,17 +17633,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>43.15</v>
+        <v>9129.07</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>98.15000000000001</v>
+        <v>10962.94</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>2274.623406720742</v>
+        <v>1200.882455715642</v>
       </c>
     </row>
     <row r="25">
@@ -17265,17 +17654,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C25" s="6" t="n">
-        <v>25.68</v>
+        <v>51.26</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>34.82</v>
+        <v>116.62</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>1355.919003115265</v>
+        <v>2275.068279360125</v>
       </c>
     </row>
     <row r="26">
@@ -17286,38 +17675,38 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>3540.700000000001</v>
+        <v>25.68</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>7802.979999999999</v>
+        <v>34.82</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>2203.79585957579</v>
+        <v>1355.919003115265</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Cold-Rolled Sheet</t>
+          <t>Steel Plate</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>13.38</v>
+        <v>4086.04</v>
       </c>
       <c r="D27" s="6" t="n">
-        <v>32.54</v>
+        <v>8883.74</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>2431.988041853513</v>
+        <v>2174.168632710399</v>
       </c>
     </row>
     <row r="28">
@@ -17328,17 +17717,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>1477.26</v>
+        <v>18.13</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>2260.03</v>
+        <v>42.97</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>1529.879642039993</v>
+        <v>2370.104798676227</v>
       </c>
     </row>
     <row r="29">
@@ -17349,17 +17738,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>645.8000000000001</v>
+        <v>2042.58</v>
       </c>
       <c r="D29" s="6" t="n">
-        <v>786.75</v>
+        <v>3118.93</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>1218.256426138123</v>
+        <v>1526.956104534461</v>
       </c>
     </row>
     <row r="30">
@@ -17370,17 +17759,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>424.12</v>
+        <v>645.8000000000001</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>761.33</v>
+        <v>786.75</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>1795.081580684712</v>
+        <v>1218.256426138123</v>
       </c>
     </row>
     <row r="31">
@@ -17391,17 +17780,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C31" s="6" t="n">
-        <v>2851.83</v>
+        <v>424.12</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>3001.82</v>
+        <v>761.33</v>
       </c>
       <c r="E31" s="6" t="n">
-        <v>1052.594299099175</v>
+        <v>1795.081580684712</v>
       </c>
     </row>
     <row r="32">
@@ -17412,17 +17801,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>0.04</v>
+        <v>3051.02</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>0.19</v>
+        <v>3183.75</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>4750</v>
+        <v>1043.503484080733</v>
       </c>
     </row>
     <row r="33">
@@ -17433,17 +17822,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C33" s="6" t="n">
-        <v>1641.42</v>
+        <v>0.04</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>1690.42</v>
+        <v>0.19</v>
       </c>
       <c r="E33" s="6" t="n">
-        <v>1029.852201142913</v>
+        <v>4750</v>
       </c>
     </row>
     <row r="34">
@@ -17454,38 +17843,38 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C34" s="6" t="n">
-        <v>4452.63</v>
+        <v>2248.09</v>
       </c>
       <c r="D34" s="6" t="n">
-        <v>8263.219999999999</v>
+        <v>2309.75</v>
       </c>
       <c r="E34" s="6" t="n">
-        <v>1855.80656825292</v>
+        <v>1027.427727537599</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Coated Steel Sheet</t>
+          <t>Cold-Rolled Sheet</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C35" s="6" t="n">
-        <v>1110.32</v>
+        <v>6118.5</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>1790.26</v>
+        <v>11433.96</v>
       </c>
       <c r="E35" s="6" t="n">
-        <v>1612.382015995388</v>
+        <v>1868.752145133612</v>
       </c>
     </row>
     <row r="36">
@@ -17496,17 +17885,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C36" s="6" t="n">
-        <v>824.96</v>
+        <v>1121.86</v>
       </c>
       <c r="D36" s="6" t="n">
-        <v>1032.88</v>
+        <v>1811.53</v>
       </c>
       <c r="E36" s="6" t="n">
-        <v>1252.036462373933</v>
+        <v>1614.755851888827</v>
       </c>
     </row>
     <row r="37">
@@ -17517,17 +17906,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C37" s="6" t="n">
-        <v>40.24</v>
+        <v>1165.83</v>
       </c>
       <c r="D37" s="6" t="n">
-        <v>88.01000000000001</v>
+        <v>1487.11</v>
       </c>
       <c r="E37" s="6" t="n">
-        <v>2187.127236580517</v>
+        <v>1275.580487721194</v>
       </c>
     </row>
     <row r="38">
@@ -17538,17 +17927,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C38" s="6" t="n">
-        <v>2907.21</v>
+        <v>40.24</v>
       </c>
       <c r="D38" s="6" t="n">
-        <v>5548.78</v>
+        <v>88.01000000000001</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>1908.627171755738</v>
+        <v>2187.127236580517</v>
       </c>
     </row>
     <row r="39">
@@ -17559,17 +17948,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C39" s="6" t="n">
-        <v>246.5</v>
+        <v>2907.21</v>
       </c>
       <c r="D39" s="6" t="n">
-        <v>602.38</v>
+        <v>5548.78</v>
       </c>
       <c r="E39" s="6" t="n">
-        <v>2443.732251521298</v>
+        <v>1908.627171755738</v>
       </c>
     </row>
     <row r="40">
@@ -17580,17 +17969,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C40" s="6" t="n">
-        <v>447.02</v>
+        <v>246.68</v>
       </c>
       <c r="D40" s="6" t="n">
-        <v>827.6900000000001</v>
+        <v>603.6799999999999</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>1851.572636571071</v>
+        <v>2447.219069239501</v>
       </c>
     </row>
     <row r="41">
@@ -17601,17 +17990,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C41" s="6" t="n">
-        <v>14339.53</v>
+        <v>487.1799999999999</v>
       </c>
       <c r="D41" s="6" t="n">
-        <v>23370.68</v>
+        <v>953.9400000000001</v>
       </c>
       <c r="E41" s="6" t="n">
-        <v>1629.807950469785</v>
+        <v>1958.085307278624</v>
       </c>
     </row>
     <row r="42">
@@ -17622,17 +18011,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C42" s="6" t="n">
-        <v>160.98</v>
+        <v>15708.75</v>
       </c>
       <c r="D42" s="6" t="n">
-        <v>274.8</v>
+        <v>26118.7</v>
       </c>
       <c r="E42" s="6" t="n">
-        <v>1707.044353335818</v>
+        <v>1662.684809421501</v>
       </c>
     </row>
     <row r="43">
@@ -17643,17 +18032,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C43" s="6" t="n">
-        <v>284.88</v>
+        <v>160.98</v>
       </c>
       <c r="D43" s="6" t="n">
-        <v>577.25</v>
+        <v>274.8</v>
       </c>
       <c r="E43" s="6" t="n">
-        <v>2026.291771974165</v>
+        <v>1707.044353335818</v>
       </c>
     </row>
     <row r="44">
@@ -17664,17 +18053,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C44" s="6" t="n">
-        <v>3609.36</v>
+        <v>284.88</v>
       </c>
       <c r="D44" s="6" t="n">
-        <v>4508.49</v>
+        <v>577.25</v>
       </c>
       <c r="E44" s="6" t="n">
-        <v>1249.110645654631</v>
+        <v>2026.291771974165</v>
       </c>
     </row>
     <row r="45">
@@ -17685,17 +18074,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="C45" s="6" t="n">
-        <v>144.18</v>
+        <v>3609.36</v>
       </c>
       <c r="D45" s="6" t="n">
-        <v>204.36</v>
+        <v>4508.49</v>
       </c>
       <c r="E45" s="6" t="n">
-        <v>1417.394923012901</v>
+        <v>1249.110645654631</v>
       </c>
     </row>
     <row r="46">
@@ -17706,17 +18095,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="C46" s="6" t="n">
-        <v>0.12</v>
+        <v>144.18</v>
       </c>
       <c r="D46" s="6" t="n">
-        <v>0.25</v>
+        <v>204.36</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>2083.333333333333</v>
+        <v>1417.394923012901</v>
       </c>
     </row>
     <row r="47">
@@ -17727,17 +18116,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C47" s="6" t="n">
-        <v>5138.799999999999</v>
+        <v>0.12</v>
       </c>
       <c r="D47" s="6" t="n">
-        <v>8197.349999999999</v>
+        <v>0.25</v>
       </c>
       <c r="E47" s="6" t="n">
-        <v>1595.187592434031</v>
+        <v>2083.333333333333</v>
       </c>
     </row>
     <row r="48">
@@ -17748,17 +18137,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C48" s="6" t="n">
-        <v>542.15</v>
+        <v>5138.799999999999</v>
       </c>
       <c r="D48" s="6" t="n">
-        <v>737.62</v>
+        <v>8197.349999999999</v>
       </c>
       <c r="E48" s="6" t="n">
-        <v>1360.545974361339</v>
+        <v>1595.187592434031</v>
       </c>
     </row>
     <row r="49">
@@ -17769,17 +18158,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C49" s="6" t="n">
-        <v>1412.89</v>
+        <v>542.15</v>
       </c>
       <c r="D49" s="6" t="n">
-        <v>1664.87</v>
+        <v>737.62</v>
       </c>
       <c r="E49" s="6" t="n">
-        <v>1178.343678559548</v>
+        <v>1360.545974361339</v>
       </c>
     </row>
     <row r="50">
@@ -17790,17 +18179,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C50" s="6" t="n">
-        <v>0.33</v>
+        <v>1412.89</v>
       </c>
       <c r="D50" s="6" t="n">
-        <v>1.37</v>
+        <v>1664.87</v>
       </c>
       <c r="E50" s="6" t="n">
-        <v>4151.515151515151</v>
+        <v>1178.343678559548</v>
       </c>
     </row>
     <row r="51">
@@ -17811,17 +18200,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="C51" s="6" t="n">
-        <v>0.63</v>
+        <v>0.33</v>
       </c>
       <c r="D51" s="6" t="n">
         <v>1.37</v>
       </c>
       <c r="E51" s="6" t="n">
-        <v>2174.603174603174</v>
+        <v>4151.515151515151</v>
       </c>
     </row>
     <row r="52">
@@ -17832,17 +18221,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C52" s="6" t="n">
-        <v>14911.05</v>
+        <v>0.63</v>
       </c>
       <c r="D52" s="6" t="n">
-        <v>31301.04</v>
+        <v>1.37</v>
       </c>
       <c r="E52" s="6" t="n">
-        <v>2099.184162081141</v>
+        <v>2174.603174603174</v>
       </c>
     </row>
     <row r="53">
@@ -17853,38 +18242,38 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C53" s="6" t="n">
-        <v>1281.18</v>
+        <v>19566.25</v>
       </c>
       <c r="D53" s="6" t="n">
-        <v>1691.49</v>
+        <v>41493.37</v>
       </c>
       <c r="E53" s="6" t="n">
-        <v>1320.259448321079</v>
+        <v>2120.660320705296</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C54" s="6" t="n">
-        <v>25.53</v>
+        <v>1315.71</v>
       </c>
       <c r="D54" s="6" t="n">
-        <v>42.55</v>
+        <v>1732.85</v>
       </c>
       <c r="E54" s="6" t="n">
-        <v>1666.666666666667</v>
+        <v>1317.045549551193</v>
       </c>
     </row>
     <row r="55">
@@ -17895,17 +18284,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C55" s="6" t="n">
-        <v>19.72</v>
+        <v>65.06</v>
       </c>
       <c r="D55" s="6" t="n">
-        <v>39.63</v>
+        <v>74.83</v>
       </c>
       <c r="E55" s="6" t="n">
-        <v>2009.634888438134</v>
+        <v>1150.169074700277</v>
       </c>
     </row>
     <row r="56">
@@ -17916,17 +18305,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="C56" s="6" t="n">
-        <v>7.25</v>
+        <v>19.72</v>
       </c>
       <c r="D56" s="6" t="n">
-        <v>19.82</v>
+        <v>39.63</v>
       </c>
       <c r="E56" s="6" t="n">
-        <v>2733.793103448276</v>
+        <v>2009.634888438134</v>
       </c>
     </row>
     <row r="57">
@@ -17937,17 +18326,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C57" s="6" t="n">
-        <v>1721.39</v>
+        <v>7.25</v>
       </c>
       <c r="D57" s="6" t="n">
-        <v>1312.5</v>
+        <v>19.82</v>
       </c>
       <c r="E57" s="6" t="n">
-        <v>762.465217062955</v>
+        <v>2733.793103448276</v>
       </c>
     </row>
     <row r="58">
@@ -17958,17 +18347,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C58" s="6" t="n">
-        <v>5026.549999999999</v>
+        <v>1721.39</v>
       </c>
       <c r="D58" s="6" t="n">
-        <v>6984.03</v>
+        <v>1312.5</v>
       </c>
       <c r="E58" s="6" t="n">
-        <v>1389.428136594682</v>
+        <v>762.465217062955</v>
       </c>
     </row>
     <row r="59">
@@ -17979,38 +18368,38 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C59" s="6" t="n">
-        <v>228.32</v>
+        <v>6110.48</v>
       </c>
       <c r="D59" s="6" t="n">
-        <v>339.98</v>
+        <v>8452.559999999999</v>
       </c>
       <c r="E59" s="6" t="n">
-        <v>1489.050455501051</v>
+        <v>1383.289037849727</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C60" s="6" t="n">
-        <v>86.63</v>
+        <v>257.66</v>
       </c>
       <c r="D60" s="6" t="n">
-        <v>188.27</v>
+        <v>391.03</v>
       </c>
       <c r="E60" s="6" t="n">
-        <v>2173.265612374466</v>
+        <v>1517.620119537375</v>
       </c>
     </row>
     <row r="61">
@@ -18021,17 +18410,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C61" s="6" t="n">
-        <v>25.8</v>
+        <v>124.07</v>
       </c>
       <c r="D61" s="6" t="n">
-        <v>47.1</v>
+        <v>266.46</v>
       </c>
       <c r="E61" s="6" t="n">
-        <v>1825.581395348837</v>
+        <v>2147.658579833965</v>
       </c>
     </row>
     <row r="62">
@@ -18042,17 +18431,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C62" s="6" t="n">
-        <v>112.54</v>
+        <v>25.8</v>
       </c>
       <c r="D62" s="6" t="n">
-        <v>228.5</v>
+        <v>47.1</v>
       </c>
       <c r="E62" s="6" t="n">
-        <v>2030.389194952905</v>
+        <v>1825.581395348837</v>
       </c>
     </row>
     <row r="63">
@@ -18063,17 +18452,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C63" s="6" t="n">
-        <v>0.01</v>
+        <v>112.54</v>
       </c>
       <c r="D63" s="6" t="n">
-        <v>0.01</v>
+        <v>228.5</v>
       </c>
       <c r="E63" s="6" t="n">
-        <v>1000</v>
+        <v>2030.389194952905</v>
       </c>
     </row>
     <row r="64">
@@ -18084,17 +18473,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C64" s="6" t="n">
-        <v>273.96</v>
+        <v>0.01</v>
       </c>
       <c r="D64" s="6" t="n">
-        <v>412.03</v>
+        <v>0.01</v>
       </c>
       <c r="E64" s="6" t="n">
-        <v>1503.978683019419</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="65">
@@ -18105,17 +18494,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Slovakia</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C65" s="6" t="n">
-        <v>0</v>
+        <v>432.72</v>
       </c>
       <c r="D65" s="6" t="n">
-        <v>1.29</v>
+        <v>652.62</v>
       </c>
       <c r="E65" s="6" t="n">
-        <v>0</v>
+        <v>1508.180809761508</v>
       </c>
     </row>
     <row r="66">
@@ -18130,13 +18519,13 @@
         </is>
       </c>
       <c r="C66" s="6" t="n">
-        <v>61.92</v>
+        <v>62.77</v>
       </c>
       <c r="D66" s="6" t="n">
-        <v>127.05</v>
+        <v>131.18</v>
       </c>
       <c r="E66" s="6" t="n">
-        <v>2051.841085271318</v>
+        <v>2089.851840050979</v>
       </c>
     </row>
     <row r="67">
@@ -18147,17 +18536,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C67" s="6" t="n">
-        <v>278.34</v>
+        <v>1313.86</v>
       </c>
       <c r="D67" s="6" t="n">
-        <v>281.93</v>
+        <v>1346.46</v>
       </c>
       <c r="E67" s="6" t="n">
-        <v>1012.897894661206</v>
+        <v>1024.81238488119</v>
       </c>
     </row>
     <row r="68">
@@ -18168,38 +18557,38 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C68" s="6" t="n">
-        <v>1389.84</v>
+        <v>278.34</v>
       </c>
       <c r="D68" s="6" t="n">
-        <v>3032.35</v>
+        <v>281.93</v>
       </c>
       <c r="E68" s="6" t="n">
-        <v>2181.797904794797</v>
+        <v>1012.897894661206</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C69" s="6" t="n">
-        <v>145.18</v>
+        <v>1611.75</v>
       </c>
       <c r="D69" s="6" t="n">
-        <v>179.39</v>
+        <v>3542.18</v>
       </c>
       <c r="E69" s="6" t="n">
-        <v>1235.638517702163</v>
+        <v>2197.722971924926</v>
       </c>
     </row>
     <row r="70">
@@ -18210,17 +18599,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C70" s="6" t="n">
-        <v>1378.34</v>
+        <v>72.08</v>
       </c>
       <c r="D70" s="6" t="n">
-        <v>1751.17</v>
+        <v>104.06</v>
       </c>
       <c r="E70" s="6" t="n">
-        <v>1270.492041150949</v>
+        <v>1443.673695893452</v>
       </c>
     </row>
     <row r="71">
@@ -18231,17 +18620,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C71" s="6" t="n">
-        <v>76.91</v>
+        <v>265.87</v>
       </c>
       <c r="D71" s="6" t="n">
-        <v>229.62</v>
+        <v>328.8</v>
       </c>
       <c r="E71" s="6" t="n">
-        <v>2985.567546482902</v>
+        <v>1236.694625192763</v>
       </c>
     </row>
     <row r="72">
@@ -18252,17 +18641,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C72" s="6" t="n">
-        <v>169.23</v>
+        <v>1455.29</v>
       </c>
       <c r="D72" s="6" t="n">
-        <v>230.99</v>
+        <v>1846.57</v>
       </c>
       <c r="E72" s="6" t="n">
-        <v>1364.94711339597</v>
+        <v>1268.867373513183</v>
       </c>
     </row>
     <row r="73">
@@ -18273,17 +18662,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C73" s="6" t="n">
-        <v>93.3</v>
+        <v>88.08000000000001</v>
       </c>
       <c r="D73" s="6" t="n">
-        <v>138.03</v>
+        <v>147.89</v>
       </c>
       <c r="E73" s="6" t="n">
-        <v>1479.421221864952</v>
+        <v>1679.041780199818</v>
       </c>
     </row>
     <row r="74">
@@ -18294,80 +18683,80 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C74" s="6" t="n">
-        <v>3006.56</v>
+        <v>76.91</v>
       </c>
       <c r="D74" s="6" t="n">
-        <v>4648.9</v>
+        <v>229.62</v>
       </c>
       <c r="E74" s="6" t="n">
-        <v>1546.252195199829</v>
+        <v>2985.567546482902</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C75" s="6" t="n">
-        <v>74.12</v>
+        <v>193.25</v>
       </c>
       <c r="D75" s="6" t="n">
-        <v>65.39</v>
+        <v>263.71</v>
       </c>
       <c r="E75" s="6" t="n">
-        <v>882.2180248246087</v>
+        <v>1364.605433376456</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C76" s="6" t="n">
-        <v>99.94</v>
+        <v>93.3</v>
       </c>
       <c r="D76" s="6" t="n">
-        <v>281.04</v>
+        <v>138.03</v>
       </c>
       <c r="E76" s="6" t="n">
-        <v>2812.087252351411</v>
+        <v>1479.421221864952</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C77" s="6" t="n">
-        <v>55.54</v>
+        <v>4096.100000000001</v>
       </c>
       <c r="D77" s="6" t="n">
-        <v>81.45</v>
+        <v>6237.090000000001</v>
       </c>
       <c r="E77" s="6" t="n">
-        <v>1466.510622974433</v>
+        <v>1522.689875735455</v>
       </c>
     </row>
     <row r="78">
@@ -18378,17 +18767,17 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C78" s="6" t="n">
-        <v>4.75</v>
+        <v>74.12</v>
       </c>
       <c r="D78" s="6" t="n">
-        <v>28.52</v>
+        <v>65.39</v>
       </c>
       <c r="E78" s="6" t="n">
-        <v>6004.210526315789</v>
+        <v>882.2180248246087</v>
       </c>
     </row>
     <row r="79">
@@ -18399,17 +18788,17 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C79" s="6" t="n">
-        <v>23499.35</v>
+        <v>99.94</v>
       </c>
       <c r="D79" s="6" t="n">
-        <v>24530.11</v>
+        <v>281.04</v>
       </c>
       <c r="E79" s="6" t="n">
-        <v>1043.863340900919</v>
+        <v>2812.087252351411</v>
       </c>
     </row>
     <row r="80">
@@ -18420,17 +18809,17 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C80" s="6" t="n">
-        <v>4817.210000000001</v>
+        <v>55.54</v>
       </c>
       <c r="D80" s="6" t="n">
-        <v>8156.56</v>
+        <v>81.45</v>
       </c>
       <c r="E80" s="6" t="n">
-        <v>1693.2124611549</v>
+        <v>1466.510622974433</v>
       </c>
     </row>
     <row r="81">
@@ -18441,17 +18830,17 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C81" s="6" t="n">
-        <v>3325.159999999999</v>
+        <v>14.68</v>
       </c>
       <c r="D81" s="6" t="n">
-        <v>5062.68</v>
+        <v>69.22000000000001</v>
       </c>
       <c r="E81" s="6" t="n">
-        <v>1522.537261364867</v>
+        <v>4715.258855585833</v>
       </c>
     </row>
     <row r="82">
@@ -18462,17 +18851,17 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C82" s="6" t="n">
-        <v>2</v>
+        <v>329.64</v>
       </c>
       <c r="D82" s="6" t="n">
-        <v>3.57</v>
+        <v>359.81</v>
       </c>
       <c r="E82" s="6" t="n">
-        <v>1785</v>
+        <v>1091.52408688266</v>
       </c>
     </row>
     <row r="83">
@@ -18483,17 +18872,17 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C83" s="6" t="n">
-        <v>6088.31</v>
+        <v>28413.96</v>
       </c>
       <c r="D83" s="6" t="n">
-        <v>7011.77</v>
+        <v>29077.1</v>
       </c>
       <c r="E83" s="6" t="n">
-        <v>1151.677559125603</v>
+        <v>1023.338527963015</v>
       </c>
     </row>
     <row r="84">
@@ -18504,17 +18893,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Luxembourg</t>
         </is>
       </c>
       <c r="C84" s="6" t="n">
-        <v>0.03</v>
+        <v>6806.030000000001</v>
       </c>
       <c r="D84" s="6" t="n">
-        <v>0.18</v>
+        <v>10908.33</v>
       </c>
       <c r="E84" s="6" t="n">
-        <v>6000</v>
+        <v>1602.744918844025</v>
       </c>
     </row>
     <row r="85">
@@ -18525,17 +18914,17 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C85" s="6" t="n">
-        <v>1.52</v>
+        <v>4442.499999999999</v>
       </c>
       <c r="D85" s="6" t="n">
-        <v>12.48</v>
+        <v>6812.01</v>
       </c>
       <c r="E85" s="6" t="n">
-        <v>8210.526315789473</v>
+        <v>1533.37310073157</v>
       </c>
     </row>
     <row r="86">
@@ -18546,17 +18935,17 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C86" s="6" t="n">
-        <v>350.4399999999999</v>
+        <v>2</v>
       </c>
       <c r="D86" s="6" t="n">
-        <v>340.99</v>
+        <v>3.57</v>
       </c>
       <c r="E86" s="6" t="n">
-        <v>973.0339002396988</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="87">
@@ -18567,17 +18956,17 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C87" s="6" t="n">
-        <v>628.9299999999999</v>
+        <v>6088.349999999999</v>
       </c>
       <c r="D87" s="6" t="n">
-        <v>972.9</v>
+        <v>7011.969999999999</v>
       </c>
       <c r="E87" s="6" t="n">
-        <v>1546.913010986915</v>
+        <v>1151.702842313599</v>
       </c>
     </row>
     <row r="88">
@@ -18588,17 +18977,17 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C88" s="6" t="n">
-        <v>0.4</v>
+        <v>0.05</v>
       </c>
       <c r="D88" s="6" t="n">
-        <v>1.97</v>
+        <v>0.24</v>
       </c>
       <c r="E88" s="6" t="n">
-        <v>4925</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="89">
@@ -18609,17 +18998,17 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="C89" s="6" t="n">
-        <v>2966.21</v>
+        <v>0</v>
       </c>
       <c r="D89" s="6" t="n">
-        <v>7558.589999999999</v>
+        <v>0.23</v>
       </c>
       <c r="E89" s="6" t="n">
-        <v>2548.231581715387</v>
+        <v>0</v>
       </c>
     </row>
     <row r="90">
@@ -18630,17 +19019,101 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="C90" s="6" t="n">
+        <v>653.25</v>
+      </c>
+      <c r="D90" s="6" t="n">
+        <v>636.14</v>
+      </c>
+      <c r="E90" s="6" t="n">
+        <v>973.80788365863</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Türkiye</t>
+        </is>
+      </c>
+      <c r="C91" s="6" t="n">
+        <v>628.9399999999999</v>
+      </c>
+      <c r="D91" s="6" t="n">
+        <v>962.17</v>
+      </c>
+      <c r="E91" s="6" t="n">
+        <v>1529.827964511718</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="D92" s="6" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="E92" s="6" t="n">
+        <v>4758.620689655173</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C93" s="6" t="n">
+        <v>3599.73</v>
+      </c>
+      <c r="D93" s="6" t="n">
+        <v>9278.840000000006</v>
+      </c>
+      <c r="E93" s="6" t="n">
+        <v>2577.648879221499</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
           <t>Vietnam</t>
         </is>
       </c>
-      <c r="C90" s="6" t="n">
-        <v>446.88</v>
-      </c>
-      <c r="D90" s="6" t="n">
-        <v>374.9</v>
-      </c>
-      <c r="E90" s="6" t="n">
-        <v>838.9276763336914</v>
+      <c r="C94" s="6" t="n">
+        <v>690.49</v>
+      </c>
+      <c r="D94" s="6" t="n">
+        <v>579.4100000000001</v>
+      </c>
+      <c r="E94" s="6" t="n">
+        <v>839.1287346666861</v>
       </c>
     </row>
   </sheetData>

</xml_diff>